<commit_message>
docs(fonctionnalites): inventaire des lots Syndic S1 à S3
21 sous-fonctionnalités ajoutées (agences mandantes et identité des
documents, paiement par lot avec affectation et avance, suivi mensuel,
reçus et quittances, impression groupée) et 7 lignes mises à jour
(rattachement du mandant, bornes de période, excédent devenu avance,
appels couverts non relancés). Miroir régénéré.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -189,7 +189,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O620" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O641" headerRowCount="1">
   <autoFilter ref="A1:O620"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Domaine (regroupement agent)"/>
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O620"/>
+  <dimension ref="A1:O641"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -31179,7 +31179,7 @@
       </c>
       <c r="G396" s="2" t="inlineStr">
         <is>
-          <t>name (obligatoire), address, registrationNo, fiscalYear, syndicManagerId, cadastralReference, totalLots, totalBuildings, propertyId (optionnel)</t>
+          <t>name (obligatoire), address, registrationNo, fiscalYear, syndicManagerId, cadastralReference, totalLots, totalBuildings, propertyId (optionnel), mandatingAgencyId (optionnel, lot S1)</t>
         </is>
       </c>
       <c r="H396" s="2" t="inlineStr">
@@ -31333,7 +31333,7 @@
       </c>
       <c r="G398" s="2" t="inlineStr">
         <is>
-          <t>Au moins un champ parmi name, address, registrationNo, fiscalYear, syndicManagerId, cadastralReference, totalLots, totalBuildings, status, regulationDocUrl, propertyId</t>
+          <t>Au moins un champ parmi name, address, registrationNo, fiscalYear, syndicManagerId, cadastralReference, totalLots, totalBuildings, status, regulationDocUrl, propertyId, mandatingAgencyId (lot S1, rattachement/détachement d'un mandant)</t>
         </is>
       </c>
       <c r="H398" s="2" t="inlineStr">
@@ -33797,7 +33797,7 @@
       </c>
       <c r="G430" s="2" t="inlineStr">
         <is>
-          <t>syndicateId, period, amount, currency, dueDate, lotId ou lotIds ou applyToAllLots, isRecurring, recurrenceFrequency, recurrenceCount</t>
+          <t>syndicateId, period, amount, currency, dueDate, lotId ou lotIds ou applyToAllLots, isRecurring, recurrenceFrequency, recurrenceCount, periodStart/periodEnd (optionnels, lot S2 ; déduits du libellé quand ils manquent)</t>
         </is>
       </c>
       <c r="H430" s="2" t="inlineStr">
@@ -33946,7 +33946,7 @@
       </c>
       <c r="F432" s="2" t="inlineStr">
         <is>
-          <t>Enregistrer un paiement reçu sur un appel de charges, avec mise à jour du statut (PENDING/PARTIAL/PAID)</t>
+          <t>Enregistrer un paiement reçu sur un appel de charges désigné (route historique) : passe par le même moteur d'affectation que le paiement par lot (lot S2) — l'excédent n'est plus refusé, il s'impute sur les autres appels ouverts du lot puis reste en avance ; émet reçu et quittances (lot S3)</t>
         </is>
       </c>
       <c r="G432" s="2" t="inlineStr">
@@ -33956,12 +33956,12 @@
       </c>
       <c r="H432" s="2" t="inlineStr">
         <is>
-          <t>`ChargePayment` créé ; `ChargeCall.status` mis à jour ; crédite le compte propriétaire du lot</t>
+          <t>`ChargePayment` créé ; `allocations[]`, `advance`, `lotAdvanceBalance` ; `ChargeCall.status` mis à jour ; crédite le compte propriétaire du lot ; reçu/quittances émis</t>
         </is>
       </c>
       <c r="I432" s="2" t="inlineStr">
         <is>
-          <t>Créer un appel de charges. Le paiement ne doit pas dépasser le reste dû (sinon 422)</t>
+          <t>Créer un appel de charges</t>
         </is>
       </c>
       <c r="J432" s="2" t="inlineStr">
@@ -34105,7 +34105,7 @@
       </c>
       <c r="G434" s="2" t="inlineStr">
         <is>
-          <t>label, period, dueDate, batchType, totalAmount, currency, budgetId (optionnel)</t>
+          <t>label, period, dueDate, batchType, totalAmount, currency, budgetId (optionnel), periodStart/periodEnd (optionnels, lot S2)</t>
         </is>
       </c>
       <c r="H434" s="2" t="inlineStr">
@@ -34490,7 +34490,7 @@
       </c>
       <c r="G439" s="2" t="inlineStr">
         <is>
-          <t>label, period, dueDate, batchType, currency (optionnel)</t>
+          <t>label, period, dueDate, batchType, currency (optionnel), periodStart/periodEnd (optionnels, lot S2)</t>
         </is>
       </c>
       <c r="H439" s="2" t="inlineStr">
@@ -34793,7 +34793,7 @@
       </c>
       <c r="F443" s="2" t="inlineStr">
         <is>
-          <t>Relancer en masse tous les appels de charges en retard et non soldés (niveau incrémenté auto, plafonné à 4)</t>
+          <t>Relancer en masse tous les appels de charges en retard et non soldés (niveau incrémenté auto, plafonné à 4) ; un appel entièrement couvert (par un paiement ou par l'avance du lot, lot S2) n'est jamais relancé</t>
         </is>
       </c>
       <c r="G443" s="2" t="inlineStr">
@@ -48468,6 +48468,1623 @@
       <c r="O620" s="2" t="inlineStr">
         <is>
           <t>Assemblées (`/copropriete/assemblees`)</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>Syndic copropriete</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>Syndic, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>SYNDIC</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>Identité des documents (agences mandantes)</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>Lister les agences mandantes</t>
+        </is>
+      </c>
+      <c r="F621" t="inlineStr">
+        <is>
+          <t>Afficher les agences mandantes pour le compte de qui le cabinet gère des copropriétés</t>
+        </is>
+      </c>
+      <c r="G621" t="inlineStr">
+        <is>
+          <t>tenantId (URL)</t>
+        </is>
+      </c>
+      <c r="H621" t="inlineStr">
+        <is>
+          <t>Liste de `MandatingAgency` (coordonnées, indicateurs hasLogo/hasSignature/hasStamp)</t>
+        </is>
+      </c>
+      <c r="I621" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J621" t="inlineStr">
+        <is>
+          <t>Collaborateur (accès agence)</t>
+        </is>
+      </c>
+      <c r="K621" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L621" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/syndic-mandating-agencies</t>
+        </is>
+      </c>
+      <c r="M621" t="inlineStr">
+        <is>
+          <t>requireAnyPropertyPermission(['PROPERTIES_VIEW'])</t>
+        </is>
+      </c>
+      <c r="N621" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O621" t="inlineStr">
+        <is>
+          <t>Syndic &gt; Agences mandantes</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>Syndic copropriete</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>Syndic, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>SYNDIC</t>
+        </is>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>Identité des documents (agences mandantes)</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>Créer une agence mandante</t>
+        </is>
+      </c>
+      <c r="F622" t="inlineStr">
+        <is>
+          <t>Enregistrer un mandant (nom, coordonnées, RCCM, identifiant fiscal) dont le cabinet gère des copropriétés</t>
+        </is>
+      </c>
+      <c r="G622" t="inlineStr">
+        <is>
+          <t>name (obligatoire), legalName, address, phone, email, rccm, taxId (optionnels)</t>
+        </is>
+      </c>
+      <c r="H622" t="inlineStr">
+        <is>
+          <t>`MandatingAgency` créé</t>
+        </is>
+      </c>
+      <c r="I622" t="inlineStr">
+        <is>
+          <t>Nom unique dans l'agence, insensible à la casse (sinon 409)</t>
+        </is>
+      </c>
+      <c r="J622" t="inlineStr">
+        <is>
+          <t>Collaborateur (accès agence)</t>
+        </is>
+      </c>
+      <c r="K622" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L622" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/syndic-mandating-agencies</t>
+        </is>
+      </c>
+      <c r="M622" t="inlineStr">
+        <is>
+          <t>requireAnyPropertyPermission(['PROPERTIES_CREATE'])</t>
+        </is>
+      </c>
+      <c r="N622" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O622" t="inlineStr">
+        <is>
+          <t>Syndic &gt; Agences mandantes</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>Syndic copropriete</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>Syndic, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>SYNDIC</t>
+        </is>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>Identité des documents (agences mandantes)</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>Consulter une agence mandante</t>
+        </is>
+      </c>
+      <c r="F623" t="inlineStr">
+        <is>
+          <t>Détail d'un mandant</t>
+        </is>
+      </c>
+      <c r="G623" t="inlineStr">
+        <is>
+          <t>agencyId (URL)</t>
+        </is>
+      </c>
+      <c r="H623" t="inlineStr">
+        <is>
+          <t>`MandatingAgency`</t>
+        </is>
+      </c>
+      <c r="I623" t="inlineStr">
+        <is>
+          <t>Créer une agence mandante</t>
+        </is>
+      </c>
+      <c r="J623" t="inlineStr">
+        <is>
+          <t>Collaborateur (accès agence)</t>
+        </is>
+      </c>
+      <c r="K623" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L623" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/syndic-mandating-agencies/:agencyId</t>
+        </is>
+      </c>
+      <c r="M623" t="inlineStr">
+        <is>
+          <t>requireAnyPropertyPermission(['PROPERTIES_VIEW'])</t>
+        </is>
+      </c>
+      <c r="N623" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O623" t="inlineStr">
+        <is>
+          <t>Syndic &gt; Agences mandantes</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>Syndic copropriete</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>Syndic, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>SYNDIC</t>
+        </is>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>Identité des documents (agences mandantes)</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>Modifier une agence mandante</t>
+        </is>
+      </c>
+      <c r="F624" t="inlineStr">
+        <is>
+          <t>Mettre à jour les coordonnées d'un mandant</t>
+        </is>
+      </c>
+      <c r="G624" t="inlineStr">
+        <is>
+          <t>Au moins un champ parmi name, legalName, address, phone, email, rccm, taxId</t>
+        </is>
+      </c>
+      <c r="H624" t="inlineStr">
+        <is>
+          <t>`MandatingAgency` mis à jour</t>
+        </is>
+      </c>
+      <c r="I624" t="inlineStr">
+        <is>
+          <t>Créer une agence mandante. Nom unique dans l'agence si modifié (sinon 409)</t>
+        </is>
+      </c>
+      <c r="J624" t="inlineStr">
+        <is>
+          <t>Collaborateur (accès agence)</t>
+        </is>
+      </c>
+      <c r="K624" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L624" t="inlineStr">
+        <is>
+          <t>PATCH /tenants/:tenantId/syndic-mandating-agencies/:agencyId</t>
+        </is>
+      </c>
+      <c r="M624" t="inlineStr">
+        <is>
+          <t>requirePropertyPermission('PROPERTIES_EDIT')</t>
+        </is>
+      </c>
+      <c r="N624" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O624" t="inlineStr">
+        <is>
+          <t>Syndic &gt; Agences mandantes</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>Syndic copropriete</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>Syndic, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>SYNDIC</t>
+        </is>
+      </c>
+      <c r="D625" t="inlineStr">
+        <is>
+          <t>Identité des documents (agences mandantes)</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>Supprimer une agence mandante</t>
+        </is>
+      </c>
+      <c r="F625" t="inlineStr">
+        <is>
+          <t>Retirer un mandant qui ne rend plus service au cabinet</t>
+        </is>
+      </c>
+      <c r="G625" t="inlineStr">
+        <is>
+          <t>agencyId (URL)</t>
+        </is>
+      </c>
+      <c r="H625" t="inlineStr">
+        <is>
+          <t>Confirmation ; `MandatingAgency` supprimé, ses images (logo, signature, cachet) effacées du disque</t>
+        </is>
+      </c>
+      <c r="I625" t="inlineStr">
+        <is>
+          <t>Créer une agence mandante. Aucune copropriété rattachée (sinon 409, à détacher avant suppression)</t>
+        </is>
+      </c>
+      <c r="J625" t="inlineStr">
+        <is>
+          <t>Collaborateur (accès agence)</t>
+        </is>
+      </c>
+      <c r="K625" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L625" t="inlineStr">
+        <is>
+          <t>DELETE /tenants/:tenantId/syndic-mandating-agencies/:agencyId</t>
+        </is>
+      </c>
+      <c r="M625" t="inlineStr">
+        <is>
+          <t>requirePropertyPermission('PROPERTIES_EDIT')</t>
+        </is>
+      </c>
+      <c r="N625" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O625" t="inlineStr">
+        <is>
+          <t>Syndic &gt; Agences mandantes</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>Syndic copropriete</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>Syndic, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>SYNDIC</t>
+        </is>
+      </c>
+      <c r="D626" t="inlineStr">
+        <is>
+          <t>Identité des documents (agences mandantes)</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>Gérer le logo d'un mandant</t>
+        </is>
+      </c>
+      <c r="F626" t="inlineStr">
+        <is>
+          <t>Déposer, remplacer ou supprimer le logo du mandant, apposé sur les documents des copropriétés qu'il mandate</t>
+        </is>
+      </c>
+      <c r="G626" t="inlineStr">
+        <is>
+          <t>Fichier image (PNG/JPG, type vérifié par octets magiques, taille bornée) en PUT ; aucun corps en DELETE</t>
+        </is>
+      </c>
+      <c r="H626" t="inlineStr">
+        <is>
+          <t>`{hasLogo, logoUrl}` mis à jour ; image privée, jamais servie en statique</t>
+        </is>
+      </c>
+      <c r="I626" t="inlineStr">
+        <is>
+          <t>Créer une agence mandante</t>
+        </is>
+      </c>
+      <c r="J626" t="inlineStr">
+        <is>
+          <t>Collaborateur (accès agence)</t>
+        </is>
+      </c>
+      <c r="K626" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L626" t="inlineStr">
+        <is>
+          <t>GET/PUT/DELETE /tenants/:tenantId/syndic-mandating-agencies/:agencyId/images/logo</t>
+        </is>
+      </c>
+      <c r="M626" t="inlineStr">
+        <is>
+          <t>requireAnyPropertyPermission(['PROPERTIES_VIEW']) (GET) / requirePropertyPermission('PROPERTIES_EDIT') (PUT, DELETE)</t>
+        </is>
+      </c>
+      <c r="N626" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O626" t="inlineStr">
+        <is>
+          <t>Syndic &gt; Agences mandantes</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>Syndic copropriete</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>Syndic, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>SYNDIC</t>
+        </is>
+      </c>
+      <c r="D627" t="inlineStr">
+        <is>
+          <t>Identité des documents (agences mandantes)</t>
+        </is>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>Gérer la signature et le cachet d'un mandant</t>
+        </is>
+      </c>
+      <c r="F627" t="inlineStr">
+        <is>
+          <t>Déposer, remplacer ou supprimer la signature et le cachet du mandant, apposés sur les documents des copropriétés qu'il mandate</t>
+        </is>
+      </c>
+      <c r="G627" t="inlineStr">
+        <is>
+          <t>`:kind` = signature ou stamp (URL) ; fichier image en PUT, aucun corps en DELETE</t>
+        </is>
+      </c>
+      <c r="H627" t="inlineStr">
+        <is>
+          <t>`{hasSignature/hasStamp, ...Url}` mis à jour</t>
+        </is>
+      </c>
+      <c r="I627" t="inlineStr">
+        <is>
+          <t>Créer une agence mandante</t>
+        </is>
+      </c>
+      <c r="J627" t="inlineStr">
+        <is>
+          <t>Collaborateur (accès agence)</t>
+        </is>
+      </c>
+      <c r="K627" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L627" t="inlineStr">
+        <is>
+          <t>GET/PUT/DELETE /tenants/:tenantId/syndic-mandating-agencies/:agencyId/images/:kind</t>
+        </is>
+      </c>
+      <c r="M627" t="inlineStr">
+        <is>
+          <t>requireAnyPropertyPermission(['PROPERTIES_VIEW']) (GET) / requirePermission('TENANT_SETTINGS_EDIT') (PUT, DELETE) — écriture plus restrictive que le reste de la fiche (audit sécurité S1)</t>
+        </is>
+      </c>
+      <c r="N627" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O627" t="inlineStr">
+        <is>
+          <t>Syndic &gt; Agences mandantes</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>Syndic copropriete</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>Syndic, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>SYNDIC</t>
+        </is>
+      </c>
+      <c r="D628" t="inlineStr">
+        <is>
+          <t>Identité des documents (copropriété)</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>Gérer le logo d'une copropriété</t>
+        </is>
+      </c>
+      <c r="F628" t="inlineStr">
+        <is>
+          <t>Déposer, remplacer ou supprimer le logo propre à la copropriété, affiché en complément du logo du mandant (ou de l'agence) sur ses documents</t>
+        </is>
+      </c>
+      <c r="G628" t="inlineStr">
+        <is>
+          <t>Fichier image (PNG/JPG, borné) en PUT ; aucun corps en DELETE</t>
+        </is>
+      </c>
+      <c r="H628" t="inlineStr">
+        <is>
+          <t>`{hasLogo, logoUrl}` mis à jour</t>
+        </is>
+      </c>
+      <c r="I628" t="inlineStr">
+        <is>
+          <t>Créer une copropriété</t>
+        </is>
+      </c>
+      <c r="J628" t="inlineStr">
+        <is>
+          <t>Collaborateur (accès agence)</t>
+        </is>
+      </c>
+      <c r="K628" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L628" t="inlineStr">
+        <is>
+          <t>GET/PUT/DELETE /tenants/:tenantId/syndics/:syndicId/logo</t>
+        </is>
+      </c>
+      <c r="M628" t="inlineStr">
+        <is>
+          <t>requireAnyPropertyPermission(['PROPERTIES_VIEW']) (GET) / requirePropertyPermission('PROPERTIES_EDIT') (PUT, DELETE)</t>
+        </is>
+      </c>
+      <c r="N628" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O628" t="inlineStr">
+        <is>
+          <t>Syndic &gt; Copropriété &gt; Fiche</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>Syndic copropriete</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="D629" t="inlineStr">
+        <is>
+          <t>Identité des documents (agence)</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>Consulter la signature et le cachet de l'agence pour ses documents</t>
+        </is>
+      </c>
+      <c r="F629" t="inlineStr">
+        <is>
+          <t>Afficher si l'agence a déjà une signature/un cachet pour ses documents (utilisés quand une copropriété n'a pas de mandant)</t>
+        </is>
+      </c>
+      <c r="G629" t="inlineStr">
+        <is>
+          <t>tenantId (URL)</t>
+        </is>
+      </c>
+      <c r="H629" t="inlineStr">
+        <is>
+          <t>`{hasSignature, hasStamp, signatureUrl, stampUrl}`</t>
+        </is>
+      </c>
+      <c r="I629" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J629" t="inlineStr">
+        <is>
+          <t>Collaborateur (accès agence)</t>
+        </is>
+      </c>
+      <c r="K629" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L629" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/document-identity</t>
+        </is>
+      </c>
+      <c r="M629" t="inlineStr">
+        <is>
+          <t>requirePermission('TENANT_SETTINGS_VIEW')</t>
+        </is>
+      </c>
+      <c r="N629" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O629" t="inlineStr">
+        <is>
+          <t>Agence &gt; Paramètres de l'agence</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>Syndic copropriete</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>Identité des documents (agence)</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>Gérer la signature et le cachet de l'agence pour ses documents</t>
+        </is>
+      </c>
+      <c r="F630" t="inlineStr">
+        <is>
+          <t>Déposer, remplacer ou supprimer la signature et le cachet apposés sur les documents de l'agence (relevés, PV d'AG, reçus et quittances) quand une copropriété n'a pas de mandant</t>
+        </is>
+      </c>
+      <c r="G630" t="inlineStr">
+        <is>
+          <t>`:kind` = signature ou stamp (URL) ; fichier image en PUT</t>
+        </is>
+      </c>
+      <c r="H630" t="inlineStr">
+        <is>
+          <t>`{hasSignature/hasStamp, ...Url}` mis à jour</t>
+        </is>
+      </c>
+      <c r="I630" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J630" t="inlineStr">
+        <is>
+          <t>Collaborateur avec TENANT_SETTINGS_EDIT (typiquement TENANT_ADMIN)</t>
+        </is>
+      </c>
+      <c r="K630" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L630" t="inlineStr">
+        <is>
+          <t>GET/PUT/DELETE /tenants/:tenantId/document-identity/images/:kind</t>
+        </is>
+      </c>
+      <c r="M630" t="inlineStr">
+        <is>
+          <t>requirePermission('TENANT_SETTINGS_VIEW') (GET) / requirePermission('TENANT_SETTINGS_EDIT') (PUT, DELETE)</t>
+        </is>
+      </c>
+      <c r="N630" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O630" t="inlineStr">
+        <is>
+          <t>Agence &gt; Paramètres de l'agence</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>Syndic copropriete</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>Syndic, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>SYNDIC</t>
+        </is>
+      </c>
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>Finances</t>
+        </is>
+      </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>Enregistrer un paiement de lot avec affectation</t>
+        </is>
+      </c>
+      <c r="F631" t="inlineStr">
+        <is>
+          <t>Enregistrer un paiement reçu d'un lot : affecte le montant aux appels cochés, sinon du plus ancien au plus récent ; l'excédent devient une avance du lot ; émet le reçu puis la quittance de chaque appel soldé (lot S3)</t>
+        </is>
+      </c>
+      <c r="G631" t="inlineStr">
+        <is>
+          <t>lotId (URL) ; amount, paidAt, method, reference (optionnel), chargeCallIds (optionnel, mois cochés)</t>
+        </is>
+      </c>
+      <c r="H631" t="inlineStr">
+        <is>
+          <t>`LotPaymentResult` (paiement, `allocations[]` par appel, `advance`, `lotAdvanceBalance`) ; documents de recouvrement émis (voir S3)</t>
+        </is>
+      </c>
+      <c r="I631" t="inlineStr">
+        <is>
+          <t>Créer une copropriété et le lot</t>
+        </is>
+      </c>
+      <c r="J631" t="inlineStr">
+        <is>
+          <t>Collaborateur (accès agence)</t>
+        </is>
+      </c>
+      <c r="K631" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L631" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/syndics/:syndicId/lots/:lotId/paiements</t>
+        </is>
+      </c>
+      <c r="M631" t="inlineStr">
+        <is>
+          <t>requirePropertyPermission('PROPERTIES_EDIT')</t>
+        </is>
+      </c>
+      <c r="N631" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O631" t="inlineStr">
+        <is>
+          <t>Syndic &gt; Finances &gt; Appels de charges</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>Syndic copropriete</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>Syndic, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>SYNDIC</t>
+        </is>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>Finances</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>Prévisualiser l'affectation d'un paiement de lot</t>
+        </is>
+      </c>
+      <c r="F632" t="inlineStr">
+        <is>
+          <t>Simuler l'affectation d'un paiement avant de l'enregistrer (même moteur que l'enregistrement, sans écriture)</t>
+        </is>
+      </c>
+      <c r="G632" t="inlineStr">
+        <is>
+          <t>lotId (URL) ; amount, paidAt, method, reference (optionnel), chargeCallIds (optionnel)</t>
+        </is>
+      </c>
+      <c r="H632" t="inlineStr">
+        <is>
+          <t>`LotPaymentResult` prévisionnel (aucune écriture, `payment.id` null)</t>
+        </is>
+      </c>
+      <c r="I632" t="inlineStr">
+        <is>
+          <t>Créer une copropriété et le lot</t>
+        </is>
+      </c>
+      <c r="J632" t="inlineStr">
+        <is>
+          <t>Collaborateur (accès agence)</t>
+        </is>
+      </c>
+      <c r="K632" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L632" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/syndics/:syndicId/lots/:lotId/paiements/apercu</t>
+        </is>
+      </c>
+      <c r="M632" t="inlineStr">
+        <is>
+          <t>requirePropertyPermission('PROPERTIES_EDIT')</t>
+        </is>
+      </c>
+      <c r="N632" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O632" t="inlineStr">
+        <is>
+          <t>Syndic &gt; Finances &gt; Appels de charges</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>Syndic copropriete</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>Syndic, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>SYNDIC</t>
+        </is>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>Finances</t>
+        </is>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>Consulter l'avance d'un lot</t>
+        </is>
+      </c>
+      <c r="F633" t="inlineStr">
+        <is>
+          <t>Afficher le crédit non affecté d'un lot (excédent de paiements passés), imputé automatiquement sur chaque nouvel appel</t>
+        </is>
+      </c>
+      <c r="G633" t="inlineStr">
+        <is>
+          <t>lotId (URL)</t>
+        </is>
+      </c>
+      <c r="H633" t="inlineStr">
+        <is>
+          <t>`{advance, currency}`</t>
+        </is>
+      </c>
+      <c r="I633" t="inlineStr">
+        <is>
+          <t>Créer une copropriété et le lot</t>
+        </is>
+      </c>
+      <c r="J633" t="inlineStr">
+        <is>
+          <t>Collaborateur (accès agence)</t>
+        </is>
+      </c>
+      <c r="K633" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L633" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/syndics/:syndicId/lots/:lotId/avance</t>
+        </is>
+      </c>
+      <c r="M633" t="inlineStr">
+        <is>
+          <t>requireAnyPropertyPermission(['PROPERTIES_VIEW'])</t>
+        </is>
+      </c>
+      <c r="N633" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O633" t="inlineStr">
+        <is>
+          <t>Syndic &gt; Finances &gt; Appels de charges</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>Syndic copropriete</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>Syndic, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>SYNDIC</t>
+        </is>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>Finances</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>Lister les appels ouverts d'un lot</t>
+        </is>
+      </c>
+      <c r="F634" t="inlineStr">
+        <is>
+          <t>Afficher les appels de charges non soldés du lot, pour cocher les mois à couvrir lors d'un paiement</t>
+        </is>
+      </c>
+      <c r="G634" t="inlineStr">
+        <is>
+          <t>lotId (URL)</t>
+        </is>
+      </c>
+      <c r="H634" t="inlineStr">
+        <is>
+          <t>Liste d'appels ouverts (période, bornes, échéance, montant, payé, reste dû, devise, statut recalculé)</t>
+        </is>
+      </c>
+      <c r="I634" t="inlineStr">
+        <is>
+          <t>Créer une copropriété et le lot</t>
+        </is>
+      </c>
+      <c r="J634" t="inlineStr">
+        <is>
+          <t>Collaborateur (accès agence)</t>
+        </is>
+      </c>
+      <c r="K634" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L634" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/syndics/:syndicId/lots/:lotId/appels-ouverts</t>
+        </is>
+      </c>
+      <c r="M634" t="inlineStr">
+        <is>
+          <t>requireAnyPropertyPermission(['PROPERTIES_VIEW'])</t>
+        </is>
+      </c>
+      <c r="N634" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O634" t="inlineStr">
+        <is>
+          <t>Syndic &gt; Finances &gt; Appels de charges</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>Syndic copropriete</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>Syndic, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>SYNDIC</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>Finances</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>Consulter le suivi mensuel d'une copropriété</t>
+        </is>
+      </c>
+      <c r="F635" t="inlineStr">
+        <is>
+          <t>Grille lot × mois d'un exercice : statut de chaque mois (réglé, partiel, dû, en retard) et avance de chaque lot</t>
+        </is>
+      </c>
+      <c r="G635" t="inlineStr">
+        <is>
+          <t>syndicId (URL) ; year (query, année civile par défaut)</t>
+        </is>
+      </c>
+      <c r="H635" t="inlineStr">
+        <is>
+          <t>`{year, currency, months[1..12], lots[{lotId, lotNumber, ownerName, advance, months[]}]}`</t>
+        </is>
+      </c>
+      <c r="I635" t="inlineStr">
+        <is>
+          <t>Créer une copropriété</t>
+        </is>
+      </c>
+      <c r="J635" t="inlineStr">
+        <is>
+          <t>Collaborateur (accès agence)</t>
+        </is>
+      </c>
+      <c r="K635" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L635" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/syndics/:syndicId/suivi-mensuel</t>
+        </is>
+      </c>
+      <c r="M635" t="inlineStr">
+        <is>
+          <t>requireAnyPropertyPermission(['PROPERTIES_VIEW'])</t>
+        </is>
+      </c>
+      <c r="N635" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O635" t="inlineStr">
+        <is>
+          <t>Syndic &gt; Finances &gt; Suivi mensuel</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>Syndic copropriete</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>Syndic, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>SYNDIC</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>Finances</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>Lister les quittances et reçus d'une copropriété</t>
+        </is>
+      </c>
+      <c r="F636" t="inlineStr">
+        <is>
+          <t>Afficher l'historique des reçus de paiement et quittances de charges de la copropriété, filtrable et paginé</t>
+        </is>
+      </c>
+      <c r="G636" t="inlineStr">
+        <is>
+          <t>syndicId (URL) ; lotId, contactId, kind (RECEIPT/QUITTANCE), from, to, page, limit (optionnels)</t>
+        </is>
+      </c>
+      <c r="H636" t="inlineStr">
+        <is>
+          <t>Page de `SyndicChargeReceipt` (numéro, période, montant, dates d'émission/envoi, erreur d'e-mail éventuelle)</t>
+        </is>
+      </c>
+      <c r="I636" t="inlineStr">
+        <is>
+          <t>Créer une copropriété</t>
+        </is>
+      </c>
+      <c r="J636" t="inlineStr">
+        <is>
+          <t>Collaborateur (accès agence)</t>
+        </is>
+      </c>
+      <c r="K636" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L636" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/syndics/:syndicId/quittances</t>
+        </is>
+      </c>
+      <c r="M636" t="inlineStr">
+        <is>
+          <t>requireAnyPropertyPermission(['PROPERTIES_VIEW'])</t>
+        </is>
+      </c>
+      <c r="N636" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O636" t="inlineStr">
+        <is>
+          <t>Syndic &gt; Finances &gt; Quittances</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>Syndic copropriete</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>Syndic, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>SYNDIC</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>Finances</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>Lister les quittances et reçus d'un lot</t>
+        </is>
+      </c>
+      <c r="F637" t="inlineStr">
+        <is>
+          <t>Afficher l'historique des reçus et quittances d'un lot précis</t>
+        </is>
+      </c>
+      <c r="G637" t="inlineStr">
+        <is>
+          <t>lotId (URL) ; lotId, contactId, kind, from, to, page, limit (optionnels)</t>
+        </is>
+      </c>
+      <c r="H637" t="inlineStr">
+        <is>
+          <t>Page de `SyndicChargeReceipt` du lot</t>
+        </is>
+      </c>
+      <c r="I637" t="inlineStr">
+        <is>
+          <t>Créer une copropriété et le lot</t>
+        </is>
+      </c>
+      <c r="J637" t="inlineStr">
+        <is>
+          <t>Collaborateur (accès agence)</t>
+        </is>
+      </c>
+      <c r="K637" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L637" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/syndics/:syndicId/lots/:lotId/quittances</t>
+        </is>
+      </c>
+      <c r="M637" t="inlineStr">
+        <is>
+          <t>requireAnyPropertyPermission(['PROPERTIES_VIEW'])</t>
+        </is>
+      </c>
+      <c r="N637" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O637" t="inlineStr">
+        <is>
+          <t>Syndic &gt; Copropriété (section compte du lot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>Syndic copropriete</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>Syndic, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>SYNDIC</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>Finances</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>Télécharger un reçu ou une quittance</t>
+        </is>
+      </c>
+      <c r="F638" t="inlineStr">
+        <is>
+          <t>Récupérer le PDF d'un reçu de paiement ou d'une quittance déjà émise</t>
+        </is>
+      </c>
+      <c r="G638" t="inlineStr">
+        <is>
+          <t>receiptId (URL)</t>
+        </is>
+      </c>
+      <c r="H638" t="inlineStr">
+        <is>
+          <t>Fichier PDF (fichier privé, servi par route authentifiée, jamais en statique)</t>
+        </is>
+      </c>
+      <c r="I638" t="inlineStr">
+        <is>
+          <t>Un reçu ou une quittance émis (paiement ou rattrapage)</t>
+        </is>
+      </c>
+      <c r="J638" t="inlineStr">
+        <is>
+          <t>Collaborateur (accès agence)</t>
+        </is>
+      </c>
+      <c r="K638" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L638" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/syndics/:syndicId/quittances/:receiptId/fichier</t>
+        </is>
+      </c>
+      <c r="M638" t="inlineStr">
+        <is>
+          <t>requireAnyPropertyPermission(['PROPERTIES_VIEW'])</t>
+        </is>
+      </c>
+      <c r="N638" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O638" t="inlineStr">
+        <is>
+          <t>Syndic &gt; Finances &gt; Quittances</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>Syndic copropriete</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>Syndic, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>SYNDIC</t>
+        </is>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>Finances</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>Renvoyer une quittance ou un reçu par e-mail</t>
+        </is>
+      </c>
+      <c r="F639" t="inlineStr">
+        <is>
+          <t>Renvoyer le PDF d'un reçu ou d'une quittance au copropriétaire, sur le modèle CHARGE_PAYMENT_RECEIPT ou CHARGE_CALL_SETTLED</t>
+        </is>
+      </c>
+      <c r="G639" t="inlineStr">
+        <is>
+          <t>receiptId (URL)</t>
+        </is>
+      </c>
+      <c r="H639" t="inlineStr">
+        <is>
+          <t>Confirmation d'envoi ; `emailedAt` / `emailErrorCode` mis à jour</t>
+        </is>
+      </c>
+      <c r="I639" t="inlineStr">
+        <is>
+          <t>Un reçu ou une quittance émis. Limité par utilisateur et agence (receiptResendRateLimiter)</t>
+        </is>
+      </c>
+      <c r="J639" t="inlineStr">
+        <is>
+          <t>Collaborateur (accès agence)</t>
+        </is>
+      </c>
+      <c r="K639" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L639" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/syndics/:syndicId/quittances/:receiptId/envoi</t>
+        </is>
+      </c>
+      <c r="M639" t="inlineStr">
+        <is>
+          <t>requirePropertyPermission('PROPERTIES_EDIT')</t>
+        </is>
+      </c>
+      <c r="N639" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O639" t="inlineStr">
+        <is>
+          <t>Syndic &gt; Finances &gt; Quittances</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>Syndic copropriete</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>Syndic, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>SYNDIC</t>
+        </is>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>Finances</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>Imprimer les quittances en grille</t>
+        </is>
+      </c>
+      <c r="F640" t="inlineStr">
+        <is>
+          <t>Composer un PDF imprimable A4 de plusieurs quittances (ou reçus, ou les deux) d'une période, pour tous les copropriétaires ou un seul, en grille 1×1 à 3×4 par feuille</t>
+        </is>
+      </c>
+      <c r="G640" t="inlineStr">
+        <is>
+          <t>from, to (obligatoires) ; kind (QUITTANCE/RECEIPT/ALL, défaut QUITTANCE), lotId, contactId (optionnels), cols (1-3), rows (1-4)</t>
+        </is>
+      </c>
+      <c r="H640" t="inlineStr">
+        <is>
+          <t>Fichier PDF (une grille par feuille, texte adapté à la cellule, traits de coupe)</t>
+        </is>
+      </c>
+      <c r="I640" t="inlineStr">
+        <is>
+          <t>Des quittances ou reçus émis sur la période. Limité par utilisateur et agence (receiptPrintRateLimiter)</t>
+        </is>
+      </c>
+      <c r="J640" t="inlineStr">
+        <is>
+          <t>Collaborateur (accès agence)</t>
+        </is>
+      </c>
+      <c r="K640" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L640" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/syndics/:syndicId/quittances/impression</t>
+        </is>
+      </c>
+      <c r="M640" t="inlineStr">
+        <is>
+          <t>requireAnyPropertyPermission(['PROPERTIES_VIEW'])</t>
+        </is>
+      </c>
+      <c r="N640" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O640" t="inlineStr">
+        <is>
+          <t>Syndic &gt; Finances &gt; Quittances</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>Syndic copropriete</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>Syndic, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>SYNDIC</t>
+        </is>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>Finances</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>Générer les quittances manquantes</t>
+        </is>
+      </c>
+      <c r="F641" t="inlineStr">
+        <is>
+          <t>Rattrapage : émet une quittance pour chaque appel de charges déjà soldé (PAID) qui n'en a pas encore, sans jamais régénérer un original existant</t>
+        </is>
+      </c>
+      <c r="G641" t="inlineStr">
+        <is>
+          <t>syndicId (URL)</t>
+        </is>
+      </c>
+      <c r="H641" t="inlineStr">
+        <is>
+          <t>`{created, skipped, remaining}` (borné par lot, en plusieurs appels si beaucoup d'appels restent à traiter)</t>
+        </is>
+      </c>
+      <c r="I641" t="inlineStr">
+        <is>
+          <t>Créer une copropriété. Pas de quittance rétroactive pour les paiements historiques non tracés par appel</t>
+        </is>
+      </c>
+      <c r="J641" t="inlineStr">
+        <is>
+          <t>Collaborateur (accès agence)</t>
+        </is>
+      </c>
+      <c r="K641" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L641" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/syndics/:syndicId/quittances/generer-manquantes</t>
+        </is>
+      </c>
+      <c r="M641" t="inlineStr">
+        <is>
+          <t>requirePropertyPermission('PROPERTIES_EDIT')</t>
+        </is>
+      </c>
+      <c r="N641" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O641" t="inlineStr">
+        <is>
+          <t>Syndic &gt; Finances &gt; Quittances</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(patrimoine): alerte quotidienne d'expiration des pièces du bien et relevés en asyncHandler
- alertExpiringDocuments porte sur PropertyDocument (et non plus
  PatrimonyDocument, abandonné au lot P0) : documents qui expirent dans les
  30 jours, e-mail aux propriétaires du bien (indivision comprise) reliés à
  un contact CRM avec consentement e-mail ; HTML échappé, sujet brut.
- Anti-doublon par warningSentAt, réservé atomiquement avant l'envoi et
  retiré si aucun envoi n'aboutit ; un document sans destinataire éligible
  n'est pas marqué et reste retenté.
- Tâche planifiée quotidienne (7 h UTC) : agences actives une par une, dans
  leur contexte d'agence ; une agence en échec n'arrête pas les suivantes.
- owner-statements-controller : asyncHandler et erreurs typées à la place
  des try/catch qui devinaient le statut ; tests 400, 404 et 409.
- Wiki : ligne « Alerter les propriétaires d'un document qui arrive à
  échéance ».

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -189,7 +189,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O661" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O662" headerRowCount="1">
   <autoFilter ref="A1:O661"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Domaine (regroupement agent)"/>
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O661"/>
+  <dimension ref="A1:O662"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -51625,6 +51625,83 @@
       <c r="O661" s="2" t="inlineStr">
         <is>
           <t>Syndic &gt; Budgets (bouton « Postes et fonds »)</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>Documents patrimoniaux</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>Alerter les propriétaires d'un document qui arrive à échéance</t>
+        </is>
+      </c>
+      <c r="F662" t="inlineStr">
+        <is>
+          <t>Tâche quotidienne (7 h UTC), agence par agence dans son contexte : chaque document de bien (`PropertyDocument`) dont la date d'expiration tombe dans les 30 prochains jours déclenche un e-mail aux propriétaires du bien (indivision comprise), une seule fois par document (`warningSentAt`) ; un document sans destinataire éligible est retenté le lendemain</t>
+        </is>
+      </c>
+      <c r="G662" t="inlineStr">
+        <is>
+          <t>Aucune (tâche planifiée `document-expiry-alert-job`) ; lit `expirationDate` des documents du bien</t>
+        </is>
+      </c>
+      <c r="H662" t="inlineStr">
+        <is>
+          <t>E-mail « Document patrimoine expirant » (gabarit `DOCUMENT_EXPIRY_ALERT`, personnalisable) ; `warningSentAt` posé sur le document</t>
+        </is>
+      </c>
+      <c r="I662" t="inlineStr">
+        <is>
+          <t>Ajouter un document patrimonial (avec date d'expiration) ; propriétaire relié à un contact CRM (`details.crmContactId`) ayant une adresse e-mail et le consentement e-mail ; notification `DOCUMENT_EXPIRY_ALERT` activée</t>
+        </is>
+      </c>
+      <c r="J662" t="inlineStr">
+        <is>
+          <t>Système (tâche planifiée)</t>
+        </is>
+      </c>
+      <c r="K662" t="inlineStr">
+        <is>
+          <t>— (job serveur)</t>
+        </is>
+      </c>
+      <c r="L662" t="inlineStr">
+        <is>
+          <t>N/A — job cron interne (`packages/api/src/jobs/document-expiry-alert-job.ts`), pas de route API</t>
+        </is>
+      </c>
+      <c r="M662" t="inlineStr">
+        <is>
+          <t>Aucune (exécution serveur, hors requête HTTP)</t>
+        </is>
+      </c>
+      <c r="N662" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O662" t="inlineStr">
+        <is>
+          <t>Aucun (technique)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(patrimoine): exports PDF/Excel du patrimoine par agence et par bien
Ajoute la route d'export authentifiee (PDF et Excel) protegee par la
permission PROPERTIES_VIEW et l'isolation tenant, le bouton d'export sur
les pages patrimoine, et les tests associes (controleur, generation PDF,
generation classeur, devises).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -189,7 +189,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O661" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O663" headerRowCount="1">
   <autoFilter ref="A1:O661"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Domaine (regroupement agent)"/>
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O661"/>
+  <dimension ref="A1:O663"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -51625,6 +51625,160 @@
       <c r="O661" s="2" t="inlineStr">
         <is>
           <t>Syndic &gt; Budgets (bouton « Postes et fonds »)</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>Exports du patrimoine</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>Exporter le patrimoine de l'agence (PDF ou Excel)</t>
+        </is>
+      </c>
+      <c r="F662" t="inlineStr">
+        <is>
+          <t>Télécharger une synthèse PDF (vue consolidée, performance par bien : rendements brut/net/net-net, plus-value latente, puis une section par bien) ou un classeur Excel (synthèse, biens, valorisations, emprunts, dépenses, travaux, documents avec échéances) pour tous les biens de l'agence hors brouillon, vendu et archivé</t>
+        </is>
+      </c>
+      <c r="G662" t="inlineStr">
+        <is>
+          <t>Query `format` = `pdf` ou `xlsx` (obligatoire)</t>
+        </is>
+      </c>
+      <c r="H662" t="inlineStr">
+        <is>
+          <t>Fichier en pièce jointe (`Content-Disposition: attachment`, `Cache-Control: no-store`), généré en mémoire, jamais servi en statique ; PDF en français si l'interface est en arabe (police sans glyphes arabes), Excel dans la langue de l'interface ; au-delà de 500 biens → 400</t>
+        </is>
+      </c>
+      <c r="I662" t="inlineStr">
+        <is>
+          <t>Consulter la vue consolidée</t>
+        </is>
+      </c>
+      <c r="J662" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K662" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L662" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/patrimoine/export</t>
+        </is>
+      </c>
+      <c r="M662" t="inlineStr">
+        <is>
+          <t>PROPERTIES_VIEW (`requireAnyPropertyPermission`)</t>
+        </is>
+      </c>
+      <c r="N662" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O662" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Vue consolidée &gt; bouton Exporter</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>Exports du patrimoine</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>Exporter le patrimoine d'un bien (PDF ou Excel)</t>
+        </is>
+      </c>
+      <c r="F663" t="inlineStr">
+        <is>
+          <t>Télécharger la synthèse PDF ou le classeur Excel du patrimoine d'un seul bien (mêmes contenus que l'export d'agence, limités au bien)</t>
+        </is>
+      </c>
+      <c r="G663" t="inlineStr">
+        <is>
+          <t>Param `propertyId`, query `format` = `pdf` ou `xlsx` (obligatoire)</t>
+        </is>
+      </c>
+      <c r="H663" t="inlineStr">
+        <is>
+          <t>Fichier en pièce jointe `patrimoine-&lt;référence du bien&gt;-&lt;date&gt;.pdf|xlsx`, généré en mémoire, jamais servi en statique</t>
+        </is>
+      </c>
+      <c r="I663" t="inlineStr">
+        <is>
+          <t>Le bien doit appartenir au tenant (sinon 404, comme un bien inexistant)</t>
+        </is>
+      </c>
+      <c r="J663" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K663" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L663" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/properties/:propertyId/patrimoine/export</t>
+        </is>
+      </c>
+      <c r="M663" t="inlineStr">
+        <is>
+          <t>PROPERTIES_VIEW (`requireAnyPropertyPermission`)</t>
+        </is>
+      </c>
+      <c r="N663" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O663" t="inlineStr">
+        <is>
+          <t>Biens &gt; fiche bien &gt; onglet Patrimoine &gt; bouton Exporter</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(patrimoine): alertes d'echeance etendues (bail, emprunt, travaux) et wiki
Etend le job quotidien d'alerte patrimoine (PR #40) : en plus des documents
arrivant a expiration (assurance comprise, deja couvert sans filtre sur le
type), alerte desormais les proprietaires des baux actifs dont la fin
approche, et l'agence (administrateurs actifs, repli sur l'e-mail de contact)
des emprunts actifs et des programmes de travaux planifies dont l'echeance
approche. Anti-doublon via AuditLog (nouvelles cles PATRIMOINE_*_ALERT_SENT)
en l'absence de colonne dediee sur ces modeles, documente dans le code.

Met a jour le classeur des fonctionnalites (export patrimoine PDF/Excel deja
livre, alertes etendues) et regenere son miroir texte.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -189,7 +189,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O662" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O667" headerRowCount="1">
   <autoFilter ref="A1:O661"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Domaine (regroupement agent)"/>
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O662"/>
+  <dimension ref="A1:O667"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -51700,6 +51700,391 @@
         </is>
       </c>
       <c r="O662" t="inlineStr">
+        <is>
+          <t>Aucun (technique)</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>Export du patrimoine</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>Exporter le patrimoine de toute l'agence (PDF ou Excel)</t>
+        </is>
+      </c>
+      <c r="F663" t="inlineStr">
+        <is>
+          <t>Telecharger, en un fichier, une synthese (PDF) ou un classeur detaille (Excel) du patrimoine de l'agence : biens hors DRAFT/SOLD/ARCHIVED, valorisations, emprunts, depenses, travaux, documents et rendement par bien</t>
+        </is>
+      </c>
+      <c r="G663" t="inlineStr">
+        <is>
+          <t>Query `format` (obligatoire, `pdf` ou `xlsx`)</t>
+        </is>
+      </c>
+      <c r="H663" t="inlineStr">
+        <is>
+          <t>Fichier PDF ou XLSX en piece jointe (`Content-Disposition: attachment`), genere en memoire, jamais ecrit sur disque</t>
+        </is>
+      </c>
+      <c r="I663" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J663" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K663" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L663" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/patrimoine/export</t>
+        </is>
+      </c>
+      <c r="M663" t="inlineStr">
+        <is>
+          <t>PROPERTIES_VIEW (`requireAnyPropertyPermission`)</t>
+        </is>
+      </c>
+      <c r="N663" t="inlineStr">
+        <is>
+          <t>Disponible (borne a 500 biens — `MAX_EXPORT_PROPERTIES` — au-dela, exporter par bien)</t>
+        </is>
+      </c>
+      <c r="O663" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Vue consolidée (bouton Exporter)</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>Export du patrimoine</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>Exporter le patrimoine d'un bien (PDF ou Excel)</t>
+        </is>
+      </c>
+      <c r="F664" t="inlineStr">
+        <is>
+          <t>Telecharger la synthese (PDF) ou le classeur detaille (Excel) patrimoine d'un seul bien</t>
+        </is>
+      </c>
+      <c r="G664" t="inlineStr">
+        <is>
+          <t>Query `format` (obligatoire, `pdf` ou `xlsx`)</t>
+        </is>
+      </c>
+      <c r="H664" t="inlineStr">
+        <is>
+          <t>Fichier PDF ou XLSX en piece jointe, nomme d'apres la reference interne du bien</t>
+        </is>
+      </c>
+      <c r="I664" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J664" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K664" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L664" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/properties/:propertyId/patrimoine/export</t>
+        </is>
+      </c>
+      <c r="M664" t="inlineStr">
+        <is>
+          <t>PROPERTIES_VIEW (`requireAnyPropertyPermission`)</t>
+        </is>
+      </c>
+      <c r="N664" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O664" t="inlineStr">
+        <is>
+          <t>Biens &gt; fiche bien &gt; onglet Patrimoine (bouton Exporter)</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>Alertes d'échéance patrimoine</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>Alerter les propriétaires d'un bail qui arrive à échéance</t>
+        </is>
+      </c>
+      <c r="F665" t="inlineStr">
+        <is>
+          <t>Prevenir par e-mail le(s) proprietaire(s) d'un bien qu'un bail actif de ce bien se termine dans les 30 prochains jours, pour anticiper le renouvellement ou la recherche d'un nouveau locataire</t>
+        </is>
+      </c>
+      <c r="G665" t="inlineStr">
+        <is>
+          <t>Aucune (tache planifiee `document-expiry-alert-job`) ; lit `RentalLease.end_date` des baux actifs</t>
+        </is>
+      </c>
+      <c r="H665" t="inlineStr">
+        <is>
+          <t>E-mail « Fin de bail prochaine » (gabarit `LEASE_ENDING_SOON`, personnalisable) ; entree `AuditLog` (`PATRIMOINE_LEASE_END_ALERT_SENT`) posee comme marque anti-doublon</t>
+        </is>
+      </c>
+      <c r="I665" t="inlineStr">
+        <is>
+          <t>Créer un bail ; proprietaire relie a un contact CRM (`details.crmContactId`) ayant une adresse e-mail et le consentement e-mail ; notification `LEASE_ENDING_SOON` activee</t>
+        </is>
+      </c>
+      <c r="J665" t="inlineStr">
+        <is>
+          <t>Système (tâche planifiée)</t>
+        </is>
+      </c>
+      <c r="K665" t="inlineStr">
+        <is>
+          <t>— (job serveur)</t>
+        </is>
+      </c>
+      <c r="L665" t="inlineStr">
+        <is>
+          <t>N/A — job cron interne (`packages/api/src/jobs/document-expiry-alert-job.ts`), pas de route API</t>
+        </is>
+      </c>
+      <c r="M665" t="inlineStr">
+        <is>
+          <t>Aucune (exécution serveur, hors requête HTTP)</t>
+        </is>
+      </c>
+      <c r="N665" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O665" t="inlineStr">
+        <is>
+          <t>Aucun (technique)</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>Alertes d'échéance patrimoine</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>Alerter l'agence d'un emprunt qui arrive à échéance</t>
+        </is>
+      </c>
+      <c r="F666" t="inlineStr">
+        <is>
+          <t>Prevenir par e-mail les administrateurs actifs de l'agence (repli sur l'e-mail de contact de l'agence si aucun) qu'un emprunt actif lie a un bien arrive a echeance dans les 30 prochains jours</t>
+        </is>
+      </c>
+      <c r="G666" t="inlineStr">
+        <is>
+          <t>Aucune (tache planifiee) ; lit `PropertyLoan.endDate` des emprunts au statut `ACTIVE`</t>
+        </is>
+      </c>
+      <c r="H666" t="inlineStr">
+        <is>
+          <t>E-mail « Alerte fin de prêt » (gabarit `LOAN_MATURITY_ALERT`, personnalisable) ; entree `AuditLog` (`PATRIMOINE_LOAN_MATURITY_ALERT_SENT`) posee comme marque anti-doublon</t>
+        </is>
+      </c>
+      <c r="I666" t="inlineStr">
+        <is>
+          <t>Ajouter un emprunt ; notification `LOAN_MATURITY_ALERT` activee</t>
+        </is>
+      </c>
+      <c r="J666" t="inlineStr">
+        <is>
+          <t>Système (tâche planifiée)</t>
+        </is>
+      </c>
+      <c r="K666" t="inlineStr">
+        <is>
+          <t>— (job serveur)</t>
+        </is>
+      </c>
+      <c r="L666" t="inlineStr">
+        <is>
+          <t>N/A — job cron interne (`packages/api/src/jobs/document-expiry-alert-job.ts`), pas de route API</t>
+        </is>
+      </c>
+      <c r="M666" t="inlineStr">
+        <is>
+          <t>Aucune (exécution serveur, hors requête HTTP)</t>
+        </is>
+      </c>
+      <c r="N666" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O666" t="inlineStr">
+        <is>
+          <t>Aucun (technique)</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>Alertes d'échéance patrimoine</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>Alerter l'agence d'un programme de travaux planifié qui approche</t>
+        </is>
+      </c>
+      <c r="F667" t="inlineStr">
+        <is>
+          <t>Prevenir par e-mail les administrateurs actifs de l'agence qu'un programme de travaux au statut `PLANNED` a une date prevue dans les 30 prochains jours</t>
+        </is>
+      </c>
+      <c r="G667" t="inlineStr">
+        <is>
+          <t>Aucune (tache planifiee) ; lit `WorkProgram.plannedDate` des programmes `PLANNED`</t>
+        </is>
+      </c>
+      <c r="H667" t="inlineStr">
+        <is>
+          <t>E-mail « Rappel programme de travaux » (gabarit `WORK_PROGRAM_REMINDER`, personnalisable) ; entree `AuditLog` (`PATRIMOINE_WORK_UPCOMING_ALERT_SENT`) posee comme marque anti-doublon</t>
+        </is>
+      </c>
+      <c r="I667" t="inlineStr">
+        <is>
+          <t>Ajouter un programme de travaux ; notification `WORK_PROGRAM_REMINDER` activee</t>
+        </is>
+      </c>
+      <c r="J667" t="inlineStr">
+        <is>
+          <t>Système (tâche planifiée)</t>
+        </is>
+      </c>
+      <c r="K667" t="inlineStr">
+        <is>
+          <t>— (job serveur)</t>
+        </is>
+      </c>
+      <c r="L667" t="inlineStr">
+        <is>
+          <t>N/A — job cron interne (`packages/api/src/jobs/document-expiry-alert-job.ts`), pas de route API</t>
+        </is>
+      </c>
+      <c r="M667" t="inlineStr">
+        <is>
+          <t>Aucune (exécution serveur, hors requête HTTP)</t>
+        </is>
+      </c>
+      <c r="N667" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O667" t="inlineStr">
         <is>
           <t>Aucun (technique)</t>
         </is>

</xml_diff>

<commit_message>
chore(i18n,wiki): libellés traduits et inventaire des fonctionnalités à jour
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -189,7 +189,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O662" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O663" headerRowCount="1">
   <autoFilter ref="A1:O661"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Domaine (regroupement agent)"/>
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O662"/>
+  <dimension ref="A1:O663"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -32759,7 +32759,7 @@
       </c>
       <c r="O416" s="2" t="inlineStr">
         <is>
-          <t>Syndic &gt; Copropriété</t>
+          <t>Syndic &gt; Copropriété &gt; Profils et incidents (bouton « Modifier l'incident » et colonne Prestataire)</t>
         </is>
       </c>
     </row>
@@ -34249,12 +34249,12 @@
       </c>
       <c r="E436" s="2" t="inlineStr">
         <is>
-          <t>Voter / approuver un budget (changement de statut)</t>
+          <t>Approuver, réviser ou clôturer un budget (changement de statut)</t>
         </is>
       </c>
       <c r="F436" s="2" t="inlineStr">
         <is>
-          <t>Faire évoluer le statut (DRAFT → APPROVED → REVISED/CLOSED), en le liant en option à la résolution d'AG qui l'a voté</t>
+          <t>Faire évoluer le statut selon des transitions contrôlées : Brouillon → Approuvé ; Approuvé ↔ Révisé ; Approuvé ou Révisé → Clôturé (définitif). La clôture affiche d'abord le budgété, le réalisé et l'écart ; un budget clôturé n'est plus modifiable (libellé, montant, répartition, fonds des postes, génération d'appels)</t>
         </is>
       </c>
       <c r="G436" s="2" t="inlineStr">
@@ -34264,7 +34264,7 @@
       </c>
       <c r="H436" s="2" t="inlineStr">
         <is>
-          <t>`SyndicateBudget` mis à jour (approvedAt daté si APPROVED)</t>
+          <t>`SyndicateBudget` mis à jour (approvedAt daté si APPROVED) ; 409 si la transition est interdite, si le budget est clôturé ou si une programmation d'appels active et non terminée l'utilise encore</t>
         </is>
       </c>
       <c r="I436" s="2" t="inlineStr">
@@ -34299,7 +34299,7 @@
       </c>
       <c r="O436" s="2" t="inlineStr">
         <is>
-          <t>Syndic &gt; Finances</t>
+          <t>Syndic &gt; Finances &gt; Budgets (boutons Approuver, Réviser, Clôturer)</t>
         </is>
       </c>
     </row>
@@ -36646,7 +36646,7 @@
       </c>
       <c r="G467" s="2" t="inlineStr">
         <is>
-          <t>type, scheduledAt, startTime, endTime, location, resolutions[] (titre, description, règle de majorité optionnels)</t>
+          <t>type, date + heure de début (obligatoires, combinées en scheduledAt), heure de fin optionnelle, location, resolutions[] (titre, description, règle de majorité optionnels)</t>
         </is>
       </c>
       <c r="H467" s="2" t="inlineStr">
@@ -49741,7 +49741,7 @@
       </c>
       <c r="H637" t="inlineStr">
         <is>
-          <t>Fichier PDF (fichier privé, servi par route authentifiée, jamais en statique)</t>
+          <t>Fichier PDF (fichier privé, servi par route authentifiée, jamais en statique). Côté écran : délai de 120 s pour un téléchargement, message d'échec qualifié (délai, connexion, document introuvable, erreur serveur)</t>
         </is>
       </c>
       <c r="I637" t="inlineStr">
@@ -51050,7 +51050,7 @@
       </c>
       <c r="H654" t="inlineStr">
         <is>
-          <t>`{run, schedule}` : statut SUCCESS/FAILED/SKIPPED, appels créés, appels couverts par une avance, notifications envoyées et non envoyées</t>
+          <t>`{run, schedule}` : statut SUCCESS/FAILED/SKIPPED, appels créés, appels couverts par une avance, avis envoyés et non envoyés avec leur raison affichée en clair (pas de copropriétaire, copropriétaire changé, pas d'e-mail, notification désactivée, envoi d'e-mails non configuré, échec de l'envoi) ; date d'envoi de l'avis notée sur chaque appel</t>
         </is>
       </c>
       <c r="I654" t="inlineStr">
@@ -51112,32 +51112,32 @@
       </c>
       <c r="E655" t="inlineStr">
         <is>
-          <t>Émettre automatiquement les appels de charges programmés</t>
+          <t>Renvoyer les avis non envoyés d'une exécution de programmation</t>
         </is>
       </c>
       <c r="F655" t="inlineStr">
         <is>
-          <t>Tâche quotidienne (6 h UTC) : chaque programmation active dont la date d'émission est arrivée émet sa période comme « Exécuter maintenant » ; rattrape dans l'ordre les périodes manquées (12 au plus par programmation et par passage) ; un échec est consigné sans arrêter les autres</t>
+          <t>Après correction de la cause (e-mail du copropriétaire, réglage de notification…), renvoyer l'avis d'appel PDF aux seuls appels de l'exécution encore dus dont l'avis n'est jamais parti</t>
         </is>
       </c>
       <c r="G655" t="inlineStr">
         <is>
-          <t>Aucune (tâche planifiée `syndic-charge-call-scheduler`)</t>
+          <t>scheduleId, runId (URL)</t>
         </is>
       </c>
       <c r="H655" t="inlineStr">
         <is>
-          <t>Exécutions `SyndicChargeScheduleRun` (déclencheur CRON), appels de charges, quittances et avis d'appel envoyés</t>
+          <t>Résumé : avis envoyés, avis toujours non envoyés et leurs raisons ; compteurs et notes de l'exécution mis à jour. 409 si rien à renvoyer ou si un renvoi a eu lieu il y a moins d'une minute</t>
         </is>
       </c>
       <c r="I655" t="inlineStr">
         <is>
-          <t>Créer une programmation d'appels de charges (active)</t>
+          <t>Exécuter maintenant une programmation d'appels de charges (ou exécution automatique)</t>
         </is>
       </c>
       <c r="J655" t="inlineStr">
         <is>
-          <t>Système (tâche planifiée)</t>
+          <t>Collaborateur (accès agence)</t>
         </is>
       </c>
       <c r="K655" t="inlineStr">
@@ -51147,12 +51147,12 @@
       </c>
       <c r="L655" t="inlineStr">
         <is>
-          <t>— (tâche node-cron, pas de route)</t>
+          <t>POST /tenants/:tenantId/syndics/:syndicId/programmations/:scheduleId/executions/:runId/renvoyer-avis</t>
         </is>
       </c>
       <c r="M655" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>requirePropertyPermission('PROPERTIES_EDIT')</t>
         </is>
       </c>
       <c r="N655" t="inlineStr">
@@ -51162,7 +51162,7 @@
       </c>
       <c r="O655" t="inlineStr">
         <is>
-          <t>Syndic &gt; Finances &gt; Programmation</t>
+          <t>Syndic &gt; Finances &gt; Programmation (bouton « Renvoyer les avis non envoyés »)</t>
         </is>
       </c>
     </row>
@@ -51189,32 +51189,32 @@
       </c>
       <c r="E656" t="inlineStr">
         <is>
-          <t>Consulter l'historique d'exécution d'une programmation</t>
+          <t>Émettre automatiquement les appels de charges programmés</t>
         </is>
       </c>
       <c r="F656" t="inlineStr">
         <is>
-          <t>Afficher les exécutions d'une programmation (automatiques ou manuelles) avec leur résultat et l'erreur éventuelle</t>
+          <t>Tâche quotidienne (6 h UTC) : chaque programmation active dont la date d'émission est arrivée émet sa période comme « Exécuter maintenant » ; rattrape dans l'ordre les périodes manquées (12 au plus par programmation et par passage) ; un échec est consigné sans arrêter les autres</t>
         </is>
       </c>
       <c r="G656" t="inlineStr">
         <is>
-          <t>scheduleId (URL) ; limit (1-100, défaut 50)</t>
+          <t>Aucune (tâche planifiée `syndic-charge-call-scheduler`)</t>
         </is>
       </c>
       <c r="H656" t="inlineStr">
         <is>
-          <t>Liste de `SyndicChargeScheduleRun` (période, statut, déclencheur, lot d'appels, appels créés/couverts, notifications envoyées/non envoyées, remarque, erreur)</t>
+          <t>Exécutions `SyndicChargeScheduleRun` (déclencheur CRON), appels de charges, quittances et avis d'appel envoyés</t>
         </is>
       </c>
       <c r="I656" t="inlineStr">
         <is>
-          <t>Créer une programmation d'appels de charges</t>
+          <t>Créer une programmation d'appels de charges (active)</t>
         </is>
       </c>
       <c r="J656" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Système (tâche planifiée)</t>
         </is>
       </c>
       <c r="K656" t="inlineStr">
@@ -51224,12 +51224,12 @@
       </c>
       <c r="L656" t="inlineStr">
         <is>
-          <t>GET /tenants/:tenantId/syndics/:syndicId/programmations/:scheduleId/executions</t>
+          <t>— (tâche node-cron, pas de route)</t>
         </is>
       </c>
       <c r="M656" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission(['PROPERTIES_VIEW'])</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N656" t="inlineStr">
@@ -51266,22 +51266,22 @@
       </c>
       <c r="E657" t="inlineStr">
         <is>
-          <t>Prévisualiser les prochaines périodes d'une programmation</t>
+          <t>Consulter l'historique d'exécution d'une programmation</t>
         </is>
       </c>
       <c r="F657" t="inlineStr">
         <is>
-          <t>Afficher les 3 prochaines périodes à émettre avec leurs dates (émission, échéance) et montants, total et par lot, sans rien écrire ; un budget non approuvé ou sans répartition donne une erreur sur la période</t>
+          <t>Afficher les exécutions d'une programmation (automatiques ou manuelles) avec leur résultat et l'erreur éventuelle</t>
         </is>
       </c>
       <c r="G657" t="inlineStr">
         <is>
-          <t>scheduleId (URL)</t>
+          <t>scheduleId (URL) ; limit (1-100, défaut 50)</t>
         </is>
       </c>
       <c r="H657" t="inlineStr">
         <is>
-          <t>`{scheduleId, active, periods[{label, periodStart, periodEnd, issueDate, dueDate, totalAmount, currency, budgetId, lots[], error}]}`</t>
+          <t>Liste de `SyndicChargeScheduleRun` (période, statut, déclencheur, lot d'appels, appels créés/couverts, notifications envoyées/non envoyées, remarque, erreur)</t>
         </is>
       </c>
       <c r="I657" t="inlineStr">
@@ -51301,7 +51301,7 @@
       </c>
       <c r="L657" t="inlineStr">
         <is>
-          <t>GET /tenants/:tenantId/syndics/:syndicId/programmations/:scheduleId/apercu</t>
+          <t>GET /tenants/:tenantId/syndics/:syndicId/programmations/:scheduleId/executions</t>
         </is>
       </c>
       <c r="M657" t="inlineStr">
@@ -51343,27 +51343,27 @@
       </c>
       <c r="E658" t="inlineStr">
         <is>
-          <t>Télécharger l'avis d'appel de charges (PDF)</t>
+          <t>Prévisualiser les prochaines périodes d'une programmation</t>
         </is>
       </c>
       <c r="F658" t="inlineStr">
         <is>
-          <t>Récupérer l'avis d'appel PDF d'un appel de charges (montant, avance imputée, reste à payer, échéance), le même que celui joint à l'e-mail du copropriétaire</t>
+          <t>Afficher les 3 prochaines périodes à émettre avec leurs dates (émission, échéance) et montants, total et par lot, sans rien écrire ; un budget non approuvé ou sans répartition donne une erreur sur la période</t>
         </is>
       </c>
       <c r="G658" t="inlineStr">
         <is>
-          <t>chargeId (URL)</t>
+          <t>scheduleId (URL)</t>
         </is>
       </c>
       <c r="H658" t="inlineStr">
         <is>
-          <t>Fichier PDF (fichier privé, servi par route authentifiée)</t>
+          <t>`{scheduleId, active, periods[{label, periodStart, periodEnd, issueDate, dueDate, totalAmount, currency, budgetId, lots[], error}]}`</t>
         </is>
       </c>
       <c r="I658" t="inlineStr">
         <is>
-          <t>Créer un appel de charges</t>
+          <t>Créer une programmation d'appels de charges</t>
         </is>
       </c>
       <c r="J658" t="inlineStr">
@@ -51378,7 +51378,7 @@
       </c>
       <c r="L658" t="inlineStr">
         <is>
-          <t>GET /tenants/:tenantId/syndics/:syndicId/charges/:chargeId/avis</t>
+          <t>GET /tenants/:tenantId/syndics/:syndicId/programmations/:scheduleId/apercu</t>
         </is>
       </c>
       <c r="M658" t="inlineStr">
@@ -51393,161 +51393,161 @@
       </c>
       <c r="O658" t="inlineStr">
         <is>
-          <t>Syndic &gt; Finances &gt; Appels de charges</t>
+          <t>Syndic &gt; Finances &gt; Programmation</t>
         </is>
       </c>
     </row>
     <row r="659">
       <c r="A659" t="inlineStr">
         <is>
+          <t>Syndic copropriete</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>Syndic, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>SYNDIC</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>Finances</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>Télécharger l'avis d'appel de charges (PDF)</t>
+        </is>
+      </c>
+      <c r="F659" t="inlineStr">
+        <is>
+          <t>Récupérer l'avis d'appel PDF d'un appel de charges (montant, avance imputée, reste à payer, échéance), le même que celui joint à l'e-mail du copropriétaire</t>
+        </is>
+      </c>
+      <c r="G659" t="inlineStr">
+        <is>
+          <t>chargeId (URL)</t>
+        </is>
+      </c>
+      <c r="H659" t="inlineStr">
+        <is>
+          <t>Fichier PDF (fichier privé, servi par route authentifiée)</t>
+        </is>
+      </c>
+      <c r="I659" t="inlineStr">
+        <is>
+          <t>Créer un appel de charges</t>
+        </is>
+      </c>
+      <c r="J659" t="inlineStr">
+        <is>
+          <t>Collaborateur (accès agence)</t>
+        </is>
+      </c>
+      <c r="K659" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L659" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/syndics/:syndicId/charges/:chargeId/avis</t>
+        </is>
+      </c>
+      <c r="M659" t="inlineStr">
+        <is>
+          <t>requireAnyPropertyPermission(['PROPERTIES_VIEW'])</t>
+        </is>
+      </c>
+      <c r="N659" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O659" t="inlineStr">
+        <is>
+          <t>Syndic &gt; Finances &gt; Appels de charges</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
           <t>Portails externes</t>
         </is>
       </c>
-      <c r="B659" t="inlineStr">
+      <c r="B660" t="inlineStr">
         <is>
           <t>Syndic, Opérateur intégré</t>
         </is>
       </c>
-      <c r="C659" t="inlineStr">
+      <c r="C660" t="inlineStr">
         <is>
           <t>MODULE_SYNDIC (SYNDIC)</t>
         </is>
       </c>
-      <c r="D659" t="inlineStr">
+      <c r="D660" t="inlineStr">
         <is>
           <t>Portail Copropriétaire</t>
         </is>
       </c>
-      <c r="E659" t="inlineStr">
+      <c r="E660" t="inlineStr">
         <is>
           <t>Télécharger l'avis d'appel de charges (portail copropriétaire)</t>
         </is>
       </c>
-      <c r="F659" t="inlineStr">
+      <c r="F660" t="inlineStr">
         <is>
           <t>Récupérer l'avis d'appel PDF d'un appel de charges de ses lots, depuis la liste de ses appels</t>
         </is>
       </c>
-      <c r="G659" t="inlineStr">
+      <c r="G660" t="inlineStr">
         <is>
           <t>Param `chargeId` (UUID)</t>
         </is>
       </c>
-      <c r="H659" t="inlineStr">
+      <c r="H660" t="inlineStr">
         <is>
           <t>Fichier PDF ; 404 si l'appel est hors du périmètre du copropriétaire ou antérieur à l'acquisition du lot (`ownedSince`), même réponse qu'un appel inexistant</t>
         </is>
       </c>
-      <c r="I659" t="inlineStr">
+      <c r="I660" t="inlineStr">
         <is>
           <t>Consulter mes appels de charges</t>
         </is>
       </c>
-      <c r="J659" t="inlineStr">
+      <c r="J660" t="inlineStr">
         <is>
           <t>Copropriétaire, uniquement pour les appels de ses lots depuis leur acquisition (`ownedSince`) ; 20 téléchargements par minute (coOwnerChargeNoticeRateLimiter)</t>
         </is>
       </c>
-      <c r="K659" t="inlineStr">
+      <c r="K660" t="inlineStr">
         <is>
           <t>Copropriétaire</t>
         </is>
       </c>
-      <c r="L659" t="inlineStr">
+      <c r="L660" t="inlineStr">
         <is>
           <t>GET /api/portal/copropriete/appels/:chargeId/avis</t>
         </is>
       </c>
-      <c r="M659" t="inlineStr">
+      <c r="M660" t="inlineStr">
         <is>
           <t>authenticate + requireCoOwnerPortalAccess</t>
         </is>
       </c>
-      <c r="N659" t="inlineStr">
-        <is>
-          <t>Disponible</t>
-        </is>
-      </c>
-      <c r="O659" t="inlineStr">
+      <c r="N660" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O660" t="inlineStr">
         <is>
           <t>Appels de charges (`/copropriete/appels`) → bouton « Avis d'appel (PDF) »</t>
-        </is>
-      </c>
-    </row>
-    <row r="660">
-      <c r="A660" s="2" t="inlineStr">
-        <is>
-          <t>Syndic copropriete</t>
-        </is>
-      </c>
-      <c r="B660" s="2" t="inlineStr">
-        <is>
-          <t>Syndic, Opérateur intégré</t>
-        </is>
-      </c>
-      <c r="C660" s="2" t="inlineStr">
-        <is>
-          <t>SYNDIC</t>
-        </is>
-      </c>
-      <c r="D660" s="2" t="inlineStr">
-        <is>
-          <t>Finances</t>
-        </is>
-      </c>
-      <c r="E660" s="2" t="inlineStr">
-        <is>
-          <t>Affecter un appel de charges à un fonds</t>
-        </is>
-      </c>
-      <c r="F660" s="2" t="inlineStr">
-        <is>
-          <t>Désigner le fonds qui recevra en entier ce qui sera payé ensuite sur un appel (appel de fonds travaux), ou retirer l'affectation ; les paiements déjà reçus ne sont pas repris</t>
-        </is>
-      </c>
-      <c r="G660" s="2" t="inlineStr">
-        <is>
-          <t>chargeId (URL) ; fundId (UUID ou null) — corps strict</t>
-        </is>
-      </c>
-      <c r="H660" s="2" t="inlineStr">
-        <is>
-          <t>`{ id, fundId }` ; évènement d'audit SYNDICATE_FUND_ASSIGNMENT_CHANGED</t>
-        </is>
-      </c>
-      <c r="I660" s="2" t="inlineStr">
-        <is>
-          <t>Créer un appel de charges ; Créer un fonds (même copropriété, même devise, sinon 404 / 422)</t>
-        </is>
-      </c>
-      <c r="J660" s="2" t="inlineStr">
-        <is>
-          <t>Collaborateur (accès agence)</t>
-        </is>
-      </c>
-      <c r="K660" s="2" t="inlineStr">
-        <is>
-          <t>Agence</t>
-        </is>
-      </c>
-      <c r="L660" s="2" t="inlineStr">
-        <is>
-          <t>PATCH /tenants/:tenantId/syndics/:syndicId/charges/:chargeId/fonds</t>
-        </is>
-      </c>
-      <c r="M660" s="2" t="inlineStr">
-        <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
-        </is>
-      </c>
-      <c r="N660" s="2" t="inlineStr">
-        <is>
-          <t>Disponible</t>
-        </is>
-      </c>
-      <c r="O660" s="2" t="inlineStr">
-        <is>
-          <t>Syndic &gt; Finances &gt; Appels de charges (action « Affecter à un fonds »)</t>
         </is>
       </c>
     </row>
@@ -51574,132 +51574,209 @@
       </c>
       <c r="E661" s="2" t="inlineStr">
         <is>
+          <t>Affecter un appel de charges à un fonds</t>
+        </is>
+      </c>
+      <c r="F661" s="2" t="inlineStr">
+        <is>
+          <t>Désigner le fonds qui recevra en entier ce qui sera payé ensuite sur un appel (appel de fonds travaux), ou retirer l'affectation ; les paiements déjà reçus ne sont pas repris</t>
+        </is>
+      </c>
+      <c r="G661" s="2" t="inlineStr">
+        <is>
+          <t>chargeId (URL) ; fundId (UUID ou null) — corps strict</t>
+        </is>
+      </c>
+      <c r="H661" s="2" t="inlineStr">
+        <is>
+          <t>`{ id, fundId }` ; évènement d'audit SYNDICATE_FUND_ASSIGNMENT_CHANGED</t>
+        </is>
+      </c>
+      <c r="I661" s="2" t="inlineStr">
+        <is>
+          <t>Créer un appel de charges ; Créer un fonds (même copropriété, même devise, sinon 404 / 422)</t>
+        </is>
+      </c>
+      <c r="J661" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur (accès agence)</t>
+        </is>
+      </c>
+      <c r="K661" s="2" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L661" s="2" t="inlineStr">
+        <is>
+          <t>PATCH /tenants/:tenantId/syndics/:syndicId/charges/:chargeId/fonds</t>
+        </is>
+      </c>
+      <c r="M661" s="2" t="inlineStr">
+        <is>
+          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+        </is>
+      </c>
+      <c r="N661" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O661" s="2" t="inlineStr">
+        <is>
+          <t>Syndic &gt; Finances &gt; Appels de charges (action « Affecter à un fonds »)</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" s="2" t="inlineStr">
+        <is>
+          <t>Syndic copropriete</t>
+        </is>
+      </c>
+      <c r="B662" s="2" t="inlineStr">
+        <is>
+          <t>Syndic, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C662" s="2" t="inlineStr">
+        <is>
+          <t>SYNDIC</t>
+        </is>
+      </c>
+      <c r="D662" s="2" t="inlineStr">
+        <is>
+          <t>Finances</t>
+        </is>
+      </c>
+      <c r="E662" s="2" t="inlineStr">
+        <is>
           <t>Affecter un poste de budget à un fonds</t>
         </is>
       </c>
-      <c r="F661" s="2" t="inlineStr">
+      <c r="F662" s="2" t="inlineStr">
         <is>
           <t>Désigner le fonds alimenté par un poste du budget : il recevra la part de ce poste dans chaque paiement de charges enregistré ensuite, au prorata de la répartition du lot ; ou retirer l'affectation</t>
         </is>
       </c>
-      <c r="G661" s="2" t="inlineStr">
+      <c r="G662" s="2" t="inlineStr">
         <is>
           <t>budgetId, lineId (URL) ; fundId (UUID ou null) — corps strict</t>
         </is>
       </c>
-      <c r="H661" s="2" t="inlineStr">
+      <c r="H662" s="2" t="inlineStr">
         <is>
           <t>`{ id, fundId }` ; évènement d'audit SYNDICATE_FUND_ASSIGNMENT_CHANGED</t>
         </is>
       </c>
-      <c r="I661" s="2" t="inlineStr">
+      <c r="I662" s="2" t="inlineStr">
         <is>
           <t>Créer un budget ; Créer un fonds (même copropriété, devise du budget, sinon 404 / 422)</t>
         </is>
       </c>
-      <c r="J661" s="2" t="inlineStr">
+      <c r="J662" s="2" t="inlineStr">
         <is>
           <t>Collaborateur (accès agence)</t>
         </is>
       </c>
-      <c r="K661" s="2" t="inlineStr">
+      <c r="K662" s="2" t="inlineStr">
         <is>
           <t>Agence</t>
         </is>
       </c>
-      <c r="L661" s="2" t="inlineStr">
+      <c r="L662" s="2" t="inlineStr">
         <is>
           <t>PATCH /tenants/:tenantId/syndics/:syndicId/budgets/:budgetId/lignes/:lineId/fonds</t>
         </is>
       </c>
-      <c r="M661" s="2" t="inlineStr">
+      <c r="M662" s="2" t="inlineStr">
         <is>
           <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
         </is>
       </c>
-      <c r="N661" s="2" t="inlineStr">
-        <is>
-          <t>Disponible</t>
-        </is>
-      </c>
-      <c r="O661" s="2" t="inlineStr">
+      <c r="N662" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O662" s="2" t="inlineStr">
         <is>
           <t>Syndic &gt; Budgets (bouton « Postes et fonds »)</t>
         </is>
       </c>
     </row>
-    <row r="662">
-      <c r="A662" t="inlineStr">
+    <row r="663">
+      <c r="A663" t="inlineStr">
         <is>
           <t>Parc immobilier</t>
         </is>
       </c>
-      <c r="B662" t="inlineStr">
+      <c r="B663" t="inlineStr">
         <is>
           <t>Agence, Promoteur, Opérateur intégré</t>
         </is>
       </c>
-      <c r="C662" t="inlineStr">
+      <c r="C663" t="inlineStr">
         <is>
           <t>PATRIMOINE</t>
         </is>
       </c>
-      <c r="D662" t="inlineStr">
+      <c r="D663" t="inlineStr">
         <is>
           <t>Documents patrimoniaux</t>
         </is>
       </c>
-      <c r="E662" t="inlineStr">
+      <c r="E663" t="inlineStr">
         <is>
           <t>Alerter les propriétaires d'un document qui arrive à échéance</t>
         </is>
       </c>
-      <c r="F662" t="inlineStr">
+      <c r="F663" t="inlineStr">
         <is>
           <t>Tâche quotidienne (7 h UTC), agence par agence dans son contexte : chaque document de bien (`PropertyDocument`) dont la date d'expiration tombe dans les 30 prochains jours déclenche un e-mail aux propriétaires du bien (indivision comprise), une seule fois par document (`warningSentAt`) ; un document sans destinataire éligible est retenté le lendemain</t>
         </is>
       </c>
-      <c r="G662" t="inlineStr">
+      <c r="G663" t="inlineStr">
         <is>
           <t>Aucune (tâche planifiée `document-expiry-alert-job`) ; lit `expirationDate` des documents du bien</t>
         </is>
       </c>
-      <c r="H662" t="inlineStr">
+      <c r="H663" t="inlineStr">
         <is>
           <t>E-mail « Document patrimoine expirant » (gabarit `DOCUMENT_EXPIRY_ALERT`, personnalisable) ; `warningSentAt` posé sur le document</t>
         </is>
       </c>
-      <c r="I662" t="inlineStr">
+      <c r="I663" t="inlineStr">
         <is>
           <t>Ajouter un document patrimonial (avec date d'expiration) ; propriétaire relié à un contact CRM (`details.crmContactId`) ayant une adresse e-mail et le consentement e-mail ; notification `DOCUMENT_EXPIRY_ALERT` activée</t>
         </is>
       </c>
-      <c r="J662" t="inlineStr">
+      <c r="J663" t="inlineStr">
         <is>
           <t>Système (tâche planifiée)</t>
         </is>
       </c>
-      <c r="K662" t="inlineStr">
+      <c r="K663" t="inlineStr">
         <is>
           <t>— (job serveur)</t>
         </is>
       </c>
-      <c r="L662" t="inlineStr">
+      <c r="L663" t="inlineStr">
         <is>
           <t>N/A — job cron interne (`packages/api/src/jobs/document-expiry-alert-job.ts`), pas de route API</t>
         </is>
       </c>
-      <c r="M662" t="inlineStr">
+      <c r="M663" t="inlineStr">
         <is>
           <t>Aucune (exécution serveur, hors requête HTTP)</t>
         </is>
       </c>
-      <c r="N662" t="inlineStr">
-        <is>
-          <t>Disponible</t>
-        </is>
-      </c>
-      <c r="O662" t="inlineStr">
+      <c r="N663" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O663" t="inlineStr">
         <is>
           <t>Aucun (technique)</t>
         </is>

</xml_diff>

<commit_message>
docs(copilot): wiki, sécurité, runbook, spec 022, ADR-004 et passation
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NipnEzc6N8uvDDXG2M7jms
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sous-fonctionnalites" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legende Packs-Modules" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes et points ouverts" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sous-fonctionnalites" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Legende Packs-Modules" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Notes et points ouverts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -189,8 +189,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O689" headerRowCount="1">
-  <autoFilter ref="A1:O688"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O698" headerRowCount="1">
+  <autoFilter ref="A1:O698"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Domaine (regroupement agent)"/>
     <tableColumn id="2" name="Pack(s)"/>
@@ -242,8 +242,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotesPointsOuverts" displayName="NotesPointsOuverts" ref="A1:D19" headerRowCount="1">
-  <autoFilter ref="A1:D19"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotesPointsOuverts" displayName="NotesPointsOuverts" ref="A1:D22" headerRowCount="1">
+  <autoFilter ref="A1:D22"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Domaine"/>
     <tableColumn id="2" name="Sujet"/>
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O689"/>
+  <dimension ref="A1:O698"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -30424,7 +30424,7 @@
       </c>
       <c r="J386" s="2" t="inlineStr">
         <is>
-          <t>Collaborateurs du tenant (contexte tenant requis, pas de garde RBAC nommée dans la route, uniquement `requireTenantAccess`)</t>
+          <t>Détenteurs de la permission — TENANT_ADMIN, TENANT_MANAGER par défaut ; pas TENANT_AGENT</t>
         </is>
       </c>
       <c r="K386" s="2" t="inlineStr">
@@ -30439,7 +30439,7 @@
       </c>
       <c r="M386" s="2" t="inlineStr">
         <is>
-          <t>`authenticate` + `requireTenantAccess` + `enforceTenantIsolation` (pas de `requireTenantCollaborator` sur `document-routes.ts` — accès potentiellement plus large que les autres routes communication, voir Notes)</t>
+          <t>`authenticate` + `requireTenantAccess` + `enforceTenantIsolation` + `requireDocumentsEdit`</t>
         </is>
       </c>
       <c r="N386" s="2" t="inlineStr">
@@ -30501,7 +30501,7 @@
       </c>
       <c r="J387" s="2" t="inlineStr">
         <is>
-          <t>Collaborateurs du tenant</t>
+          <t>Détenteurs de `RENTAL_DOCUMENTS_VIEW` ou de `RENTAL_DOCUMENTS_GENERATE` — TENANT_ADMIN, TENANT_MANAGER par défaut ; pas TENANT_AGENT</t>
         </is>
       </c>
       <c r="K387" s="2" t="inlineStr">
@@ -30516,7 +30516,7 @@
       </c>
       <c r="M387" s="2" t="inlineStr">
         <is>
-          <t>idem</t>
+          <t>`authenticate` + `requireTenantAccess` + `enforceTenantIsolation` + `requireAnyPermission(['RENTAL_DOCUMENTS_VIEW', 'RENTAL_DOCUMENTS_GENERATE'])`</t>
         </is>
       </c>
       <c r="N387" s="2" t="inlineStr">
@@ -30563,47 +30563,47 @@
       </c>
       <c r="G388" s="2" t="inlineStr">
         <is>
-          <t>PATCH `{status: 'ACTIVE'</t>
+          <t>PATCH `{status: 'ACTIVE' | 'INACTIVE'}`</t>
         </is>
       </c>
       <c r="H388" s="2" t="inlineStr">
         <is>
-          <t>'INACTIVE'}`</t>
+          <t>Modèle mis à jour</t>
         </is>
       </c>
       <c r="I388" s="2" t="inlineStr">
         <is>
-          <t>Modèle mis à jour</t>
+          <t>Un modèle doit avoir été uploadé</t>
         </is>
       </c>
       <c r="J388" s="2" t="inlineStr">
         <is>
-          <t>Un modèle doit avoir été uploadé</t>
+          <t>Détenteurs de la permission — TENANT_ADMIN, TENANT_MANAGER par défaut ; pas TENANT_AGENT</t>
         </is>
       </c>
       <c r="K388" s="2" t="inlineStr">
         <is>
-          <t>Collaborateurs du tenant</t>
+          <t>Agence (collaborateur)</t>
         </is>
       </c>
       <c r="L388" s="2" t="inlineStr">
         <is>
-          <t>Agence (collaborateur)</t>
+          <t>PATCH `/api/tenants/:tenantId/documents/templates/:id`</t>
         </is>
       </c>
       <c r="M388" s="2" t="inlineStr">
         <is>
-          <t>PATCH `/api/tenants/:tenantId/documents/templates/:id`</t>
+          <t>`authenticate` + `requireTenantAccess` + `enforceTenantIsolation` + `requireDocumentsEdit`</t>
         </is>
       </c>
       <c r="N388" s="2" t="inlineStr">
         <is>
-          <t>idem</t>
+          <t>Disponible</t>
         </is>
       </c>
       <c r="O388" s="2" t="inlineStr">
         <is>
-          <t>Disponible</t>
+          <t>Documents &gt; Modèles de documents</t>
         </is>
       </c>
     </row>
@@ -30655,7 +30655,7 @@
       </c>
       <c r="J389" s="2" t="inlineStr">
         <is>
-          <t>Collaborateurs du tenant</t>
+          <t>Détenteurs de la permission — TENANT_ADMIN, TENANT_MANAGER par défaut ; pas TENANT_AGENT</t>
         </is>
       </c>
       <c r="K389" s="2" t="inlineStr">
@@ -30670,7 +30670,7 @@
       </c>
       <c r="M389" s="2" t="inlineStr">
         <is>
-          <t>idem</t>
+          <t>`authenticate` + `requireTenantAccess` + `enforceTenantIsolation` + `requireDocumentsEdit`</t>
         </is>
       </c>
       <c r="N389" s="2" t="inlineStr">
@@ -30732,7 +30732,7 @@
       </c>
       <c r="J390" s="2" t="inlineStr">
         <is>
-          <t>Collaborateurs du tenant</t>
+          <t>Détenteurs de la permission — TENANT_ADMIN, TENANT_MANAGER par défaut ; pas TENANT_AGENT</t>
         </is>
       </c>
       <c r="K390" s="2" t="inlineStr">
@@ -30747,7 +30747,7 @@
       </c>
       <c r="M390" s="2" t="inlineStr">
         <is>
-          <t>idem</t>
+          <t>`authenticate` + `requireTenantAccess` + `enforceTenantIsolation` + `requireDocumentsEdit`</t>
         </is>
       </c>
       <c r="N390" s="2" t="inlineStr">
@@ -30809,7 +30809,7 @@
       </c>
       <c r="J391" s="2" t="inlineStr">
         <is>
-          <t>Collaborateurs du tenant (déclenché typiquement depuis les écrans de gestion locative, pas depuis le menu "Documents")</t>
+          <t>Détenteurs de la permission — TENANT_ADMIN, TENANT_MANAGER par défaut ; pas TENANT_AGENT</t>
         </is>
       </c>
       <c r="K391" s="2" t="inlineStr">
@@ -30824,7 +30824,7 @@
       </c>
       <c r="M391" s="2" t="inlineStr">
         <is>
-          <t>`authenticate` + `requireTenantAccess` + `enforceTenantIsolation`</t>
+          <t>`authenticate` + `requireTenantAccess` + `enforceTenantIsolation` + `requireDocumentsGenerate`</t>
         </is>
       </c>
       <c r="N391" s="2" t="inlineStr">
@@ -30886,7 +30886,7 @@
       </c>
       <c r="J392" s="2" t="inlineStr">
         <is>
-          <t>Collaborateurs du tenant</t>
+          <t>Détenteurs de la permission — TENANT_ADMIN, TENANT_MANAGER par défaut ; pas TENANT_AGENT</t>
         </is>
       </c>
       <c r="K392" s="2" t="inlineStr">
@@ -30901,7 +30901,7 @@
       </c>
       <c r="M392" s="2" t="inlineStr">
         <is>
-          <t>idem</t>
+          <t>`authenticate` + `requireTenantAccess` + `enforceTenantIsolation` + `requireDocumentsGenerate`</t>
         </is>
       </c>
       <c r="N392" s="2" t="inlineStr">
@@ -30963,7 +30963,7 @@
       </c>
       <c r="J393" s="2" t="inlineStr">
         <is>
-          <t>Collaborateurs du tenant</t>
+          <t>Détenteurs de la permission — TENANT_ADMIN, TENANT_MANAGER par défaut ; pas TENANT_AGENT</t>
         </is>
       </c>
       <c r="K393" s="2" t="inlineStr">
@@ -30978,7 +30978,7 @@
       </c>
       <c r="M393" s="2" t="inlineStr">
         <is>
-          <t>idem</t>
+          <t>`authenticate` + `requireTenantAccess` + `enforceTenantIsolation` + `requireDocumentsView`</t>
         </is>
       </c>
       <c r="N393" s="2" t="inlineStr">
@@ -30988,7 +30988,7 @@
       </c>
       <c r="O393" s="2" t="inlineStr">
         <is>
-          <t>Non affiché dans le menu "Documents"</t>
+          <t>Non affiché dans le menu "Documents" (téléchargement proposé par les écrans Location et par l'Assistant IA ImmoCopilot)</t>
         </is>
       </c>
     </row>
@@ -53781,6 +53781,699 @@
       <c r="O689" t="inlineStr">
         <is>
           <t>Aucun (technique)</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" s="2" t="inlineStr">
+        <is>
+          <t>Communication et Documents</t>
+        </is>
+      </c>
+      <c r="B690" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Syndic, Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C690" s="2" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="D690" s="2" t="inlineStr">
+        <is>
+          <t>Assistant IA ImmoCopilot</t>
+        </is>
+      </c>
+      <c r="E690" s="2" t="inlineStr">
+        <is>
+          <t>Connaître l'état de l'assistant et les outils permis</t>
+        </is>
+      </c>
+      <c r="F690" s="2" t="inlineStr">
+        <is>
+          <t>Interroge l'assistant à l'ouverture de la coquille d'agence : indique s'il est activé et quels outils l'utilisateur peut employer (permissions RBAC et, en mode `enforce`, modules de l'abonnement). Le bouton flottant « Assistant » (raccourci Ctrl/Cmd+J) n'apparaît que si `enabled` est vrai ; toute erreur de statut le masque</t>
+        </is>
+      </c>
+      <c r="G690" s="2" t="inlineStr">
+        <is>
+          <t>GET (aucun corps)</t>
+        </is>
+      </c>
+      <c r="H690" s="2" t="inlineStr">
+        <is>
+          <t>`{success, data: {enabled, reason? (NOT_CONFIGURED | NO_TOOLS), provider (fake | anthropic | null), tools[], limits {maxMessages, maxMessageChars}}}`</t>
+        </is>
+      </c>
+      <c r="I690" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J690" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateurs de l'agence, tous rôles ; refusé au super-admin et aux clients de portail</t>
+        </is>
+      </c>
+      <c r="K690" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L690" s="2" t="inlineStr">
+        <is>
+          <t>GET `/api/tenants/:tenantId/ai/status`</t>
+        </is>
+      </c>
+      <c r="M690" s="2" t="inlineStr">
+        <is>
+          <t>`authenticate` + `requireTenantAccess` + `requireTenantCollaborator` + `requireAiStatusAccess` (aucune permission dédiée ; répond `enabled: false` quand l'assistant est désactivé)</t>
+        </is>
+      </c>
+      <c r="N690" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O690" s="2" t="inlineStr">
+        <is>
+          <t>Bouton flottant Assistant (Ctrl/Cmd+J), toutes pages d'agence</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" s="2" t="inlineStr">
+        <is>
+          <t>Communication et Documents</t>
+        </is>
+      </c>
+      <c r="B691" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Syndic, Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C691" s="2" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="D691" s="2" t="inlineStr">
+        <is>
+          <t>Assistant IA ImmoCopilot</t>
+        </is>
+      </c>
+      <c r="E691" s="2" t="inlineStr">
+        <is>
+          <t>Discuter avec l'assistant (flux en direct)</t>
+        </is>
+      </c>
+      <c r="F691" s="2" t="inlineStr">
+        <is>
+          <t>Ouvre le tiroir de conversation (côté « fin » : à droite en français, à gauche en arabe) et envoie l'échange au fournisseur LLM en flux SSE : texte progressif, cartes de résultats (biens, baux, documents, proposition), suggestions selon l'écran courant, arrêt de la réponse et nouvelle conversation. Conversation non persistée ; l'assistant n'écrit jamais lui-même. Limites : 20 messages, 4 000 caractères chacun, 24 000 au total ; 20 requêtes/min et 300/jour par utilisateur et par agence ; 4 tours et 8 appels d'outils maximum</t>
+        </is>
+      </c>
+      <c r="G691" s="2" t="inlineStr">
+        <is>
+          <t>POST `{conversationId?, messages[{role, content}] (1 à 20), context? {currentPath?, activeEntityType? (PROPERTY | LEASE), activeEntityId?}}`</t>
+        </is>
+      </c>
+      <c r="H691" s="2" t="inlineStr">
+        <is>
+          <t>Flux `text/event-stream` : `meta`, `text_delta`, `tool_status`, `property_results`, `lease_results`, `document_list`, `action_proposal`, `error`, `done` (ping toutes les 15 s). Avant l'ouverture du flux : JSON typé (400 corps invalide, 403, 429 `RATE_LIMITED`, 503 `AI_DISABLED`)</t>
+        </is>
+      </c>
+      <c r="I691" s="2" t="inlineStr">
+        <is>
+          <t>Statut de l'assistant (activé)</t>
+        </is>
+      </c>
+      <c r="J691" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateurs de l'agence ; chaque outil vérifie sa propre permission ; refusé au super-admin et aux clients de portail</t>
+        </is>
+      </c>
+      <c r="K691" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L691" s="2" t="inlineStr">
+        <is>
+          <t>POST `/api/tenants/:tenantId/ai/chat`</t>
+        </is>
+      </c>
+      <c r="M691" s="2" t="inlineStr">
+        <is>
+          <t>`authenticate` + `requireTenantAccess` + `requireTenantCollaborator` + `requireAiAssistantAccess` + limiteurs `aiChatRateLimiter` et `aiChatDailyLimiter` ; pas de permission unique : chaque outil vérifie la sienne (voir les lignes suivantes)</t>
+        </is>
+      </c>
+      <c r="N691" s="2" t="inlineStr">
+        <is>
+          <t>Disponible (désactivé par défaut, AI_PROVIDER)</t>
+        </is>
+      </c>
+      <c r="O691" s="2" t="inlineStr">
+        <is>
+          <t>Bouton flottant Assistant (Ctrl/Cmd+J), toutes pages d'agence</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" s="2" t="inlineStr">
+        <is>
+          <t>Communication et Documents</t>
+        </is>
+      </c>
+      <c r="B692" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Syndic, Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C692" s="2" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="D692" s="2" t="inlineStr">
+        <is>
+          <t>Assistant IA ImmoCopilot</t>
+        </is>
+      </c>
+      <c r="E692" s="2" t="inlineStr">
+        <is>
+          <t>Rechercher des biens en langage naturel</t>
+        </is>
+      </c>
+      <c r="F692" s="2" t="inlineStr">
+        <is>
+          <t>Outil `search_properties` : filtre les biens de l'agence (texte, commune ou zone, type, statut, mode de transaction, prix, chambres), au plus 10 résultats, affichés en cartes cliquables vers la fiche du bien. Les biens publics d'autres agences sont exclus ; jamais d'e-mail, de téléphone ni de propriétaire transmis au fournisseur</t>
+        </is>
+      </c>
+      <c r="G692" s="2" t="inlineStr">
+        <is>
+          <t>Demande en langage naturel (ex. « appartements disponibles à Cocody »)</t>
+        </is>
+      </c>
+      <c r="H692" s="2" t="inlineStr">
+        <is>
+          <t>Événement `property_results` (cartes : référence, titre, type, statut, zone, prix, chambres, surface, vignette) et texte de synthèse</t>
+        </is>
+      </c>
+      <c r="I692" s="2" t="inlineStr">
+        <is>
+          <t>Discuter avec l'assistant (flux en direct)</t>
+        </is>
+      </c>
+      <c r="J692" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateurs de l'agence détenteurs de la permission — TENANT_ADMIN, TENANT_MANAGER, TENANT_AGENT par défaut ; refusé au super-admin et aux clients de portail</t>
+        </is>
+      </c>
+      <c r="K692" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L692" s="2" t="inlineStr">
+        <is>
+          <t>POST `/api/tenants/:tenantId/ai/chat` (outil `search_properties`)</t>
+        </is>
+      </c>
+      <c r="M692" s="2" t="inlineStr">
+        <is>
+          <t>`PROPERTIES_VIEW` (outil `search_properties`) + `authenticate` + `requireTenantAccess` + `requireTenantCollaborator` + `requireAiAssistantAccess`</t>
+        </is>
+      </c>
+      <c r="N692" s="2" t="inlineStr">
+        <is>
+          <t>Disponible (désactivé par défaut, AI_PROVIDER)</t>
+        </is>
+      </c>
+      <c r="O692" s="2" t="inlineStr">
+        <is>
+          <t>Bouton flottant Assistant (Ctrl/Cmd+J), toutes pages d'agence</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" s="2" t="inlineStr">
+        <is>
+          <t>Communication et Documents</t>
+        </is>
+      </c>
+      <c r="B693" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C693" s="2" t="inlineStr">
+        <is>
+          <t>RENTAL</t>
+        </is>
+      </c>
+      <c r="D693" s="2" t="inlineStr">
+        <is>
+          <t>Assistant IA ImmoCopilot</t>
+        </is>
+      </c>
+      <c r="E693" s="2" t="inlineStr">
+        <is>
+          <t>Retrouver un bail</t>
+        </is>
+      </c>
+      <c r="F693" s="2" t="inlineStr">
+        <is>
+          <t>Outil `search_leases` : retrouve les baux de l'agence par numéro de bail (recherche partielle), nom du locataire (filtre en mémoire sur les 200 premiers baux), bien ou statut ; au plus 10 résultats. Un bien d'une autre agence est refusé comme un bien inexistant</t>
+        </is>
+      </c>
+      <c r="G693" s="2" t="inlineStr">
+        <is>
+          <t>Numéro de bail, nom du locataire, `propertyId` ou statut</t>
+        </is>
+      </c>
+      <c r="H693" s="2" t="inlineStr">
+        <is>
+          <t>Événement `lease_results` (cartes : numéro, statut, bien, locataire, loyer, date de début)</t>
+        </is>
+      </c>
+      <c r="I693" s="2" t="inlineStr">
+        <is>
+          <t>Discuter avec l'assistant (flux en direct)</t>
+        </is>
+      </c>
+      <c r="J693" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateurs de l'agence détenteurs de la permission — TENANT_ADMIN, TENANT_MANAGER par défaut ; pas TENANT_AGENT ; refusé au super-admin et aux clients de portail</t>
+        </is>
+      </c>
+      <c r="K693" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L693" s="2" t="inlineStr">
+        <is>
+          <t>POST `/api/tenants/:tenantId/ai/chat` (outil `search_leases`)</t>
+        </is>
+      </c>
+      <c r="M693" s="2" t="inlineStr">
+        <is>
+          <t>`RENTAL_LEASES_VIEW` (outil `search_leases`) + `authenticate` + `requireTenantAccess` + `requireTenantCollaborator` + `requireAiAssistantAccess`</t>
+        </is>
+      </c>
+      <c r="N693" s="2" t="inlineStr">
+        <is>
+          <t>Disponible (désactivé par défaut, AI_PROVIDER)</t>
+        </is>
+      </c>
+      <c r="O693" s="2" t="inlineStr">
+        <is>
+          <t>Bouton flottant Assistant (Ctrl/Cmd+J), toutes pages d'agence</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" s="2" t="inlineStr">
+        <is>
+          <t>Communication et Documents</t>
+        </is>
+      </c>
+      <c r="B694" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C694" s="2" t="inlineStr">
+        <is>
+          <t>RENTAL</t>
+        </is>
+      </c>
+      <c r="D694" s="2" t="inlineStr">
+        <is>
+          <t>Assistant IA ImmoCopilot</t>
+        </is>
+      </c>
+      <c r="E694" s="2" t="inlineStr">
+        <is>
+          <t>Lister les documents d'un bail</t>
+        </is>
+      </c>
+      <c r="F694" s="2" t="inlineStr">
+        <is>
+          <t>Outil `list_lease_documents` : liste les documents locatifs d'un bail de l'agence (quittances, contrat, relevés…), filtrables par type (`LEASE_CONTRACT`, `LEASE_ADDENDUM`, `RENT_RECEIPT`, `RENT_QUITTANCE`, `DEPOSIT_RECEIPT`, `STATEMENT`, `OTHER`), au plus 10</t>
+        </is>
+      </c>
+      <c r="G694" s="2" t="inlineStr">
+        <is>
+          <t>`leaseId` (obtenu par « Retrouver un bail » ou l'écran courant), type facultatif</t>
+        </is>
+      </c>
+      <c r="H694" s="2" t="inlineStr">
+        <is>
+          <t>Événement `document_list` (portée bail : libellé, type, statut, date, téléchargeable)</t>
+        </is>
+      </c>
+      <c r="I694" s="2" t="inlineStr">
+        <is>
+          <t>Retrouver un bail</t>
+        </is>
+      </c>
+      <c r="J694" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateurs de l'agence détenteurs de la permission — TENANT_ADMIN, TENANT_MANAGER par défaut ; pas TENANT_AGENT ; refusé au super-admin et aux clients de portail</t>
+        </is>
+      </c>
+      <c r="K694" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L694" s="2" t="inlineStr">
+        <is>
+          <t>POST `/api/tenants/:tenantId/ai/chat` (outil `list_lease_documents`)</t>
+        </is>
+      </c>
+      <c r="M694" s="2" t="inlineStr">
+        <is>
+          <t>`RENTAL_DOCUMENTS_VIEW` (outil `list_lease_documents`) + `authenticate` + `requireTenantAccess` + `requireTenantCollaborator` + `requireAiAssistantAccess`</t>
+        </is>
+      </c>
+      <c r="N694" s="2" t="inlineStr">
+        <is>
+          <t>Disponible (désactivé par défaut, AI_PROVIDER)</t>
+        </is>
+      </c>
+      <c r="O694" s="2" t="inlineStr">
+        <is>
+          <t>Bouton flottant Assistant (Ctrl/Cmd+J), toutes pages d'agence</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" s="2" t="inlineStr">
+        <is>
+          <t>Communication et Documents</t>
+        </is>
+      </c>
+      <c r="B695" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Syndic, Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C695" s="2" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="D695" s="2" t="inlineStr">
+        <is>
+          <t>Assistant IA ImmoCopilot</t>
+        </is>
+      </c>
+      <c r="E695" s="2" t="inlineStr">
+        <is>
+          <t>Lister les documents d'un bien</t>
+        </is>
+      </c>
+      <c r="F695" s="2" t="inlineStr">
+        <is>
+          <t>Outil `list_property_documents` : liste les pièces du dossier d'un bien de l'agence (titre foncier, mandat, plans…), expirées comprises par défaut, au plus 10 ; jamais de chemin de fichier transmis</t>
+        </is>
+      </c>
+      <c r="G695" s="2" t="inlineStr">
+        <is>
+          <t>`propertyId` (obtenu par « Rechercher des biens » ou l'écran courant), `includeExpired` facultatif</t>
+        </is>
+      </c>
+      <c r="H695" s="2" t="inlineStr">
+        <is>
+          <t>Événement `document_list` (portée bien : nom du fichier, type, statut valide ou expiré, date)</t>
+        </is>
+      </c>
+      <c r="I695" s="2" t="inlineStr">
+        <is>
+          <t>Rechercher des biens en langage naturel</t>
+        </is>
+      </c>
+      <c r="J695" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateurs de l'agence détenteurs de la permission — TENANT_ADMIN, TENANT_MANAGER, TENANT_AGENT par défaut ; refusé au super-admin et aux clients de portail</t>
+        </is>
+      </c>
+      <c r="K695" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L695" s="2" t="inlineStr">
+        <is>
+          <t>POST `/api/tenants/:tenantId/ai/chat` (outil `list_property_documents`)</t>
+        </is>
+      </c>
+      <c r="M695" s="2" t="inlineStr">
+        <is>
+          <t>`PROPERTIES_VIEW` (outil `list_property_documents`) + `authenticate` + `requireTenantAccess` + `requireTenantCollaborator` + `requireAiAssistantAccess`</t>
+        </is>
+      </c>
+      <c r="N695" s="2" t="inlineStr">
+        <is>
+          <t>Disponible (désactivé par défaut, AI_PROVIDER)</t>
+        </is>
+      </c>
+      <c r="O695" s="2" t="inlineStr">
+        <is>
+          <t>Bouton flottant Assistant (Ctrl/Cmd+J), toutes pages d'agence</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" s="2" t="inlineStr">
+        <is>
+          <t>Communication et Documents</t>
+        </is>
+      </c>
+      <c r="B696" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C696" s="2" t="inlineStr">
+        <is>
+          <t>RENTAL</t>
+        </is>
+      </c>
+      <c r="D696" s="2" t="inlineStr">
+        <is>
+          <t>Assistant IA ImmoCopilot</t>
+        </is>
+      </c>
+      <c r="E696" s="2" t="inlineStr">
+        <is>
+          <t>Préparer une quittance ou un relevé de compte (proposition)</t>
+        </is>
+      </c>
+      <c r="F696" s="2" t="inlineStr">
+        <is>
+          <t>Outil `propose_rental_document` : prépare une PROPOSITION, sans aucune écriture. Quittance (`RENT_RECEIPT`, période AAAA-MM) : le serveur retrouve l'échéance de la période puis le paiement encaissé (SUCCESS) qui l'alloue ; sans paiement, sans échéance ou sans modèle actif, aucune proposition (« impossible ») ; une quittance FINAL déjà émise est montrée au lieu d'être reproposée. Relevé (`RENT_STATEMENT`, dates de début et de fin, 12 mois maximum). Renvoie une carte de récapitulatif et un jeton signé valable 300 s (`AI_PROPOSAL_TTL_SECONDS`). Le jeton n'est jamais transmis au fournisseur LLM</t>
+        </is>
+      </c>
+      <c r="G696" s="2" t="inlineStr">
+        <is>
+          <t>`leaseId`, `docType`, période (quittance) ou dates (relevé)</t>
+        </is>
+      </c>
+      <c r="H696" s="2" t="inlineStr">
+        <is>
+          <t>Événement `action_proposal` (bail, bien, locataire, période, montant, expiration, jeton) ou `document_list` si la quittance existe déjà ; audit `AI_PROPOSAL_ISSUED`</t>
+        </is>
+      </c>
+      <c r="I696" s="2" t="inlineStr">
+        <is>
+          <t>Retrouver un bail</t>
+        </is>
+      </c>
+      <c r="J696" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateurs de l'agence détenteurs de la permission — TENANT_ADMIN, TENANT_MANAGER par défaut ; pas TENANT_AGENT ; refusé au super-admin et aux clients de portail</t>
+        </is>
+      </c>
+      <c r="K696" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L696" s="2" t="inlineStr">
+        <is>
+          <t>POST `/api/tenants/:tenantId/ai/chat` (outil `propose_rental_document`)</t>
+        </is>
+      </c>
+      <c r="M696" s="2" t="inlineStr">
+        <is>
+          <t>`RENTAL_DOCUMENTS_GENERATE` (outil `propose_rental_document`) + `authenticate` + `requireTenantAccess` + `requireTenantCollaborator` + `requireAiAssistantAccess`</t>
+        </is>
+      </c>
+      <c r="N696" s="2" t="inlineStr">
+        <is>
+          <t>Disponible (désactivé par défaut, AI_PROVIDER)</t>
+        </is>
+      </c>
+      <c r="O696" s="2" t="inlineStr">
+        <is>
+          <t>Bouton flottant Assistant (Ctrl/Cmd+J), toutes pages d'agence</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" s="2" t="inlineStr">
+        <is>
+          <t>Communication et Documents</t>
+        </is>
+      </c>
+      <c r="B697" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C697" s="2" t="inlineStr">
+        <is>
+          <t>RENTAL</t>
+        </is>
+      </c>
+      <c r="D697" s="2" t="inlineStr">
+        <is>
+          <t>Assistant IA ImmoCopilot</t>
+        </is>
+      </c>
+      <c r="E697" s="2" t="inlineStr">
+        <is>
+          <t>Confirmer et générer le document proposé</t>
+        </is>
+      </c>
+      <c r="F697" s="2" t="inlineStr">
+        <is>
+          <t>Action humaine sur la carte de proposition (« Confirmer et générer ») : rejoue authentification, agence, collaborateur et `RENTAL_DOCUMENTS_GENERATE`, vérifie le jeton (signature, expiration, utilisateur, agence, usage unique) et l'appartenance de chaque identifiant, puis génère le `.docx` via le générateur existant. Idempotent (une quittance FINAL déjà émise est renvoyée) ; 10 confirmations par minute ; audit `AI_PROPOSAL_REDEEMED` et `AI_ACTION_EXECUTED`. Seule porte de génération de l'assistant</t>
+        </is>
+      </c>
+      <c r="G697" s="2" t="inlineStr">
+        <is>
+          <t>POST `{proposalToken}`</t>
+        </is>
+      </c>
+      <c r="H697" s="2" t="inlineStr">
+        <is>
+          <t>201 `{success, data: {proposalId, alreadyExisted, document {id, documentNumber, type, mimeType, filename, downloadPath}}}` ; erreurs `PROPOSAL_INVALID` (400), `PROPOSAL_EXPIRED` (410), `PROPOSAL_ALREADY_USED` (409), 503 `AI_DISABLED`</t>
+        </is>
+      </c>
+      <c r="I697" s="2" t="inlineStr">
+        <is>
+          <t>Préparer une quittance ou un relevé de compte (proposition)</t>
+        </is>
+      </c>
+      <c r="J697" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateurs de l'agence détenteurs de la permission — TENANT_ADMIN, TENANT_MANAGER par défaut ; pas TENANT_AGENT ; refusé au super-admin et aux clients de portail</t>
+        </is>
+      </c>
+      <c r="K697" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L697" s="2" t="inlineStr">
+        <is>
+          <t>POST `/api/tenants/:tenantId/ai/actions/execute`</t>
+        </is>
+      </c>
+      <c r="M697" s="2" t="inlineStr">
+        <is>
+          <t>`RENTAL_DOCUMENTS_GENERATE` (`requireDocumentsGenerate`) + `authenticate` + `requireTenantAccess` + `requireTenantCollaborator` + `requireAiAssistantAccess` + `aiActionRateLimiter`</t>
+        </is>
+      </c>
+      <c r="N697" s="2" t="inlineStr">
+        <is>
+          <t>Disponible (désactivé par défaut, AI_PROVIDER)</t>
+        </is>
+      </c>
+      <c r="O697" s="2" t="inlineStr">
+        <is>
+          <t>Bouton flottant Assistant (Ctrl/Cmd+J), toutes pages d'agence</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" s="2" t="inlineStr">
+        <is>
+          <t>Communication et Documents</t>
+        </is>
+      </c>
+      <c r="B698" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Syndic, Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C698" s="2" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="D698" s="2" t="inlineStr">
+        <is>
+          <t>Assistant IA ImmoCopilot</t>
+        </is>
+      </c>
+      <c r="E698" s="2" t="inlineStr">
+        <is>
+          <t>Télécharger le document généré</t>
+        </is>
+      </c>
+      <c r="F698" s="2" t="inlineStr">
+        <is>
+          <t>Carte de téléchargement affichée après la confirmation : télécharge le `.docx` (« Word (.docx) ») par la route authentifiée existante, qui vérifie l'appartenance à l'agence avant lecture disque ; jamais de chemin de fichier dans la réponse. Pour une pièce de bien, la carte passe par la route de fichier du bien</t>
+        </is>
+      </c>
+      <c r="G698" s="2" t="inlineStr">
+        <is>
+          <t>GET (identifiant du document)</t>
+        </is>
+      </c>
+      <c r="H698" s="2" t="inlineStr">
+        <is>
+          <t>Flux binaire `.docx` (`Content-Disposition: attachment`)</t>
+        </is>
+      </c>
+      <c r="I698" s="2" t="inlineStr">
+        <is>
+          <t>Confirmer et générer le document proposé</t>
+        </is>
+      </c>
+      <c r="J698" s="2" t="inlineStr">
+        <is>
+          <t>Détenteurs de la permission — TENANT_ADMIN, TENANT_MANAGER par défaut ; pas TENANT_AGENT</t>
+        </is>
+      </c>
+      <c r="K698" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L698" s="2" t="inlineStr">
+        <is>
+          <t>GET `/api/tenants/:tenantId/documents/:id/download`</t>
+        </is>
+      </c>
+      <c r="M698" s="2" t="inlineStr">
+        <is>
+          <t>`authenticate` + `requireTenantAccess` + `enforceTenantIsolation` + `requireDocumentsView`</t>
+        </is>
+      </c>
+      <c r="N698" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O698" s="2" t="inlineStr">
+        <is>
+          <t>Bouton flottant Assistant (Ctrl/Cmd+J), toutes pages d'agence</t>
         </is>
       </c>
     </row>
@@ -54386,7 +55079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -54835,6 +55528,50 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Assistant IA ImmoCopilot : données transmises au fournisseur LLM (minimisation, désactivé par défaut)</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Quand AI_PROVIDER=anthropic, chaque échange envoie au fournisseur (Anthropic) le texte saisi et des résultats d'outils projetés : références et titres de biens, adresses, prix, numéros de bail, NOM du locataire principal, montant et période d'une quittance. Jamais d'e-mail, de téléphone, de chemin de fichier, de notes ni de propriétaire ; sorties d'outils plafonnées à 10 éléments et 8 Ko ; le jeton de proposition ne part pas. L'assistant est désactivé par défaut (AI_PROVIDER=disabled), refusé au super-admin et aux clients de portail, et rien n'est conservé côté navigateur.</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>L'activation en production relève d'une décision juridique et contractuelle (transfert de données personnelles à un tiers, accord de traitement avec le fournisseur) : à trancher avant d'activer. Voir docs/governance/SECURITY.md, section « Assistant IA ».</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Gestion locative</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Avis d'échéance non générable (pas de DocumentType)</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Aucun avis d'échéance ni relance n'existe : les types générables (`DocumentType`) sont LEASE_HABITATION, LEASE_COMMERCIAL, RENT_RECEIPT et RENT_STATEMENT, en sortie DOCX uniquement. L'assistant ImmoCopilot ne peut donc proposer que la quittance (à partir d'un paiement encaissé) et le relevé de compte.</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Phase 2 : nouveau `DocumentType`, modèle DOCX et constructeur de contexte, avant d'ajouter l'avis d'échéance à l'assistant.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
fix(web): tenir le budget d'entree, wiki du lot 1, spec du lot 2
Ecrans du patrimoine multi-actifs rattaches a la route patrimoine existante
(joker) au lieu de trois React.lazy, repartition par classe en barre CSS,
liste des entites detentrices dans le service des actifs : le chemin
critique repasse sous le budget du 8.1. Wiki des fonctionnalites mis a jour
(19 sous-fonctionnalites). Spec du lot 2 : valorisation par classe.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PxDVZM8akvCsSCfK3Cgg19
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -189,8 +189,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O698" headerRowCount="1">
-  <autoFilter ref="A1:O698"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O717" headerRowCount="1">
+  <autoFilter ref="A1:O717"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Domaine (regroupement agent)"/>
     <tableColumn id="2" name="Pack(s)"/>
@@ -242,8 +242,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotesPointsOuverts" displayName="NotesPointsOuverts" ref="A1:D22" headerRowCount="1">
-  <autoFilter ref="A1:D22"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotesPointsOuverts" displayName="NotesPointsOuverts" ref="A1:D23" headerRowCount="1">
+  <autoFilter ref="A1:D23"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Domaine"/>
     <tableColumn id="2" name="Sujet"/>
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O698"/>
+  <dimension ref="A1:O717"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -54474,6 +54474,1465 @@
       <c r="O698" s="2" t="inlineStr">
         <is>
           <t>Bouton flottant Assistant (Ctrl/Cmd+J), toutes pages d'agence</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B699" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C699" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D699" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Actifs</t>
+        </is>
+      </c>
+      <c r="E699" s="2" t="inlineStr">
+        <is>
+          <t>Lister les actifs</t>
+        </is>
+      </c>
+      <c r="F699" s="2" t="inlineStr">
+        <is>
+          <t>Parcourir les actifs du patrimoine de l'agence, toutes classes confondues, avec filtres par classe, statut et recherche par nom</t>
+        </is>
+      </c>
+      <c r="G699" s="2" t="inlineStr">
+        <is>
+          <t>Query facultatives : `assetClass` (une des 10 classes), `status` (`ACTIVE`, `DISPOSED`, `ARCHIVED`), `search` (texte, insensible à la casse, sur le nom) ; sans filtre de statut, les actifs archivés sont masqués</t>
+        </is>
+      </c>
+      <c r="H699" s="2" t="inlineStr">
+        <is>
+          <t>Liste d'actifs, du plus récent au plus ancien, chacun avec sa valeur courante et son capital restant dû adossé</t>
+        </is>
+      </c>
+      <c r="I699" s="2" t="inlineStr"/>
+      <c r="J699" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K699" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L699" s="2" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/patrimoine/assets</t>
+        </is>
+      </c>
+      <c r="M699" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_VIEW (`requireAnyPropertyPermission`)</t>
+        </is>
+      </c>
+      <c r="N699" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O699" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Mes actifs (/tenant/:tenantId/patrimoine/actifs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B700" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C700" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D700" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Actifs</t>
+        </is>
+      </c>
+      <c r="E700" s="2" t="inlineStr">
+        <is>
+          <t>Créer un actif</t>
+        </is>
+      </c>
+      <c r="F700" s="2" t="inlineStr">
+        <is>
+          <t>Enregistrer un actif de l'une des 10 classes : immobilier, entreprises et parts de sociétés, stocks et marchandises, véhicules et équipements, comptes et mobile money, épargne et placements, créances, agriculture et élevage, biens meubles de valeur, autre ; avec une première valorisation facultative</t>
+        </is>
+      </c>
+      <c r="G700" s="2" t="inlineStr">
+        <is>
+          <t>Body Zod `.strict()` : `name` (1 à 200 car.), `assetClass` (obligatoire), `currency` (ISO 3 lettres) et `exchangeRateToXof` (&gt;0) facultatifs, `acquisitionCost` (&gt;=0), `acquisitionDate`, `holdingEntityId`, `details` (validé selon la classe), `notes`, `propertyId` (obligatoire et réservé à la classe immobilière), `initialValuation` facultative `{valuatedAt, estimatedValue (&gt;0), method, source, notes}`</t>
+        </is>
+      </c>
+      <c r="H700" s="2" t="inlineStr">
+        <is>
+          <t>201 — Actif (id, nom, classe, statut, devise, taux de change vers XOF, coût et date d'acquisition, date de cession, entité détentrice, bien lié, détails propres à la classe, notes, valeur courante avec sa date et sa valeur en XOF, capital restant dû des prêts adossés en XOF) ; la valorisation initiale, si fournie, est créée dans la même transaction</t>
+        </is>
+      </c>
+      <c r="I700" s="2" t="inlineStr">
+        <is>
+          <t>Un actif immobilier exige un bien de l'agence non déjà rattaché à un actif (409 sinon) ; `holdingEntityId` doit appartenir à l'agence ; une devise autre que le XOF exige un taux de change</t>
+        </is>
+      </c>
+      <c r="J700" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="K700" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L700" s="2" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/patrimoine/assets</t>
+        </is>
+      </c>
+      <c r="M700" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="N700" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O700" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Mes actifs (/tenant/:tenantId/patrimoine/actifs) — bouton « Ajouter un actif » (tiroir de saisie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B701" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C701" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D701" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Actifs</t>
+        </is>
+      </c>
+      <c r="E701" s="2" t="inlineStr">
+        <is>
+          <t>Consulter la fiche d'un actif</t>
+        </is>
+      </c>
+      <c r="F701" s="2" t="inlineStr">
+        <is>
+          <t>Afficher un actif avec sa valeur courante, ses informations, ses valeurs, ses dettes et, hors immobilier, ses détenteurs</t>
+        </is>
+      </c>
+      <c r="G701" s="2" t="inlineStr">
+        <is>
+          <t>Param `assetId`</t>
+        </is>
+      </c>
+      <c r="H701" s="2" t="inlineStr">
+        <is>
+          <t>Actif (id, nom, classe, statut, devise, taux de change vers XOF, coût et date d'acquisition, date de cession, entité détentrice, bien lié, détails propres à la classe, notes, valeur courante avec sa date et sa valeur en XOF, capital restant dû des prêts adossés en XOF)</t>
+        </is>
+      </c>
+      <c r="I701" s="2" t="inlineStr">
+        <is>
+          <t>L'actif doit appartenir à l'agence (sinon 404, comme un actif inexistant)</t>
+        </is>
+      </c>
+      <c r="J701" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K701" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L701" s="2" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/patrimoine/assets/:assetId</t>
+        </is>
+      </c>
+      <c r="M701" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_VIEW (`requireAnyPropertyPermission`)</t>
+        </is>
+      </c>
+      <c r="N701" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O701" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Mes actifs &gt; fiche d'un actif, onglet Informations (/tenant/:tenantId/patrimoine/actifs/:assetId)</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B702" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C702" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D702" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Actifs</t>
+        </is>
+      </c>
+      <c r="E702" s="2" t="inlineStr">
+        <is>
+          <t>Modifier un actif</t>
+        </is>
+      </c>
+      <c r="F702" s="2" t="inlineStr">
+        <is>
+          <t>Corriger les informations d'un actif (la classe et le bien lié ne changent pas)</t>
+        </is>
+      </c>
+      <c r="G702" s="2" t="inlineStr">
+        <is>
+          <t>Body Zod partiel `.strict()` (au moins un champ) : `name`, `currency`, `exchangeRateToXof`, `acquisitionCost`, `acquisitionDate`, `holdingEntityId`, `details` (validé selon la classe de l'actif), `notes`</t>
+        </is>
+      </c>
+      <c r="H702" s="2" t="inlineStr">
+        <is>
+          <t>Actif (id, nom, classe, statut, devise, taux de change vers XOF, coût et date d'acquisition, date de cession, entité détentrice, bien lié, détails propres à la classe, notes, valeur courante avec sa date et sa valeur en XOF, capital restant dû des prêts adossés en XOF)</t>
+        </is>
+      </c>
+      <c r="I702" s="2" t="inlineStr">
+        <is>
+          <t>L'actif doit appartenir à l'agence (sinon 404, comme un actif inexistant) ; `holdingEntityId` doit appartenir à l'agence</t>
+        </is>
+      </c>
+      <c r="J702" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="K702" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L702" s="2" t="inlineStr">
+        <is>
+          <t>PATCH /tenants/:tenantId/patrimoine/assets/:assetId</t>
+        </is>
+      </c>
+      <c r="M702" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="N702" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O702" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Mes actifs &gt; fiche d'un actif, onglet Informations (/tenant/:tenantId/patrimoine/actifs/:assetId) — bouton « Modifier »</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B703" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C703" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D703" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Actifs</t>
+        </is>
+      </c>
+      <c r="E703" s="2" t="inlineStr">
+        <is>
+          <t>Marquer un actif comme cédé</t>
+        </is>
+      </c>
+      <c r="F703" s="2" t="inlineStr">
+        <is>
+          <t>Enregistrer la cession d'un actif : il sort de la valeur nette à la date de cession, son historique est conservé</t>
+        </is>
+      </c>
+      <c r="G703" s="2" t="inlineStr">
+        <is>
+          <t>Param `assetId`, body `{ disposedAt }` (date)</t>
+        </is>
+      </c>
+      <c r="H703" s="2" t="inlineStr">
+        <is>
+          <t>Actif au statut `DISPOSED` avec sa date de cession</t>
+        </is>
+      </c>
+      <c r="I703" s="2" t="inlineStr">
+        <is>
+          <t>L'actif doit appartenir à l'agence (sinon 404, comme un actif inexistant) ; 409 si l'actif n'est plus au statut `ACTIVE`</t>
+        </is>
+      </c>
+      <c r="J703" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="K703" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L703" s="2" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/patrimoine/assets/:assetId/dispose</t>
+        </is>
+      </c>
+      <c r="M703" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="N703" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O703" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Mes actifs &gt; fiche d'un actif, onglet Informations (/tenant/:tenantId/patrimoine/actifs/:assetId) — bouton « Marquer comme cédé »</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B704" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C704" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D704" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Actifs</t>
+        </is>
+      </c>
+      <c r="E704" s="2" t="inlineStr">
+        <is>
+          <t>Archiver un actif</t>
+        </is>
+      </c>
+      <c r="F704" s="2" t="inlineStr">
+        <is>
+          <t>Retirer un actif de la liste par défaut sans le supprimer</t>
+        </is>
+      </c>
+      <c r="G704" s="2" t="inlineStr">
+        <is>
+          <t>Param `assetId`</t>
+        </is>
+      </c>
+      <c r="H704" s="2" t="inlineStr">
+        <is>
+          <t>Actif au statut `ARCHIVED`</t>
+        </is>
+      </c>
+      <c r="I704" s="2" t="inlineStr">
+        <is>
+          <t>L'actif doit appartenir à l'agence (sinon 404, comme un actif inexistant) ; 409 s'il est déjà archivé (un actif actif ou cédé peut être archivé)</t>
+        </is>
+      </c>
+      <c r="J704" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="K704" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L704" s="2" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/patrimoine/assets/:assetId/archive</t>
+        </is>
+      </c>
+      <c r="M704" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="N704" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O704" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Mes actifs &gt; fiche d'un actif, onglet Informations (/tenant/:tenantId/patrimoine/actifs/:assetId) — bouton « Archiver »</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B705" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C705" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D705" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Valorisations d'un actif</t>
+        </is>
+      </c>
+      <c r="E705" s="2" t="inlineStr">
+        <is>
+          <t>Lister les valorisations d'un actif</t>
+        </is>
+      </c>
+      <c r="F705" s="2" t="inlineStr">
+        <is>
+          <t>Consulter l'historique des valeurs d'un actif</t>
+        </is>
+      </c>
+      <c r="G705" s="2" t="inlineStr">
+        <is>
+          <t>Param `assetId`</t>
+        </is>
+      </c>
+      <c r="H705" s="2" t="inlineStr">
+        <is>
+          <t>Liste de valorisations, la plus récente d'abord (id, date, valeur estimée, devise, méthode `MANUAL` / `MARKET_ESTIMATE` / `EXPERT_APPRAISAL`, source, notes) ; pour un actif immobilier lié à un bien, ce sont les valorisations du bien</t>
+        </is>
+      </c>
+      <c r="I705" s="2" t="inlineStr">
+        <is>
+          <t>L'actif doit appartenir à l'agence (sinon 404, comme un actif inexistant)</t>
+        </is>
+      </c>
+      <c r="J705" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K705" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L705" s="2" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/patrimoine/assets/:assetId/valuations</t>
+        </is>
+      </c>
+      <c r="M705" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_VIEW (`requireAnyPropertyPermission`)</t>
+        </is>
+      </c>
+      <c r="N705" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O705" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Mes actifs &gt; fiche d'un actif, onglet Valeurs</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B706" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C706" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D706" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Valorisations d'un actif</t>
+        </is>
+      </c>
+      <c r="E706" s="2" t="inlineStr">
+        <is>
+          <t>Ajouter une valorisation</t>
+        </is>
+      </c>
+      <c r="F706" s="2" t="inlineStr">
+        <is>
+          <t>Enregistrer une nouvelle valeur pour un actif ; le dernier relevé daté au plus tard à la date choisie devient sa valeur courante</t>
+        </is>
+      </c>
+      <c r="G706" s="2" t="inlineStr">
+        <is>
+          <t>Body Zod `.strict()` : `valuatedAt`, `estimatedValue` (&gt;0), `currency` facultative (devise de l'actif par défaut), `method` (`MANUAL` par défaut), `source`, `notes`</t>
+        </is>
+      </c>
+      <c r="H706" s="2" t="inlineStr">
+        <is>
+          <t>201 — valorisation créée</t>
+        </is>
+      </c>
+      <c r="I706" s="2" t="inlineStr">
+        <is>
+          <t>L'actif doit appartenir à l'agence (sinon 404, comme un actif inexistant) ; la devise de la ligne doit être compatible avec celle de l'actif (taux de change)</t>
+        </is>
+      </c>
+      <c r="J706" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="K706" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L706" s="2" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/patrimoine/assets/:assetId/valuations</t>
+        </is>
+      </c>
+      <c r="M706" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="N706" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O706" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Mes actifs &gt; fiche d'un actif, onglet Valeurs</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B707" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C707" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D707" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Valorisations d'un actif</t>
+        </is>
+      </c>
+      <c r="E707" s="2" t="inlineStr">
+        <is>
+          <t>Modifier une valorisation</t>
+        </is>
+      </c>
+      <c r="F707" s="2" t="inlineStr">
+        <is>
+          <t>Corriger une valeur enregistrée</t>
+        </is>
+      </c>
+      <c r="G707" s="2" t="inlineStr">
+        <is>
+          <t>Params `assetId`, `valuationId` ; body partiel `.strict()` (au moins un champ) : `valuatedAt`, `estimatedValue`, `currency`, `method`, `source`, `notes`</t>
+        </is>
+      </c>
+      <c r="H707" s="2" t="inlineStr">
+        <is>
+          <t>Valorisation mise à jour</t>
+        </is>
+      </c>
+      <c r="I707" s="2" t="inlineStr">
+        <is>
+          <t>La valorisation doit appartenir à l'actif (et à l'agence)</t>
+        </is>
+      </c>
+      <c r="J707" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="K707" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L707" s="2" t="inlineStr">
+        <is>
+          <t>PATCH /tenants/:tenantId/patrimoine/assets/:assetId/valuations/:valuationId</t>
+        </is>
+      </c>
+      <c r="M707" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="N707" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O707" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Mes actifs &gt; fiche d'un actif, onglet Valeurs</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B708" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C708" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D708" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Valorisations d'un actif</t>
+        </is>
+      </c>
+      <c r="E708" s="2" t="inlineStr">
+        <is>
+          <t>Supprimer une valorisation</t>
+        </is>
+      </c>
+      <c r="F708" s="2" t="inlineStr">
+        <is>
+          <t>Retirer une valeur enregistrée par erreur</t>
+        </is>
+      </c>
+      <c r="G708" s="2" t="inlineStr">
+        <is>
+          <t>Params `assetId`, `valuationId`</t>
+        </is>
+      </c>
+      <c r="H708" s="2" t="inlineStr">
+        <is>
+          <t>204 No Content</t>
+        </is>
+      </c>
+      <c r="I708" s="2" t="inlineStr">
+        <is>
+          <t>La valorisation doit appartenir à l'actif (et à l'agence)</t>
+        </is>
+      </c>
+      <c r="J708" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="K708" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L708" s="2" t="inlineStr">
+        <is>
+          <t>DELETE /tenants/:tenantId/patrimoine/assets/:assetId/valuations/:valuationId</t>
+        </is>
+      </c>
+      <c r="M708" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="N708" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O708" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Mes actifs &gt; fiche d'un actif, onglet Valeurs</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B709" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C709" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D709" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Parts détenues d'un actif</t>
+        </is>
+      </c>
+      <c r="E709" s="2" t="inlineStr">
+        <is>
+          <t>Lister les parts détenues d'un actif non immobilier</t>
+        </is>
+      </c>
+      <c r="F709" s="2" t="inlineStr">
+        <is>
+          <t>Voir quelles entités détentrices possèdent un actif non immobilier, et pour quelle part</t>
+        </is>
+      </c>
+      <c r="G709" s="2" t="inlineStr">
+        <is>
+          <t>Param `assetId`</t>
+        </is>
+      </c>
+      <c r="H709" s="2" t="inlineStr">
+        <is>
+          <t>Liste de parts (id, actif, entité, nom de l'entité, part en %, date d'effet, notes)</t>
+        </is>
+      </c>
+      <c r="I709" s="2" t="inlineStr">
+        <is>
+          <t>L'actif doit appartenir à l'agence ; 400 pour un actif immobilier (ses parts se gèrent depuis les entités détentrices)</t>
+        </is>
+      </c>
+      <c r="J709" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K709" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L709" s="2" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/patrimoine/assets/:assetId/holdings</t>
+        </is>
+      </c>
+      <c r="M709" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_VIEW (`requireAnyPropertyPermission`)</t>
+        </is>
+      </c>
+      <c r="N709" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O709" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Mes actifs &gt; fiche d'un actif non immobilier, onglet Détenteurs</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B710" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C710" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D710" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Parts détenues d'un actif</t>
+        </is>
+      </c>
+      <c r="E710" s="2" t="inlineStr">
+        <is>
+          <t>Poser ou mettre à jour la part d'une entité détentrice sur un actif</t>
+        </is>
+      </c>
+      <c r="F710" s="2" t="inlineStr">
+        <is>
+          <t>Attribuer, ou modifier, la part d'une entité détentrice sur un actif non immobilier</t>
+        </is>
+      </c>
+      <c r="G710" s="2" t="inlineStr">
+        <is>
+          <t>Params `assetId`, `entityId` ; body Zod `.strict()` : `sharePercent` (&gt;0 et &lt;=100), `effectiveFrom` facultative</t>
+        </is>
+      </c>
+      <c r="H710" s="2" t="inlineStr">
+        <is>
+          <t>Part créée ou mise à jour (id, actif, entité, nom de l'entité, part en %, date d'effet, notes)</t>
+        </is>
+      </c>
+      <c r="I710" s="2" t="inlineStr">
+        <is>
+          <t>L'actif et l'entité détentrice doivent appartenir à l'agence ; la somme des parts de l'actif ne peut pas dépasser 100 % (400) ; 400 pour un actif immobilier</t>
+        </is>
+      </c>
+      <c r="J710" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="K710" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L710" s="2" t="inlineStr">
+        <is>
+          <t>PUT /tenants/:tenantId/patrimoine/assets/:assetId/holdings/:entityId</t>
+        </is>
+      </c>
+      <c r="M710" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="N710" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O710" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Mes actifs &gt; fiche d'un actif non immobilier, onglet Détenteurs</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B711" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C711" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D711" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Parts détenues d'un actif</t>
+        </is>
+      </c>
+      <c r="E711" s="2" t="inlineStr">
+        <is>
+          <t>Retirer la part d'une entité détentrice</t>
+        </is>
+      </c>
+      <c r="F711" s="2" t="inlineStr">
+        <is>
+          <t>Supprimer la part d'une entité détentrice sur un actif non immobilier</t>
+        </is>
+      </c>
+      <c r="G711" s="2" t="inlineStr">
+        <is>
+          <t>Params `assetId`, `entityId`</t>
+        </is>
+      </c>
+      <c r="H711" s="2" t="inlineStr">
+        <is>
+          <t>204 No Content</t>
+        </is>
+      </c>
+      <c r="I711" s="2" t="inlineStr">
+        <is>
+          <t>L'actif doit appartenir à l'agence ; 404 si l'entité n'a pas de part sur l'actif ; 400 pour un actif immobilier</t>
+        </is>
+      </c>
+      <c r="J711" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="K711" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L711" s="2" t="inlineStr">
+        <is>
+          <t>DELETE /tenants/:tenantId/patrimoine/assets/:assetId/holdings/:entityId</t>
+        </is>
+      </c>
+      <c r="M711" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="N711" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O711" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Mes actifs &gt; fiche d'un actif non immobilier, onglet Détenteurs</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B712" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C712" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D712" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Dettes</t>
+        </is>
+      </c>
+      <c r="E712" s="2" t="inlineStr">
+        <is>
+          <t>Lister les dettes (adossées ou personnelles)</t>
+        </is>
+      </c>
+      <c r="F712" s="2" t="inlineStr">
+        <is>
+          <t>Consulter les dettes de l'agence : adossées à un actif (ou au bien d'un actif immobilier) ou personnelles</t>
+        </is>
+      </c>
+      <c r="G712" s="2" t="inlineStr">
+        <is>
+          <t>Query facultatives : `assetId` (dettes d'un actif) ou `unattached=true` (dettes personnelles) — les deux ne se combinent pas (400)</t>
+        </is>
+      </c>
+      <c r="H712" s="2" t="inlineStr">
+        <is>
+          <t>Liste de dettes, la plus récente d'abord (id, actif, bien, prêteur, capital emprunté, capital restant dû, taux, mensualité, devise, dates de début et de fin, statut `ACTIVE` / `CLOSED` / `DEFAULTED`) ; un prêt d'un bien sans actif n'apparaît pas</t>
+        </is>
+      </c>
+      <c r="I712" s="2" t="inlineStr">
+        <is>
+          <t>`assetId` doit désigner un actif de l'agence</t>
+        </is>
+      </c>
+      <c r="J712" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K712" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L712" s="2" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/patrimoine/debts</t>
+        </is>
+      </c>
+      <c r="M712" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_VIEW (`requireAnyPropertyPermission`)</t>
+        </is>
+      </c>
+      <c r="N712" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O712" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Valeur nette (panneau Dettes) ; Patrimoine &gt; Mes actifs &gt; fiche d'un actif, onglet Dettes</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B713" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C713" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D713" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Dettes</t>
+        </is>
+      </c>
+      <c r="E713" s="2" t="inlineStr">
+        <is>
+          <t>Enregistrer une dette</t>
+        </is>
+      </c>
+      <c r="F713" s="2" t="inlineStr">
+        <is>
+          <t>Saisir un prêt adossé à un actif ou une dette personnelle</t>
+        </is>
+      </c>
+      <c r="G713" s="2" t="inlineStr">
+        <is>
+          <t>Body Zod `.strict()` : `lender` (2 à 200 car.), `capitalAmount` (&gt;0), `remainingCapital` (&gt;=0), `interestRate` (&gt;=0, taux nul admis), `monthlyPayment` (&gt;=0), `startDate`, `endDate` (&gt;= début), `currency` et `status` facultatifs, `assetId` facultatif (absent = dette personnelle)</t>
+        </is>
+      </c>
+      <c r="H713" s="2" t="inlineStr">
+        <is>
+          <t>201 — dette créée ; pour l'actif d'un bien immobilier, elle est rattachée au bien</t>
+        </is>
+      </c>
+      <c r="I713" s="2" t="inlineStr">
+        <is>
+          <t>`assetId` doit appartenir à l'agence ; une dette personnelle est en XOF ; une dette adossée suit la devise de l'actif</t>
+        </is>
+      </c>
+      <c r="J713" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="K713" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L713" s="2" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/patrimoine/debts</t>
+        </is>
+      </c>
+      <c r="M713" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="N713" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O713" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Valeur nette (panneau Dettes) ; Patrimoine &gt; Mes actifs &gt; fiche d'un actif, onglet Dettes</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B714" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C714" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D714" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Dettes</t>
+        </is>
+      </c>
+      <c r="E714" s="2" t="inlineStr">
+        <is>
+          <t>Modifier une dette</t>
+        </is>
+      </c>
+      <c r="F714" s="2" t="inlineStr">
+        <is>
+          <t>Mettre à jour un prêt (capital restant dû, mensualité, statut…)</t>
+        </is>
+      </c>
+      <c r="G714" s="2" t="inlineStr">
+        <is>
+          <t>Param `debtId` ; body partiel `.strict()` (au moins un champ) : `lender`, `capitalAmount`, `remainingCapital`, `interestRate`, `monthlyPayment`, `currency`, `startDate`, `endDate`, `status` (l'actif rattaché ne change pas)</t>
+        </is>
+      </c>
+      <c r="H714" s="2" t="inlineStr">
+        <is>
+          <t>Dette mise à jour</t>
+        </is>
+      </c>
+      <c r="I714" s="2" t="inlineStr">
+        <is>
+          <t>La dette doit appartenir à l'agence ; un prêt d'un bien sans actif est introuvable par cette route</t>
+        </is>
+      </c>
+      <c r="J714" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="K714" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L714" s="2" t="inlineStr">
+        <is>
+          <t>PATCH /tenants/:tenantId/patrimoine/debts/:debtId</t>
+        </is>
+      </c>
+      <c r="M714" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="N714" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O714" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Valeur nette (panneau Dettes) ; Patrimoine &gt; Mes actifs &gt; fiche d'un actif, onglet Dettes</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B715" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C715" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D715" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Dettes</t>
+        </is>
+      </c>
+      <c r="E715" s="2" t="inlineStr">
+        <is>
+          <t>Supprimer une dette</t>
+        </is>
+      </c>
+      <c r="F715" s="2" t="inlineStr">
+        <is>
+          <t>Retirer une dette</t>
+        </is>
+      </c>
+      <c r="G715" s="2" t="inlineStr">
+        <is>
+          <t>Param `debtId`</t>
+        </is>
+      </c>
+      <c r="H715" s="2" t="inlineStr">
+        <is>
+          <t>204 No Content</t>
+        </is>
+      </c>
+      <c r="I715" s="2" t="inlineStr">
+        <is>
+          <t>La dette doit appartenir à l'agence ; un prêt d'un bien sans actif est introuvable par cette route</t>
+        </is>
+      </c>
+      <c r="J715" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="K715" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L715" s="2" t="inlineStr">
+        <is>
+          <t>DELETE /tenants/:tenantId/patrimoine/debts/:debtId</t>
+        </is>
+      </c>
+      <c r="M715" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="N715" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O715" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Valeur nette (panneau Dettes) ; Patrimoine &gt; Mes actifs &gt; fiche d'un actif, onglet Dettes</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B716" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C716" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D716" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Valeur nette</t>
+        </is>
+      </c>
+      <c r="E716" s="2" t="inlineStr">
+        <is>
+          <t>Consulter la valeur nette consolidée à une date</t>
+        </is>
+      </c>
+      <c r="F716" s="2" t="inlineStr">
+        <is>
+          <t>Voir la valeur nette de l'agence (actifs moins dettes, en XOF) à une date, avec la répartition par classe d'actif et les éléments écartés du calcul</t>
+        </is>
+      </c>
+      <c r="G716" s="2" t="inlineStr">
+        <is>
+          <t>Query facultative `asOf` (AAAA-MM-JJ, aujourd'hui par défaut ; date inexistante refusée)</t>
+        </is>
+      </c>
+      <c r="H716" s="2" t="inlineStr">
+        <is>
+          <t>Devise XOF, date, total des actifs, total des dettes, valeur nette, répartition par classe, actifs retenus (id, valeur en XOF, date de valorisation), actifs exclus avec la raison (`NO_VALUATION`, `MISSING_EXCHANGE_RATE`, `DISPOSED`, `ARCHIVED`), prêts exclus (`MISSING_EXCHANGE_RATE`)</t>
+        </is>
+      </c>
+      <c r="I716" s="2" t="inlineStr">
+        <is>
+          <t>Chaque actif retenu a au moins une valorisation datée au plus tard à la date demandée ; seuls les prêts au statut `ACTIVE` comptent ; un prêt d'un bien sans actif n'est pas compté ; les dettes personnelles le sont</t>
+        </is>
+      </c>
+      <c r="J716" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K716" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L716" s="2" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/patrimoine/net-worth</t>
+        </is>
+      </c>
+      <c r="M716" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_VIEW (`requireAnyPropertyPermission`)</t>
+        </is>
+      </c>
+      <c r="N716" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O716" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Valeur nette (/tenant/:tenantId/patrimoine/valeur-nette)</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B717" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C717" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D717" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Valeur nette</t>
+        </is>
+      </c>
+      <c r="E717" s="2" t="inlineStr">
+        <is>
+          <t>Consulter l'évolution mensuelle de la valeur nette</t>
+        </is>
+      </c>
+      <c r="F717" s="2" t="inlineStr">
+        <is>
+          <t>Suivre la valeur nette mois par mois</t>
+        </is>
+      </c>
+      <c r="G717" s="2" t="inlineStr">
+        <is>
+          <t>Query facultatives `from` et `to` (AAAA-MM-JJ), `step=month` ; par défaut les 12 derniers mois jusqu'à aujourd'hui ; 60 points au plus (400 au-delà ou si `from` suit `to`)</t>
+        </is>
+      </c>
+      <c r="H717" s="2" t="inlineStr">
+        <is>
+          <t>Série de points mensuels (date, total des actifs, total des dettes, valeur nette en XOF)</t>
+        </is>
+      </c>
+      <c r="I717" s="2" t="inlineStr">
+        <is>
+          <t>Voir « Consulter la valeur nette consolidée à une date » ; le capital restant dû des prêts est celui d'aujourd'hui pour tous les mois (voir Notes)</t>
+        </is>
+      </c>
+      <c r="J717" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K717" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L717" s="2" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/patrimoine/net-worth/history</t>
+        </is>
+      </c>
+      <c r="M717" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_VIEW (`requireAnyPropertyPermission`)</t>
+        </is>
+      </c>
+      <c r="N717" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O717" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Valeur nette (/tenant/:tenantId/patrimoine/valeur-nette) — courbe « Évolution de la valeur nette »</t>
         </is>
       </c>
     </row>
@@ -55079,7 +56538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -55572,6 +57031,28 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs (lot 1) : limites connues</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Quatre limites assumées au lot 1. (1) Les dépenses, travaux et documents ne sont gérés que pour les actifs immobiliers (depuis la fiche du bien) : un actif d'une autre classe n'a ni dépenses, ni travaux, ni documents. (2) L'historique mensuel de la valeur nette (`GET /net-worth/history`) utilise le capital restant dû d'aujourd'hui pour tous les mois passés, faute d'historique du capital ; les dettes des mois anciens sont donc approximées. (3) Les parts détenues d'un actif non immobilier (`PUT /assets/:assetId/holdings/:entityId`) ne sont pas verrouillées : deux PUT simultanés sur le même actif peuvent chacun passer le contrôle des 100 % et dépasser ce total. (4) La consolidation fiscale des entités détentrices ne couvre que l'immobilier.</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Décider si le lot suivant ajoute les dépenses/travaux/documents des autres classes, un historique du capital restant dû, un verrou sur les parts détenues et l'extension de la consolidation fiscale aux actifs non immobiliers. Aucune ligne du classeur n'est en statut « À vérifier » pour ces points : ce sont des limites de périmètre, pas des incertitudes.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
docs(patrimoine): wiki du lot 2 et spec du lot 3 (projections et simulations)
Wiki des fonctionnalites : 10 sous-fonctionnalites et une note (726 lignes).
Spec 025 : projections sur 1 a 30 ans, trois scenarios, simulations sur
copie des donnees, scenarios enregistres.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PxDVZM8akvCsSCfK3Cgg19
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -189,8 +189,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O717" headerRowCount="1">
-  <autoFilter ref="A1:O717"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O727" headerRowCount="1">
+  <autoFilter ref="A1:O727"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Domaine (regroupement agent)"/>
     <tableColumn id="2" name="Pack(s)"/>
@@ -242,8 +242,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotesPointsOuverts" displayName="NotesPointsOuverts" ref="A1:D23" headerRowCount="1">
-  <autoFilter ref="A1:D23"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotesPointsOuverts" displayName="NotesPointsOuverts" ref="A1:D24" headerRowCount="1">
+  <autoFilter ref="A1:D24"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Domaine"/>
     <tableColumn id="2" name="Sujet"/>
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O717"/>
+  <dimension ref="A1:O727"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -55933,6 +55933,776 @@
       <c r="O717" s="2" t="inlineStr">
         <is>
           <t>Patrimoine &gt; Valeur nette (/tenant/:tenantId/patrimoine/valeur-nette) — courbe « Évolution de la valeur nette »</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B718" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C718" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D718" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Valorisation et fiabilité</t>
+        </is>
+      </c>
+      <c r="E718" s="2" t="inlineStr">
+        <is>
+          <t>Suggérer la valeur d'un actif par les caractéristiques de sa classe</t>
+        </is>
+      </c>
+      <c r="F718" s="2" t="inlineStr">
+        <is>
+          <t>Obtenir une valeur calculée à partir des caractéristiques de l'actif (amortissement d'un véhicule ou équipement, quote-part d'une entreprise, quantité × coût unitaire d'un stock, épargne capitalisée, créance décotée, quantité × valeur unitaire en agriculture), sans rien enregistrer</t>
+        </is>
+      </c>
+      <c r="G718" s="2" t="inlineStr">
+        <is>
+          <t>Param `assetId` ; body Zod `.strict()` facultatif : `asOf` (AAAA-MM-JJ, aujourd'hui par défaut) ; les caractéristiques lues sont celles de l'actif (détails de sa classe, coût et date d'acquisition, dernière valorisation)</t>
+        </is>
+      </c>
+      <c r="H718" s="2" t="inlineStr">
+        <is>
+          <t>Soit `ok: true` avec le montant (arrondi au franc), la devise de l'actif, la méthode (`DEPRECIATION_LINEAR`, `DEPRECIATION_DECLINING`, `EQUITY_SHARE`, `UNIT_COST`, `ACCRUED_SAVINGS`, `DISCOUNTED_CLAIM` ou `UNIT_VALUE`) et les hypothèses retenues ; soit `ok: false` avec la liste des champs manquants (liste vide pour l'immobilier, les biens meubles et « autre », qui se valorisent par saisie ou expertise ; `balance` pour un compte, dont le solde se saisit) — jamais de valeur inventée. Aucune écriture, aucune ligne d'audit</t>
+        </is>
+      </c>
+      <c r="I718" s="2" t="inlineStr">
+        <is>
+          <t>Consulter la fiche d'un actif ; Renseigner les caractéristiques de valorisation propres à une classe</t>
+        </is>
+      </c>
+      <c r="J718" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K718" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L718" s="2" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/patrimoine/assets/:assetId/valuations/suggest</t>
+        </is>
+      </c>
+      <c r="M718" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_VIEW (`requireAnyPropertyPermission`)</t>
+        </is>
+      </c>
+      <c r="N718" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O718" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Mes actifs &gt; fiche d'un actif, onglet Valeurs (/tenant/:tenantId/patrimoine/actifs/:assetId) — bouton « Calculer une valeur »</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B719" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C719" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D719" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Valorisation et fiabilité</t>
+        </is>
+      </c>
+      <c r="E719" s="2" t="inlineStr">
+        <is>
+          <t>Enregistrer la valeur suggérée après confirmation</t>
+        </is>
+      </c>
+      <c r="F719" s="2" t="inlineStr">
+        <is>
+          <t>Transformer la valeur calculée en valorisation de l'historique, après une confirmation explicite ; le bouton « Modifier » du résultat ouvre le formulaire de valorisation pré-rempli plutôt que d'enregistrer</t>
+        </is>
+      </c>
+      <c r="G719" s="2" t="inlineStr">
+        <is>
+          <t>Résultat d'une suggestion (`ok: true`) ; clic sur « Enregistrer cette valeur », puis confirmation « Enregistrer cette valeur de {montant} ? » (« Une valeur datée d'aujourd'hui sera ajoutée à l'historique. ») ; le corps envoyé est `valuatedAt` (aujourd'hui), `estimatedValue` (montant suggéré), `currency` et `method` (méthode suggérée)</t>
+        </is>
+      </c>
+      <c r="H719" s="2" t="inlineStr">
+        <is>
+          <t>Valorisation créée avec la méthode suggérée (201), message « Valeur ajoutée. », historique et valeur courante rafraîchis ; sa fiabilité est calculée par le serveur (voir « Consulter la fiabilité d'une valorisation »)</t>
+        </is>
+      </c>
+      <c r="I719" s="2" t="inlineStr">
+        <is>
+          <t>Suggérer la valeur d'un actif par les caractéristiques de sa classe ; Ajouter une valorisation</t>
+        </is>
+      </c>
+      <c r="J719" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="K719" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L719" s="2" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/patrimoine/assets/:assetId/valuations (route existante « Ajouter une valorisation »)</t>
+        </is>
+      </c>
+      <c r="M719" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="N719" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O719" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Mes actifs &gt; fiche d'un actif, onglet Valeurs — résultat de « Calculer une valeur », bouton « Enregistrer cette valeur »</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B720" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C720" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D720" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Valorisation et fiabilité</t>
+        </is>
+      </c>
+      <c r="E720" s="2" t="inlineStr">
+        <is>
+          <t>Consulter la fiabilité d'une valorisation</t>
+        </is>
+      </c>
+      <c r="F720" s="2" t="inlineStr">
+        <is>
+          <t>Savoir dans quelle mesure une valeur est fiable : niveau Élevée, Moyenne ou Faible et raisons (méthode, présence d'une source, ancienneté, statut juridique d'un bien immobilier)</t>
+        </is>
+      </c>
+      <c r="G720" s="2" t="inlineStr">
+        <is>
+          <t>Aucune saisie : la fiabilité n'est jamais fournie par le client (le corps d'une valorisation est `.strict()`) ; le serveur la calcule à l'écriture et la recalcule à chaque lecture à la date du jour (ancienneté) avec le statut juridique courant de l'actif</t>
+        </is>
+      </c>
+      <c r="H720" s="2" t="inlineStr">
+        <is>
+          <t>Par valorisation : `reliability` (`HIGH`, `MEDIUM`, `LOW`) et `reliabilityReasons` (clés stables traduites côté écran : saisie manuelle avec ou sans source, expertise, solde, valeur calculée, valeur ancienne, valeur très ancienne, statut juridique fragile ou non renseigné) ; pour l'actif, la fiabilité de sa valeur courante (`currentValue.reliability`). Règle : expertise et solde partent de Élevée, saisie manuelle avec source de Moyenne, sans source de Faible, valeur calculée de Moyenne ; un niveau de perdu au-delà du seuil de péremption de la classe, deux au-delà du double ; pour l'immobilier, plafond Faible si le statut est fragile, Moyen s'il n'est pas renseigné. Une ligne d'avant le lot 2 (fiabilité jamais stockée) reste « inconnue » et compte comme peu fiable</t>
+        </is>
+      </c>
+      <c r="I720" s="2" t="inlineStr">
+        <is>
+          <t>Lister les valorisations d'un actif ; Consulter la fiche d'un actif</t>
+        </is>
+      </c>
+      <c r="J720" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K720" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L720" s="2" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/patrimoine/assets/:assetId/valuations ; GET /tenants/:tenantId/patrimoine/assets/:assetId ; GET /tenants/:tenantId/patrimoine/assets</t>
+        </is>
+      </c>
+      <c r="M720" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_VIEW (`requireAnyPropertyPermission`)</t>
+        </is>
+      </c>
+      <c r="N720" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O720" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Mes actifs (badge sur la valeur de chaque actif) ; fiche d'un actif (badge sur la valeur courante) ; onglet Valeurs (colonne « Fiabilité » de l'historique, avec les raisons)</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B721" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C721" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D721" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Valorisation et fiabilité</t>
+        </is>
+      </c>
+      <c r="E721" s="2" t="inlineStr">
+        <is>
+          <t>Repérer une valeur périmée selon un seuil par classe</t>
+        </is>
+      </c>
+      <c r="F721" s="2" t="inlineStr">
+        <is>
+          <t>Voir d'un coup d'oeil quels actifs ont une valeur trop ancienne pour leur classe, sans réviser tous les actifs</t>
+        </is>
+      </c>
+      <c r="G721" s="2" t="inlineStr">
+        <is>
+          <t>Aucune saisie ; seuil en mois propre à la classe, fixé côté serveur : comptes et mobile money 3, stocks 3, épargne et placements 6, créances 6, agriculture et élevage 6, véhicules et équipements 12, entreprises et parts de sociétés 12, immobilier 24, biens meubles de valeur 24, autre 12</t>
+        </is>
+      </c>
+      <c r="H721" s="2" t="inlineStr">
+        <is>
+          <t>Booléen `stale` sur chaque actif : vrai si la dernière valorisation dépasse le seuil de sa classe, ou si l'actif n'a aucune valorisation ; pastille « Valeur périmée » dans la liste des actifs et sur la fiche</t>
+        </is>
+      </c>
+      <c r="I721" s="2" t="inlineStr">
+        <is>
+          <t>Lister les actifs ; Ajouter une valorisation</t>
+        </is>
+      </c>
+      <c r="J721" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K721" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L721" s="2" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/patrimoine/assets ; GET /tenants/:tenantId/patrimoine/assets/:assetId</t>
+        </is>
+      </c>
+      <c r="M721" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_VIEW (`requireAnyPropertyPermission`)</t>
+        </is>
+      </c>
+      <c r="N721" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O721" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Mes actifs (pastille « Valeur périmée » sur chaque actif concerné) ; fiche d'un actif</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B722" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C722" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D722" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Valorisation et fiabilité</t>
+        </is>
+      </c>
+      <c r="E722" s="2" t="inlineStr">
+        <is>
+          <t>Renseigner le statut juridique d'un actif immobilier</t>
+        </is>
+      </c>
+      <c r="F722" s="2" t="inlineStr">
+        <is>
+          <t>Qualifier le titre du bien (titre foncier, ACD, certificat de propriété ou de détention, lettre d'attribution, attestation villageoise ou coutumière, autre) : il conditionne le plafond de fiabilité de la valeur</t>
+        </is>
+      </c>
+      <c r="G722" s="2" t="inlineStr">
+        <is>
+          <t>Champ facultatif `details.legalStatus` du formulaire d'un actif immobilier : `TITRE_FONCIER`, `ACD`, `CERTIFICAT_PROPRIETE`, `LETTRE_ATTRIBUTION`, `ATTESTATION_COUTUMIERE` ou `AUTRE` (les détails d'un actif immobilier n'ont pas d'autre champ) ; par PATCH, corps partiel `.strict()` avec `details`</t>
+        </is>
+      </c>
+      <c r="H722" s="2" t="inlineStr">
+        <is>
+          <t>Actif mis à jour avec son statut juridique ; le formulaire affiche « Statut juridique fragile : la fiabilité de la valeur est plafonnée. » pour la lettre d'attribution et l'attestation villageoise ou coutumière (statuts fragiles : fiabilité plafonnée à Faible) ; statut non renseigné : fiabilité plafonnée à Moyenne, raison « Statut juridique non renseigné » ; « Autre » ne plafonne pas</t>
+        </is>
+      </c>
+      <c r="I722" s="2" t="inlineStr">
+        <is>
+          <t>Modifier un actif ; Créer un actif</t>
+        </is>
+      </c>
+      <c r="J722" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="K722" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L722" s="2" t="inlineStr">
+        <is>
+          <t>PATCH /tenants/:tenantId/patrimoine/assets/:assetId (champ `details`) ; POST /tenants/:tenantId/patrimoine/assets pour la création</t>
+        </is>
+      </c>
+      <c r="M722" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="N722" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O722" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Mes actifs &gt; formulaire d'actif (bouton « Ajouter un actif », ou « Modifier » de l'onglet Informations d'une fiche d'actif immobilier), champ « Statut juridique »</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B723" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C723" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D723" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Valorisation et fiabilité</t>
+        </is>
+      </c>
+      <c r="E723" s="2" t="inlineStr">
+        <is>
+          <t>Renseigner les caractéristiques de valorisation propres à une classe</t>
+        </is>
+      </c>
+      <c r="F723" s="2" t="inlineStr">
+        <is>
+          <t>Saisir dans l'actif les paramètres qui permettent de calculer sa valeur : véhicules et équipements (durée d'utilité en années, valeur résiduelle en %, méthode d'amortissement linéaire ou dégressif, taux dégressif en %), entreprises (valeur de l'entreprise, ou résultat net et multiple de résultat), stocks (décote en %), créances (capital et recouvrabilité en %), agriculture et élevage (valeur unitaire, avec surface ou effectif), épargne et placements (capital et taux attendu)</t>
+        </is>
+      </c>
+      <c r="G723" s="2" t="inlineStr">
+        <is>
+          <t>Champs facultatifs de `details` selon la classe, validés par un schéma `.strict()` : `usefulLifeYears` (1 à 50), `residualValuePercent`, `depreciationMethod`, `decliningRatePercent`, `companyValue`, `netIncome`, `earningsMultiple` (&gt;0, 100 au plus), `writeDownPercent`, `principal`, `collectibilityPercent`, `unitValue`, `expectedRatePercent` ; pourcentages de 0 à 100, montants &gt;= 0</t>
+        </is>
+      </c>
+      <c r="H723" s="2" t="inlineStr">
+        <is>
+          <t>Actif créé (201) ou mis à jour avec ces détails ; ils alimentent « Suggérer la valeur d'un actif » (sans eux, la suggestion renvoie la liste des champs manquants avec le lien « Compléter les informations de l'actif »)</t>
+        </is>
+      </c>
+      <c r="I723" s="2" t="inlineStr">
+        <is>
+          <t>Créer un actif ; Modifier un actif</t>
+        </is>
+      </c>
+      <c r="J723" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="K723" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L723" s="2" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/patrimoine/assets ; PATCH /tenants/:tenantId/patrimoine/assets/:assetId</t>
+        </is>
+      </c>
+      <c r="M723" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="N723" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O723" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Mes actifs &gt; formulaire d'actif (« Ajouter un actif » ou « Modifier » de l'onglet Informations)</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B724" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C724" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D724" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Valorisation et fiabilité</t>
+        </is>
+      </c>
+      <c r="E724" s="2" t="inlineStr">
+        <is>
+          <t>Consulter la part de la valeur nette reposant sur des valeurs peu fiables</t>
+        </is>
+      </c>
+      <c r="F724" s="2" t="inlineStr">
+        <is>
+          <t>Mesurer le risque d'imprécision de la valeur nette : quelle part des actifs retenus repose sur des valeurs de fiabilité Faible ou inconnue</t>
+        </is>
+      </c>
+      <c r="G724" s="2" t="inlineStr">
+        <is>
+          <t>Aucune saisie ; même requête que « Consulter la valeur nette consolidée à une date » (`asOf` facultative)</t>
+        </is>
+      </c>
+      <c r="H724" s="2" t="inlineStr">
+        <is>
+          <t>Champ `lowReliabilityShare` : pourcentage (arrondi) du total des actifs retenus, en XOF, dont la valeur est de fiabilité Faible ou sans fiabilité connue ; 0 si le total des actifs est nul. L'écran affiche la ligne « {part} % de la valeur repose sur des valeurs peu fiables » avec le lien « Voir les actifs » seulement quand la part est supérieure à 0</t>
+        </is>
+      </c>
+      <c r="I724" s="2" t="inlineStr">
+        <is>
+          <t>Consulter la valeur nette consolidée à une date ; Consulter la fiabilité d'une valorisation</t>
+        </is>
+      </c>
+      <c r="J724" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K724" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L724" s="2" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/patrimoine/net-worth (champ `lowReliabilityShare`)</t>
+        </is>
+      </c>
+      <c r="M724" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_VIEW (`requireAnyPropertyPermission`)</t>
+        </is>
+      </c>
+      <c r="N724" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O724" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Valeur nette (/tenant/:tenantId/patrimoine/valeur-nette) — ligne d'alerte sous les indicateurs</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B725" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C725" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D725" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Cycle de vie</t>
+        </is>
+      </c>
+      <c r="E725" s="2" t="inlineStr">
+        <is>
+          <t>Créer automatiquement l'actif immobilier d'un bien</t>
+        </is>
+      </c>
+      <c r="F725" s="2" t="inlineStr">
+        <is>
+          <t>Faire apparaître un bien dans le patrimoine multi-actifs (liste des actifs, valeur nette) sans geste de l'utilisateur, dès qu'il porte une donnée patrimoniale</t>
+        </is>
+      </c>
+      <c r="G725" s="2" t="inlineStr">
+        <is>
+          <t>Aucune saisie propre : déclenchée par la première valorisation du bien, son premier prêt, sa première part détenue (entité détentrice) ou la bascule d'un lot de chantier au patrimoine</t>
+        </is>
+      </c>
+      <c r="H725" s="2" t="inlineStr">
+        <is>
+          <t>Actif de classe immobilier, statut actif, devise XOF, lié au bien et nommé d'après sa référence interne (à défaut son titre, sinon « Bien ») ; opération idempotente, sans doublon même en cas de requêtes concurrentes ; no-op si le bien n'appartient pas à l'agence ; les valorisations, prêts et parts existants restent rattachés au bien</t>
+        </is>
+      </c>
+      <c r="I725" s="2" t="inlineStr">
+        <is>
+          <t>Ajouter une valorisation à un bien ; Enregistrer un prêt d'un bien ; Poser les parts détenues d'un bien ; Basculer un lot au patrimoine</t>
+        </is>
+      </c>
+      <c r="J725" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — permission de la route déclenchante</t>
+        </is>
+      </c>
+      <c r="K725" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L725" s="2" t="inlineStr">
+        <is>
+          <t>Sans objet (effet de bord) : POST /tenants/:tenantId/properties/:propertyId/valuations ; POST /tenants/:tenantId/properties/:propertyId/loans ; POST /tenants/:tenantId/patrimoine/entities/:entityId/holdings ; PUT /tenants/:tenantId/patrimoine/properties/:propertyId/holdings ; POST /tenants/:tenantId/finance/sites/:siteId/lots/:lotId/capitalize</t>
+        </is>
+      </c>
+      <c r="M725" s="2" t="inlineStr">
+        <is>
+          <t>Celle de la route déclenchante (PROPERTIES_EDIT ; FINANCE_DOCUMENTS_VALIDATE pour la bascule d'un lot)</t>
+        </is>
+      </c>
+      <c r="N725" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O725" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Mes actifs (l'actif apparaît après l'action déclenchante)</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B726" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C726" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D726" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Cycle de vie</t>
+        </is>
+      </c>
+      <c r="E726" s="2" t="inlineStr">
+        <is>
+          <t>Supprimer un bien avec son actif immobilier</t>
+        </is>
+      </c>
+      <c r="F726" s="2" t="inlineStr">
+        <is>
+          <t>Ne laisser aucun actif orphelin ni aucune valeur fantôme dans la valeur nette lorsqu'un bien est supprimé</t>
+        </is>
+      </c>
+      <c r="G726" s="2" t="inlineStr">
+        <is>
+          <t>Aucune saisie propre : effet de la suppression définitive d'un bien</t>
+        </is>
+      </c>
+      <c r="H726" s="2" t="inlineStr">
+        <is>
+          <t>L'actif immobilier lié au bien est supprimé avec lui (clé étrangère en cascade sur `assets.property_id`), comme les valorisations, prêts et parts du bien (tous supprimés en cascade avec lui) ; le bien disparaît donc de la valeur nette</t>
+        </is>
+      </c>
+      <c r="I726" s="2" t="inlineStr">
+        <is>
+          <t>Supprimer un bien</t>
+        </is>
+      </c>
+      <c r="J726" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="K726" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L726" s="2" t="inlineStr">
+        <is>
+          <t>DELETE /tenants/:tenantId/properties/:id (route existante « Supprimer un bien »)</t>
+        </is>
+      </c>
+      <c r="M726" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="N726" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O726" s="2" t="inlineStr">
+        <is>
+          <t>Biens &gt; Toutes les propriétés &gt; fiche bien</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B727" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C727" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D727" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Cycle de vie</t>
+        </is>
+      </c>
+      <c r="E727" s="2" t="inlineStr">
+        <is>
+          <t>Refuser la suppression d'une entité détentrice qui porte encore des biens ou des actifs</t>
+        </is>
+      </c>
+      <c r="F727" s="2" t="inlineStr">
+        <is>
+          <t>Empêcher qu'une entité détentrice supprimée détache silencieusement les actifs qu'elle possède (la référence de l'actif passerait à vide)</t>
+        </is>
+      </c>
+      <c r="G727" s="2" t="inlineStr">
+        <is>
+          <t>Param `entityId`</t>
+        </is>
+      </c>
+      <c r="H727" s="2" t="inlineStr">
+        <is>
+          <t>409 « Cette entité porte encore des rattachements à des biens ou actifs : détachez-les avant de la supprimer. » si l'entité a des parts sur des biens ou porte des actifs ; sinon 204 No Content</t>
+        </is>
+      </c>
+      <c r="I727" s="2" t="inlineStr">
+        <is>
+          <t>Supprimer une entité détentrice</t>
+        </is>
+      </c>
+      <c r="J727" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="K727" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L727" s="2" t="inlineStr">
+        <is>
+          <t>DELETE /tenants/:tenantId/patrimoine/entities/:entityId (route existante « Supprimer une entité détentrice »)</t>
+        </is>
+      </c>
+      <c r="M727" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="N727" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O727" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Entités détentrices &gt; fiche entité</t>
         </is>
       </c>
     </row>
@@ -56538,7 +57308,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -57053,6 +57823,28 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — règles de gestion</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Règles transverses du patrimoine multi-actifs, communes aux écrans et routes décrits ci-dessus. (1) Plafonds par agence : 500 actifs non archivés et 1 000 valorisations par actif ; au-delà, 409. (2) Toute écriture sur un actif archivé est refusée (409). (3) Le changement de devise d'un actif est refusé (409) tant que des lignes (valorisations, dettes) existent dans une autre devise. (4) Les écritures sont auditées (clés `PATRIMOINE_ASSET_CREATED`, `_UPDATED`, `_DISPOSED`, `_ARCHIVED`, `PATRIMOINE_VALUATION_CREATED`, `_UPDATED`, `_DELETED`, `PATRIMOINE_DEBT_CREATED`, `_UPDATED`, `_DELETED`, `PATRIMOINE_HOLDING_SET`, `PATRIMOINE_HOLDING_DELETED`) ; le journal ne porte que des identifiants, types, classes et noms de champs, jamais un montant, un nom ou une note ; la suggestion de valeur n'écrit rien et n'est pas auditée. (5) La fiabilité d'une valorisation est calculée par le serveur (à l'écriture, puis recalculée à la lecture selon l'ancienneté et le statut juridique courant) et n'est jamais fournie par le client. (6) La liste des statuts juridiques fonciers (titre foncier, ACD, certificat de propriété ou de détention, lettre d'attribution, attestation villageoise ou coutumière, autre) et le classement de la lettre d'attribution et de l'attestation villageoise ou coutumière comme statuts fragiles sont une hypothèse métier.</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Faire valider par un juriste local la liste des statuts juridiques fonciers et le classement « fragile » avant toute communication grand public (page vitrine, supports commerciaux). Les autres règles sont vérifiées dans le code (`services/patrimoine-assets/limits.ts`, `audit.ts`, `lib/patrimoine/assets/reliability.ts`) ; aucune ligne du classeur n'est en statut « À vérifier » pour ces points.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
docs(patrimoine): wiki du lot 3, projections et simulations
11 sous-fonctionnalites, une note, trois lignes du lot 2 precisees.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PxDVZM8akvCsSCfK3Cgg19
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -189,8 +189,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O727" headerRowCount="1">
-  <autoFilter ref="A1:O727"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O738" headerRowCount="1">
+  <autoFilter ref="A1:O738"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Domaine (regroupement agent)"/>
     <tableColumn id="2" name="Pack(s)"/>
@@ -242,8 +242,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotesPointsOuverts" displayName="NotesPointsOuverts" ref="A1:D24" headerRowCount="1">
-  <autoFilter ref="A1:D24"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotesPointsOuverts" displayName="NotesPointsOuverts" ref="A1:D25" headerRowCount="1">
+  <autoFilter ref="A1:D25"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Domaine"/>
     <tableColumn id="2" name="Sujet"/>
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O727"/>
+  <dimension ref="A1:O738"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -55974,7 +55974,7 @@
       </c>
       <c r="H718" s="2" t="inlineStr">
         <is>
-          <t>Soit `ok: true` avec le montant (arrondi au franc), la devise de l'actif, la méthode (`DEPRECIATION_LINEAR`, `DEPRECIATION_DECLINING`, `EQUITY_SHARE`, `UNIT_COST`, `ACCRUED_SAVINGS`, `DISCOUNTED_CLAIM` ou `UNIT_VALUE`) et les hypothèses retenues ; soit `ok: false` avec la liste des champs manquants (liste vide pour l'immobilier, les biens meubles et « autre », qui se valorisent par saisie ou expertise ; `balance` pour un compte, dont le solde se saisit) — jamais de valeur inventée. Aucune écriture, aucune ligne d'audit</t>
+          <t>Soit `ok: true` avec le montant (arrondi au franc), la devise de l'actif, la méthode (`DEPRECIATION_LINEAR`, `DEPRECIATION_DECLINING`, `EQUITY_SHARE`, `UNIT_COST`, `ACCRUED_SAVINGS`, `DISCOUNTED_CLAIM` ou `UNIT_VALUE`) et les hypothèses retenues ; soit `ok: false` avec la liste des champs manquants (liste vide pour l'immobilier, les biens meubles et « autre », qui se valorisent par saisie ou expertise ; `balance` pour un compte, dont le solde se saisit) — jamais de valeur inventée ; soit `ok: false` avec un `reason` et une liste `missing` vide quand le calcul aboutit à un refus motivé : valeur nulle (`ZERO_VALUE`), montant non fini ou hors limites, au-delà de 999 999 999 999,99 (`OUT_OF_RANGE`), ou date d'acquisition postérieure à la date de calcul (`ACQUISITION_DATE_IN_FUTURE`, pour les classes qui l'utilisent : véhicule ou équipement, épargne sans valorisation antérieure) ; l'écran affiche un message explicatif pour chaque cas. Aucune écriture, aucune ligne d'audit</t>
         </is>
       </c>
       <c r="I718" s="2" t="inlineStr">
@@ -56046,12 +56046,12 @@
       </c>
       <c r="G719" s="2" t="inlineStr">
         <is>
-          <t>Résultat d'une suggestion (`ok: true`) ; clic sur « Enregistrer cette valeur », puis confirmation « Enregistrer cette valeur de {montant} ? » (« Une valeur datée d'aujourd'hui sera ajoutée à l'historique. ») ; le corps envoyé est `valuatedAt` (aujourd'hui), `estimatedValue` (montant suggéré), `currency` et `method` (méthode suggérée)</t>
+          <t>Résultat d'une suggestion (`ok: true`) ; clic sur « Enregistrer cette valeur », puis confirmation « Enregistrer cette valeur de {montant} ? » (« Une valeur datée d'aujourd'hui sera ajoutée à l'historique. ») ; le corps envoyé est `valuatedAt` (aujourd'hui), `estimatedValue` (montant suggéré), `currency` et `method` (méthode suggérée, revérifiée par le serveur à l'écriture)</t>
         </is>
       </c>
       <c r="H719" s="2" t="inlineStr">
         <is>
-          <t>Valorisation créée avec la méthode suggérée (201), message « Valeur ajoutée. », historique et valeur courante rafraîchis ; sa fiabilité est calculée par le serveur (voir « Consulter la fiabilité d'une valorisation »)</t>
+          <t>Valorisation créée (201) ; la méthode calculée n'est conservée que si le serveur retrouve le montant (recalcul à la date de la ligne, tolérance de 1 en XOF ou de 0,01 dans une autre devise) : si le montant a été modifié, la ligne repasse en saisie manuelle (`MANUAL`), message « Valeur ajoutée. », historique et valeur courante rafraîchis ; sa fiabilité est calculée par le serveur (voir « Consulter la fiabilité d'une valorisation »)</t>
         </is>
       </c>
       <c r="I719" s="2" t="inlineStr">
@@ -56128,7 +56128,7 @@
       </c>
       <c r="H720" s="2" t="inlineStr">
         <is>
-          <t>Par valorisation : `reliability` (`HIGH`, `MEDIUM`, `LOW`) et `reliabilityReasons` (clés stables traduites côté écran : saisie manuelle avec ou sans source, expertise, solde, valeur calculée, valeur ancienne, valeur très ancienne, statut juridique fragile ou non renseigné) ; pour l'actif, la fiabilité de sa valeur courante (`currentValue.reliability`). Règle : expertise et solde partent de Élevée, saisie manuelle avec source de Moyenne, sans source de Faible, valeur calculée de Moyenne ; un niveau de perdu au-delà du seuil de péremption de la classe, deux au-delà du double ; pour l'immobilier, plafond Faible si le statut est fragile, Moyen s'il n'est pas renseigné. Une ligne d'avant le lot 2 (fiabilité jamais stockée) reste « inconnue » et compte comme peu fiable</t>
+          <t>Par valorisation : `reliability` (`HIGH`, `MEDIUM`, `LOW`) et `reliabilityReasons` (clés stables traduites côté écran : saisie manuelle avec ou sans source, expertise, solde, valeur calculée, valeur ancienne, valeur très ancienne, statut juridique fragile ou non renseigné) ; pour l'actif, la fiabilité de sa valeur courante (`currentValue.reliability`). Règle : expertise et solde partent de Élevée, saisie manuelle avec source de Moyenne, sans source de Faible (une estimation de marché est traitée comme une saisie manuelle : même niveau, avec ou sans source), valeur calculée de Moyenne ; une expertise exige une source : sans source, l'écriture est refusée avec une erreur de validation sur `source` ; un niveau de perdu au-delà du seuil de péremption de la classe, deux au-delà du double ; pour l'immobilier, plafond Faible si le statut est fragile, Moyen s'il n'est pas renseigné. Une ligne d'avant le lot 2 (fiabilité jamais stockée) reste « inconnue » et compte comme peu fiable</t>
         </is>
       </c>
       <c r="I720" s="2" t="inlineStr">
@@ -56703,6 +56703,853 @@
       <c r="O727" s="2" t="inlineStr">
         <is>
           <t>Patrimoine &gt; Entités détentrices &gt; fiche entité</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B728" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C728" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D728" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Projections et simulations</t>
+        </is>
+      </c>
+      <c r="E728" s="2" t="inlineStr">
+        <is>
+          <t>Projeter la valeur nette sur 1 à 30 ans</t>
+        </is>
+      </c>
+      <c r="F728" s="2" t="inlineStr">
+        <is>
+          <t>Voir comment la valeur nette de l'agence évolue année par année selon trois scénarios (prudent, central, optimiste), avec des hypothèses de croissance par classe d'actifs et d'inflation modifiables ; aucune donnée réelle n'est écrite</t>
+        </is>
+      </c>
+      <c r="G728" s="2" t="inlineStr">
+        <is>
+          <t>Body Zod `.strict()` : `horizonYears` (entier de 1 à 30, obligatoire ; 10 par défaut à l'écran), `baseScenario` (`PRUDENT`, `CENTRAL` ou `OPTIMISTIC`, obligatoire ; Central par défaut à l'écran), `assumptions` facultatif `{ growthPercentByClass (croissance annuelle nominale de −50 à 100 % pour chacune des 10 classes ; une classe absente prend le taux du scénario de base), inflationPercent (0 à 100) }`</t>
+        </is>
+      </c>
+      <c r="H728" s="2" t="inlineStr">
+        <is>
+          <t>`assumptionsUsed` (hypothèses complètes retenues) et `base` : `points` (année 0 = aujourd'hui puis une ligne par année jusqu'à l'horizon : total des actifs, total des dettes, valeur nette, valeur réelle en pouvoir d'achat d'aujourd'hui, ventilation par classe, en XOF) et `warnings`. Chaque année : croissance composée par classe (un véhicule ou équipement s'amortit selon ses caractéristiques, une épargne suit son taux attendu), 12 mensualités de chaque dette active. Actifs cédés, archivés ou sans valeur exclus. Aucune écriture, aucune ligne d'audit</t>
+        </is>
+      </c>
+      <c r="I728" s="2" t="inlineStr">
+        <is>
+          <t>Consulter la valeur nette consolidée à une date ; Consulter la fiabilité d'une valorisation ; Lister les dettes (adossées ou personnelles)</t>
+        </is>
+      </c>
+      <c r="J728" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K728" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L728" s="2" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/patrimoine/projections</t>
+        </is>
+      </c>
+      <c r="M728" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_VIEW (`requireAnyPropertyPermission`)</t>
+        </is>
+      </c>
+      <c r="N728" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O728" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Projections (/tenant/:tenantId/patrimoine/projections) — carte « Valeur nette par année », « Tableau annuel », panneau « Hypothèses » (boutons « Appliquer les hypothèses » et « Rétablir les hypothèses par défaut »)</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B729" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C729" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D729" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Projections et simulations</t>
+        </is>
+      </c>
+      <c r="E729" s="2" t="inlineStr">
+        <is>
+          <t>Comparer les trois scénarios sur le même horizon</t>
+        </is>
+      </c>
+      <c r="F729" s="2" t="inlineStr">
+        <is>
+          <t>Afficher sur une même courbe les trajectoires de valeur nette des scénarios prudent, central et optimiste</t>
+        </is>
+      </c>
+      <c r="G729" s="2" t="inlineStr">
+        <is>
+          <t>Même body que la projection avec `compareScenarios: true` ; les surcharges d'hypothèses éventuelles s'appliquent aux trois scénarios</t>
+        </is>
+      </c>
+      <c r="H729" s="2" t="inlineStr">
+        <is>
+          <t>Champ `byScenario` : pour chaque clé `PRUDENT`, `CENTRAL`, `OPTIMISTIC`, les `points` et les `warnings` de la projection à cet horizon. Aucune écriture</t>
+        </is>
+      </c>
+      <c r="I729" s="2" t="inlineStr">
+        <is>
+          <t>Projeter la valeur nette sur 1 à 30 ans</t>
+        </is>
+      </c>
+      <c r="J729" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K729" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L729" s="2" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/patrimoine/projections (champ `compareScenarios`)</t>
+        </is>
+      </c>
+      <c r="M729" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_VIEW (`requireAnyPropertyPermission`)</t>
+        </is>
+      </c>
+      <c r="N729" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O729" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Projections (/tenant/:tenantId/patrimoine/projections) — interrupteur « Comparer les trois scénarios » (trois courbes « Scénario Prudent / Central / Optimiste »)</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B730" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C730" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D730" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Projections et simulations</t>
+        </is>
+      </c>
+      <c r="E730" s="2" t="inlineStr">
+        <is>
+          <t>Simuler des opérations sur une copie du patrimoine</t>
+        </is>
+      </c>
+      <c r="F730" s="2" t="inlineStr">
+        <is>
+          <t>Tester l'effet d'une vente, d'un achat, d'un emprunt, d'un remboursement anticipé ou d'une épargne mensuelle sur la valeur nette future, sans modifier aucune donnée réelle ; le calcul travaille sur une copie en mémoire</t>
+        </is>
+      </c>
+      <c r="G730" s="2" t="inlineStr">
+        <is>
+          <t>Champ `operations` (50 au plus, chacune avec `year` de 1 à l'horizon) : `SELL_ASSET` (`assetId`, `salePrice` facultatif — valeur projetée par défaut —, `feesPercent` 0 à 100), `BUY_ASSET` (`assetClass`, `name` 1 à 200 car., `price` &gt;0, `growthPercent` facultatif), `TAKE_LOAN` (`amount` &gt;0, `annualRatePercent` 0 à 100, `termYears` 1 à 30), `PREPAY_LOAN` (`loanId`, `amount` &gt;0, au plus le capital restant dû projeté), `MONTHLY_SAVING` (`fromYear`, `toYear` facultatif — horizon par défaut —, `amount` par mois &gt;0)</t>
+        </is>
+      </c>
+      <c r="H730" s="2" t="inlineStr">
+        <is>
+          <t>`simulated` (`points` et `warnings`, même forme que la base) et `delta`. Le produit d'une vente, l'emprunt et l'épargne alimentent une trésorerie simulée, que les achats et remboursements débitent. Corps invalide : 400 ; opération incohérente (actif ou dette introuvable, actif déjà vendu ou plus actif, remboursement supérieur au capital dû) : 422 avec l'indice de l'opération. Aucune écriture, aucune ligne d'audit</t>
+        </is>
+      </c>
+      <c r="I730" s="2" t="inlineStr">
+        <is>
+          <t>Projeter la valeur nette sur 1 à 30 ans ; Créer un actif ; Enregistrer une dette</t>
+        </is>
+      </c>
+      <c r="J730" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K730" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L730" s="2" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/patrimoine/projections (champ `operations`)</t>
+        </is>
+      </c>
+      <c r="M730" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_VIEW (`requireAnyPropertyPermission`)</t>
+        </is>
+      </c>
+      <c r="N730" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O730" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Projections (/tenant/:tenantId/patrimoine/projections) — panneau « Simuler » (types « Vente d'un actif », « Achat d'un actif », « Nouvel emprunt », « Remboursement anticipé », « Épargne mensuelle » ; boutons « Ajouter l'opération », « Retirer », « Lancer la simulation »)</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B731" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C731" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D731" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Projections et simulations</t>
+        </is>
+      </c>
+      <c r="E731" s="2" t="inlineStr">
+        <is>
+          <t>Consulter l'écart de valeur nette entre la trajectoire simulée et la base</t>
+        </is>
+      </c>
+      <c r="F731" s="2" t="inlineStr">
+        <is>
+          <t>Mesurer année par année ce que les opérations simulées changent par rapport à la projection sans opération</t>
+        </is>
+      </c>
+      <c r="G731" s="2" t="inlineStr">
+        <is>
+          <t>Aucune saisie propre : présent dès que la requête porte au moins une opération</t>
+        </is>
+      </c>
+      <c r="H731" s="2" t="inlineStr">
+        <is>
+          <t>Champ `delta` : une entrée par année (`year`, `netWorth` = valeur nette simulée moins valeur nette de base, en XOF). L'écran affiche la carte « Écart avec la base » (phrase de synthèse à l'horizon et tableau Année, Base, Simulation, Écart) et la courbe « Simulation »</t>
+        </is>
+      </c>
+      <c r="I731" s="2" t="inlineStr">
+        <is>
+          <t>Simuler des opérations sur une copie du patrimoine</t>
+        </is>
+      </c>
+      <c r="J731" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K731" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L731" s="2" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/patrimoine/projections (champ `delta`) ; POST /tenants/:tenantId/patrimoine/scenarios/:scenarioId/run</t>
+        </is>
+      </c>
+      <c r="M731" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_VIEW (`requireAnyPropertyPermission`)</t>
+        </is>
+      </c>
+      <c r="N731" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O731" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Projections (/tenant/:tenantId/patrimoine/projections) — carte « Écart avec la base »</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B732" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C732" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D732" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Projections et simulations</t>
+        </is>
+      </c>
+      <c r="E732" s="2" t="inlineStr">
+        <is>
+          <t>Enregistrer un scénario</t>
+        </is>
+      </c>
+      <c r="F732" s="2" t="inlineStr">
+        <is>
+          <t>Conserver les hypothèses, les opérations et l'horizon d'une simulation pour la rejouer plus tard</t>
+        </is>
+      </c>
+      <c r="G732" s="2" t="inlineStr">
+        <is>
+          <t>Body Zod `.strict()` : `name` (1 à 120 car., espaces retirés), `horizonYears` (1 à 30), `baseScenario`, `assumptions` et `operations` (50 au plus) facultatifs, avec les mêmes contrôles que la projection ; seule la forme est validée, les actifs et dettes visés ne sont revérifiés qu'à l'exécution</t>
+        </is>
+      </c>
+      <c r="H732" s="2" t="inlineStr">
+        <is>
+          <t>201 — scénario (id, nom, horizon, scénario de base, hypothèses, opérations, dates de création et de modification) ; aucun résultat de calcul n'est stocké. 409 si le nom est déjà pris dans l'agence (« Un scénario porte déjà ce nom. ») ou si l'agence a atteint 100 scénarios. Ligne d'audit `PATRIMOINE_SCENARIO_CREATED` (identifiants seulement)</t>
+        </is>
+      </c>
+      <c r="I732" s="2" t="inlineStr">
+        <is>
+          <t>Projeter la valeur nette sur 1 à 30 ans</t>
+        </is>
+      </c>
+      <c r="J732" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="K732" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L732" s="2" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/patrimoine/scenarios</t>
+        </is>
+      </c>
+      <c r="M732" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="N732" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O732" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Projections (/tenant/:tenantId/patrimoine/projections) — panneau « Scénarios enregistrés », champ « Nom du scénario » et bouton « Enregistrer ce scénario » (message « Scénario enregistré. »)</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B733" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C733" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D733" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Projections et simulations</t>
+        </is>
+      </c>
+      <c r="E733" s="2" t="inlineStr">
+        <is>
+          <t>Lister les scénarios enregistrés</t>
+        </is>
+      </c>
+      <c r="F733" s="2" t="inlineStr">
+        <is>
+          <t>Retrouver les scénarios de l'agence</t>
+        </is>
+      </c>
+      <c r="G733" s="2" t="inlineStr">
+        <is>
+          <t>Aucune saisie</t>
+        </is>
+      </c>
+      <c r="H733" s="2" t="inlineStr">
+        <is>
+          <t>Liste de scénarios complets (id, nom, horizon, scénario de base, hypothèses, opérations, dates), du plus récemment modifié au plus ancien, 100 au plus</t>
+        </is>
+      </c>
+      <c r="I733" s="2" t="inlineStr">
+        <is>
+          <t>Enregistrer un scénario</t>
+        </is>
+      </c>
+      <c r="J733" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K733" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L733" s="2" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/patrimoine/scenarios</t>
+        </is>
+      </c>
+      <c r="M733" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_VIEW (`requireAnyPropertyPermission`)</t>
+        </is>
+      </c>
+      <c r="N733" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O733" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Projections (/tenant/:tenantId/patrimoine/projections) — panneau « Scénarios enregistrés » (« Aucun scénario enregistré pour l'instant. » quand la liste est vide)</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B734" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C734" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D734" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Projections et simulations</t>
+        </is>
+      </c>
+      <c r="E734" s="2" t="inlineStr">
+        <is>
+          <t>Consulter un scénario enregistré</t>
+        </is>
+      </c>
+      <c r="F734" s="2" t="inlineStr">
+        <is>
+          <t>Lire les réglages d'un scénario précis</t>
+        </is>
+      </c>
+      <c r="G734" s="2" t="inlineStr">
+        <is>
+          <t>Param `scenarioId` (UUID, sinon 400)</t>
+        </is>
+      </c>
+      <c r="H734" s="2" t="inlineStr">
+        <is>
+          <t>Scénario complet (même forme qu'un élément de la liste) ; 404 « Scénario introuvable. » s'il n'existe pas ou appartient à une autre agence</t>
+        </is>
+      </c>
+      <c r="I734" s="2" t="inlineStr">
+        <is>
+          <t>Enregistrer un scénario</t>
+        </is>
+      </c>
+      <c r="J734" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K734" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L734" s="2" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/patrimoine/scenarios/:scenarioId</t>
+        </is>
+      </c>
+      <c r="M734" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_VIEW (`requireAnyPropertyPermission`)</t>
+        </is>
+      </c>
+      <c r="N734" s="2" t="inlineStr">
+        <is>
+          <t>Disponible (route API sans écran dédié)</t>
+        </is>
+      </c>
+      <c r="O734" s="2" t="inlineStr">
+        <is>
+          <t>Aucun écran ne l'appelle : Patrimoine &gt; Projections (/tenant/:tenantId/patrimoine/projections) ouvre un scénario depuis la liste déjà chargée (bouton « Ouvrir »)</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B735" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C735" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D735" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Projections et simulations</t>
+        </is>
+      </c>
+      <c r="E735" s="2" t="inlineStr">
+        <is>
+          <t>Modifier ou renommer un scénario</t>
+        </is>
+      </c>
+      <c r="F735" s="2" t="inlineStr">
+        <is>
+          <t>Changer le nom d'un scénario ou remplacer ses réglages (horizon, scénario de base, hypothèses, opérations)</t>
+        </is>
+      </c>
+      <c r="G735" s="2" t="inlineStr">
+        <is>
+          <t>Param `scenarioId` ; body Zod `.strict()` : les champs de la création, tous facultatifs, au moins un (sinon 400 « Aucun champ à modifier. ») ; un nouvel horizon sans nouvelles opérations doit rester compatible avec les années des opérations enregistrées</t>
+        </is>
+      </c>
+      <c r="H735" s="2" t="inlineStr">
+        <is>
+          <t>200 — scénario mis à jour ; 404 s'il est introuvable ; 409 si le nom est déjà pris ; 422 si l'horizon est trop court pour les opérations enregistrées. Ligne d'audit `PATRIMOINE_SCENARIO_UPDATED` (noms des champs modifiés seulement)</t>
+        </is>
+      </c>
+      <c r="I735" s="2" t="inlineStr">
+        <is>
+          <t>Enregistrer un scénario</t>
+        </is>
+      </c>
+      <c r="J735" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="K735" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L735" s="2" t="inlineStr">
+        <is>
+          <t>PATCH /tenants/:tenantId/patrimoine/scenarios/:scenarioId</t>
+        </is>
+      </c>
+      <c r="M735" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="N735" s="2" t="inlineStr">
+        <is>
+          <t>À vérifier — bug probable (bouton « Mettre à jour », voir Notes)</t>
+        </is>
+      </c>
+      <c r="O735" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Projections (/tenant/:tenantId/patrimoine/projections) — panneau « Scénarios enregistrés », boutons « Renommer » (champ « Nouveau nom du scénario », « Valider », « Annuler ») et « Mettre à jour » (confirmation « Mettre à jour « {name} » avec les réglages actuels ? »)</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B736" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C736" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D736" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Projections et simulations</t>
+        </is>
+      </c>
+      <c r="E736" s="2" t="inlineStr">
+        <is>
+          <t>Supprimer un scénario</t>
+        </is>
+      </c>
+      <c r="F736" s="2" t="inlineStr">
+        <is>
+          <t>Retirer un scénario devenu inutile (et libérer une place sous le plafond de 100)</t>
+        </is>
+      </c>
+      <c r="G736" s="2" t="inlineStr">
+        <is>
+          <t>Param `scenarioId`</t>
+        </is>
+      </c>
+      <c r="H736" s="2" t="inlineStr">
+        <is>
+          <t>204 No Content ; 404 s'il est introuvable. Ligne d'audit `PATRIMOINE_SCENARIO_DELETED` (identifiants seulement)</t>
+        </is>
+      </c>
+      <c r="I736" s="2" t="inlineStr">
+        <is>
+          <t>Enregistrer un scénario</t>
+        </is>
+      </c>
+      <c r="J736" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="K736" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L736" s="2" t="inlineStr">
+        <is>
+          <t>DELETE /tenants/:tenantId/patrimoine/scenarios/:scenarioId</t>
+        </is>
+      </c>
+      <c r="M736" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="N736" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O736" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Projections (/tenant/:tenantId/patrimoine/projections) — panneau « Scénarios enregistrés », bouton « Supprimer » (confirmation « Supprimer « {name} » ? », message « Scénario supprimé. »)</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B737" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C737" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D737" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Projections et simulations</t>
+        </is>
+      </c>
+      <c r="E737" s="2" t="inlineStr">
+        <is>
+          <t>Rejouer un scénario enregistré sur le patrimoine actuel</t>
+        </is>
+      </c>
+      <c r="F737" s="2" t="inlineStr">
+        <is>
+          <t>Relancer un scénario enregistré avec les actifs, dettes et valeurs d'aujourd'hui pour voir son résultat à jour</t>
+        </is>
+      </c>
+      <c r="G737" s="2" t="inlineStr">
+        <is>
+          <t>Param `scenarioId` ; body `.strict()` facultatif : `compareScenarios` (booléen)</t>
+        </is>
+      </c>
+      <c r="H737" s="2" t="inlineStr">
+        <is>
+          <t>Même réponse qu'une projection (`assumptionsUsed`, `base`, `simulated` et `delta` si le scénario a des opérations, `byScenario` si comparaison). Une opération dont l'actif ou la dette a disparu (ou n'est plus actif) devient un avertissement `OPERATION_NOT_APPLICABLE` au lieu d'une erreur ; un scénario stocké devenu illisible répond 422 (« Le scénario enregistré est invalide : corrigez-le ou recréez-le. »). Aucune écriture, aucune ligne d'audit</t>
+        </is>
+      </c>
+      <c r="I737" s="2" t="inlineStr">
+        <is>
+          <t>Enregistrer un scénario ; Projeter la valeur nette sur 1 à 30 ans</t>
+        </is>
+      </c>
+      <c r="J737" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K737" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L737" s="2" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/patrimoine/scenarios/:scenarioId/run</t>
+        </is>
+      </c>
+      <c r="M737" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_VIEW (`requireAnyPropertyPermission`)</t>
+        </is>
+      </c>
+      <c r="N737" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O737" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Projections (/tenant/:tenantId/patrimoine/projections) — panneau « Scénarios enregistrés », bouton « Ouvrir » (les résultats affichés viennent de l'exécution du scénario tant que les réglages ne sont pas modifiés)</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B738" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C738" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D738" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — Projections et simulations</t>
+        </is>
+      </c>
+      <c r="E738" s="2" t="inlineStr">
+        <is>
+          <t>Consulter les avertissements d'une projection</t>
+        </is>
+      </c>
+      <c r="F738" s="2" t="inlineStr">
+        <is>
+          <t>Savoir quand un résultat repose sur des données fragiles ou incohérentes</t>
+        </is>
+      </c>
+      <c r="G738" s="2" t="inlineStr">
+        <is>
+          <t>Aucune saisie</t>
+        </is>
+      </c>
+      <c r="H738" s="2" t="inlineStr">
+        <is>
+          <t>Champ `warnings` de `base`, de `simulated` et de chaque scénario de `byScenario` : `LOW_RELIABILITY_START` (`sharePercent`, part de la valeur de départ peu fiable, seulement si &gt;0), `ASSET_WITHOUT_VALUE` (actif sans valeur, non compté), `LOAN_PAYMENT_TOO_LOW` (mensualité inférieure aux intérêts), `NEGATIVE_CASH` (`year`, trésorerie simulée négative), `OPERATION_NOT_APPLICABLE` (`index`, `reason` : `ASSET_NOT_FOUND`, `ASSET_NOT_ACTIVE`, `LOAN_NOT_FOUND`)</t>
+        </is>
+      </c>
+      <c r="I738" s="2" t="inlineStr">
+        <is>
+          <t>Projeter la valeur nette sur 1 à 30 ans ; Consulter la part de la valeur nette reposant sur des valeurs peu fiables</t>
+        </is>
+      </c>
+      <c r="J738" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K738" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L738" s="2" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/patrimoine/projections (champ `warnings`) ; POST /tenants/:tenantId/patrimoine/scenarios/:scenarioId/run</t>
+        </is>
+      </c>
+      <c r="M738" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_VIEW (`requireAnyPropertyPermission`)</t>
+        </is>
+      </c>
+      <c r="N738" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O738" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine &gt; Projections (/tenant/:tenantId/patrimoine/projections) — bandeau « À savoir sur ces résultats » (avertissements de la base et de la simulation, sans doublon) ; bandeau permanent « Ces projections reposent sur des hypothèses indicatives, elles ne sont pas une prévision. »</t>
         </is>
       </c>
     </row>
@@ -57308,7 +58155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -57836,12 +58683,34 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Règles transverses du patrimoine multi-actifs, communes aux écrans et routes décrits ci-dessus. (1) Plafonds par agence : 500 actifs non archivés et 1 000 valorisations par actif ; au-delà, 409. (2) Toute écriture sur un actif archivé est refusée (409). (3) Le changement de devise d'un actif est refusé (409) tant que des lignes (valorisations, dettes) existent dans une autre devise. (4) Les écritures sont auditées (clés `PATRIMOINE_ASSET_CREATED`, `_UPDATED`, `_DISPOSED`, `_ARCHIVED`, `PATRIMOINE_VALUATION_CREATED`, `_UPDATED`, `_DELETED`, `PATRIMOINE_DEBT_CREATED`, `_UPDATED`, `_DELETED`, `PATRIMOINE_HOLDING_SET`, `PATRIMOINE_HOLDING_DELETED`) ; le journal ne porte que des identifiants, types, classes et noms de champs, jamais un montant, un nom ou une note ; la suggestion de valeur n'écrit rien et n'est pas auditée. (5) La fiabilité d'une valorisation est calculée par le serveur (à l'écriture, puis recalculée à la lecture selon l'ancienneté et le statut juridique courant) et n'est jamais fournie par le client. (6) La liste des statuts juridiques fonciers (titre foncier, ACD, certificat de propriété ou de détention, lettre d'attribution, attestation villageoise ou coutumière, autre) et le classement de la lettre d'attribution et de l'attestation villageoise ou coutumière comme statuts fragiles sont une hypothèse métier.</t>
+          <t>Règles transverses du patrimoine multi-actifs, communes aux écrans et routes décrits ci-dessus. (1) Plafonds par agence : 500 actifs non archivés et 1 000 valorisations par actif ; au-delà, 409. (2) Toute écriture sur un actif archivé est refusée (409). (3) Le changement de devise d'un actif est refusé (409) tant que des lignes (valorisations, dettes) existent dans une autre devise. (4) Les écritures sont auditées (clés `PATRIMOINE_ASSET_CREATED`, `_UPDATED`, `_DISPOSED`, `_ARCHIVED`, `PATRIMOINE_VALUATION_CREATED`, `_UPDATED`, `_DELETED`, `PATRIMOINE_DEBT_CREATED`, `_UPDATED`, `_DELETED`, `PATRIMOINE_HOLDING_SET`, `PATRIMOINE_HOLDING_DELETED`) ; le journal ne porte que des identifiants, types, classes et noms de champs, jamais un montant, un nom ou une note ; la suggestion de valeur n'écrit rien et n'est pas auditée. (5) La fiabilité d'une valorisation est calculée par le serveur (à l'écriture, puis recalculée à la lecture selon l'ancienneté et le statut juridique courant) et n'est jamais fournie par le client. (6) Les valorisations saisies par le module Bien (création et modification d'une valorisation depuis la fiche d'un bien, `lib/patrimoine/queries.ts`) reçoivent elles aussi une fiabilité stockée, calculée par le serveur avec le même barème : sans source à la création (le module Bien n'en saisit pas ; à la modification, la source déjà portée par la ligne est conservée), avec le statut juridique courant du bien. (7) La liste des statuts juridiques fonciers (titre foncier, ACD, certificat de propriété ou de détention, lettre d'attribution, attestation villageoise ou coutumière, autre) et le classement de la lettre d'attribution et de l'attestation villageoise ou coutumière comme statuts fragiles sont une hypothèse métier.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
           <t>Faire valider par un juriste local la liste des statuts juridiques fonciers et le classement « fragile » avant toute communication grand public (page vitrine, supports commerciaux). Les autres règles sont vérifiées dans le code (`services/patrimoine-assets/limits.ts`, `audit.ts`, `lib/patrimoine/assets/reliability.ts`) ; aucune ligne du classeur n'est en statut « À vérifier » pour ces points.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine multi-actifs — projections</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Limites et choix à confirmer du lot 3 (projections et simulations). (1) Les hypothèses de croissance et d'inflation par défaut sont indicatives et à confirmer par le produit (prudent : immobilier 2 %, épargne 2 %, autres classes 0 %, inflation 4 % ; central : immobilier 4 %, entreprises 5 %, épargne 4 %, stocks 2 %, agriculture 3 %, biens meubles 2 %, inflation 3 % ; optimiste : immobilier 6 %, entreprises 10 %, épargne 6 %, stocks 4 %, agriculture 6 %, biens meubles 4 %, inflation 2 % ; trésorerie, créances, véhicules et autre à 0 %, les véhicules s'amortissant d'après leurs caractéristiques) ; constantes de `lib/patrimoine/projection/assumptions.ts`, modifiables sans migration et corrigeables à l'écran. (2) Les mensualités de dettes ne sont pas prélevées sur la trésorerie, car les revenus ne sont pas modélisés : la valeur nette augmente donc du capital remboursé (l'écran l'annonce dans un bandeau). (3) Pas de projection de change : chaque valeur est convertie en XOF au taux d'aujourd'hui. (4) Le plafond de 100 scénarios par agence est contrôlé sans verrou (comptage puis création) : deux créations simultanées peuvent le dépasser d'une unité. (5) Les scénarios sont audités : `PATRIMOINE_SCENARIO_CREATED`, `PATRIMOINE_SCENARIO_UPDATED`, `PATRIMOINE_SCENARIO_DELETED` (identifiants, scénario de base et noms de champs seulement, jamais un nom, un montant ou une opération) ; les projections, simulations et exécutions de scénario n'écrivent rien et ne sont pas auditées. (6) À vérifier, bug probable : le bouton « Mettre à jour » d'un scénario enregistré envoie au PATCH les réglages courants avec un `name` vide (`ProjectionsPage.tsx`, `current.name = ''`, transmis tel quel par `ScenariosPanel.tsx`), que `scenarioUpdateSchema` refuse (nom de 1 à 120 caractères) : la mise à jour depuis l'écran échouerait donc en 400 ; en outre, des hypothèses vides ne sont pas envoyées et ne remplaceraient pas celles déjà enregistrées. Le renommage (`{ name }`) n'est pas concerné et la route elle-même est correcte. Constat de lecture du code, non rejoué dans l'application.</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Faire confirmer par le produit les hypothèses par défaut avant toute communication grand public, décider s'il faut modéliser les revenus (et donc prélever les mensualités), un verrou sur le plafond de scénarios et, plus tard, une projection de change. Corriger ou confirmer le bouton « Mettre à jour » (omettre `name` du corps envoyé, et envoyer `assumptions: {}` pour effacer des hypothèses), puis repasser la ligne « Modifier ou renommer un scénario » en `Disponible`.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(copilot): durcissements de l'audit (atomicité, plafond par agence, garde bail, permissions, logs)
Usage unique du jeton et idempotence des quittances sous verrou consultatif PostgreSQL
(sémaphore de processus contre la saturation du pool), plafond de débit par agence,
garde « bail vu » contre l'injection de prompt, GENERATE et VIEW exigés, faux
fournisseur limité à development/test, entityId d'audit généré côté serveur, messages
d'erreur de génération sans chemin disque, logs sans coordonnées personnelles.
Docs, wiki et passation mis à jour.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NipnEzc6N8uvDDXG2M7jms
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -53889,7 +53889,7 @@
       </c>
       <c r="F691" s="2" t="inlineStr">
         <is>
-          <t>Ouvre le tiroir de conversation (côté « fin » : à droite en français, à gauche en arabe) et envoie l'échange au fournisseur LLM en flux SSE : texte progressif, cartes de résultats (biens, baux, documents, proposition), suggestions selon l'écran courant, arrêt de la réponse et nouvelle conversation. Conversation non persistée ; l'assistant n'écrit jamais lui-même. Limites : 20 messages, 4 000 caractères chacun, 24 000 au total ; 20 requêtes/min et 300/jour par utilisateur et par agence ; 4 tours et 8 appels d'outils maximum</t>
+          <t>Ouvre le tiroir de conversation (côté « fin » : à droite en français, à gauche en arabe) et envoie l'échange au fournisseur LLM en flux SSE : texte progressif, cartes de résultats (biens, baux, documents, proposition), suggestions selon l'écran courant, arrêt de la réponse et nouvelle conversation. Conversation non persistée ; l'assistant n'écrit jamais lui-même. Limites : 20 messages, 4 000 caractères chacun, 24 000 au total ; 20 requêtes/min et 300/jour par utilisateur et par agence, plus un plafond par agence tous collaborateurs confondus (`AI_TENANT_MINUTE_LIMIT` 100/min, `AI_TENANT_DAILY_LIMIT` 3000/jour) ; limiteurs en mémoire, par instance d'API ; 4 tours et 8 appels d'outils maximum</t>
         </is>
       </c>
       <c r="G691" s="2" t="inlineStr">
@@ -53924,7 +53924,7 @@
       </c>
       <c r="M691" s="2" t="inlineStr">
         <is>
-          <t>`authenticate` + `requireTenantAccess` + `requireTenantCollaborator` + `requireAiAssistantAccess` + limiteurs `aiChatRateLimiter` et `aiChatDailyLimiter` ; pas de permission unique : chaque outil vérifie la sienne (voir les lignes suivantes)</t>
+          <t>`authenticate` + `requireTenantAccess` + `requireTenantCollaborator` + `requireAiAssistantAccess` + limiteurs `aiChatRateLimiter`, `aiChatDailyLimiter` (par utilisateur) puis `aiTenantChatRateLimiter` et `aiTenantDailyLimiter` (par agence) ; pas de permission unique : chaque outil vérifie la sienne (voir les lignes suivantes)</t>
         </is>
       </c>
       <c r="N691" s="2" t="inlineStr">
@@ -54274,7 +54274,7 @@
       </c>
       <c r="F696" s="2" t="inlineStr">
         <is>
-          <t>Outil `propose_rental_document` : prépare une PROPOSITION, sans aucune écriture. Quittance (`RENT_RECEIPT`, période AAAA-MM) : le serveur retrouve l'échéance de la période puis le paiement encaissé (SUCCESS) qui l'alloue ; sans paiement, sans échéance ou sans modèle actif, aucune proposition (« impossible ») ; une quittance FINAL déjà émise est montrée au lieu d'être reproposée. Relevé (`RENT_STATEMENT`, dates de début et de fin, 12 mois maximum). Renvoie une carte de récapitulatif et un jeton signé valable 300 s (`AI_PROPOSAL_TTL_SECONDS`). Le jeton n'est jamais transmis au fournisseur LLM</t>
+          <t>Outil `propose_rental_document` : prépare une PROPOSITION, sans aucune écriture. Quittance (`RENT_RECEIPT`, période AAAA-MM) : le serveur retrouve l'échéance de la période puis le paiement encaissé (SUCCESS) qui l'alloue ; sans paiement, sans échéance ou sans modèle actif, aucune proposition (« impossible ») ; une quittance FINAL déjà émise est montrée au lieu d'être reproposée. Relevé (`RENT_STATEMENT`, dates de début et de fin, 12 mois maximum). Le bail doit avoir été vu dans la même requête (résultat de `search_leases` ou `list_lease_documents`, ou écran vérifié), sinon « impossible » (`lease_not_seen`). Renvoie une carte de récapitulatif et un jeton signé valable 300 s (`AI_PROPOSAL_TTL_SECONDS`). Le jeton n'est jamais transmis au fournisseur LLM</t>
         </is>
       </c>
       <c r="G696" s="2" t="inlineStr">
@@ -54294,7 +54294,7 @@
       </c>
       <c r="J696" s="2" t="inlineStr">
         <is>
-          <t>Collaborateurs de l'agence détenteurs de la permission — TENANT_ADMIN, TENANT_MANAGER par défaut ; pas TENANT_AGENT ; refusé au super-admin et aux clients de portail</t>
+          <t>Collaborateurs de l'agence détenteurs des permissions `RENTAL_DOCUMENTS_GENERATE` et `RENTAL_DOCUMENTS_VIEW` — TENANT_ADMIN, TENANT_MANAGER par défaut ; pas TENANT_AGENT ; refusé au super-admin et aux clients de portail</t>
         </is>
       </c>
       <c r="K696" s="2" t="inlineStr">
@@ -54309,7 +54309,7 @@
       </c>
       <c r="M696" s="2" t="inlineStr">
         <is>
-          <t>`RENTAL_DOCUMENTS_GENERATE` (outil `propose_rental_document`) + `authenticate` + `requireTenantAccess` + `requireTenantCollaborator` + `requireAiAssistantAccess`</t>
+          <t>`RENTAL_DOCUMENTS_GENERATE` et `RENTAL_DOCUMENTS_VIEW` (outil `propose_rental_document`, les deux exigées) + `authenticate` + `requireTenantAccess` + `requireTenantCollaborator` + `requireAiAssistantAccess`</t>
         </is>
       </c>
       <c r="N696" s="2" t="inlineStr">
@@ -54351,7 +54351,7 @@
       </c>
       <c r="F697" s="2" t="inlineStr">
         <is>
-          <t>Action humaine sur la carte de proposition (« Confirmer et générer ») : rejoue authentification, agence, collaborateur et `RENTAL_DOCUMENTS_GENERATE`, vérifie le jeton (signature, expiration, utilisateur, agence, usage unique) et l'appartenance de chaque identifiant, puis génère le `.docx` via le générateur existant. Idempotent (une quittance FINAL déjà émise est renvoyée) ; 10 confirmations par minute ; audit `AI_PROPOSAL_REDEEMED` et `AI_ACTION_EXECUTED`. Seule porte de génération de l'assistant</t>
+          <t>Action humaine sur la carte de proposition (« Confirmer et générer ») : rejoue authentification, agence, collaborateur, `RENTAL_DOCUMENTS_GENERATE` et `RENTAL_DOCUMENTS_VIEW` (le téléchargement exige VIEW), vérifie le jeton (signature, expiration, utilisateur, agence, usage unique, atomique entre instances : verrou consultatif PostgreSQL) et l'appartenance de chaque identifiant, puis génère le `.docx` via le générateur existant. Idempotent (une quittance FINAL déjà émise est renvoyée ; section critique par paiement, verrou consultatif) ; 10 confirmations par minute ; audit `AI_PROPOSAL_REDEEMED` et `AI_ACTION_EXECUTED`. Seule porte de génération de l'assistant</t>
         </is>
       </c>
       <c r="G697" s="2" t="inlineStr">
@@ -54371,7 +54371,7 @@
       </c>
       <c r="J697" s="2" t="inlineStr">
         <is>
-          <t>Collaborateurs de l'agence détenteurs de la permission — TENANT_ADMIN, TENANT_MANAGER par défaut ; pas TENANT_AGENT ; refusé au super-admin et aux clients de portail</t>
+          <t>Collaborateurs de l'agence détenteurs des permissions `RENTAL_DOCUMENTS_GENERATE` et `RENTAL_DOCUMENTS_VIEW` — TENANT_ADMIN, TENANT_MANAGER par défaut ; pas TENANT_AGENT ; refusé au super-admin et aux clients de portail</t>
         </is>
       </c>
       <c r="K697" s="2" t="inlineStr">
@@ -54386,7 +54386,7 @@
       </c>
       <c r="M697" s="2" t="inlineStr">
         <is>
-          <t>`RENTAL_DOCUMENTS_GENERATE` (`requireDocumentsGenerate`) + `authenticate` + `requireTenantAccess` + `requireTenantCollaborator` + `requireAiAssistantAccess` + `aiActionRateLimiter`</t>
+          <t>`RENTAL_DOCUMENTS_GENERATE` (`requireDocumentsGenerate`) + `RENTAL_DOCUMENTS_VIEW` (`requireDocumentsView`) + `authenticate` + `requireTenantAccess` + `requireTenantCollaborator` + `requireAiAssistantAccess` + `aiActionRateLimiter`</t>
         </is>
       </c>
       <c r="N697" s="2" t="inlineStr">

</xml_diff>

<commit_message>
docs(patrimoine): wiki et passation du lot 4 (espace particulier)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PxDVZM8akvCsSCfK3Cgg19
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -189,8 +189,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O738" headerRowCount="1">
-  <autoFilter ref="A1:O738"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O743" headerRowCount="1">
+  <autoFilter ref="A1:O743"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Domaine (regroupement agent)"/>
     <tableColumn id="2" name="Pack(s)"/>
@@ -242,8 +242,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotesPointsOuverts" displayName="NotesPointsOuverts" ref="A1:D25" headerRowCount="1">
-  <autoFilter ref="A1:D25"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotesPointsOuverts" displayName="NotesPointsOuverts" ref="A1:D26" headerRowCount="1">
+  <autoFilter ref="A1:D26"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Domaine"/>
     <tableColumn id="2" name="Sujet"/>
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O738"/>
+  <dimension ref="A1:O743"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -40039,7 +40039,7 @@
       </c>
       <c r="H511" s="2" t="inlineStr">
         <is>
-          <t>Utilisateur créé (non vérifié)</t>
+          <t>Utilisateur créé (non vérifié) Réponse neutre identique que l'adresse existe ou non (« Si cette adresse est valide… ») ; pour un compte existant non vérifié, le mot de passe et le nom de la dernière inscription remplacent les anciens et les sessions sont révoquées avant le nouvel e-mail. Limite de 3 inscriptions par heure et par adresse IP (IPv6 regroupée par /64), état conservé en base sous forme d'empreinte ; le comptage ne concerne que les requêtes valides. Réponse 503 en production sans serveur d'e-mails.</t>
         </is>
       </c>
       <c r="I511" s="2" t="inlineStr">
@@ -40270,7 +40270,7 @@
       </c>
       <c r="H514" s="2" t="inlineStr">
         <is>
-          <t>`{user}` + cookies</t>
+          <t>`{user}` + cookies Réponse uniforme « Email ou mot de passe incorrect. » tant que le mot de passe n'est pas correct (compte inconnu, non vérifié ou désactivé indistinguables sans le mot de passe) ; l'état du compte n'est révélé qu'après un mot de passe valide.</t>
         </is>
       </c>
       <c r="I514" s="2" t="inlineStr">
@@ -57550,6 +57550,391 @@
       <c r="O738" s="2" t="inlineStr">
         <is>
           <t>Patrimoine &gt; Projections (/tenant/:tenantId/patrimoine/projections) — bandeau « À savoir sur ces résultats » (avertissements de la base et de la simulation, sans doublon) ; bandeau permanent « Ces projections reposent sur des hypothèses indicatives, elles ne sont pas une prévision. »</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" s="2" t="inlineStr">
+        <is>
+          <t>Administration plateforme</t>
+        </is>
+      </c>
+      <c r="B739" s="2" t="inlineStr">
+        <is>
+          <t>Particulier gratuit, Particulier plus</t>
+        </is>
+      </c>
+      <c r="C739" s="2" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="D739" s="2" t="inlineStr">
+        <is>
+          <t>Espace particulier — Création et palier</t>
+        </is>
+      </c>
+      <c r="E739" s="2" t="inlineStr">
+        <is>
+          <t>Créer son espace personnel</t>
+        </is>
+      </c>
+      <c r="F739" s="2" t="inlineStr">
+        <is>
+          <t>Un utilisateur connecté à l'e-mail vérifié et sans espace obtient son espace de patrimoine en quelques champs, sans intervention d'un administrateur</t>
+        </is>
+      </c>
+      <c r="G739" s="2" t="inlineStr">
+        <is>
+          <t>Body Zod `.strict()` : `displayName` (1 à 120 caractères), `country` (CI, SN, BF, ML, NE, TG, BJ, GW), `phone` facultatif (format international UEMOA, 8 à 15 chiffres) ; en-tête facultatif `Idempotency-Key`</t>
+        </is>
+      </c>
+      <c r="H739" s="2" t="inlineStr">
+        <is>
+          <t>201 `{ tenantId, slug, name }` ; espace de type PARTICULIER avec le module Patrimoine seul, abonnement gratuit actif, adhésion active et rôle administrateur, créés en une transaction. 409 `PERSONAL_SPACE_EXISTS` (avec `tenantId`) si l'utilisateur a déjà un espace personnel (verrou consultatif, un seul espace même en cas de double clic ou de requêtes simultanées) ; 403 `EMAIL_NOT_VERIFIED` ; 503 `SIGNUP_UNAVAILABLE` en production sans serveur d'e-mails. Ligne d'audit `PERSONAL_SPACE_CREATED` (identifiants, pays et pack, jamais le nom ni le téléphone)</t>
+        </is>
+      </c>
+      <c r="I739" s="2" t="inlineStr">
+        <is>
+          <t>S'inscrire ; Se connecter</t>
+        </is>
+      </c>
+      <c r="J739" s="2" t="inlineStr">
+        <is>
+          <t>Utilisateur connecté sans espace</t>
+        </is>
+      </c>
+      <c r="K739" s="2" t="inlineStr">
+        <is>
+          <t>Utilisateur connecté (e-mail vérifié)</t>
+        </is>
+      </c>
+      <c r="L739" s="2" t="inlineStr">
+        <is>
+          <t>POST /api/personal-space</t>
+        </is>
+      </c>
+      <c r="M739" s="2" t="inlineStr">
+        <is>
+          <t>Authentifié, e-mail vérifié</t>
+        </is>
+      </c>
+      <c r="N739" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O739" s="2" t="inlineStr">
+        <is>
+          <t>Écran « Créer mon espace » affiché à la place de « compte non rattaché » (champs « Nom affiché », pays, « Téléphone » ; bouton « Créer mon espace »)</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B740" s="2" t="inlineStr">
+        <is>
+          <t>Particulier gratuit, Particulier plus</t>
+        </is>
+      </c>
+      <c r="C740" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D740" s="2" t="inlineStr">
+        <is>
+          <t>Espace particulier — Création et palier</t>
+        </is>
+      </c>
+      <c r="E740" s="2" t="inlineStr">
+        <is>
+          <t>Consulter l'usage du palier (actifs suivis)</t>
+        </is>
+      </c>
+      <c r="F740" s="2" t="inlineStr">
+        <is>
+          <t>Savoir combien d'actifs sont suivis sur la limite du palier et si l'ajout est encore possible</t>
+        </is>
+      </c>
+      <c r="G740" s="2" t="inlineStr">
+        <is>
+          <t>Aucune saisie</t>
+        </is>
+      </c>
+      <c r="H740" s="2" t="inlineStr">
+        <is>
+          <t>`{ plan: FREE | PAID | AGENCY, limit (null hors palier particulier), used, canAdd, upgrade }` ; `used` compte les actifs non archivés et les biens non archivés sans actif lié, chacun une fois ; `upgrade` (cible, prix mensuel, plafond) n'est proposé que sur le palier gratuit, lu dans le catalogue</t>
+        </is>
+      </c>
+      <c r="I740" s="2" t="inlineStr">
+        <is>
+          <t>Créer son espace personnel</t>
+        </is>
+      </c>
+      <c r="J740" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur — PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K740" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Particulier</t>
+        </is>
+      </c>
+      <c r="L740" s="2" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/patrimoine/usage</t>
+        </is>
+      </c>
+      <c r="M740" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="N740" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O740" s="2" t="inlineStr">
+        <is>
+          <t>Bandeau « X actifs sur N » de Patrimoine &gt; Valeur nette et Mes actifs (alerte avec lien vers l'abonnement sur le palier gratuit, ligne discrète sur le palier payant, rien pour une agence)</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B741" s="2" t="inlineStr">
+        <is>
+          <t>Particulier gratuit, Particulier plus</t>
+        </is>
+      </c>
+      <c r="C741" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D741" s="2" t="inlineStr">
+        <is>
+          <t>Espace particulier — Création et palier</t>
+        </is>
+      </c>
+      <c r="E741" s="2" t="inlineStr">
+        <is>
+          <t>Être refusé au-delà de la limite du palier gratuit</t>
+        </is>
+      </c>
+      <c r="F741" s="2" t="inlineStr">
+        <is>
+          <t>Empêcher l'ajout d'un actif ou d'un bien au-delà de 10 sur le palier gratuit, la lecture, la modification, l'archivage et les projections restant possibles</t>
+        </is>
+      </c>
+      <c r="G741" s="2" t="inlineStr">
+        <is>
+          <t>Création d'un actif ou d'un bien (routes existantes)</t>
+        </is>
+      </c>
+      <c r="H741" s="2" t="inlineStr">
+        <is>
+          <t>409 `FREE_TIER_LIMIT` avec `limit` et `used`, quel que soit `SUBSCRIPTION_ENFORCEMENT`, sans rien créer ; les actifs archivés ne comptent pas ; la garde est prise sous verrou consultatif ; les agences (plafond de 500 du lot 1) ne sont pas concernées ; la valorisation d'un bien reste enregistrée même quand l'actif lié ne peut pas être créé</t>
+        </is>
+      </c>
+      <c r="I741" s="2" t="inlineStr">
+        <is>
+          <t>Consulter l'usage du palier</t>
+        </is>
+      </c>
+      <c r="J741" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur — PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="K741" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Particulier</t>
+        </is>
+      </c>
+      <c r="L741" s="2" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/patrimoine/assets ; POST /tenants/:tenantId/properties</t>
+        </is>
+      </c>
+      <c r="M741" s="2" t="inlineStr">
+        <is>
+          <t>PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="N741" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O741" s="2" t="inlineStr">
+        <is>
+          <t>Tiroir de création d'un actif : alerte « Limite du palier gratuit atteinte » avec bouton vers l'abonnement, saisie conservée</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" s="2" t="inlineStr">
+        <is>
+          <t>Administration plateforme</t>
+        </is>
+      </c>
+      <c r="B742" s="2" t="inlineStr">
+        <is>
+          <t>Particulier gratuit, Particulier plus</t>
+        </is>
+      </c>
+      <c r="C742" s="2" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="D742" s="2" t="inlineStr">
+        <is>
+          <t>Espace particulier — Création et palier</t>
+        </is>
+      </c>
+      <c r="E742" s="2" t="inlineStr">
+        <is>
+          <t>Passer au palier payant (facture et paiement mobile money)</t>
+        </is>
+      </c>
+      <c r="F742" s="2" t="inlineStr">
+        <is>
+          <t>Faire monter le plafond d'actifs en payant le palier particulier plus par mobile money ou carte via PaySecureHub</t>
+        </is>
+      </c>
+      <c r="G742" s="2" t="inlineStr">
+        <is>
+          <t>Body Zod `.strict()` : `target` (`PARTICULIER_PLUS`) ; le téléphone de l'espace doit être renseigné</t>
+        </is>
+      </c>
+      <c r="H742" s="2" t="inlineStr">
+        <is>
+          <t>201 `{ invoiceId, checkoutUrl, code }` ; le pack ne change qu'à la confirmation du paiement par la réconciliation serveur (idempotent, sous verrou), jamais avant ; paiement annulé ou échoué : l'espace reste gratuit. 409 `ALREADY_ON_TARGET` ; 409 `PAYMENT_IN_PROGRESS` avec les données de reprise ; 422 `PHONE_REQUIRED` ; 403 pour un espace non particulier ; 503 si les paiements sont indisponibles. Paiement encaissé sans changement de pack : paiement en REVIEW et audit `SUBSCRIPTION_UPGRADE_NOT_APPLIED`</t>
+        </is>
+      </c>
+      <c r="I742" s="2" t="inlineStr">
+        <is>
+          <t>Créer son espace personnel</t>
+        </is>
+      </c>
+      <c r="J742" s="2" t="inlineStr">
+        <is>
+          <t>Administrateur de l'espace (TENANT_ADMIN)</t>
+        </is>
+      </c>
+      <c r="K742" s="2" t="inlineStr">
+        <is>
+          <t>Particulier (espace personnel)</t>
+        </is>
+      </c>
+      <c r="L742" s="2" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/subscription/upgrade</t>
+        </is>
+      </c>
+      <c r="M742" s="2" t="inlineStr">
+        <is>
+          <t>TENANT_SETTINGS_EDIT (exemptée de la lecture seule)</t>
+        </is>
+      </c>
+      <c r="N742" s="2" t="inlineStr">
+        <is>
+          <t>Disponible (paiement réel non testé sans identifiants de production ; tarif provisoire)</t>
+        </is>
+      </c>
+      <c r="O742" s="2" t="inlineStr">
+        <is>
+          <t>Paramètres &gt; Abonnement : carte « Palier de votre espace » (palier actuel, usage, offre « Tarif provisoire », bouton « Passer au palier payant », champ « Téléphone » obligatoire avant de payer, « Reprendre le paiement », suivi du retour de paiement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" s="2" t="inlineStr">
+        <is>
+          <t>Administration plateforme</t>
+        </is>
+      </c>
+      <c r="B743" s="2" t="inlineStr">
+        <is>
+          <t>Particulier gratuit, Particulier plus</t>
+        </is>
+      </c>
+      <c r="C743" s="2" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="D743" s="2" t="inlineStr">
+        <is>
+          <t>Espace particulier — Navigation</t>
+        </is>
+      </c>
+      <c r="E743" s="2" t="inlineStr">
+        <is>
+          <t>Naviguer dans un espace particulier (menu réduit et accueil valeur nette)</t>
+        </is>
+      </c>
+      <c r="F743" s="2" t="inlineStr">
+        <is>
+          <t>Ne voir que ce qui sert un particulier : patrimoine, biens, baux, paramètres et abonnement</t>
+        </is>
+      </c>
+      <c r="G743" s="2" t="inlineStr">
+        <is>
+          <t>Aucune saisie ; le type de l'espace vient de `tenant.type`</t>
+        </is>
+      </c>
+      <c r="H743" s="2" t="inlineStr">
+        <is>
+          <t>Menu réduit (Accueil, Biens, Baux, Plus), tableau de bord redirigé vers Patrimoine &gt; Valeur nette, copilote masqué ; décidé par le type de l'espace, y compris en mode global `warn`. Côté API, une liste blanche de routes est appliquée au type PARTICULIER quel que soit le mode : tout le reste (newsletter, invitations, utilisateurs, CRM, finance, syndic, notifications, réglages, IA) répond 403 `PERSONAL_SPACE_ROUTE_FORBIDDEN`</t>
+        </is>
+      </c>
+      <c r="I743" s="2" t="inlineStr">
+        <is>
+          <t>Créer son espace personnel</t>
+        </is>
+      </c>
+      <c r="J743" s="2" t="inlineStr">
+        <is>
+          <t>Administrateur de l'espace (TENANT_ADMIN)</t>
+        </is>
+      </c>
+      <c r="K743" s="2" t="inlineStr">
+        <is>
+          <t>Particulier (espace personnel)</t>
+        </is>
+      </c>
+      <c r="L743" s="2" t="inlineStr">
+        <is>
+          <t>GET /tenants/my-memberships (champ `tenant.type`) ; GET /tenants/:tenantId</t>
+        </is>
+      </c>
+      <c r="M743" s="2" t="inlineStr">
+        <is>
+          <t>Authentifié ; membre de l'espace</t>
+        </is>
+      </c>
+      <c r="N743" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O743" s="2" t="inlineStr">
+        <is>
+          <t>Menu d'un espace particulier ; accueil « Valeur nette »</t>
         </is>
       </c>
     </row>
@@ -58155,7 +58540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -58714,6 +59099,28 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Administration plateforme</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Espace particulier — points ouverts du lot 4</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Limites et décisions à confirmer du lot 4. (1) Le prix (2 900 FCFA HT par mois) et le plafond (100 actifs) du pack Particulier plus sont provisoires ; `db:seed:catalog` sans `--missing-only` écrase les valeurs ajustées. (2) La suppression ou l'anonymisation d'un compte ou d'un espace, l'export libre-service, la conservation des données, les consentements et conditions d'utilisation ne sont pas traités. (3) L'inscription est limitée par adresse IP (3 par heure, dépend de `trust proxy = 1`, un CGNAT partage une IP, fail-open en cas de panne de base) ; pas de captcha, de filtre de domaines jetables ni de normalisation des alias e-mail. (4) L'IP est encore journalisée en clair par le middleware de journalisation. (5) Le paiement mobile money réel n'est pas testé sans identifiants PaySecureHub de production ; la notification de paiement n'est pas signée (constat antérieur). (6) L'idempotence de la création d'espace est en mémoire du processus ; la garde d'unicité en base reste la référence. (7) Aucune rétrogradation payant vers gratuit ; aucun rôle dédié « particulier » (le créateur est TENANT_ADMIN, encadré par la liste blanche de routes). (8) Recette manuelle dans un navigateur non faite : parcours vérifié par tests et build seulement.</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Faire fixer par le produit le prix et le plafond du palier payant, la conservation et la suppression des données, les conditions d'utilisation et la protection des données par pays ; obtenir les identifiants PaySecureHub pour tester le paiement réel ; décider d'un captcha.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
feat(patrimoine): suppression d'un bien refusée avec un prêt actif ; décisions métier du 2026-09-29
- deleteProperty : 409 tant qu'un prêt ACTIF est adossé au bien (test, traductions en/ar, wiki)
- docx du fournisseur de paiement retiré du suivi git et ignoré
- décisions consignées : spec 026, HANDOFF, notes du wiki

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PxDVZM8akvCsSCfK3Cgg19
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -1154,7 +1154,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>204 No Content</t>
+          <t>204 No Content 409 « Ce bien porte un prêt actif : soldez-le ou supprimez-le avant de supprimer le bien. » quand un prêt ACTIF porte sur le bien (la suppression emporterait le prêt en cascade).</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -56590,7 +56590,7 @@
       </c>
       <c r="H726" s="2" t="inlineStr">
         <is>
-          <t>L'actif immobilier lié au bien est supprimé avec lui (clé étrangère en cascade sur `assets.property_id`), comme les valorisations, prêts et parts du bien (tous supprimés en cascade avec lui) ; le bien disparaît donc de la valeur nette</t>
+          <t>L'actif immobilier lié au bien est supprimé avec lui (clé étrangère en cascade sur `assets.property_id`), comme les valorisations, prêts et parts du bien (tous supprimés en cascade avec lui) ; le bien disparaît donc de la valeur nette 409 « Ce bien porte un prêt actif : soldez-le ou supprimez-le avant de supprimer le bien. » quand un prêt ACTIF porte sur le bien (la suppression emporterait le prêt en cascade).</t>
         </is>
       </c>
       <c r="I726" s="2" t="inlineStr">
@@ -59112,12 +59112,12 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Limites et décisions à confirmer du lot 4. (1) Le prix (2 900 FCFA HT par mois) et le plafond (100 actifs) du pack Particulier plus sont provisoires ; `db:seed:catalog` sans `--missing-only` écrase les valeurs ajustées. (2) La suppression ou l'anonymisation d'un compte ou d'un espace, l'export libre-service, la conservation des données, les consentements et conditions d'utilisation ne sont pas traités. (3) L'inscription est limitée par adresse IP (3 par heure, dépend de `trust proxy = 1`, un CGNAT partage une IP, fail-open en cas de panne de base) ; pas de captcha, de filtre de domaines jetables ni de normalisation des alias e-mail. (4) L'IP est encore journalisée en clair par le middleware de journalisation. (5) Le paiement mobile money réel n'est pas testé sans identifiants PaySecureHub de production ; la notification de paiement n'est pas signée (constat antérieur). (6) L'idempotence de la création d'espace est en mémoire du processus ; la garde d'unicité en base reste la référence. (7) Aucune rétrogradation payant vers gratuit ; aucun rôle dédié « particulier » (le créateur est TENANT_ADMIN, encadré par la liste blanche de routes). (8) Recette manuelle dans un navigateur non faite : parcours vérifié par tests et build seulement.</t>
+          <t>Limites et décisions à confirmer du lot 4. (1) Décision du 2026-09-29 : le prix (2 900 FCFA HT par mois) et le plafond (100 actifs) du pack Particulier plus sont conservés, restant modifiables dans le catalogue ; `db:seed:catalog` sans `--missing-only` écrase les valeurs ajustées. (2) Décision du 2026-09-29 : conservation des données, suppression sur demande à l'équipe ; la suppression ou l'anonymisation libre-service, l'export libre-service, les consentements et conditions d'utilisation ne sont pas traités. (3) L'inscription est limitée par adresse IP (3 par heure, dépend de `trust proxy = 1`, un CGNAT partage une IP, fail-open en cas de panne de base) ; pas de captcha (décision du 2026-09-29 : pas maintenant), de filtre de domaines jetables ni de normalisation des alias e-mail. (4) L'IP est encore journalisée en clair par le middleware de journalisation. (5) Le paiement mobile money réel n'est pas testé sans identifiants PaySecureHub de production ; la notification de paiement n'est pas signée (constat antérieur). (6) L'idempotence de la création d'espace est en mémoire du processus ; la garde d'unicité en base reste la référence. (7) Aucune rétrogradation payant vers gratuit ; aucun rôle dédié « particulier » (le créateur est TENANT_ADMIN, encadré par la liste blanche de routes). (8) Recette manuelle dans un navigateur non faite : parcours vérifié par tests et build seulement.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Faire fixer par le produit le prix et le plafond du palier payant, la conservation et la suppression des données, les conditions d'utilisation et la protection des données par pays ; obtenir les identifiants PaySecureHub pour tester le paiement réel ; décider d'un captcha.</t>
+          <t>Faire relire par un juriste les conditions d'utilisation, la conservation et la protection des données par pays ; obtenir les identifiants PaySecureHub pour tester le paiement réel ; revoir le captcha avant l'ouverture publique.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(copilot): wiki des fonctionnalités (réglages IA) et passation
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sous-fonctionnalites" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Legende Packs-Modules" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Notes et points ouverts" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sous-fonctionnalites" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legende Packs-Modules" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes et points ouverts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -189,7 +189,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O698" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O701" headerRowCount="1">
   <autoFilter ref="A1:O698"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Domaine (regroupement agent)"/>
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O698"/>
+  <dimension ref="A1:O701"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -53812,7 +53812,7 @@
       </c>
       <c r="F690" s="2" t="inlineStr">
         <is>
-          <t>Interroge l'assistant à l'ouverture de la coquille d'agence : indique s'il est activé et quels outils l'utilisateur peut employer (permissions RBAC et, en mode `enforce`, modules de l'abonnement). Le bouton flottant « Assistant » (raccourci Ctrl/Cmd+J) n'apparaît que si `enabled` est vrai ; toute erreur de statut le masque</t>
+          <t>Interroge l'assistant à l'ouverture de la coquille d'agence : indique s'il est activé et quels outils l'utilisateur peut employer (permissions RBAC et, en mode `enforce`, modules de l'abonnement). Le bouton flottant « Assistant » (raccourci Ctrl/Cmd+J) n'apparaît que si `enabled` est vrai ; toute erreur de statut le masque Le fournisseur et le modèle effectifs viennent du réglage plateforme (écran « Assistant IA » de l'administration) ou, à défaut, des variables AI_*.</t>
         </is>
       </c>
       <c r="G690" s="2" t="inlineStr">
@@ -53822,7 +53822,7 @@
       </c>
       <c r="H690" s="2" t="inlineStr">
         <is>
-          <t>`{success, data: {enabled, reason? (NOT_CONFIGURED | NO_TOOLS), provider (fake | anthropic | null), tools[], limits {maxMessages, maxMessageChars}}}`</t>
+          <t>`{success, data: {enabled, reason? (NOT_CONFIGURED | NO_TOOLS), provider (fake | anthropic | openrouter | null), tools[], limits {maxMessages, maxMessageChars}}}`</t>
         </is>
       </c>
       <c r="I690" s="2" t="inlineStr">
@@ -54474,6 +54474,237 @@
       <c r="O698" s="2" t="inlineStr">
         <is>
           <t>Bouton flottant Assistant (Ctrl/Cmd+J), toutes pages d'agence</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" s="2" t="inlineStr">
+        <is>
+          <t>Administration plateforme</t>
+        </is>
+      </c>
+      <c r="B699" s="2" t="inlineStr">
+        <is>
+          <t>N/A (plateforme)</t>
+        </is>
+      </c>
+      <c r="C699" s="2" t="inlineStr">
+        <is>
+          <t>Administration plateforme</t>
+        </is>
+      </c>
+      <c r="D699" s="2" t="inlineStr">
+        <is>
+          <t>Réglages de l'Assistant IA</t>
+        </is>
+      </c>
+      <c r="E699" s="2" t="inlineStr">
+        <is>
+          <t>Consulter le réglage IA de la plateforme</t>
+        </is>
+      </c>
+      <c r="F699" s="2" t="inlineStr">
+        <is>
+          <t>Affiche le fournisseur (désactivé, OpenRouter, Anthropic, faux fournisseur de recette), le modèle, l'effort et le repli, la source du réglage (base de données ou variables d'environnement), qui l'a modifié en dernier, et la disponibilité de chaque fournisseur (clé présente ou non dans le .env du serveur ; `fake` refusé en production). Aucune clé n'est renvoyée</t>
+        </is>
+      </c>
+      <c r="G699" s="2" t="inlineStr">
+        <is>
+          <t>GET (aucun corps)</t>
+        </is>
+      </c>
+      <c r="H699" s="2" t="inlineStr">
+        <is>
+          <t>`{success, data: {provider, model, effort, refusalFallback, updatedAt, updatedByName, providers[{id,label,available,reason?}], keys{openrouter,anthropic}, source}}`</t>
+        </is>
+      </c>
+      <c r="I699" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J699" s="2" t="inlineStr">
+        <is>
+          <t>Super-admin</t>
+        </is>
+      </c>
+      <c r="K699" s="2" t="inlineStr">
+        <is>
+          <t>Plateforme</t>
+        </is>
+      </c>
+      <c r="L699" s="2" t="inlineStr">
+        <is>
+          <t>GET `/api/platform/ai-settings`</t>
+        </is>
+      </c>
+      <c r="M699" s="2" t="inlineStr">
+        <is>
+          <t>`authenticate` + `requirePermission('PLATFORM_TENANTS_VIEW')` + `requireSuperAdmin`</t>
+        </is>
+      </c>
+      <c r="N699" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O699" s="2" t="inlineStr">
+        <is>
+          <t>Administration &gt; Assistant IA</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" s="2" t="inlineStr">
+        <is>
+          <t>Administration plateforme</t>
+        </is>
+      </c>
+      <c r="B700" s="2" t="inlineStr">
+        <is>
+          <t>N/A (plateforme)</t>
+        </is>
+      </c>
+      <c r="C700" s="2" t="inlineStr">
+        <is>
+          <t>Administration plateforme</t>
+        </is>
+      </c>
+      <c r="D700" s="2" t="inlineStr">
+        <is>
+          <t>Réglages de l'Assistant IA</t>
+        </is>
+      </c>
+      <c r="E700" s="2" t="inlineStr">
+        <is>
+          <t>Choisir le fournisseur et le modèle de l'assistant</t>
+        </is>
+      </c>
+      <c r="F700" s="2" t="inlineStr">
+        <is>
+          <t>Enregistre le réglage unique de la plateforme (valable pour toutes les agences, effet à chaud sous 30 s). OpenRouter exige OPENROUTER_API_KEY côté serveur et un identifiant `fournisseur/modèle` ; Anthropic exige ANTHROPIC_API_KEY ; l'effort et le repli ne valent que pour Anthropic. La modification est tracée au journal d'audit (`AI_SETTINGS_UPDATED`, sans secret)</t>
+        </is>
+      </c>
+      <c r="G700" s="2" t="inlineStr">
+        <is>
+          <t>`{provider (disabled | fake | anthropic | openrouter), model, effort (low | medium | high), refusalFallback}` — schéma strict</t>
+        </is>
+      </c>
+      <c r="H700" s="2" t="inlineStr">
+        <is>
+          <t>Même forme que la consultation ; 422 avec `errors[{field,message}]` si une règle métier est violée</t>
+        </is>
+      </c>
+      <c r="I700" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J700" s="2" t="inlineStr">
+        <is>
+          <t>Super-admin</t>
+        </is>
+      </c>
+      <c r="K700" s="2" t="inlineStr">
+        <is>
+          <t>Plateforme</t>
+        </is>
+      </c>
+      <c r="L700" s="2" t="inlineStr">
+        <is>
+          <t>PUT `/api/platform/ai-settings`</t>
+        </is>
+      </c>
+      <c r="M700" s="2" t="inlineStr">
+        <is>
+          <t>`authenticate` + `requirePermission('PLATFORM_TENANTS_EDIT')` + `requireSuperAdmin`</t>
+        </is>
+      </c>
+      <c r="N700" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O700" s="2" t="inlineStr">
+        <is>
+          <t>Administration &gt; Assistant IA &gt; Enregistrer</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" s="2" t="inlineStr">
+        <is>
+          <t>Administration plateforme</t>
+        </is>
+      </c>
+      <c r="B701" s="2" t="inlineStr">
+        <is>
+          <t>N/A (plateforme)</t>
+        </is>
+      </c>
+      <c r="C701" s="2" t="inlineStr">
+        <is>
+          <t>Administration plateforme</t>
+        </is>
+      </c>
+      <c r="D701" s="2" t="inlineStr">
+        <is>
+          <t>Réglages de l'Assistant IA</t>
+        </is>
+      </c>
+      <c r="E701" s="2" t="inlineStr">
+        <is>
+          <t>Rechercher un modèle dans le catalogue OpenRouter</t>
+        </is>
+      </c>
+      <c r="F701" s="2" t="inlineStr">
+        <is>
+          <t>Alimente la recherche de modèle de l'écran : liste publique des modèles OpenRouter (sans clé, délai de 5 s, cache de 10 minutes). Si le catalogue est injoignable, la liste est vide et `unavailable` vaut vrai : l'identifiant se saisit alors à la main</t>
+        </is>
+      </c>
+      <c r="G701" s="2" t="inlineStr">
+        <is>
+          <t>GET (aucun corps)</t>
+        </is>
+      </c>
+      <c r="H701" s="2" t="inlineStr">
+        <is>
+          <t>`{success, data: {models[{id,name,contextLength|null}], unavailable}}`</t>
+        </is>
+      </c>
+      <c r="I701" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J701" s="2" t="inlineStr">
+        <is>
+          <t>Super-admin</t>
+        </is>
+      </c>
+      <c r="K701" s="2" t="inlineStr">
+        <is>
+          <t>Plateforme</t>
+        </is>
+      </c>
+      <c r="L701" s="2" t="inlineStr">
+        <is>
+          <t>GET `/api/platform/ai-settings/models`</t>
+        </is>
+      </c>
+      <c r="M701" s="2" t="inlineStr">
+        <is>
+          <t>`authenticate` + `requirePermission('PLATFORM_TENANTS_VIEW')` + `requireSuperAdmin`</t>
+        </is>
+      </c>
+      <c r="N701" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O701" s="2" t="inlineStr">
+        <is>
+          <t>Administration &gt; Assistant IA &gt; champ Modèle</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(recette): rapport final, scénarios des six packs, wiki et passation
Scénarios et journaux des six packs, index des anomalies, rapport final de la
recette, classeur des fonctionnalités et son miroir (wiki:export), RUNBOOK
(migration et rattrapage des permissions Syndic) et HANDOFF.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -189,8 +189,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O701" headerRowCount="1">
-  <autoFilter ref="A1:O698"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O711" headerRowCount="1">
+  <autoFilter ref="A1:O711"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Domaine (regroupement agent)"/>
     <tableColumn id="2" name="Pack(s)"/>
@@ -617,7 +617,7 @@
     <row r="12" ht="34" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>1. Sous-fonctionnalites : le tableau complet (619 lignes), une ligne par action. Colonnes demandees (Pack, Module, Fonctionnalite, Sous-fonctionnalite, Objectif, Donnees d'entree/sortie, Dependances, Fait partie de) + colonnes ajoutees utiles pour le wiki : Roles/profils, Portail, Route API, Permission technique, Statut, Menu affiche.</t>
+          <t>1. Sous-fonctionnalites : le tableau complet (710 lignes), une ligne par action. Colonnes demandees (Pack, Module, Fonctionnalite, Sous-fonctionnalite, Objectif, Donnees d'entree/sortie, Dependances, Fait partie de) + colonnes ajoutees utiles pour le wiki : Roles/profils, Portail, Route API, Permission technique, Statut, Menu affiche.</t>
         </is>
       </c>
     </row>
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O701"/>
+  <dimension ref="A1:O711"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -836,7 +836,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Ajouter un bien au portefeuille de l'agence (ou un bien privé/CLIENT selon `ownershipType`)</t>
+          <t>Ajouter un bien au portefeuille de l'agence (ou un bien privé/CLIENT selon `ownershipType`). Dans l'assistant de création, le champ « Propriétaire » propose « L'agence » (bien détenu en propre) ou « Un client » (bien `CLIENT`, client propriétaire à choisir ; choix absent d'un compte Patrimoine seul) ; le type « Boutique / Commercial » est proposé. Le nom du propriétaire choisi est enregistré avec le bien.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Suppression définitive (cascade médias/documents/lots) ; bloquée si affaires CRM actives liées</t>
+          <t>Suppression définitive (cascade médias/documents/lots) ; bloquée si affaires CRM actives liées. Refus 409 détaillé (bail, mandat, ticket, compromis ou mandat de vente, visite planifiée, document, lot rattaché, affaire active) avec invitation à archiver le bien (statut « Archivé »), affiché tel quel dans la fiche.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1154,7 +1154,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>204 No Content</t>
+          <t>204 No Content. 409 listant les blocages en cas de refus</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Uploader un fichier (photo JPEG/PNG/WebP ou vidéo MP4/WebM/QuickTime) rattaché au bien</t>
+          <t>Uploader un fichier (photo JPEG/PNG/WebP ou vidéo MP4/WebM/QuickTime) rattaché au bien. Un type de fichier qui ne correspond pas à `mediaType` est refusé en 400 avec un message traduit, affiché à l'utilisateur ; les réponses sur les médias n'exposent plus le chemin disque.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -2299,7 +2299,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Uploader une pièce (PDF/Word/image, TIFF/DWG pour les plans) avec type, expiration, caractère obligatoire</t>
+          <t>Uploader une pièce (PDF/Word/image, TIFF/DWG pour les plans) avec type, expiration, caractère obligatoire. Depuis l'onglet « Documents » de la fiche bien (liste, dépôt, téléchargement, suppression).</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -2607,7 +2607,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Faire prendre en gestion, par l'agence, un bien à propriétaire privé (`ownershipType=CLIENT`)</t>
+          <t>Faire prendre en gestion, par l'agence, un bien à propriétaire privé (`ownershipType=CLIENT`). Depuis l'onglet « Mandat de gestion » de la fiche d'un bien client, bouton « Confier ce bien » (onglet absent d'un compte Patrimoine seul). Le mandat et le registre des lots sont écrits dans la même transaction : un bien client loué entre tout de suite dans la réserve LOTS ; en mode Bloquer, un quota plein répond 409 `QUOTA_EXCEEDED` et annule le mandat.</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -2617,7 +2617,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Mandat créé (`isActive:true`)</t>
+          <t>Mandat créé (`isActive:true`). Erreurs typées et traduites : bien introuvable 404, bien non CLIENT 400, mandat actif déjà présent 409, agence sans droit 403 ; refus 403 `OWN_ASSETS_ONLY` avant toute lecture du bien pour un compte Patrimoine seul.</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -2684,7 +2684,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Lister les mandats actifs du tenant sur ce bien (jamais ceux d'une autre agence)</t>
+          <t>Lister les mandats actifs du tenant sur ce bien (jamais ceux d'une autre agence). Affichés dans l'onglet « Mandat de gestion » de la fiche bien.</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -3069,12 +3069,12 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Programmer une visite (type, objectif, contact/affaire CRM liés, collaborateurs, assigné) pour un bien</t>
+          <t>Programmer une visite (type, objectif, contact/affaire CRM liés, collaborateurs, assigné) pour un bien. Refus 409 si le bien a déjà une visite active qui chevauche le créneau (créneaux contigus acceptés ; le créneau en conflit est renvoyé dans `data.conflict`).</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Body : `contactId`/`dealId` optionnels, `visitType`, `goal` optionnel, `scheduledAt` (doit être future), `duration`, `location`, `assignedToUserId`, `collaboratorIds[]`, `notes`</t>
+          <t>Body : `contactId`/`dealId` optionnels, `visitType`, `goal` optionnel, `scheduledAt` (doit être future), `duration`, `location`, `assignedToUserId`, `collaboratorIds[]`, `notes`. Corps validé : statut, type ou objectif inconnus, ou date illisible, répondent 400 `VALIDATION_ERROR`</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -3223,7 +3223,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Faire évoluer le statut d'une visite (ex. confirmée, annulée)</t>
+          <t>Faire évoluer le statut d'une visite (ex. confirmée, annulée). Statut validé : une valeur inconnue répond 400 `VALIDATION_ERROR` (plus d'erreur brute).</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -4003,7 +4003,7 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Agrégat patrimoine (voir `getPatrimoineOverview`)</t>
+          <t>Agrégat patrimoine (voir `getPatrimoineOverview`). La valeur courante d'un bien est sa dernière valorisation (date, puis horodatage de création, puis identifiant) : deux valorisations du même jour sont départagées par la plus récente saisie.</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
@@ -4070,7 +4070,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Calculer rendement brut/net/net-net, plus-value latente, projection à horizon, pour tout le portefeuille (sans `propertyId`) ou pour un bien précis ; avec `propertyId`, le net-net et la plus-value latente sont `null` tant que le prix d'acquisition du bien est inconnu</t>
+          <t>Calculer rendement brut/net/net-net, plus-value latente, projection à horizon, pour tout le portefeuille (sans `propertyId`) ou pour un bien précis ; avec `propertyId`, le net-net et la plus-value latente sont `null` tant que le prix d'acquisition du bien est inconnu. Rendements arrondis (et non tronqués), affichés au format français ; le net-net projeté se rapporte au plus élevé du coût de revient et de la valeur projetée, si bien que brut ≥ net ≥ net-net à tout horizon.</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -4147,7 +4147,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Calculer les rendements et la projection pour un bien donné (variante par bien de la performance) ; loyer annuel = somme des loyers annualisés de chaque bail actif selon sa périodicité (mensuelle/trimestrielle/semestrielle/annuelle) ; charges annuelles = dépenses non capitalisées payées dans les 12 derniers mois glissants ; `netNetYield` et la plus-value latente valent `null` (affichés « — » à l'écran) tant qu'aucun prix d'acquisition n'est connu</t>
+          <t>Calculer les rendements et la projection pour un bien donné (variante par bien de la performance) ; loyer annuel = somme des loyers annualisés de chaque bail actif selon sa périodicité (mensuelle/trimestrielle/semestrielle/annuelle) ; charges annuelles = dépenses non capitalisées payées dans les 12 derniers mois glissants ; `netNetYield` et la plus-value latente valent `null` (affichés « — » à l'écran) tant qu'aucun prix d'acquisition n'est connu. Rendements arrondis (et non tronqués), affichés au format français ; le net-net projeté se rapporte au plus élevé du coût de revient et de la valeur projetée, si bien que brut ≥ net ≥ net-net à tout horizon.</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -4224,7 +4224,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Lister l'historique des estimations de valeur d'un bien</t>
+          <t>Lister l'historique des estimations de valeur d'un bien. Ordre unique : date de valorisation, puis horodatage de création, puis identifiant (la plus récente d'abord).</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -4696,7 +4696,7 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>Dépense créée</t>
+          <t>Dépense créée. Pour un bien détenu en propre, la dépense est écrite au journal dans la même transaction (charge / trésorerie, ou 401 si l'agence doit la facture), contre-passée si elle est modifiée ou supprimée.</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
@@ -4850,7 +4850,7 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>Dépense mise à jour</t>
+          <t>Dépense mise à jour. Pour un bien détenu en propre, la dépense est écrite au journal dans la même transaction (charge / trésorerie, ou 401 si l'agence doit la facture), contre-passée si elle est modifiée ou supprimée.</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
@@ -4927,7 +4927,7 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>204 No Content</t>
+          <t>204 No Content. Pour un bien détenu en propre, la dépense est écrite au journal dans la même transaction (charge / trésorerie, ou 401 si l'agence doit la facture), contre-passée si elle est modifiée ou supprimée.</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
@@ -6149,7 +6149,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Ouvrir un nouveau bail sur un bien</t>
+          <t>Ouvrir un nouveau bail sur un bien. Création atomique : le client et le compte du locataire ou du bailleur issus d'un contact sont créés dans la même transaction que le bail, et les refus (barrière « détenu en propre » 403 `OWN_ASSETS_ONLY`, bien ou client d'une autre agence) interviennent avant toute écriture. Un compte Patrimoine seul ne voit pas le champ Propriétaire du formulaire.</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -6236,7 +6236,7 @@
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>Liste paginée / fiche bail (co-locataires, dépôt, documents inclus)</t>
+          <t>Liste paginée / fiche bail (co-locataires, dépôt, documents inclus). Documents du bail renvoyés sans chemin disque.</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
@@ -6842,7 +6842,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Appliquer un nouveau loyer/charges à partir d'un mois donné</t>
+          <t>Appliquer un nouveau loyer/charges à partir d'un mois donné. Une révision à date d'effet future est « planifiée » : le loyer du bail et les indicateurs (vue consolidée, rendement) gardent l'ancien montant jusqu'à cette date, puis le job quotidien l'applique ; la facturation d'une période utilise le loyer effectif de la période.</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -6919,7 +6919,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>Repousser la fin du bail et générer les échéances de la nouvelle période</t>
+          <t>Repousser la fin du bail et générer les échéances de la nouvelle période. Un nouveau loyer à date d'effet future est planifié de la même façon (le bail garde l'ancien loyer jusqu'à la première période concernée).</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -7853,7 +7853,7 @@
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>Mouvement créé, montants agrégés du dépôt mis à jour</t>
+          <t>Mouvement créé, montants agrégés du dépôt mis à jour. Solde détenu = collecté − remboursé − retenu : une restitution ou une retenue n'est décomptée qu'une fois. Un dépôt ne s'encaisse qu'en un seul paiement (seconde collecte refusée en 400 traduit) et un solde insuffisant est refusé (400 traduit).</t>
         </is>
       </c>
       <c r="I93" s="2" t="inlineStr">
@@ -8084,7 +8084,7 @@
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>Liste / détail du document</t>
+          <t>Liste / détail du document. Sans chemin disque.</t>
         </is>
       </c>
       <c r="I96" s="2" t="inlineStr">
@@ -8228,7 +8228,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>Créer la totalité des échéances (loyer + charges) du bail selon sa fréquence</t>
+          <t>Créer la totalité des échéances (loyer + charges) du bail selon sa fréquence. Les échéances sont créées à l'état « Brouillon » ; la campagne de facturation du mois les émet.</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -8305,7 +8305,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>Suivre les échéances (par bail, par locataire, en retard...)</t>
+          <t>Suivre les échéances (par bail, par locataire, en retard...). Le statut est reclassé à l'affichage : une échéance échue et non soldée apparaît « En retard » (Brouillon comprise) même si le job quotidien n'a pas tourné.</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -8382,7 +8382,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>Remettre à jour les statuts (DRAFT/DUE/OVERDUE/PARTIAL/PAID) d'un bail</t>
+          <t>Remettre à jour les statuts (DRAFT/DUE/OVERDUE/PARTIAL/PAID) d'un bail. Les échéances Brouillon ou « À payer » échues passent « En retard ».</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -8536,7 +8536,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>Saisir un règlement reçu du locataire</t>
+          <t>Saisir un règlement reçu du locataire. Sur l'écran Échéances, « Encaisser » demande confirmation (montant, locataire, échéance, mode espèces) avant d'enregistrer ; la liste des paiements affiche le locataire et des montants en FCFA.</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -9152,7 +9152,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>Chiffrer la pénalité due sur une échéance en retard, ou lancer le calcul en masse</t>
+          <t>Chiffrer la pénalité due sur une échéance en retard, ou lancer le calcul en masse. Les échéances Brouillon échues sont comptées comme les autres ; le délai de grâce est celui du bail, sinon celui de la règle de pénalité de l'agence.</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -9537,7 +9537,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>Voir, pour chaque propriétaire, le solde dû (loyers encaissés − honoraires − TVA − dépenses − reversements)</t>
+          <t>Voir, pour chaque propriétaire, le solde dû (loyers encaissés − honoraires − TVA − dépenses − reversements). Refusé (403 `OWN_ASSETS_ONLY`) à un compte Patrimoine seul : les comptes propriétaires tiers exigent le pack Agence.</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>Enregistrer le paiement du solde dû à un propriétaire</t>
+          <t>Enregistrer le paiement du solde dû à un propriétaire. Refusé (403 `OWN_ASSETS_ONLY`) à un compte Patrimoine seul : les comptes propriétaires tiers exigent le pack Agence.</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -9691,7 +9691,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>Défaire un reversement erroné</t>
+          <t>Défaire un reversement erroné. Refusé (403 `OWN_ASSETS_ONLY`) à un compte Patrimoine seul : les comptes propriétaires tiers exigent le pack Agence.</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -9922,7 +9922,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>Fixer le mode (taux ou montant fixe), la base de calcul, et le statut fiscal (retenue à la source) par propriétaire</t>
+          <t>Fixer le mode (taux ou montant fixe), la base de calcul, et le statut fiscal (retenue à la source) par propriétaire. Refusé (403 `OWN_ASSETS_ONLY`) à un compte Patrimoine seul ; section masquée sans gestion locative.</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -9999,7 +9999,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>Supprimer la dérogation propriétaire, retomber sur les réglages de l'agence</t>
+          <t>Supprimer la dérogation propriétaire, retomber sur les réglages de l'agence. Refusé (403 `OWN_ASSETS_ONLY`) à un compte Patrimoine seul.</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -10076,7 +10076,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>Fixer la part de commission (%) de chaque collaborateur actif sur les honoraires</t>
+          <t>Fixer la part de commission (%) de chaque collaborateur actif sur les honoraires. Refusé (403 `OWN_ASSETS_ONLY`) à un compte Patrimoine seul ; section masquée sans gestion locative.</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -10173,7 +10173,7 @@
       </c>
       <c r="J123" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — OWNER_STATEMENTS_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K123" s="2" t="inlineStr">
@@ -10188,7 +10188,7 @@
       </c>
       <c r="M123" s="2" t="inlineStr">
         <is>
-          <t>PROPERTIES_VIEW</t>
+          <t>OWNER_STATEMENTS_VIEW</t>
         </is>
       </c>
       <c r="N123" s="2" t="inlineStr">
@@ -10230,7 +10230,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>Calculer le relevé mensuel de gérance d'un propriétaire sur un ensemble de biens</t>
+          <t>Calculer le relevé mensuel de gérance d'un propriétaire sur un ensemble de biens. Refusé (403 `OWN_ASSETS_ONLY`) à un compte Patrimoine seul (création et envoi d'un relevé de gérance pour un tiers exigent le pack Agence).</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -10250,7 +10250,7 @@
       </c>
       <c r="J124" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — OWNER_STATEMENTS_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K124" s="2" t="inlineStr">
@@ -10265,7 +10265,7 @@
       </c>
       <c r="M124" s="2" t="inlineStr">
         <is>
-          <t>PROPERTIES_EDIT</t>
+          <t>OWNER_STATEMENTS_EDIT</t>
         </is>
       </c>
       <c r="N124" s="2" t="inlineStr">
@@ -10327,7 +10327,7 @@
       </c>
       <c r="J125" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — OWNER_STATEMENTS_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K125" s="2" t="inlineStr">
@@ -10342,7 +10342,7 @@
       </c>
       <c r="M125" s="2" t="inlineStr">
         <is>
-          <t>PROPERTIES_EDIT</t>
+          <t>OWNER_STATEMENTS_EDIT</t>
         </is>
       </c>
       <c r="N125" s="2" t="inlineStr">
@@ -10404,7 +10404,7 @@
       </c>
       <c r="J126" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — OWNER_STATEMENTS_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K126" s="2" t="inlineStr">
@@ -10419,7 +10419,7 @@
       </c>
       <c r="M126" s="2" t="inlineStr">
         <is>
-          <t>PROPERTIES_EDIT</t>
+          <t>OWNER_STATEMENTS_EDIT</t>
         </is>
       </c>
       <c r="N126" s="2" t="inlineStr">
@@ -10461,7 +10461,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>Transmettre le relevé (notification) au propriétaire</t>
+          <t>Transmettre le relevé (notification) au propriétaire. Refusé (403 `OWN_ASSETS_ONLY`) à un compte Patrimoine seul.</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -10481,7 +10481,7 @@
       </c>
       <c r="J127" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — OWNER_STATEMENTS_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K127" s="2" t="inlineStr">
@@ -10496,7 +10496,7 @@
       </c>
       <c r="M127" s="2" t="inlineStr">
         <is>
-          <t>PROPERTIES_EDIT</t>
+          <t>OWNER_STATEMENTS_EDIT</t>
         </is>
       </c>
       <c r="N127" s="2" t="inlineStr">
@@ -11924,7 +11924,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>Lister les écritures comptables d'une période, par journal</t>
+          <t>Lister les écritures comptables d'une période, par journal. Reprend les écritures automatiques de la gestion locative directe (voir « Écrire automatiquement la comptabilité de la gestion locative directe »).</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -12078,7 +12078,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>Balance des comptes sur une période</t>
+          <t>Balance des comptes sur une période. Intitulés du plan de comptes accentués (par exemple « Tâcherons », « Stocks de matières et fournitures »).</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -12463,7 +12463,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>Générer les factures de loyer du mois pour les baux actifs</t>
+          <t>Générer les factures de loyer du mois pour les baux actifs. Une échéance déjà générée en Brouillon pour la période est émise (« À payer », ou « En retard » si la date est passée) et inscrite au compte du locataire ; une échéance déjà émise est exclue sans doublon. Le loyer facturé est le loyer effectif de la période (révisions datées). Sans gestion locative, l'écran est remplacé par « Fonction non comprise dans votre abonnement ».</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -12540,7 +12540,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>Solde facturé/réglé par locataire, exportable CSV</t>
+          <t>Solde facturé/réglé par locataire, exportable CSV. Une échéance ne compte au solde qu'à sa date d'exigibilité (règle commune au relevé du portail locataire, au compte du locataire et au relevé DOCX) ; écran remplacé par « Fonction non comprise dans votre abonnement » sans gestion locative.</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -12617,7 +12617,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>Ancienneté des impayés (tranches d'âge) à une date donnée</t>
+          <t>Ancienneté des impayés (tranches d'âge) à une date donnée. Écran remplacé par « Fonction non comprise dans votre abonnement » sans gestion locative.</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -12694,7 +12694,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>Détail des mouvements d'un compte (client/mandant) sur une période, paginé</t>
+          <t>Détail des mouvements d'un compte (client/mandant) sur une période, paginé. Même règle d'exigibilité que la balance clients et le relevé du portail locataire.</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -13541,7 +13541,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>Solde dû par fournisseur sur une période, filtrable par chantier</t>
+          <t>Solde dû par fournisseur sur une période, filtrable par chantier. Une facture annulée et sa contrepassation sont écartées des cumuls « Facturé » et « Réglé ».</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -13772,7 +13772,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>Enregistrer une facture en brouillon, avec ses lignes et imputations chantier/poste</t>
+          <t>Enregistrer une facture en brouillon, avec ses lignes et imputations chantier/poste. Les imputations doivent totaliser le montant de la facture (refus 400 dès l'enregistrement : un brouillon mal imputé ne peut plus exister) ; une facture sans imputation (prestation) reste permise. Un fournisseur « Matériaux » n'impose un chantier que si l'agence possède la fonction Chantiers (CONSTRUCTION) ; sans elle, l'écran masque les imputations chantier.</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -14003,7 +14003,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>Contre-passer une facture validée par erreur</t>
+          <t>Contre-passer une facture validée par erreur. Un brouillon (jamais validé) peut aussi être annulé : il passe à annulé, ses imputations sont écartées et le chantier est libéré, sans écriture comptable.</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -14018,7 +14018,7 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>La facture doit être validée et pas déjà annulée (correction par annulation, jamais par modification)</t>
+          <t>La facture doit être validée (ou en brouillon) et pas déjà annulée (correction par annulation, jamais par modification)</t>
         </is>
       </c>
       <c r="J173" s="2" t="inlineStr">
@@ -21857,7 +21857,7 @@
       </c>
       <c r="F275" s="2" t="inlineStr">
         <is>
-          <t>Enregistrer un lead/client (personne ou société)</t>
+          <t>Enregistrer un lead/client (personne ou société). Formulaire à onglets : la commune reste requise même si l'onglet Contact n'a pas été ouvert. Un contact Entreprise s'affiche sous sa raison sociale (listes, sélecteurs). Un doublon d'e-mail est refusé par un message français.</t>
         </is>
       </c>
       <c r="G275" s="2" t="inlineStr">
@@ -23330,7 +23330,7 @@
       </c>
       <c r="H294" s="2" t="inlineStr">
         <is>
-          <t>Fichier CSV (téléchargement)</t>
+          <t>Fichier CSV (téléchargement). Cellules échappées (virgules, guillemets, préfixe anti-formule).</t>
         </is>
       </c>
       <c r="I294" s="2" t="inlineStr">
@@ -23397,7 +23397,7 @@
       </c>
       <c r="F295" s="2" t="inlineStr">
         <is>
-          <t>KPIs (nouveaux leads, conversions, deals créés/gagnés, actions en retard), pipeline, funnel, séries temporelles, insights contacts, workbench, perf équipe</t>
+          <t>KPIs (nouveaux leads, conversions, deals créés/gagnés, actions en retard), pipeline, funnel, séries temporelles, insights contacts, workbench, perf équipe. Types, étapes du pipeline et sources en libellés français (aucun code technique affiché).</t>
         </is>
       </c>
       <c r="G295" s="2" t="inlineStr">
@@ -23479,7 +23479,7 @@
       </c>
       <c r="G296" s="2" t="inlineStr">
         <is>
-          <t>`from`, `to` (obligatoires), `scope?`, `types?` (query)</t>
+          <t>`from`, `to` (obligatoires), `scope?`, `types?` (query). `from` et `to` obligatoires, date ISO valide, intervalle de 366 jours au plus : sinon 400 immédiat (plus de requête pendante)</t>
         </is>
       </c>
       <c r="H296" s="2" t="inlineStr">
@@ -24090,7 +24090,7 @@
       </c>
       <c r="F304" s="2" t="inlineStr">
         <is>
-          <t>Vue paginée par contact, affaire, type, auteur, période</t>
+          <t>Vue paginée par contact, affaire, type, auteur, période. Types d'activité et d'action en libellés français.</t>
         </is>
       </c>
       <c r="G304" s="2" t="inlineStr">
@@ -24860,7 +24860,7 @@
       </c>
       <c r="F314" s="2" t="inlineStr">
         <is>
-          <t>Mandater l'agence pour vendre un bien (prix demandé/plancher, mode et taux de commission, négociateur), un seul mandat ACTIF par bien</t>
+          <t>Mandater l'agence pour vendre un bien (prix demandé/plancher, mode et taux de commission, négociateur), un seul mandat ACTIF par bien. En mode Pourcentage, le taux d'honoraires doit être supérieur à 0 et au plus 20 %.</t>
         </is>
       </c>
       <c r="G314" s="2" t="inlineStr">
@@ -25014,7 +25014,7 @@
       </c>
       <c r="F316" s="2" t="inlineStr">
         <is>
-          <t>Ajuster prix, commission, dates, négociateur</t>
+          <t>Ajuster prix, commission, dates, négociateur. Même règle sur le taux d'honoraires (&gt; 0, ≤ 20 %).</t>
         </is>
       </c>
       <c r="G316" s="2" t="inlineStr">
@@ -25168,7 +25168,7 @@
       </c>
       <c r="F318" s="2" t="inlineStr">
         <is>
-          <t>Déposer une offre d'un acquéreur sur un mandat actif, avec financement, conditions, validité</t>
+          <t>Déposer une offre d'un acquéreur sur un mandat actif, avec financement, conditions, validité. Le sélecteur « Affaire CRM d'origine » affiche contact, type et montant lisibles, sans les affaires perdues ni gagnées.</t>
         </is>
       </c>
       <c r="G318" s="2" t="inlineStr">
@@ -25630,7 +25630,7 @@
       </c>
       <c r="F324" s="2" t="inlineStr">
         <is>
-          <t>Passer le compromis en SIGNED, réserver le bien (UNDER_OFFER)</t>
+          <t>Passer le compromis en SIGNED, réserver le bien (UNDER_OFFER). La fiche compromis se met à jour juste après la signature et la conclusion (frise, boutons, bloc Commission).</t>
         </is>
       </c>
       <c r="G324" s="2" t="inlineStr">
@@ -26477,7 +26477,7 @@
       </c>
       <c r="F335" s="2" t="inlineStr">
         <is>
-          <t>Créer un ticket d'incident pour un bien loué</t>
+          <t>Créer un ticket d'incident pour un bien loué. Un agent de l'agence peut déclarer un ticket sur un bien sans bail (bien en vente, détenu en propre…) ; le bail actif n'est exigé que pour une demande de locataire (contact ou client du portail) ; s'il existe un bail actif, le ticket d'agence s'y rattache. Un bien d'une autre agence reste introuvable.</t>
         </is>
       </c>
       <c r="G335" s="2" t="inlineStr">
@@ -27632,7 +27632,7 @@
       </c>
       <c r="F350" s="2" t="inlineStr">
         <is>
-          <t>Créer un prestataire de maintenance (miroir de `ServiceProvider`, partagé avec le module Syndic)</t>
+          <t>Créer un prestataire de maintenance (miroir de `ServiceProvider`, partagé avec le module Syndic). Le nom est unique dans l'agence (409 « Un prestataire nommé … existe déjà dans votre agence », casse et espaces de bord ignorés).</t>
         </is>
       </c>
       <c r="G350" s="2" t="inlineStr">
@@ -27863,7 +27863,7 @@
       </c>
       <c r="F353" s="2" t="inlineStr">
         <is>
-          <t>Mettre à jour les coordonnées/spécialités d'un prestataire</t>
+          <t>Mettre à jour les coordonnées/spécialités d'un prestataire. Même unicité du nom (409).</t>
         </is>
       </c>
       <c r="G353" s="2" t="inlineStr">
@@ -28941,7 +28941,7 @@
       </c>
       <c r="F367" s="2" t="inlineStr">
         <is>
-          <t>Lister/activer/désactiver, personnaliser sujet+corps HTML, ou réinitialiser un type de notification e-mail (parmi ~38 clés en dur : maintenance, paiements, baux, CRM, syndic, patrimoine, invitation, reset mdp…)</t>
+          <t>Lister/activer/désactiver, personnaliser sujet+corps HTML, ou réinitialiser un type de notification e-mail (parmi ~38 clés en dur : maintenance, paiements, baux, CRM, syndic, patrimoine, invitation, reset mdp…). En mode `enforce`, la liste ne montre et ne laisse modifier que les événements des modules souscrits (locatif, CRM, syndic, patrimoine) : un événement hors pack est masqué et sa modification répond 403 `MODULE_NOT_INCLUDED` ; pour un module retiré en lecture seule, l'événement reste listé s'il reste des données mais n'est plus modifiable (`MODULE_READ_ONLY`). Textes par défaut accentués.</t>
         </is>
       </c>
       <c r="G367" s="2" t="inlineStr">
@@ -29018,7 +29018,7 @@
       </c>
       <c r="F368" s="2" t="inlineStr">
         <is>
-          <t>Lister/activer/désactiver, personnaliser corps (+ `contentSid`/`contentVariablesJson` pour templates WhatsApp Business), ou réinitialiser un type de notification WhatsApp (parmi ~22 clés : maintenance, paiements, baux, CRM, invite groupe, compte portail, syndic…)</t>
+          <t>Lister/activer/désactiver, personnaliser corps (+ `contentSid`/`contentVariablesJson` pour templates WhatsApp Business), ou réinitialiser un type de notification WhatsApp (parmi ~22 clés : maintenance, paiements, baux, CRM, invite groupe, compte portail, syndic…). En mode `enforce`, la liste ne montre et ne laisse modifier que les événements des modules souscrits (locatif, CRM, syndic, patrimoine) : un événement hors pack est masqué et sa modification répond 403 `MODULE_NOT_INCLUDED` ; pour un module retiré en lecture seule, l'événement reste listé s'il reste des données mais n'est plus modifiable (`MODULE_READ_ONLY`). Textes par défaut accentués.</t>
         </is>
       </c>
       <c r="G368" s="2" t="inlineStr">
@@ -29403,7 +29403,7 @@
       </c>
       <c r="F373" s="2" t="inlineStr">
         <is>
-          <t>CRUD des listes (`MANUAL`, `FROM_OWNERS`, `FROM_RENTERS`, `FROM_CRM_CONTACTS`), gestion des abonnés d'une liste manuelle (ajout unitaire, ajout depuis contacts CRM, import CSV, export CSV, retrait) ; les listes dérivées calculent leurs compteurs depuis `TenantClient`/`CrmContact` (consentement) et ne peuvent pas recevoir d'ajout manuel</t>
+          <t>CRUD des listes (`MANUAL`, `FROM_OWNERS`, `FROM_RENTERS`, `FROM_CRM_CONTACTS`), gestion des abonnés d'une liste manuelle (ajout unitaire, ajout depuis contacts CRM, import CSV, export CSV, retrait) ; les listes dérivées calculent leurs compteurs depuis `TenantClient`/`CrmContact` (consentement) et ne peuvent pas recevoir d'ajout manuel. Corps validé : une entrée invalide répond 400 `VALIDATION_ERROR` (plus d'erreur brute).</t>
         </is>
       </c>
       <c r="G373" s="2" t="inlineStr">
@@ -29865,7 +29865,7 @@
       </c>
       <c r="F379" s="2" t="inlineStr">
         <is>
-          <t>Crée une campagne en brouillon (`DRAFT`) rattachée à une liste et (optionnellement) un modèle ; le corps HTML est assaini (DOMPurify) ; modification possible uniquement tant que `DRAFT`</t>
+          <t>Crée une campagne en brouillon (`DRAFT`) rattachée à une liste et (optionnellement) un modèle ; le corps HTML est assaini (DOMPurify) ; modification possible uniquement tant que `DRAFT`. Une campagne sans liste ou aux champs invalides est refusée en 400 `VALIDATION_ERROR`.</t>
         </is>
       </c>
       <c r="G379" s="2" t="inlineStr">
@@ -30255,7 +30255,7 @@
       </c>
       <c r="G384" s="2" t="inlineStr">
         <is>
-          <t>GET `?page&amp;limit`</t>
+          <t>GET `?page&amp;limit`. `page` et `limit` facultatifs (par défaut 1 et 20)</t>
         </is>
       </c>
       <c r="H384" s="2" t="inlineStr">
@@ -30481,7 +30481,7 @@
       </c>
       <c r="F387" s="2" t="inlineStr">
         <is>
-          <t>Liste les modèles actifs/inactifs (hors supprimés) d'un tenant, filtrables par type de document et statut ; si aucun contexte tenant, retourne les modèles globaux (`tenant_id: null`)</t>
+          <t>Liste les modèles actifs/inactifs (hors supprimés) d'un tenant, filtrables par type de document et statut ; si aucun contexte tenant, retourne les modèles globaux (`tenant_id: null`). Les modèles par défaut livrés (bail habitation, bail commercial) sont rafraîchis au seed tant qu'ils n'ont pas été personnalisés ; un modèle d'agence n'est jamais remplacé.</t>
         </is>
       </c>
       <c r="G387" s="2" t="inlineStr">
@@ -30789,17 +30789,17 @@
       </c>
       <c r="F391" s="2" t="inlineStr">
         <is>
-          <t>Génère un `.docx` (bail, quittance, relevé) en résolvant le modèle (`templateId` explicite → modèle par défaut du tenant → dernier modèle actif), en construisant le contexte de fusion depuis le bail/paiement source, en validant les placeholders critiques, puis en enregistrant un `RentalDocument` numéroté (ex. `BAIL-2026-0001`, `RCU-202609-0001`)</t>
+          <t>Génère un `.docx` (bail, quittance, relevé) en résolvant le modèle (`templateId` explicite → modèle par défaut du tenant → dernier modèle actif), en construisant le contexte de fusion depuis le bail/paiement source, en validant les placeholders critiques, puis en enregistrant un `RentalDocument` numéroté (ex. `BAIL-2026-0001`, `RCU-202609-0001`). Avec `docType` `LEASE_CONTRACT`, le modèle suit le type du bien : bail commercial pour Bureau, Boutique / Commercial et Entrepôt industriel, bail habitation sinon. Un contrat par bail (son numéro est celui du bail). Quittance générable depuis un bail : le paiement retenu est le dernier encaissé, ou celui affecté à `installmentId`. Bailleur du document : entité détentrice du bien (SCI, holding, société), sinon client propriétaire (l'agence figure comme mandataire), sinon l'agence (« — » pour une coordonnée absente). La clause de pénalité du contrat reprend le mode du bail (forfait, % du loyer, % du solde, plafond). Le relevé de loyer ne compte une échéance qu'à sa date d'exigibilité, comme le compte du locataire.</t>
         </is>
       </c>
       <c r="G391" s="2" t="inlineStr">
         <is>
-          <t>POST `{docType, sourceKey (leaseId ou paymentId), templateId?, installmentId?, startDate?, endDate?}`</t>
+          <t>POST `{docType, sourceKey (leaseId ou paymentId), templateId?, installmentId?, startDate?, endDate?}`. `docType` accepte aussi `LEASE_CONTRACT` ; `sourceKey` est un paiement ou, pour une quittance, un bail (alors `installmentId` facultatif précise le paiement)</t>
         </is>
       </c>
       <c r="H391" s="2" t="inlineStr">
         <is>
-          <t>`{success, data: document, message}` (ou 400 avec `help`/`action:'upload_template'` si aucun modèle disponible)</t>
+          <t>`{success, data: document, message}` (ou 400 avec `help`/`action:'upload_template'` si aucun modèle disponible). 409 si un contrat existe déjà pour le bail, avec `data.existingDocumentId` (l'écran Documents propose « Régénérer ») ; 400 pour une quittance sans aucun paiement encaissé ; document renvoyé sans chemin disque</t>
         </is>
       </c>
       <c r="I391" s="2" t="inlineStr">
@@ -30866,7 +30866,7 @@
       </c>
       <c r="F392" s="2" t="inlineStr">
         <is>
-          <t>Recrée le fichier `.docx` d'un document existant (ex. après correction du contexte ou changement de modèle), incrémente la révision, recalcule les hash fichier/modèle</t>
+          <t>Recrée le fichier `.docx` d'un document existant (ex. après correction du contexte ou changement de modèle), incrémente la révision, recalcule les hash fichier/modèle. Proposé par l'écran Documents quand la génération d'un second contrat d'un même bail est refusée en 409.</t>
         </is>
       </c>
       <c r="G392" s="2" t="inlineStr">
@@ -31040,7 +31040,7 @@
       </c>
       <c r="J394" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW ou SYNDIC_CREATE (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K394" s="2" t="inlineStr">
@@ -31055,7 +31055,7 @@
       </c>
       <c r="M394" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW, PROPERTIES_CREATE])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW, SYNDIC_CREATE])</t>
         </is>
       </c>
       <c r="N394" s="2" t="inlineStr">
@@ -31117,7 +31117,7 @@
       </c>
       <c r="J395" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_CREATE (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K395" s="2" t="inlineStr">
@@ -31132,7 +31132,7 @@
       </c>
       <c r="M395" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_CREATE])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_CREATE])</t>
         </is>
       </c>
       <c r="N395" s="2" t="inlineStr">
@@ -31194,7 +31194,7 @@
       </c>
       <c r="J396" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K396" s="2" t="inlineStr">
@@ -31209,7 +31209,7 @@
       </c>
       <c r="M396" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N396" s="2" t="inlineStr">
@@ -31271,7 +31271,7 @@
       </c>
       <c r="J397" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW ou SYNDIC_CREATE (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K397" s="2" t="inlineStr">
@@ -31286,7 +31286,7 @@
       </c>
       <c r="M397" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW, PROPERTIES_CREATE])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW, SYNDIC_CREATE])</t>
         </is>
       </c>
       <c r="N397" s="2" t="inlineStr">
@@ -31348,7 +31348,7 @@
       </c>
       <c r="J398" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K398" s="2" t="inlineStr">
@@ -31363,7 +31363,7 @@
       </c>
       <c r="M398" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N398" s="2" t="inlineStr">
@@ -31425,7 +31425,7 @@
       </c>
       <c r="J399" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K399" s="2" t="inlineStr">
@@ -31440,7 +31440,7 @@
       </c>
       <c r="M399" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N399" s="2" t="inlineStr">
@@ -31482,7 +31482,7 @@
       </c>
       <c r="F400" s="2" t="inlineStr">
         <is>
-          <t>Afficher les lots d'une copropriété</t>
+          <t>Afficher les lots d'une copropriété. Le propriétaire affiché d'un lot vient des profils propriétaires actuels (plus forte part ; en indivision, plusieurs profils).</t>
         </is>
       </c>
       <c r="G400" s="2" t="inlineStr">
@@ -31502,7 +31502,7 @@
       </c>
       <c r="J400" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K400" s="2" t="inlineStr">
@@ -31517,7 +31517,7 @@
       </c>
       <c r="M400" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N400" s="2" t="inlineStr">
@@ -31559,7 +31559,7 @@
       </c>
       <c r="F401" s="2" t="inlineStr">
         <is>
-          <t>Ajouter un lot (appartement, parking, cave, bureau, commercial, autre) à une copropriété, avec ses tantièmes</t>
+          <t>Ajouter un lot (appartement, parking, cave, bureau, commercial, autre) à une copropriété, avec ses tantièmes. Le numéro de lot est unique dans la copropriété (409 en cas de doublon, casse et espaces de bord ignorés).</t>
         </is>
       </c>
       <c r="G401" s="2" t="inlineStr">
@@ -31579,7 +31579,7 @@
       </c>
       <c r="J401" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_CREATE (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K401" s="2" t="inlineStr">
@@ -31594,7 +31594,7 @@
       </c>
       <c r="M401" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_CREATE])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_CREATE])</t>
         </is>
       </c>
       <c r="N401" s="2" t="inlineStr">
@@ -31656,7 +31656,7 @@
       </c>
       <c r="J402" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_CREATE (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K402" s="2" t="inlineStr">
@@ -31671,7 +31671,7 @@
       </c>
       <c r="M402" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_CREATE])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_CREATE])</t>
         </is>
       </c>
       <c r="N402" s="2" t="inlineStr">
@@ -31713,7 +31713,7 @@
       </c>
       <c r="F403" s="2" t="inlineStr">
         <is>
-          <t>Modifier numéro, type, tantièmes, bien lié, copropriétaire d'un lot</t>
+          <t>Modifier numéro, type, tantièmes, bien lié, copropriétaire d'un lot. Un lot désactivé (tantièmes à 0) sort de la clé de répartition, de la réserve de lots et des appels futurs, mais reste conservé.</t>
         </is>
       </c>
       <c r="G403" s="2" t="inlineStr">
@@ -31733,7 +31733,7 @@
       </c>
       <c r="J403" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K403" s="2" t="inlineStr">
@@ -31748,7 +31748,7 @@
       </c>
       <c r="M403" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N403" s="2" t="inlineStr">
@@ -31810,7 +31810,7 @@
       </c>
       <c r="J404" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K404" s="2" t="inlineStr">
@@ -31825,7 +31825,7 @@
       </c>
       <c r="M404" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N404" s="2" t="inlineStr">
@@ -31887,7 +31887,7 @@
       </c>
       <c r="J405" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K405" s="2" t="inlineStr">
@@ -31902,7 +31902,7 @@
       </c>
       <c r="M405" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N405" s="2" t="inlineStr">
@@ -31954,7 +31954,7 @@
       </c>
       <c r="H406" s="2" t="inlineStr">
         <is>
-          <t>Liste de `LotOwnerProfile`</t>
+          <t>Liste de `LotOwnerProfile`. `summary.incompleteLots` : lots dont les parts actuelles totalisent moins de 100 % (bandeau « quotes-parts incomplètes » de l'écran).</t>
         </is>
       </c>
       <c r="I406" s="2" t="inlineStr">
@@ -31964,7 +31964,7 @@
       </c>
       <c r="J406" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K406" s="2" t="inlineStr">
@@ -31979,7 +31979,7 @@
       </c>
       <c r="M406" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N406" s="2" t="inlineStr">
@@ -32021,7 +32021,7 @@
       </c>
       <c r="F407" s="2" t="inlineStr">
         <is>
-          <t>Enregistrer qui détient un lot, avec sa quote-part et l'accès portail</t>
+          <t>Enregistrer qui détient un lot, avec sa quote-part et l'accès portail. Le total des parts actuelles d'un lot ne peut dépasser 100 % : 409 avec le détail des parts déjà attribuées et demandées.</t>
         </is>
       </c>
       <c r="G407" s="2" t="inlineStr">
@@ -32041,7 +32041,7 @@
       </c>
       <c r="J407" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K407" s="2" t="inlineStr">
@@ -32056,7 +32056,7 @@
       </c>
       <c r="M407" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N407" s="2" t="inlineStr">
@@ -32098,7 +32098,7 @@
       </c>
       <c r="F408" s="2" t="inlineStr">
         <is>
-          <t>Modifier quote-part, dates de détention, activation, accès portail</t>
+          <t>Modifier quote-part, dates de détention, activation, accès portail. Même plafond de 100 % pour les parts d'un lot.</t>
         </is>
       </c>
       <c r="G408" s="2" t="inlineStr">
@@ -32118,7 +32118,7 @@
       </c>
       <c r="J408" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K408" s="2" t="inlineStr">
@@ -32133,7 +32133,7 @@
       </c>
       <c r="M408" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N408" s="2" t="inlineStr">
@@ -32195,7 +32195,7 @@
       </c>
       <c r="J409" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K409" s="2" t="inlineStr">
@@ -32210,7 +32210,7 @@
       </c>
       <c r="M409" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N409" s="2" t="inlineStr">
@@ -32272,7 +32272,7 @@
       </c>
       <c r="J410" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K410" s="2" t="inlineStr">
@@ -32287,7 +32287,7 @@
       </c>
       <c r="M410" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N410" s="2" t="inlineStr">
@@ -32349,7 +32349,7 @@
       </c>
       <c r="J411" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K411" s="2" t="inlineStr">
@@ -32364,7 +32364,7 @@
       </c>
       <c r="M411" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N411" s="2" t="inlineStr">
@@ -32426,7 +32426,7 @@
       </c>
       <c r="J412" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K412" s="2" t="inlineStr">
@@ -32441,7 +32441,7 @@
       </c>
       <c r="M412" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N412" s="2" t="inlineStr">
@@ -32503,7 +32503,7 @@
       </c>
       <c r="J413" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K413" s="2" t="inlineStr">
@@ -32518,7 +32518,7 @@
       </c>
       <c r="M413" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N413" s="2" t="inlineStr">
@@ -32580,7 +32580,7 @@
       </c>
       <c r="J414" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K414" s="2" t="inlineStr">
@@ -32595,7 +32595,7 @@
       </c>
       <c r="M414" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N414" s="2" t="inlineStr">
@@ -32657,7 +32657,7 @@
       </c>
       <c r="J415" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K415" s="2" t="inlineStr">
@@ -32672,7 +32672,7 @@
       </c>
       <c r="M415" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N415" s="2" t="inlineStr">
@@ -32734,7 +32734,7 @@
       </c>
       <c r="J416" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K416" s="2" t="inlineStr">
@@ -32749,7 +32749,7 @@
       </c>
       <c r="M416" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N416" s="2" t="inlineStr">
@@ -32811,7 +32811,7 @@
       </c>
       <c r="J417" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K417" s="2" t="inlineStr">
@@ -32826,7 +32826,7 @@
       </c>
       <c r="M417" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N417" s="2" t="inlineStr">
@@ -32888,7 +32888,7 @@
       </c>
       <c r="J418" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K418" s="2" t="inlineStr">
@@ -32903,7 +32903,7 @@
       </c>
       <c r="M418" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N418" s="2" t="inlineStr">
@@ -32965,7 +32965,7 @@
       </c>
       <c r="J419" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K419" s="2" t="inlineStr">
@@ -32980,7 +32980,7 @@
       </c>
       <c r="M419" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N419" s="2" t="inlineStr">
@@ -33022,7 +33022,7 @@
       </c>
       <c r="F420" s="2" t="inlineStr">
         <is>
-          <t>Ajouter un prestataire de l'agence, réutilisable partout</t>
+          <t>Ajouter un prestataire de l'agence, réutilisable partout. Le nom est unique dans l'agence (casse et espaces de bord ignorés ; partagé avec les prestataires de maintenance) : 409 lisible en cas de doublon.</t>
         </is>
       </c>
       <c r="G420" s="2" t="inlineStr">
@@ -33042,7 +33042,7 @@
       </c>
       <c r="J420" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K420" s="2" t="inlineStr">
@@ -33057,7 +33057,7 @@
       </c>
       <c r="M420" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N420" s="2" t="inlineStr">
@@ -33099,7 +33099,7 @@
       </c>
       <c r="F421" s="2" t="inlineStr">
         <is>
-          <t>Modifier nom, spécialité, coordonnées</t>
+          <t>Modifier nom, spécialité, coordonnées. Même unicité du nom (409).</t>
         </is>
       </c>
       <c r="G421" s="2" t="inlineStr">
@@ -33119,7 +33119,7 @@
       </c>
       <c r="J421" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K421" s="2" t="inlineStr">
@@ -33134,7 +33134,7 @@
       </c>
       <c r="M421" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N421" s="2" t="inlineStr">
@@ -33196,7 +33196,7 @@
       </c>
       <c r="J422" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K422" s="2" t="inlineStr">
@@ -33211,7 +33211,7 @@
       </c>
       <c r="M422" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N422" s="2" t="inlineStr">
@@ -33273,7 +33273,7 @@
       </c>
       <c r="J423" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K423" s="2" t="inlineStr">
@@ -33288,7 +33288,7 @@
       </c>
       <c r="M423" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N423" s="2" t="inlineStr">
@@ -33350,7 +33350,7 @@
       </c>
       <c r="J424" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K424" s="2" t="inlineStr">
@@ -33365,7 +33365,7 @@
       </c>
       <c r="M424" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N424" s="2" t="inlineStr">
@@ -33427,7 +33427,7 @@
       </c>
       <c r="J425" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K425" s="2" t="inlineStr">
@@ -33442,7 +33442,7 @@
       </c>
       <c r="M425" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N425" s="2" t="inlineStr">
@@ -33504,7 +33504,7 @@
       </c>
       <c r="J426" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K426" s="2" t="inlineStr">
@@ -33519,7 +33519,7 @@
       </c>
       <c r="M426" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N426" s="2" t="inlineStr">
@@ -33581,7 +33581,7 @@
       </c>
       <c r="J427" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K427" s="2" t="inlineStr">
@@ -33596,7 +33596,7 @@
       </c>
       <c r="M427" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N427" s="2" t="inlineStr">
@@ -33658,7 +33658,7 @@
       </c>
       <c r="J428" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K428" s="2" t="inlineStr">
@@ -33673,7 +33673,7 @@
       </c>
       <c r="M428" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N428" s="2" t="inlineStr">
@@ -33725,7 +33725,7 @@
       </c>
       <c r="H429" s="2" t="inlineStr">
         <is>
-          <t>Liste de `ChargeCall` (+ paiements, lot, propriétaire)</t>
+          <t>Liste de `ChargeCall` (+ paiements, lot, propriétaire). Inclut `summary`, calculé sur tous les appels filtrés (montant appelé, dossiers en attente, en retard), jamais sur la seule page renvoyée.</t>
         </is>
       </c>
       <c r="I429" s="2" t="inlineStr">
@@ -33735,7 +33735,7 @@
       </c>
       <c r="J429" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K429" s="2" t="inlineStr">
@@ -33750,7 +33750,7 @@
       </c>
       <c r="M429" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N429" s="2" t="inlineStr">
@@ -33812,7 +33812,7 @@
       </c>
       <c r="J430" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_CREATE ou SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K430" s="2" t="inlineStr">
@@ -33827,7 +33827,7 @@
       </c>
       <c r="M430" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_CREATE]) ; en plus requirePropertyPermission(PROPERTIES_EDIT) quand fundId est fourni</t>
+          <t>requireAnyPropertyPermission([SYNDIC_CREATE]) ; en plus requirePropertyPermission(SYNDIC_EDIT) quand fundId est fourni</t>
         </is>
       </c>
       <c r="N430" s="2" t="inlineStr">
@@ -33889,7 +33889,7 @@
       </c>
       <c r="J431" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K431" s="2" t="inlineStr">
@@ -33904,7 +33904,7 @@
       </c>
       <c r="M431" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N431" s="2" t="inlineStr">
@@ -33956,7 +33956,7 @@
       </c>
       <c r="H432" s="2" t="inlineStr">
         <is>
-          <t>`ChargePayment` créé ; `allocations[]`, `advance`, `lotAdvanceBalance` ; `ChargeCall.status` mis à jour ; crédite le compte propriétaire du lot ; reçu/quittances émis ; crédite dans la même transaction les fonds de la copropriété des appels touchés (en entier si l'appel est affecté à un fonds, sinon la part des postes de budget qui alimentent un fonds, au prorata de la répartition du lot) — mouvement `CHARGE_PAYMENT` au journal du fonds</t>
+          <t>`ChargePayment` créé ; `allocations[]`, `advance`, `lotAdvanceBalance` ; `ChargeCall.status` mis à jour ; crédite le compte propriétaire du lot ; reçu/quittances émis ; crédite dans la même transaction les fonds de la copropriété des appels touchés (en entier si l'appel est affecté à un fonds, sinon la part des postes de budget qui alimentent un fonds, au prorata de la répartition du lot) — mouvement `CHARGE_PAYMENT` au journal du fonds. Une écriture comptable de copropriété par encaissement (débit 521 Banque, ou 571 Caisse en espèces / crédit 450 Copropriétaires sur le lot payeur), idempotente ; l'affectation aux fonds reste tracée par les mouvements de fonds.</t>
         </is>
       </c>
       <c r="I432" s="2" t="inlineStr">
@@ -33966,7 +33966,7 @@
       </c>
       <c r="J432" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K432" s="2" t="inlineStr">
@@ -33981,7 +33981,7 @@
       </c>
       <c r="M432" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N432" s="2" t="inlineStr">
@@ -34043,7 +34043,7 @@
       </c>
       <c r="J433" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K433" s="2" t="inlineStr">
@@ -34058,7 +34058,7 @@
       </c>
       <c r="M433" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N433" s="2" t="inlineStr">
@@ -34120,7 +34120,7 @@
       </c>
       <c r="J434" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K434" s="2" t="inlineStr">
@@ -34135,7 +34135,7 @@
       </c>
       <c r="M434" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N434" s="2" t="inlineStr">
@@ -34197,7 +34197,7 @@
       </c>
       <c r="J435" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K435" s="2" t="inlineStr">
@@ -34212,7 +34212,7 @@
       </c>
       <c r="M435" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N435" s="2" t="inlineStr">
@@ -34274,7 +34274,7 @@
       </c>
       <c r="J436" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K436" s="2" t="inlineStr">
@@ -34289,7 +34289,7 @@
       </c>
       <c r="M436" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N436" s="2" t="inlineStr">
@@ -34351,7 +34351,7 @@
       </c>
       <c r="J437" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K437" s="2" t="inlineStr">
@@ -34366,7 +34366,7 @@
       </c>
       <c r="M437" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N437" s="2" t="inlineStr">
@@ -34428,7 +34428,7 @@
       </c>
       <c r="J438" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K438" s="2" t="inlineStr">
@@ -34443,7 +34443,7 @@
       </c>
       <c r="M438" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N438" s="2" t="inlineStr">
@@ -34505,7 +34505,7 @@
       </c>
       <c r="J439" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K439" s="2" t="inlineStr">
@@ -34520,7 +34520,7 @@
       </c>
       <c r="M439" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N439" s="2" t="inlineStr">
@@ -34562,7 +34562,7 @@
       </c>
       <c r="F440" s="2" t="inlineStr">
         <is>
-          <t>Vue consolidée des appels de charges en retard</t>
+          <t>Vue consolidée des appels de charges en retard. Les appels de 0 FCFA (lots sans tantièmes spéciaux d'un budget en tantièmes spéciaux) ne sont ni dus ni en retard : exclus des lots en retard et des relances.</t>
         </is>
       </c>
       <c r="G440" s="2" t="inlineStr">
@@ -34582,7 +34582,7 @@
       </c>
       <c r="J440" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K440" s="2" t="inlineStr">
@@ -34597,7 +34597,7 @@
       </c>
       <c r="M440" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N440" s="2" t="inlineStr">
@@ -34659,7 +34659,7 @@
       </c>
       <c r="J441" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K441" s="2" t="inlineStr">
@@ -34674,7 +34674,7 @@
       </c>
       <c r="M441" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N441" s="2" t="inlineStr">
@@ -34736,7 +34736,7 @@
       </c>
       <c r="J442" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K442" s="2" t="inlineStr">
@@ -34751,7 +34751,7 @@
       </c>
       <c r="M442" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N442" s="2" t="inlineStr">
@@ -34813,7 +34813,7 @@
       </c>
       <c r="J443" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K443" s="2" t="inlineStr">
@@ -34828,7 +34828,7 @@
       </c>
       <c r="M443" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N443" s="2" t="inlineStr">
@@ -34890,7 +34890,7 @@
       </c>
       <c r="J444" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K444" s="2" t="inlineStr">
@@ -34905,7 +34905,7 @@
       </c>
       <c r="M444" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N444" s="2" t="inlineStr">
@@ -34947,7 +34947,7 @@
       </c>
       <c r="F445" s="2" t="inlineStr">
         <is>
-          <t>Appliquer une pénalité de retard à un appel de charges impayé</t>
+          <t>Appliquer une pénalité de retard à un appel de charges impayé. Le taux saisi est mensuel (10 % maximum), proratisé au nombre de jours de retard (mois de 30 jours, au moins un jour) et plafonné au reste dû ; l'écran affiche un aperçu du montant avant validation.</t>
         </is>
       </c>
       <c r="G445" s="2" t="inlineStr">
@@ -34967,7 +34967,7 @@
       </c>
       <c r="J445" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K445" s="2" t="inlineStr">
@@ -34982,7 +34982,7 @@
       </c>
       <c r="M445" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N445" s="2" t="inlineStr">
@@ -35044,7 +35044,7 @@
       </c>
       <c r="J446" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K446" s="2" t="inlineStr">
@@ -35059,7 +35059,7 @@
       </c>
       <c r="M446" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N446" s="2" t="inlineStr">
@@ -35121,7 +35121,7 @@
       </c>
       <c r="J447" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K447" s="2" t="inlineStr">
@@ -35136,7 +35136,7 @@
       </c>
       <c r="M447" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N447" s="2" t="inlineStr">
@@ -35198,7 +35198,7 @@
       </c>
       <c r="J448" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K448" s="2" t="inlineStr">
@@ -35213,7 +35213,7 @@
       </c>
       <c r="M448" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N448" s="2" t="inlineStr">
@@ -35255,7 +35255,7 @@
       </c>
       <c r="F449" s="2" t="inlineStr">
         <is>
-          <t>Afficher le solde et les infos du compte d'un lot, avec rapprochement automatique des écritures manquantes</t>
+          <t>Afficher le solde et les infos du compte d'un lot, avec rapprochement automatique des écritures manquantes. Le propriétaire du compte est le propriétaire principal issu des profils actuels du lot.</t>
         </is>
       </c>
       <c r="G449" s="2" t="inlineStr">
@@ -35275,7 +35275,7 @@
       </c>
       <c r="J449" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K449" s="2" t="inlineStr">
@@ -35290,7 +35290,7 @@
       </c>
       <c r="M449" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N449" s="2" t="inlineStr">
@@ -35352,7 +35352,7 @@
       </c>
       <c r="J450" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K450" s="2" t="inlineStr">
@@ -35367,7 +35367,7 @@
       </c>
       <c r="M450" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N450" s="2" t="inlineStr">
@@ -35429,7 +35429,7 @@
       </c>
       <c r="J451" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K451" s="2" t="inlineStr">
@@ -35444,7 +35444,7 @@
       </c>
       <c r="M451" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N451" s="2" t="inlineStr">
@@ -35506,7 +35506,7 @@
       </c>
       <c r="J452" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K452" s="2" t="inlineStr">
@@ -35521,7 +35521,7 @@
       </c>
       <c r="M452" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N452" s="2" t="inlineStr">
@@ -35563,7 +35563,7 @@
       </c>
       <c r="F453" s="2" t="inlineStr">
         <is>
-          <t>Vue d'ensemble : soldes des fonds, total appelé/payé/restant dû, retard</t>
+          <t>Vue d'ensemble : soldes des fonds, total appelé/payé/restant dû, retard. Montants affichés en FCFA.</t>
         </is>
       </c>
       <c r="G453" s="2" t="inlineStr">
@@ -35583,7 +35583,7 @@
       </c>
       <c r="J453" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K453" s="2" t="inlineStr">
@@ -35598,7 +35598,7 @@
       </c>
       <c r="M453" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N453" s="2" t="inlineStr">
@@ -35660,7 +35660,7 @@
       </c>
       <c r="J454" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K454" s="2" t="inlineStr">
@@ -35675,7 +35675,7 @@
       </c>
       <c r="M454" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N454" s="2" t="inlineStr">
@@ -35737,7 +35737,7 @@
       </c>
       <c r="J455" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K455" s="2" t="inlineStr">
@@ -35752,7 +35752,7 @@
       </c>
       <c r="M455" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N455" s="2" t="inlineStr">
@@ -35814,7 +35814,7 @@
       </c>
       <c r="J456" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K456" s="2" t="inlineStr">
@@ -35829,7 +35829,7 @@
       </c>
       <c r="M456" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N456" s="2" t="inlineStr">
@@ -35891,7 +35891,7 @@
       </c>
       <c r="J457" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K457" s="2" t="inlineStr">
@@ -35906,7 +35906,7 @@
       </c>
       <c r="M457" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N457" s="2" t="inlineStr">
@@ -35968,7 +35968,7 @@
       </c>
       <c r="J458" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K458" s="2" t="inlineStr">
@@ -35983,7 +35983,7 @@
       </c>
       <c r="M458" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N458" s="2" t="inlineStr">
@@ -36045,7 +36045,7 @@
       </c>
       <c r="J459" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K459" s="2" t="inlineStr">
@@ -36060,7 +36060,7 @@
       </c>
       <c r="M459" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N459" s="2" t="inlineStr">
@@ -36122,7 +36122,7 @@
       </c>
       <c r="J460" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K460" s="2" t="inlineStr">
@@ -36137,7 +36137,7 @@
       </c>
       <c r="M460" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N460" s="2" t="inlineStr">
@@ -36199,7 +36199,7 @@
       </c>
       <c r="J461" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K461" s="2" t="inlineStr">
@@ -36214,7 +36214,7 @@
       </c>
       <c r="M461" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N461" s="2" t="inlineStr">
@@ -36276,7 +36276,7 @@
       </c>
       <c r="J462" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K462" s="2" t="inlineStr">
@@ -36291,7 +36291,7 @@
       </c>
       <c r="M462" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N462" s="2" t="inlineStr">
@@ -36353,7 +36353,7 @@
       </c>
       <c r="J463" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K463" s="2" t="inlineStr">
@@ -36368,7 +36368,7 @@
       </c>
       <c r="M463" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N463" s="2" t="inlineStr">
@@ -36430,7 +36430,7 @@
       </c>
       <c r="J464" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K464" s="2" t="inlineStr">
@@ -36445,7 +36445,7 @@
       </c>
       <c r="M464" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N464" s="2" t="inlineStr">
@@ -36507,7 +36507,7 @@
       </c>
       <c r="J465" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K465" s="2" t="inlineStr">
@@ -36522,7 +36522,7 @@
       </c>
       <c r="M465" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N465" s="2" t="inlineStr">
@@ -36584,7 +36584,7 @@
       </c>
       <c r="J466" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K466" s="2" t="inlineStr">
@@ -36599,7 +36599,7 @@
       </c>
       <c r="M466" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N466" s="2" t="inlineStr">
@@ -36661,7 +36661,7 @@
       </c>
       <c r="J467" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K467" s="2" t="inlineStr">
@@ -36676,7 +36676,7 @@
       </c>
       <c r="M467" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N467" s="2" t="inlineStr">
@@ -36718,7 +36718,7 @@
       </c>
       <c r="F468" s="2" t="inlineStr">
         <is>
-          <t>Créer une AG (ordinaire/extraordinaire) avec ses résolutions initiales</t>
+          <t>Créer une AG (ordinaire/extraordinaire) avec ses résolutions initiales. La réponse renvoie l'assemblée créée (`data`) et un décompte d'envoi de la convocation par e-mail aux copropriétaires (`convocation` : propriétaires, envoyés, échecs, sans adresse) ; un échec d'envoi ne défait pas l'assemblée.</t>
         </is>
       </c>
       <c r="G468" s="2" t="inlineStr">
@@ -36738,7 +36738,7 @@
       </c>
       <c r="J468" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K468" s="2" t="inlineStr">
@@ -36753,7 +36753,7 @@
       </c>
       <c r="M468" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N468" s="2" t="inlineStr">
@@ -36815,7 +36815,7 @@
       </c>
       <c r="J469" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K469" s="2" t="inlineStr">
@@ -36830,7 +36830,7 @@
       </c>
       <c r="M469" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N469" s="2" t="inlineStr">
@@ -36892,7 +36892,7 @@
       </c>
       <c r="J470" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K470" s="2" t="inlineStr">
@@ -36907,7 +36907,7 @@
       </c>
       <c r="M470" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N470" s="2" t="inlineStr">
@@ -36969,7 +36969,7 @@
       </c>
       <c r="J471" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K471" s="2" t="inlineStr">
@@ -36984,7 +36984,7 @@
       </c>
       <c r="M471" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N471" s="2" t="inlineStr">
@@ -37026,7 +37026,7 @@
       </c>
       <c r="F472" s="2" t="inlineStr">
         <is>
-          <t>Ajouter un point (titre, ordre, éléments de discussion) à l'ordre du jour de l'AG</t>
+          <t>Ajouter un point (titre, ordre, éléments de discussion) à l'ordre du jour de l'AG. Refusé (409) une fois l'assemblée clôturée ou annulée ; modifiable tant qu'elle est planifiée ou en cours.</t>
         </is>
       </c>
       <c r="G472" s="2" t="inlineStr">
@@ -37046,7 +37046,7 @@
       </c>
       <c r="J472" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K472" s="2" t="inlineStr">
@@ -37061,7 +37061,7 @@
       </c>
       <c r="M472" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N472" s="2" t="inlineStr">
@@ -37103,7 +37103,7 @@
       </c>
       <c r="F473" s="2" t="inlineStr">
         <is>
-          <t>Modifier titre, ordre ou discussions d'un point</t>
+          <t>Modifier titre, ordre ou discussions d'un point. Refusé (409) une fois l'assemblée clôturée ou annulée ; modifiable tant qu'elle est planifiée ou en cours.</t>
         </is>
       </c>
       <c r="G473" s="2" t="inlineStr">
@@ -37123,7 +37123,7 @@
       </c>
       <c r="J473" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K473" s="2" t="inlineStr">
@@ -37138,7 +37138,7 @@
       </c>
       <c r="M473" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N473" s="2" t="inlineStr">
@@ -37180,7 +37180,7 @@
       </c>
       <c r="F474" s="2" t="inlineStr">
         <is>
-          <t>Retirer un point de l'ordre du jour</t>
+          <t>Retirer un point de l'ordre du jour. Refusé (409) une fois l'assemblée clôturée ou annulée ; modifiable tant qu'elle est planifiée ou en cours.</t>
         </is>
       </c>
       <c r="G474" s="2" t="inlineStr">
@@ -37200,7 +37200,7 @@
       </c>
       <c r="J474" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K474" s="2" t="inlineStr">
@@ -37215,7 +37215,7 @@
       </c>
       <c r="M474" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N474" s="2" t="inlineStr">
@@ -37277,7 +37277,7 @@
       </c>
       <c r="J475" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K475" s="2" t="inlineStr">
@@ -37292,7 +37292,7 @@
       </c>
       <c r="M475" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N475" s="2" t="inlineStr">
@@ -37354,7 +37354,7 @@
       </c>
       <c r="J476" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K476" s="2" t="inlineStr">
@@ -37369,7 +37369,7 @@
       </c>
       <c r="M476" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N476" s="2" t="inlineStr">
@@ -37431,7 +37431,7 @@
       </c>
       <c r="J477" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K477" s="2" t="inlineStr">
@@ -37446,7 +37446,7 @@
       </c>
       <c r="M477" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N477" s="2" t="inlineStr">
@@ -37508,7 +37508,7 @@
       </c>
       <c r="J478" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K478" s="2" t="inlineStr">
@@ -37523,7 +37523,7 @@
       </c>
       <c r="M478" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N478" s="2" t="inlineStr">
@@ -37565,7 +37565,7 @@
       </c>
       <c r="F479" s="2" t="inlineStr">
         <is>
-          <t>Générer un document Word (.docx) du compte rendu d'assemblée (ordre du jour, résolutions, résultats en tantièmes, quorum)</t>
+          <t>Générer un document Word (.docx) du compte rendu d'assemblée (ordre du jour, résolutions, résultats en tantièmes, quorum). Compte rendu accentué, avec le type d'assemblée en libellé et les pouvoirs (procurations).</t>
         </is>
       </c>
       <c r="G479" s="2" t="inlineStr">
@@ -37585,7 +37585,7 @@
       </c>
       <c r="J479" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K479" s="2" t="inlineStr">
@@ -37600,7 +37600,7 @@
       </c>
       <c r="M479" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N479" s="2" t="inlineStr">
@@ -37662,7 +37662,7 @@
       </c>
       <c r="J480" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K480" s="2" t="inlineStr">
@@ -37677,7 +37677,7 @@
       </c>
       <c r="M480" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N480" s="2" t="inlineStr">
@@ -37739,7 +37739,7 @@
       </c>
       <c r="J481" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K481" s="2" t="inlineStr">
@@ -37754,7 +37754,7 @@
       </c>
       <c r="M481" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N481" s="2" t="inlineStr">
@@ -37816,7 +37816,7 @@
       </c>
       <c r="J482" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K482" s="2" t="inlineStr">
@@ -37831,7 +37831,7 @@
       </c>
       <c r="M482" s="2" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission([PROPERTIES_VIEW])</t>
+          <t>requireAnyPropertyPermission([SYNDIC_VIEW])</t>
         </is>
       </c>
       <c r="N482" s="2" t="inlineStr">
@@ -38335,7 +38335,7 @@
       </c>
       <c r="F489" s="2" t="inlineStr">
         <is>
-          <t>Crée en une transaction : tenant ACTIF, modules, abonnement d'essai (30 j), paramètres financiers par défaut, socle comptable/trésorerie/stock, et l'administrateur invité</t>
+          <t>Crée en une transaction : tenant ACTIF, modules, abonnement d'essai (30 j), paramètres financiers par défaut, socle comptable/trésorerie/stock, et l'administrateur invité. Rejouer la même création (même nom et même administrateur) : avec la même `Idempotency-Key`, la réponse d'origine est renvoyée (200) ; sinon refus 409 invitant à « Renvoyer l'invitation ». L'écran affiche « Agence déjà créée » et ne présente jamais de faux lien : l'invitation précédente reste valide.</t>
         </is>
       </c>
       <c r="G489" s="2" t="inlineStr">
@@ -38345,7 +38345,7 @@
       </c>
       <c r="H489" s="2" t="inlineStr">
         <is>
-          <t>`{tenant, modules, subscription{planKey,billingCycle,status,items[]}, admin{userId,email,existingUser}, invitation{id,expiresAt,acceptUrl}, emailSent}`</t>
+          <t>`{tenant, modules, subscription{planKey,billingCycle,status,items[]}, admin{userId,email,existingUser}, invitation{id,expiresAt,acceptUrl}, emailSent}`. `alreadyExisted: true` pour un rejeu, `invitation.acceptUrl` absent quand le lien d'origine n'est plus reconstructible</t>
         </is>
       </c>
       <c r="I489" s="2" t="inlineStr">
@@ -40029,7 +40029,7 @@
       </c>
       <c r="F511" s="2" t="inlineStr">
         <is>
-          <t>Création de compte + envoi d'un e-mail de vérification</t>
+          <t>Création de compte + envoi d'un e-mail de vérification. L'e-mail est rédigé dans la langue préférée du compte, sinon celle de la requête, sinon le français.</t>
         </is>
       </c>
       <c r="G511" s="2" t="inlineStr">
@@ -40183,7 +40183,7 @@
       </c>
       <c r="F513" s="2" t="inlineStr">
         <is>
-          <t>Réémet le jeton de vérification</t>
+          <t>Réémet le jeton de vérification. L'e-mail est rédigé dans la langue préférée du compte, sinon celle de la requête, sinon le français.</t>
         </is>
       </c>
       <c r="G513" s="2" t="inlineStr">
@@ -40270,7 +40270,7 @@
       </c>
       <c r="H514" s="2" t="inlineStr">
         <is>
-          <t>`{user}` + cookies</t>
+          <t>`{user}` + cookies. La dernière connexion réussie est enregistrée (`lastLoginAt`) ; le rafraîchissement de session ne la modifie pas.</t>
         </is>
       </c>
       <c r="I514" s="2" t="inlineStr">
@@ -40491,7 +40491,7 @@
       </c>
       <c r="F517" s="2" t="inlineStr">
         <is>
-          <t>Envoie un lien de réinitialisation si l'adresse existe (réponse toujours identique)</t>
+          <t>Envoie un lien de réinitialisation si l'adresse existe (réponse toujours identique). L'e-mail est rédigé dans la langue préférée du compte, sinon celle de la requête, sinon le français.</t>
         </is>
       </c>
       <c r="G517" s="2" t="inlineStr">
@@ -41348,7 +41348,7 @@
       </c>
       <c r="H528" s="2" t="inlineStr">
         <is>
-          <t>`{members[], pagination}`</t>
+          <t>`{members[], pagination}`. Chaque membre porte `lastLoginAt` (dernière connexion réussie).</t>
         </is>
       </c>
       <c r="I528" s="2" t="inlineStr">
@@ -41358,7 +41358,7 @@
       </c>
       <c r="J528" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur USERS_VIEW ; super-admin</t>
+          <t>Collaborateur USERS_VIEW ; super-admin. Le rôle Agent n'a plus USERS_VIEW par défaut (liste complète réservée ; les listes d'assignation passent par « membres assignables »).</t>
         </is>
       </c>
       <c r="K528" s="2" t="inlineStr">
@@ -42262,7 +42262,7 @@
       </c>
       <c r="F540" s="2" t="inlineStr">
         <is>
-          <t>Calcule le prix mensuel/annuel d'une combinaison de packs+quantités</t>
+          <t>Calcule le prix mensuel/annuel d'une combinaison de packs+quantités. Refuse en 400 les compositions non cumulables : un pack une seule fois, Intégré exclusif, Patrimoine Essentiel et Pro non cumulables (mêmes règles que la création d'agence) ; un pack non commercialisé ou inconnu est refusé.</t>
         </is>
       </c>
       <c r="G540" s="2" t="inlineStr">
@@ -42416,7 +42416,7 @@
       </c>
       <c r="F542" s="2" t="inlineStr">
         <is>
-          <t>Modules, fonctionnalités, capacités (limite/consommé), politique de quota, lecture seule</t>
+          <t>Modules, fonctionnalités, capacités (limite/consommé), politique de quota, lecture seule. Alimente le menu de l'agence (socle seul pendant la lecture des droits, puis entrées des modules souscrits) et les gardes d'écran. Un module retiré sans aucune donnée dans l'agence n'ouvre plus aucun accès ; la lecture seule d'un module retiré ne protège que des données existantes. Un refus de quota ne conseille une extension que si le pack en vend une pour cette capacité (`extensible` dans le détail `QUOTA_EXCEEDED`), sinon il renvoie vers la facturation du dépassement, le changement de pack ou le contact.</t>
         </is>
       </c>
       <c r="G542" s="2" t="inlineStr">
@@ -42493,7 +42493,7 @@
       </c>
       <c r="F543" s="2" t="inlineStr">
         <is>
-          <t>Souscrit immédiatement un élément ; prorata au jour près (sauf essai) ; refuse un pack incompatible (exclusivité Intégré)</t>
+          <t>Souscrit immédiatement un élément ; prorata au jour près (sauf essai) ; refuse un pack incompatible (exclusivité Intégré). Une extension n'est vendue qu'avec les packs de `rules.requiresAnyOf` du catalogue : le refus (400) nomme ces packs et, pour une capacité, rappelle que l'excédent est facturé selon la grille du pack.</t>
         </is>
       </c>
       <c r="G543" s="2" t="inlineStr">
@@ -42647,7 +42647,7 @@
       </c>
       <c r="F545" s="2" t="inlineStr">
         <is>
-          <t>Retrait à l'échéance par défaut, ou immédiat avec motif obligatoire ; un pack retiré entraîne ses extensions liées</t>
+          <t>Retrait à l'échéance par défaut, ou immédiat avec motif obligatoire ; un pack retiré entraîne ses extensions liées. Le module d'un pack retiré passe en lecture seule seulement s'il contient des données de l'agence (copropriété, chantier, bien détenu en propre, bien de client ou mandat selon le module) ; sinon l'accès est supprimé.</t>
         </is>
       </c>
       <c r="G545" s="2" t="inlineStr">
@@ -42724,7 +42724,7 @@
       </c>
       <c r="F546" s="2" t="inlineStr">
         <is>
-          <t>Montée de gamme immédiate (avoir au prorata) ; descente programmée à l'échéance ; extensions suivies vers le nouveau pack ou terminées</t>
+          <t>Montée de gamme immédiate (avoir au prorata) ; descente programmée à l'échéance ; extensions suivies vers le nouveau pack ou terminées. Même règle : un module quitté sans donnée dans l'agence n'est pas conservé en lecture seule.</t>
         </is>
       </c>
       <c r="G546" s="2" t="inlineStr">
@@ -43340,7 +43340,7 @@
       </c>
       <c r="F554" s="2" t="inlineStr">
         <is>
-          <t>Recalcule les activations de lots par rapport à la consommation réelle</t>
+          <t>Recalcule les activations de lots par rapport à la consommation réelle. Un mandat de gestion actif compte immédiatement dans la réserve LOTS (inscrit dans la même transaction que sa création) ; la réconciliation automatique quotidienne (03:10 UTC) retire les mandats échus et corrige toute dérive.</t>
         </is>
       </c>
       <c r="G554" s="2" t="inlineStr">
@@ -43494,7 +43494,7 @@
       </c>
       <c r="F556" s="2" t="inlineStr">
         <is>
-          <t>Un collaborateur demande une extension de l'abonnement ; notifie tous les super-admins par e-mail</t>
+          <t>Un collaborateur demande une extension de l'abonnement ; notifie tous les super-admins par e-mail. L'écran ne propose que les extensions vendables avec les packs de l'agence (`requiresAnyOf`).</t>
         </is>
       </c>
       <c r="G556" s="2" t="inlineStr">
@@ -46189,7 +46189,7 @@
       </c>
       <c r="F591" s="2" t="inlineStr">
         <is>
-          <t>Lister les biens possédés dans l'agence sélectionnée, filtrables par statut/type/mode de transaction</t>
+          <t>Lister les biens possédés dans l'agence sélectionnée, filtrables par statut/type/mode de transaction. Un bien `CLIENT` sous mandat de gestion actif de l'agence (actif, non révoqué, commencé et non échu) fait partie du périmètre du propriétaire, comme un bien de l'agence qui lui est rattaché ou un bien qu'il loue par un bail de l'agence.</t>
         </is>
       </c>
       <c r="G591" s="2" t="inlineStr">
@@ -46969,7 +46969,7 @@
       </c>
       <c r="H601" s="2" t="inlineStr">
         <is>
-          <t>Fichier binaire (pdf/csv/xlsx)</t>
+          <t>Fichier binaire (pdf/csv/xlsx). Le PDF se génère sans erreur ; le CSV échappe les cellules (virgules, guillemets, préfixe anti-formule).</t>
         </is>
       </c>
       <c r="I601" s="2" t="inlineStr">
@@ -47123,7 +47123,7 @@
       </c>
       <c r="H603" s="2" t="inlineStr">
         <is>
-          <t>Fichier binaire</t>
+          <t>Fichier binaire. CSV : cellules échappées (virgules, guillemets, préfixe anti-formule).</t>
         </is>
       </c>
       <c r="I603" s="2" t="inlineStr">
@@ -47960,7 +47960,7 @@
       </c>
       <c r="F614" s="2" t="inlineStr">
         <is>
-          <t>Solde et relevé paginé du compte de tiers du locataire connecté, lecture seule ; aucun identifiant de compte n'est accepté en entrée (résolu uniquement depuis la session)</t>
+          <t>Solde et relevé paginé du compte de tiers du locataire connecté, lecture seule ; aucun identifiant de compte n'est accepté en entrée (résolu uniquement depuis la session). Solde cohérent avec le compte du locataire, la balance clients et le relevé DOCX (une échéance ne compte qu'à sa date d'exigibilité).</t>
         </is>
       </c>
       <c r="G614" s="2" t="inlineStr">
@@ -49279,7 +49279,7 @@
       </c>
       <c r="H631" t="inlineStr">
         <is>
-          <t>`LotPaymentResult` (paiement, `allocations[]` par appel, `advance`, `lotAdvanceBalance`) ; documents de recouvrement émis (voir S3) ; crédite dans la même transaction les fonds de la copropriété des appels touchés (en entier si l'appel est affecté à un fonds, sinon la part des postes de budget qui alimentent un fonds, au prorata de la répartition du lot) — mouvement `CHARGE_PAYMENT` au journal du fonds</t>
+          <t>`LotPaymentResult` (paiement, `allocations[]` par appel, `advance`, `lotAdvanceBalance`) ; documents de recouvrement émis (voir S3) ; crédite dans la même transaction les fonds de la copropriété des appels touchés (en entier si l'appel est affecté à un fonds, sinon la part des postes de budget qui alimentent un fonds, au prorata de la répartition du lot) — mouvement `CHARGE_PAYMENT` au journal du fonds. Même écriture comptable par encaissement (un paiement = une écriture, l'imputation d'une avance n'en écrit pas).</t>
         </is>
       </c>
       <c r="I631" t="inlineStr">
@@ -49289,7 +49289,7 @@
       </c>
       <c r="J631" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K631" t="inlineStr">
@@ -49304,7 +49304,7 @@
       </c>
       <c r="M631" t="inlineStr">
         <is>
-          <t>requirePropertyPermission('PROPERTIES_EDIT')</t>
+          <t>requirePropertyPermission('SYNDIC_EDIT')</t>
         </is>
       </c>
       <c r="N631" t="inlineStr">
@@ -49366,7 +49366,7 @@
       </c>
       <c r="J632" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K632" t="inlineStr">
@@ -49381,7 +49381,7 @@
       </c>
       <c r="M632" t="inlineStr">
         <is>
-          <t>requirePropertyPermission('PROPERTIES_EDIT')</t>
+          <t>requirePropertyPermission('SYNDIC_EDIT')</t>
         </is>
       </c>
       <c r="N632" t="inlineStr">
@@ -49443,7 +49443,7 @@
       </c>
       <c r="J633" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K633" t="inlineStr">
@@ -49458,7 +49458,7 @@
       </c>
       <c r="M633" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission(['PROPERTIES_VIEW'])</t>
+          <t>requireAnyPropertyPermission(['SYNDIC_VIEW'])</t>
         </is>
       </c>
       <c r="N633" t="inlineStr">
@@ -49520,7 +49520,7 @@
       </c>
       <c r="J634" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K634" t="inlineStr">
@@ -49535,7 +49535,7 @@
       </c>
       <c r="M634" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission(['PROPERTIES_VIEW'])</t>
+          <t>requireAnyPropertyPermission(['SYNDIC_VIEW'])</t>
         </is>
       </c>
       <c r="N634" t="inlineStr">
@@ -49597,7 +49597,7 @@
       </c>
       <c r="J635" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K635" t="inlineStr">
@@ -49612,7 +49612,7 @@
       </c>
       <c r="M635" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission(['PROPERTIES_VIEW'])</t>
+          <t>requireAnyPropertyPermission(['SYNDIC_VIEW'])</t>
         </is>
       </c>
       <c r="N635" t="inlineStr">
@@ -49674,7 +49674,7 @@
       </c>
       <c r="J636" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K636" t="inlineStr">
@@ -49689,7 +49689,7 @@
       </c>
       <c r="M636" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission(['PROPERTIES_VIEW'])</t>
+          <t>requireAnyPropertyPermission(['SYNDIC_VIEW'])</t>
         </is>
       </c>
       <c r="N636" t="inlineStr">
@@ -49751,7 +49751,7 @@
       </c>
       <c r="J637" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K637" t="inlineStr">
@@ -49766,7 +49766,7 @@
       </c>
       <c r="M637" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission(['PROPERTIES_VIEW'])</t>
+          <t>requireAnyPropertyPermission(['SYNDIC_VIEW'])</t>
         </is>
       </c>
       <c r="N637" t="inlineStr">
@@ -49828,7 +49828,7 @@
       </c>
       <c r="J638" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K638" t="inlineStr">
@@ -49843,7 +49843,7 @@
       </c>
       <c r="M638" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission(['PROPERTIES_VIEW'])</t>
+          <t>requireAnyPropertyPermission(['SYNDIC_VIEW'])</t>
         </is>
       </c>
       <c r="N638" t="inlineStr">
@@ -49905,7 +49905,7 @@
       </c>
       <c r="J639" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K639" t="inlineStr">
@@ -49920,7 +49920,7 @@
       </c>
       <c r="M639" t="inlineStr">
         <is>
-          <t>requirePropertyPermission('PROPERTIES_EDIT')</t>
+          <t>requirePropertyPermission('SYNDIC_EDIT')</t>
         </is>
       </c>
       <c r="N639" t="inlineStr">
@@ -49982,7 +49982,7 @@
       </c>
       <c r="J640" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K640" t="inlineStr">
@@ -49997,7 +49997,7 @@
       </c>
       <c r="M640" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission(['PROPERTIES_VIEW'])</t>
+          <t>requireAnyPropertyPermission(['SYNDIC_VIEW'])</t>
         </is>
       </c>
       <c r="N640" t="inlineStr">
@@ -50059,7 +50059,7 @@
       </c>
       <c r="J641" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K641" t="inlineStr">
@@ -50074,7 +50074,7 @@
       </c>
       <c r="M641" t="inlineStr">
         <is>
-          <t>requirePropertyPermission('PROPERTIES_EDIT')</t>
+          <t>requirePropertyPermission('SYNDIC_EDIT')</t>
         </is>
       </c>
       <c r="N641" t="inlineStr">
@@ -50598,7 +50598,7 @@
       </c>
       <c r="J648" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K648" t="inlineStr">
@@ -50613,7 +50613,7 @@
       </c>
       <c r="M648" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission(['PROPERTIES_VIEW'])</t>
+          <t>requireAnyPropertyPermission(['SYNDIC_VIEW'])</t>
         </is>
       </c>
       <c r="N648" t="inlineStr">
@@ -50675,7 +50675,7 @@
       </c>
       <c r="J649" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K649" t="inlineStr">
@@ -50690,7 +50690,7 @@
       </c>
       <c r="M649" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission(['PROPERTIES_VIEW'])</t>
+          <t>requireAnyPropertyPermission(['SYNDIC_VIEW'])</t>
         </is>
       </c>
       <c r="N649" t="inlineStr">
@@ -50752,7 +50752,7 @@
       </c>
       <c r="J650" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K650" t="inlineStr">
@@ -50767,7 +50767,7 @@
       </c>
       <c r="M650" t="inlineStr">
         <is>
-          <t>requirePropertyPermission('PROPERTIES_EDIT')</t>
+          <t>requirePropertyPermission('SYNDIC_EDIT')</t>
         </is>
       </c>
       <c r="N650" t="inlineStr">
@@ -50829,7 +50829,7 @@
       </c>
       <c r="J651" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K651" t="inlineStr">
@@ -50844,7 +50844,7 @@
       </c>
       <c r="M651" t="inlineStr">
         <is>
-          <t>requirePropertyPermission('PROPERTIES_EDIT')</t>
+          <t>requirePropertyPermission('SYNDIC_EDIT')</t>
         </is>
       </c>
       <c r="N651" t="inlineStr">
@@ -50906,7 +50906,7 @@
       </c>
       <c r="J652" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K652" t="inlineStr">
@@ -50921,7 +50921,7 @@
       </c>
       <c r="M652" t="inlineStr">
         <is>
-          <t>requirePropertyPermission('PROPERTIES_EDIT')</t>
+          <t>requirePropertyPermission('SYNDIC_EDIT')</t>
         </is>
       </c>
       <c r="N652" t="inlineStr">
@@ -50983,7 +50983,7 @@
       </c>
       <c r="J653" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K653" t="inlineStr">
@@ -50998,7 +50998,7 @@
       </c>
       <c r="M653" t="inlineStr">
         <is>
-          <t>requirePropertyPermission('PROPERTIES_EDIT')</t>
+          <t>requirePropertyPermission('SYNDIC_EDIT')</t>
         </is>
       </c>
       <c r="N653" t="inlineStr">
@@ -51060,7 +51060,7 @@
       </c>
       <c r="J654" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K654" t="inlineStr">
@@ -51075,7 +51075,7 @@
       </c>
       <c r="M654" t="inlineStr">
         <is>
-          <t>requirePropertyPermission('PROPERTIES_EDIT')</t>
+          <t>requirePropertyPermission('SYNDIC_EDIT')</t>
         </is>
       </c>
       <c r="N654" t="inlineStr">
@@ -51137,7 +51137,7 @@
       </c>
       <c r="J655" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K655" t="inlineStr">
@@ -51152,7 +51152,7 @@
       </c>
       <c r="M655" t="inlineStr">
         <is>
-          <t>requirePropertyPermission('PROPERTIES_EDIT')</t>
+          <t>requirePropertyPermission('SYNDIC_EDIT')</t>
         </is>
       </c>
       <c r="N655" t="inlineStr">
@@ -51214,7 +51214,7 @@
       </c>
       <c r="J656" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K656" t="inlineStr">
@@ -51229,7 +51229,7 @@
       </c>
       <c r="M656" t="inlineStr">
         <is>
-          <t>requirePropertyPermission('PROPERTIES_EDIT')</t>
+          <t>requirePropertyPermission('SYNDIC_EDIT')</t>
         </is>
       </c>
       <c r="N656" t="inlineStr">
@@ -51368,7 +51368,7 @@
       </c>
       <c r="J658" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K658" t="inlineStr">
@@ -51383,7 +51383,7 @@
       </c>
       <c r="M658" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission(['PROPERTIES_VIEW'])</t>
+          <t>requireAnyPropertyPermission(['SYNDIC_VIEW'])</t>
         </is>
       </c>
       <c r="N658" t="inlineStr">
@@ -51445,7 +51445,7 @@
       </c>
       <c r="J659" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K659" t="inlineStr">
@@ -51460,7 +51460,7 @@
       </c>
       <c r="M659" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission(['PROPERTIES_VIEW'])</t>
+          <t>requireAnyPropertyPermission(['SYNDIC_VIEW'])</t>
         </is>
       </c>
       <c r="N659" t="inlineStr">
@@ -51522,7 +51522,7 @@
       </c>
       <c r="J660" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K660" t="inlineStr">
@@ -51537,7 +51537,7 @@
       </c>
       <c r="M660" t="inlineStr">
         <is>
-          <t>requireAnyPropertyPermission(['PROPERTIES_VIEW'])</t>
+          <t>requireAnyPropertyPermission(['SYNDIC_VIEW'])</t>
         </is>
       </c>
       <c r="N660" t="inlineStr">
@@ -51676,7 +51676,7 @@
       </c>
       <c r="J662" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K662" s="2" t="inlineStr">
@@ -51691,7 +51691,7 @@
       </c>
       <c r="M662" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N662" s="2" t="inlineStr">
@@ -51753,7 +51753,7 @@
       </c>
       <c r="J663" s="2" t="inlineStr">
         <is>
-          <t>Collaborateur (accès agence)</t>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
         </is>
       </c>
       <c r="K663" s="2" t="inlineStr">
@@ -51768,7 +51768,7 @@
       </c>
       <c r="M663" s="2" t="inlineStr">
         <is>
-          <t>requirePropertyPermission(PROPERTIES_EDIT)</t>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
         </is>
       </c>
       <c r="N663" s="2" t="inlineStr">
@@ -51964,7 +51964,7 @@
       </c>
       <c r="F666" t="inlineStr">
         <is>
-          <t>Voir la valeur et la performance de ses biens : derniere valorisation, plus-value latente, rendements, capital restant des emprunts</t>
+          <t>Voir la valeur et la performance de ses biens : derniere valorisation, plus-value latente, rendements, capital restant des emprunts. Un bien `CLIENT` sous mandat de gestion actif de l'agence (actif, non révoqué, commencé et non échu) fait partie du périmètre du propriétaire, comme un bien de l'agence qui lui est rattaché ou un bien qu'il loue par un bail de l'agence.</t>
         </is>
       </c>
       <c r="G666" t="inlineStr">
@@ -52041,7 +52041,7 @@
       </c>
       <c r="F667" t="inlineStr">
         <is>
-          <t>Detail patrimonial d'un de ses biens : historique des valorisations, rendements, emprunts, travaux et documents</t>
+          <t>Detail patrimonial d'un de ses biens : historique des valorisations, rendements, emprunts, travaux et documents. Un bien `CLIENT` sous mandat de gestion actif de l'agence (actif, non révoqué, commencé et non échu) fait partie du périmètre du propriétaire, comme un bien de l'agence qui lui est rattaché ou un bien qu'il loue par un bail de l'agence.</t>
         </is>
       </c>
       <c r="G667" t="inlineStr">
@@ -52821,7 +52821,7 @@
       </c>
       <c r="H677" t="inlineStr">
         <is>
-          <t>Totaux consolidés (valeur, dette, cash-flow, rendements) + détail par bien ; un rattachement à date d'effet future est exclu des totaux (`pending`)</t>
+          <t>Totaux consolidés (valeur, dette, cash-flow, rendements) + détail par bien ; un rattachement à date d'effet future est exclu des totaux (`pending`). Rendements brut, net et net-net affichés en pourcentage exact et horodatage lisible.</t>
         </is>
       </c>
       <c r="I677" t="inlineStr">
@@ -53437,7 +53437,7 @@
       </c>
       <c r="H685" t="inlineStr">
         <is>
-          <t>Fichier PDF ou XLSX en piece jointe (`Content-Disposition: attachment`), genere en memoire, jamais ecrit sur disque</t>
+          <t>Fichier PDF ou XLSX en piece jointe (`Content-Disposition: attachment`), genere en memoire, jamais ecrit sur disque. PDF : accents des saisies conservés et montants du tableau de performance complets (nom du bien et chiffres sur deux lignes).</t>
         </is>
       </c>
       <c r="I685" t="inlineStr">
@@ -53514,7 +53514,7 @@
       </c>
       <c r="H686" t="inlineStr">
         <is>
-          <t>Fichier PDF ou XLSX en piece jointe, nomme d'apres la reference interne du bien</t>
+          <t>Fichier PDF ou XLSX en piece jointe, nomme d'apres la reference interne du bien. PDF : accents conservés (recomposition Unicode).</t>
         </is>
       </c>
       <c r="I686" t="inlineStr">
@@ -53812,7 +53812,7 @@
       </c>
       <c r="F690" s="2" t="inlineStr">
         <is>
-          <t>Interroge l'assistant à l'ouverture de la coquille d'agence : indique s'il est activé et quels outils l'utilisateur peut employer (permissions RBAC et, en mode `enforce`, modules de l'abonnement). Le bouton flottant « Assistant » (raccourci Ctrl/Cmd+J) n'apparaît que si `enabled` est vrai ; toute erreur de statut le masque Le fournisseur et le modèle effectifs viennent du réglage plateforme (écran « Assistant IA » de l'administration) ou, à défaut, des variables AI_*.</t>
+          <t>Interroge l'assistant à l'ouverture de la coquille d'agence : indique s'il est activé et quels outils l'utilisateur peut employer (permissions RBAC et, en mode `enforce`, modules de l'abonnement). Le bouton flottant « Assistant » (raccourci Ctrl/Cmd+J) n'apparaît que si `enabled` est vrai ; toute erreur de statut le masque Le fournisseur et le modèle effectifs viennent du réglage plateforme (écran « Assistant IA » de l'administration) ou, à défaut, des variables AI_*. L'accueil du tiroir (message et suggestions) ne cite que les capacités des outils autorisés : sans gestion locative, ni baux ni quittances ne sont annoncés.</t>
         </is>
       </c>
       <c r="G690" s="2" t="inlineStr">
@@ -53889,7 +53889,7 @@
       </c>
       <c r="F691" s="2" t="inlineStr">
         <is>
-          <t>Ouvre le tiroir de conversation (côté « fin » : à droite en français, à gauche en arabe) et envoie l'échange au fournisseur LLM en flux SSE : texte progressif, cartes de résultats (biens, baux, documents, proposition), suggestions selon l'écran courant, arrêt de la réponse et nouvelle conversation. Conversation non persistée ; l'assistant n'écrit jamais lui-même. Limites : 20 messages, 4 000 caractères chacun, 24 000 au total ; 20 requêtes/min et 300/jour par utilisateur et par agence, plus un plafond par agence tous collaborateurs confondus (`AI_TENANT_MINUTE_LIMIT` 100/min, `AI_TENANT_DAILY_LIMIT` 3000/jour) ; limiteurs en mémoire, par instance d'API ; 4 tours et 8 appels d'outils maximum</t>
+          <t>Ouvre le tiroir de conversation (côté « fin » : à droite en français, à gauche en arabe) et envoie l'échange au fournisseur LLM en flux SSE : texte progressif, cartes de résultats (biens, baux, documents, proposition), suggestions selon l'écran courant, arrêt de la réponse et nouvelle conversation. Conversation non persistée ; l'assistant n'écrit jamais lui-même. Limites : 20 messages, 4 000 caractères chacun, 24 000 au total ; 20 requêtes/min et 300/jour par utilisateur et par agence, plus un plafond par agence tous collaborateurs confondus (`AI_TENANT_MINUTE_LIMIT` 100/min, `AI_TENANT_DAILY_LIMIT` 3000/jour) ; limiteurs en mémoire, par instance d'API ; 4 tours et 8 appels d'outils maximum. L'invite système est construite par agence et ne cite que les capacités des outils exposés (permissions et modules souscrits) ; un appel d'outil d'un module non souscrit (modèle qui en invente un) est refusé poliment (résultat `MODULE_NOT_INCLUDED`, journal d'audit `AI_TOOL_DENIED`) et n'est jamais exécuté.</t>
         </is>
       </c>
       <c r="G691" s="2" t="inlineStr">
@@ -54705,6 +54705,776 @@
       <c r="O701" s="2" t="inlineStr">
         <is>
           <t>Administration &gt; Assistant IA &gt; champ Modèle</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" s="2" t="inlineStr">
+        <is>
+          <t>Administration plateforme</t>
+        </is>
+      </c>
+      <c r="B702" s="2" t="inlineStr">
+        <is>
+          <t>Tous packs</t>
+        </is>
+      </c>
+      <c r="C702" s="2" t="inlineStr">
+        <is>
+          <t>Abonnements par packs</t>
+        </is>
+      </c>
+      <c r="D702" s="2" t="inlineStr">
+        <is>
+          <t>Droits d'accès selon le pack (côté agence)</t>
+        </is>
+      </c>
+      <c r="E702" s="2" t="inlineStr">
+        <is>
+          <t>Remplacer un écran de module non souscrit par « Fonction non comprise dans votre abonnement »</t>
+        </is>
+      </c>
+      <c r="F702" s="2" t="inlineStr">
+        <is>
+          <t>Quand un collaborateur ouvre l'adresse d'un écran d'un module absent du pack (pipeline CRM, Ventes, Gestion locative, Patrimoine, Syndic, Chantiers et stock…), l'écran du module est remplacé par un message explicatif avec lien vers Paramètres &gt; Abonnement. Même règle que le menu ; rien n'est bloqué tant que les droits se lisent, si leur lecture échoue, en lecture seule ou hors des écrans d'agence.</t>
+        </is>
+      </c>
+      <c r="G702" s="2" t="inlineStr">
+        <is>
+          <t>Adresse de l'écran (`/tenant/:tenantId/&lt;module&gt;/…`) ; droits de l'agence (`moduleAccess`)</t>
+        </is>
+      </c>
+      <c r="H702" s="2" t="inlineStr">
+        <is>
+          <t>Écran « Fonction non comprise dans votre abonnement » ; côté API, une requête du module répond 403 `MODULE_NOT_INCLUDED` en mode `enforce`</t>
+        </is>
+      </c>
+      <c r="I702" s="2" t="inlineStr">
+        <is>
+          <t>Consulter ses droits (entitlements)</t>
+        </is>
+      </c>
+      <c r="J702" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence (tout rôle)</t>
+        </is>
+      </c>
+      <c r="K702" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L702" s="2" t="inlineStr">
+        <is>
+          <t>Aucune route dédiée : garde d'écran web (`navigation/route-features.ts`, coquille `AppShell`), qui lit GET /api/tenants/:tenantId/entitlements</t>
+        </is>
+      </c>
+      <c r="M702" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N702" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O702" s="2" t="inlineStr">
+        <is>
+          <t>Entrées des modules non souscrits (adresse saisie à la main, favori)</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" s="2" t="inlineStr">
+        <is>
+          <t>Administration plateforme</t>
+        </is>
+      </c>
+      <c r="B703" s="2" t="inlineStr">
+        <is>
+          <t>Tous packs</t>
+        </is>
+      </c>
+      <c r="C703" s="2" t="inlineStr">
+        <is>
+          <t>Abonnements par packs</t>
+        </is>
+      </c>
+      <c r="D703" s="2" t="inlineStr">
+        <is>
+          <t>Droits d'accès selon le pack (côté agence)</t>
+        </is>
+      </c>
+      <c r="E703" s="2" t="inlineStr">
+        <is>
+          <t>N'afficher dans les écrans du socle que les blocs des modules souscrits</t>
+        </is>
+      </c>
+      <c r="F703" s="2" t="inlineStr">
+        <is>
+          <t>Tableau de bord (indicateurs locatifs, CRM, syndic, patrimoine), Paramètres financiers (sections gestion locative), onglets des espaces Finance (Bons de commande et Associations sans Chantiers ; Facturation et balances locatives sans gestion locative), fiche bien (ventes, indivision, mandat, patrimoine), fiche contact (affaires, activités, filtres) et modèles de documents ne montrent que ce que le pack comprend. Le menu ne montre que le socle pendant la lecture des droits, puis les modules souscrits.</t>
+        </is>
+      </c>
+      <c r="G703" s="2" t="inlineStr">
+        <is>
+          <t>Droits de l'agence (`moduleAccess`, mode `enforce`)</t>
+        </is>
+      </c>
+      <c r="H703" s="2" t="inlineStr">
+        <is>
+          <t>Blocs, onglets et entrées masqués (`NONE`) ; la lecture seule reste visible ; rien n'est masqué si les droits ne se lisent pas</t>
+        </is>
+      </c>
+      <c r="I703" s="2" t="inlineStr">
+        <is>
+          <t>Consulter ses droits (entitlements)</t>
+        </is>
+      </c>
+      <c r="J703" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence (tout rôle)</t>
+        </is>
+      </c>
+      <c r="K703" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L703" s="2" t="inlineStr">
+        <is>
+          <t>Aucune route dédiée : lecture de GET /api/tenants/:tenantId/entitlements (hook `useAgencyFeatures`, `useFeatureAccessState`)</t>
+        </is>
+      </c>
+      <c r="M703" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N703" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O703" s="2" t="inlineStr">
+        <is>
+          <t>Tableau de bord ; Paramètres &gt; Finance ; Finance (onglets) ; Biens &gt; fiche bien ; CRM &gt; fiche contact ; Documents &gt; Modèles</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" s="2" t="inlineStr">
+        <is>
+          <t>Administration plateforme</t>
+        </is>
+      </c>
+      <c r="B704" s="2" t="inlineStr">
+        <is>
+          <t>Tous packs</t>
+        </is>
+      </c>
+      <c r="C704" s="2" t="inlineStr">
+        <is>
+          <t>Abonnements par packs</t>
+        </is>
+      </c>
+      <c r="D704" s="2" t="inlineStr">
+        <is>
+          <t>Gestion de l'abonnement d'une agence</t>
+        </is>
+      </c>
+      <c r="E704" s="2" t="inlineStr">
+        <is>
+          <t>Réconcilier quotidiennement le registre des lots (tâche planifiée)</t>
+        </is>
+      </c>
+      <c r="F704" s="2" t="inlineStr">
+        <is>
+          <t>Chaque nuit à 03:10 UTC, le registre des lots de chaque agence active est réconcilié avec la réalité : les mandats échus ou résiliés sortent du décompte, les dérives (écriture hors service, reprise) sont corrigées. Une agence en échec est journalisée sans arrêter les suivantes ; le traitement est idempotent.</t>
+        </is>
+      </c>
+      <c r="G704" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H704" s="2" t="inlineStr">
+        <is>
+          <t>Registre des lots à jour (ajouts, retraits, reclassements comptés dans le journal de la tâche)</t>
+        </is>
+      </c>
+      <c r="I704" s="2" t="inlineStr">
+        <is>
+          <t>Abonnement existant</t>
+        </is>
+      </c>
+      <c r="J704" s="2" t="inlineStr">
+        <is>
+          <t>Système (tâche planifiée)</t>
+        </is>
+      </c>
+      <c r="K704" s="2" t="inlineStr">
+        <is>
+          <t>Plateforme</t>
+        </is>
+      </c>
+      <c r="L704" s="2" t="inlineStr">
+        <is>
+          <t>N/A — tâche node-cron interne (`packages/api/src/jobs/lot-reconciliation-job.ts`, 03:10 UTC)</t>
+        </is>
+      </c>
+      <c r="M704" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N704" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O704" s="2" t="inlineStr">
+        <is>
+          <t>Jauge Lots de l'onglet Abonnement (Administration &gt; Agences &gt; fiche agence ; Paramètres &gt; Abonnement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" s="2" t="inlineStr">
+        <is>
+          <t>Gestion locative</t>
+        </is>
+      </c>
+      <c r="B705" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C705" s="2" t="inlineStr">
+        <is>
+          <t>RENTAL</t>
+        </is>
+      </c>
+      <c r="D705" s="2" t="inlineStr">
+        <is>
+          <t>Encaisser — Échéances</t>
+        </is>
+      </c>
+      <c r="E705" s="2" t="inlineStr">
+        <is>
+          <t>Passer automatiquement les échéances échues en retard (tâche quotidienne)</t>
+        </is>
+      </c>
+      <c r="F705" s="2" t="inlineStr">
+        <is>
+          <t>Chaque nuit à 02:00, les révisions de loyer dont la date d'effet est arrivée sont appliquées aux baux, puis les échéances échues non soldées (Brouillon, À payer, Partiel) passent « En retard » avant le calcul des pénalités. Les listes et le tableau de bord reclassent aussi le statut à l'affichage, sans attendre la tâche.</t>
+        </is>
+      </c>
+      <c r="G705" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H705" s="2" t="inlineStr">
+        <is>
+          <t>Échéances « En retard » et pénalités à jour</t>
+        </is>
+      </c>
+      <c r="I705" s="2" t="inlineStr">
+        <is>
+          <t>Générer les échéances</t>
+        </is>
+      </c>
+      <c r="J705" s="2" t="inlineStr">
+        <is>
+          <t>Système (tâche planifiée)</t>
+        </is>
+      </c>
+      <c r="K705" s="2" t="inlineStr">
+        <is>
+          <t>Plateforme</t>
+        </is>
+      </c>
+      <c r="L705" s="2" t="inlineStr">
+        <is>
+          <t>N/A — tâche node-cron interne (`packages/api/src/jobs/penalty-calculation-job.ts`, 02:00)</t>
+        </is>
+      </c>
+      <c r="M705" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N705" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O705" s="2" t="inlineStr">
+        <is>
+          <t>Encaisser › Échéances (statut « En retard »)</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" s="2" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B706" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C706" s="2" t="inlineStr">
+        <is>
+          <t>RENTAL</t>
+        </is>
+      </c>
+      <c r="D706" s="2" t="inlineStr">
+        <is>
+          <t>Comptabilité</t>
+        </is>
+      </c>
+      <c r="E706" s="2" t="inlineStr">
+        <is>
+          <t>Écrire automatiquement la comptabilité de la gestion locative directe</t>
+        </is>
+      </c>
+      <c r="F706" s="2" t="inlineStr">
+        <is>
+          <t>Pour un bien détenu en propre (ni indivision ni bail rattaché à un propriétaire mandant), chaque événement locatif écrit au journal dans sa transaction, de façon idempotente : encaissement (débit trésorerie / crédit 411 locataire), créance du locataire (débit 411 / crédit 7083 loyer ou 7088 pénalité, l'inverse pour une remise ou une annulation, y compris une échéance Brouillon émise), dépense de bien (débit charge / crédit trésorerie, ou 401 si l'agence doit la facture). Une pièce modifiée ou supprimée est contre-passée puis réécrite ; les comptes manquants sont créés à la volée.</t>
+        </is>
+      </c>
+      <c r="G706" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H706" s="2" t="inlineStr">
+        <is>
+          <t>Écritures au journal et au grand livre ; le 411 auxiliaire du locataire se lit comme son relevé (facturé − réglé)</t>
+        </is>
+      </c>
+      <c r="I706" s="2" t="inlineStr">
+        <is>
+          <t>Enregistrer un paiement ; Générer les échéances ; Ajouter une dépense</t>
+        </is>
+      </c>
+      <c r="J706" s="2" t="inlineStr">
+        <is>
+          <t>Système (déclenché par l'événement)</t>
+        </is>
+      </c>
+      <c r="K706" s="2" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L706" s="2" t="inlineStr">
+        <is>
+          <t>N/A — écritures posées dans la transaction de l'événement (paiement, échéance, pénalité, dépense de bien) ; consultables par GET /tenants/:tenantId/finance/accounting/journal</t>
+        </is>
+      </c>
+      <c r="M706" s="2" t="inlineStr">
+        <is>
+          <t>FINANCE_REPORTS_READ (consultation du journal)</t>
+        </is>
+      </c>
+      <c r="N706" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O706" s="2" t="inlineStr">
+        <is>
+          <t>Finance &gt; Caisse et comptabilité &gt; Comptabilité</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" s="2" t="inlineStr">
+        <is>
+          <t>Syndic copropriete</t>
+        </is>
+      </c>
+      <c r="B707" s="2" t="inlineStr">
+        <is>
+          <t>Syndic, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C707" s="2" t="inlineStr">
+        <is>
+          <t>SYNDIC</t>
+        </is>
+      </c>
+      <c r="D707" s="2" t="inlineStr">
+        <is>
+          <t>Copropriété (lots, prestataires, incidents)</t>
+        </is>
+      </c>
+      <c r="E707" s="2" t="inlineStr">
+        <is>
+          <t>Supprimer ou désactiver un lot</t>
+        </is>
+      </c>
+      <c r="F707" s="2" t="inlineStr">
+        <is>
+          <t>Supprimer un lot saisi par erreur. Refusé en 409 dès qu'il porte un mouvement (appel de charges, paiement, reçu, écriture, vote, incident, relance, pénalité, échéancier, compte) : l'écran propose alors de le désactiver (tantièmes à 0), ce qui l'exclut de la clé de répartition, de la réserve de lots et des appels futurs en conservant l'historique. Sans mouvement, le lot et ses rattachements vides (répartitions de budget, profils, compte vide) sont supprimés et la place est libérée dans la jauge LOTS.</t>
+        </is>
+      </c>
+      <c r="G707" s="2" t="inlineStr">
+        <is>
+          <t>Chemin `lotId`</t>
+        </is>
+      </c>
+      <c r="H707" s="2" t="inlineStr">
+        <is>
+          <t>`{success, message}` ; 409 avec `errors[{field:'lotId'}]` si le lot a des mouvements</t>
+        </is>
+      </c>
+      <c r="I707" s="2" t="inlineStr">
+        <is>
+          <t>Créer un lot</t>
+        </is>
+      </c>
+      <c r="J707" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
+        </is>
+      </c>
+      <c r="K707" s="2" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L707" s="2" t="inlineStr">
+        <is>
+          <t>DELETE /tenants/:tenantId/syndics/:syndicId/lots/:lotId</t>
+        </is>
+      </c>
+      <c r="M707" s="2" t="inlineStr">
+        <is>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
+        </is>
+      </c>
+      <c r="N707" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O707" s="2" t="inlineStr">
+        <is>
+          <t>Syndic &gt; Copropriété</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" s="2" t="inlineStr">
+        <is>
+          <t>Syndic copropriete</t>
+        </is>
+      </c>
+      <c r="B708" s="2" t="inlineStr">
+        <is>
+          <t>Syndic, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C708" s="2" t="inlineStr">
+        <is>
+          <t>SYNDIC</t>
+        </is>
+      </c>
+      <c r="D708" s="2" t="inlineStr">
+        <is>
+          <t>Assemblées et documents</t>
+        </is>
+      </c>
+      <c r="E708" s="2" t="inlineStr">
+        <is>
+          <t>Renvoyer la convocation d'une assemblée générale</t>
+        </is>
+      </c>
+      <c r="F708" s="2" t="inlineStr">
+        <is>
+          <t>Réenvoyer par e-mail la convocation aux copropriétaires d'une assemblée planifiée (un copropriétaire sans adresse est compté à part).</t>
+        </is>
+      </c>
+      <c r="G708" s="2" t="inlineStr">
+        <is>
+          <t>Chemin `meetingId`</t>
+        </is>
+      </c>
+      <c r="H708" s="2" t="inlineStr">
+        <is>
+          <t>`{success, convocation: {owners, emailEnabled, emailSent, emailFailed, emailSkippedNoAddress, whatsappSent, failures[]}}` ; 409 si l'assemblée n'est pas planifiée ; `error: 'CONVOCATION_FAILED'` si l'envoi échoue en bloc</t>
+        </is>
+      </c>
+      <c r="I708" s="2" t="inlineStr">
+        <is>
+          <t>Convoquer une assemblée générale</t>
+        </is>
+      </c>
+      <c r="J708" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — SYNDIC_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
+        </is>
+      </c>
+      <c r="K708" s="2" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L708" s="2" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/syndics/:syndicId/assemblees/:meetingId/convocation</t>
+        </is>
+      </c>
+      <c r="M708" s="2" t="inlineStr">
+        <is>
+          <t>requirePropertyPermission(SYNDIC_EDIT)</t>
+        </is>
+      </c>
+      <c r="N708" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O708" s="2" t="inlineStr">
+        <is>
+          <t>Syndic &gt; Assemblées et documents</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" s="2" t="inlineStr">
+        <is>
+          <t>Administration plateforme</t>
+        </is>
+      </c>
+      <c r="B709" s="2" t="inlineStr">
+        <is>
+          <t>N/A (plateforme)</t>
+        </is>
+      </c>
+      <c r="C709" s="2" t="inlineStr">
+        <is>
+          <t>Administration plateforme</t>
+        </is>
+      </c>
+      <c r="D709" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateurs</t>
+        </is>
+      </c>
+      <c r="E709" s="2" t="inlineStr">
+        <is>
+          <t>Lister les membres assignables</t>
+        </is>
+      </c>
+      <c r="F709" s="2" t="inlineStr">
+        <is>
+          <t>Alimenter les listes d'assignation (CRM, biens, ventes, maintenance) avec une liste minimale des membres ACTIFS (identifiant, nom d'affichage, rôles), sans le droit de lire la liste complète des collaborateurs.</t>
+        </is>
+      </c>
+      <c r="G709" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H709" s="2" t="inlineStr">
+        <is>
+          <t>`{success, data: {members[]}}`</t>
+        </is>
+      </c>
+      <c r="I709" s="2" t="inlineStr">
+        <is>
+          <t>Inviter un collaborateur</t>
+        </is>
+      </c>
+      <c r="J709" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur de l'agence détenant l'une des permissions listées, sans USERS_VIEW</t>
+        </is>
+      </c>
+      <c r="K709" s="2" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L709" s="2" t="inlineStr">
+        <is>
+          <t>GET /api/tenants/:tenantId/members/assignable</t>
+        </is>
+      </c>
+      <c r="M709" s="2" t="inlineStr">
+        <is>
+          <t>`authenticate` + `requireTenantAccess` + `requireTenantCollaborator` + `requireAnyPermission([CRM_CONTACTS_VIEW, CRM_DEALS_VIEW, CRM_ACTIVITIES_VIEW, CRM_APPOINTMENTS_VIEW, PROPERTIES_VIEW, PROPERTIES_VISITS_SCHEDULE, MAINTENANCE_ADMIN])`</t>
+        </is>
+      </c>
+      <c r="N709" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O709" s="2" t="inlineStr">
+        <is>
+          <t>Listes « Assigné à » des écrans CRM, biens, ventes et maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" s="2" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B710" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C710" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D710" s="2" t="inlineStr">
+        <is>
+          <t>Performance du patrimoine</t>
+        </is>
+      </c>
+      <c r="E710" s="2" t="inlineStr">
+        <is>
+          <t>Conserver les hypothèses de projection d'un bien (sur l'appareil)</t>
+        </is>
+      </c>
+      <c r="F710" s="2" t="inlineStr">
+        <is>
+          <t>Les hypothèses du simulateur de rendement (horizon en années, croissance de la valeur, des loyers et des charges, vacance) se gardent par agence et par bien dans le navigateur de l'appareil : elles survivent à un rechargement, sans être enregistrées côté serveur ni partagées entre appareils.</t>
+        </is>
+      </c>
+      <c r="G710" s="2" t="inlineStr">
+        <is>
+          <t>Hypothèses saisies dans le simulateur (bornes : 1 à 30 ans ; croissances −50 % à +100 % ; vacance 0 à 100 %)</t>
+        </is>
+      </c>
+      <c r="H710" s="2" t="inlineStr">
+        <is>
+          <t>Simulateur pré-rempli à la réouverture ; valeurs hors bornes ignorées</t>
+        </is>
+      </c>
+      <c r="I710" s="2" t="inlineStr">
+        <is>
+          <t>Consulter le rendement d'un bien</t>
+        </is>
+      </c>
+      <c r="J710" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K710" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L710" s="2" t="inlineStr">
+        <is>
+          <t>Aucune route dédiée : stockage local du navigateur (`yield-assumptions-storage.ts`)</t>
+        </is>
+      </c>
+      <c r="M710" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N710" s="2" t="inlineStr">
+        <is>
+          <t>Disponible (hypothèses conservées sur l'appareil, non synchronisées)</t>
+        </is>
+      </c>
+      <c r="O710" s="2" t="inlineStr">
+        <is>
+          <t>Biens &gt; fiche bien &gt; onglet Patrimoine</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" s="2" t="inlineStr">
+        <is>
+          <t>Administration plateforme</t>
+        </is>
+      </c>
+      <c r="B711" s="2" t="inlineStr">
+        <is>
+          <t>N/A (plateforme)</t>
+        </is>
+      </c>
+      <c r="C711" s="2" t="inlineStr">
+        <is>
+          <t>Administration plateforme</t>
+        </is>
+      </c>
+      <c r="D711" s="2" t="inlineStr">
+        <is>
+          <t>Fiabilité des réponses</t>
+        </is>
+      </c>
+      <c r="E711" s="2" t="inlineStr">
+        <is>
+          <t>Recevoir une erreur lisible et traduite</t>
+        </is>
+      </c>
+      <c r="F711" s="2" t="inlineStr">
+        <is>
+          <t>Les services lèvent des erreurs typées traduites dans la langue de l'utilisateur ; une erreur inattendue n'expose plus l'invocation Prisma, un chemin de fichier, une pile d'appels ni un message multi-lignes (réponse générique, détail dans les journaux).</t>
+        </is>
+      </c>
+      <c r="G711" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H711" s="2" t="inlineStr">
+        <is>
+          <t>`{success:false, message, errors?[{field,message}]}` avec le statut HTTP de l'erreur typée (400, 403, 404, 409, 422) ; 500 générique pour une erreur inattendue</t>
+        </is>
+      </c>
+      <c r="I711" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J711" s="2" t="inlineStr">
+        <is>
+          <t>Tout utilisateur de l'API</t>
+        </is>
+      </c>
+      <c r="K711" s="2" t="inlineStr">
+        <is>
+          <t>Tous</t>
+        </is>
+      </c>
+      <c r="L711" s="2" t="inlineStr">
+        <is>
+          <t>Toutes les routes `/api` (middleware `error-middleware`)</t>
+        </is>
+      </c>
+      <c r="M711" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N711" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O711" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -55547,17 +56317,17 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Pas de permissions dediees au metier syndic</t>
+          <t>Droits du module Syndic : pas de granularité par rôle métier</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Toutes les routes de syndic-routes.ts utilisent le RBAC generique des biens (PROPERTIES_VIEW/CREATE/EDIT) : impossible de distinguer un role 'gestionnaire syndic' d'un role 'gestionnaire de biens' au niveau des permissions.</t>
+          <t>Les routes Syndic exigent SYNDIC_VIEW / SYNDIC_CREATE / SYNDIC_EDIT et les relevés de gérance OWNER_STATEMENTS_VIEW / OWNER_STATEMENTS_EDIT (Administrateur et Gestionnaire par défaut ; Agent et Comptable sans accès). Un accès en lecture pour le terrain se donne par un rôle personnalisé. Le logo de copropriété reste gardé par PROPERTIES_VIEW / PROPERTIES_EDIT.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>A considerer si le produit veut un jour des roles metier syndic dedies (ex. Assistant syndic vs Syndic senior).</t>
+          <t>A considerer si le produit veut un jour des roles metier syndic dedies (ex. Assistant syndic vs Syndic senior) : une seule paire lecture/ecriture par module aujourd'hui.</t>
         </is>
       </c>
     </row>
@@ -55684,7 +56454,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>La campagne de facturation mensuelle des loyers (billing-runs) vit dans un groupe de menu tague CORE par defaut (accessible a tous les packs), alors qu'elle est fonctionnellement RENTAL (necessite des baux, donc le module Agence).</t>
+          <t>La campagne de facturation mensuelle des loyers (billing-runs) vit dans un groupe de menu tague CORE par defaut (accessible a tous les packs), alors qu'elle est fonctionnellement RENTAL (necessite des baux, donc le module Agence). Côté écran, « Facturation et balances » (campagne du mois, balances de comptes de locataire) est remplacé par « Fonction non comprise dans votre abonnement » sans gestion locative.</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat(patrimoine): hypothèses de projection enregistrées par bien et ratios bancaires (spec 029)
- Modèle PropertyYieldAssumption (migration additive 20261007090000), routes
  GET/PUT /properties/:id/yield/assumptions, migration unique et idempotente du
  contenu du localStorage vers le serveur (le serveur fait foi).
- Ratios dans yield.ts : DSCR, LTV, cash-on-cash et TRI (avant financement) ;
  un ratio indéterminable vaut null avec une raison, jamais 0. Carte « Ratios
  bancaires » sur l'onglet Patrimoine du bien.
- Bien client sous mandat (tenantId nul) : hypothèses en 404, décision de sécurité.
- Spec 029, DATA_MODELS.md, wiki des fonctionnalités (3 lignes + 2 enrichies).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -189,8 +189,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O711" headerRowCount="1">
-  <autoFilter ref="A1:O711"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O713" headerRowCount="1">
+  <autoFilter ref="A1:O713"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Domaine (regroupement agent)"/>
     <tableColumn id="2" name="Pack(s)"/>
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O711"/>
+  <dimension ref="A1:O713"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4080,7 +4080,7 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Sans `propertyId` : aperçu portefeuille ; avec `propertyId` : rendements + projection détaillés</t>
+          <t>Sans `propertyId` : aperçu portefeuille ; avec `propertyId` : rendements + projection détaillés Avec un bien : `assumptions` appliquées (requête &gt; hypothèses enregistrées du bien &gt; défauts), `assumptionsSaved` et `ratios` bancaires (DSCR, LTV, cash-on-cash, TRI).</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
@@ -4157,7 +4157,7 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Rendements + projection</t>
+          <t>Rendements + projection + `assumptions` appliquées (requête &gt; hypothèses enregistrées du bien &gt; défauts), `assumptionsSaved` et `ratios` bancaires (DSCR, LTV, cash-on-cash, TRI).</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
@@ -55347,22 +55347,22 @@
       </c>
       <c r="E710" s="2" t="inlineStr">
         <is>
-          <t>Conserver les hypothèses de projection d'un bien (sur l'appareil)</t>
+          <t>Retrouver les hypothèses de projection d'un bien (synchronisées)</t>
         </is>
       </c>
       <c r="F710" s="2" t="inlineStr">
         <is>
-          <t>Les hypothèses du simulateur de rendement (horizon en années, croissance de la valeur, des loyers et des charges, vacance) se gardent par agence et par bien dans le navigateur de l'appareil : elles survivent à un rechargement, sans être enregistrées côté serveur ni partagées entre appareils.</t>
+          <t>Les hypothèses du simulateur de rendement (horizon en années, croissance de la valeur, des loyers et des charges, vacance) sont enregistrées sur le serveur, une ligne par bien : elles sont retrouvées sur tout appareil et partagées entre les collaborateurs de l'agence. Sans ligne enregistrée, valeurs par défaut (10 ans, +3 % valeur, +2 % loyers, +2,5 % charges, 5 % vacance). Migration unique : au premier chargement, des hypothèses valides déjà conservées dans le navigateur (`patrimoine:performance:assumptions:{tenant}:{bien}`) sont envoyées au serveur s'il n'a encore rien pour ce bien ; le serveur n'est jamais écrasé par le local, qui ne sert plus que de repli hors ligne (bandeau « non synchronisées » tant que le serveur n'est pas joignable ou que l'utilisateur n'a pas le droit d'édition).</t>
         </is>
       </c>
       <c r="G710" s="2" t="inlineStr">
         <is>
-          <t>Hypothèses saisies dans le simulateur (bornes : 1 à 30 ans ; croissances −50 % à +100 % ; vacance 0 à 100 %)</t>
+          <t>Param `propertyId` (chemin)</t>
         </is>
       </c>
       <c r="H710" s="2" t="inlineStr">
         <is>
-          <t>Simulateur pré-rempli à la réouverture ; valeurs hors bornes ignorées</t>
+          <t>`assumptions` (years, valueGrowthRate, rentGrowthRate, expenseGrowthRate, vacancyRate), `saved` (une ligne existe), `updatedAt`</t>
         </is>
       </c>
       <c r="I710" s="2" t="inlineStr">
@@ -55382,17 +55382,17 @@
       </c>
       <c r="L710" s="2" t="inlineStr">
         <is>
-          <t>Aucune route dédiée : stockage local du navigateur (`yield-assumptions-storage.ts`)</t>
+          <t>GET /tenants/:tenantId/properties/:propertyId/yield/assumptions</t>
         </is>
       </c>
       <c r="M710" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PROPERTIES_VIEW (`requireAnyPropertyPermission`)</t>
         </is>
       </c>
       <c r="N710" s="2" t="inlineStr">
         <is>
-          <t>Disponible (hypothèses conservées sur l'appareil, non synchronisées)</t>
+          <t>Disponible (hypothèses synchronisées avec le serveur)</t>
         </is>
       </c>
       <c r="O710" s="2" t="inlineStr">
@@ -55475,6 +55475,160 @@
       <c r="O711" s="2" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D712" t="inlineStr">
+        <is>
+          <t>Performance du patrimoine</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr">
+        <is>
+          <t>Enregistrer les hypothèses de projection d'un bien</t>
+        </is>
+      </c>
+      <c r="F712" t="inlineStr">
+        <is>
+          <t>Enregistrer pour un bien l'horizon, la croissance de la valeur, des loyers et des charges et la vacance, afin que le simulateur et la projection les reprennent pour tous les collaborateurs. Écriture idempotente (une seule ligne par bien, remplacée à chaque envoi) ; l'auteur de la dernière modification est conservé. Déclenchée par « Recalculer » sur l'onglet Patrimoine et la page Performance, et automatiquement une fois pour migrer les hypothèses déjà conservées dans le navigateur.</t>
+        </is>
+      </c>
+      <c r="G712" t="inlineStr">
+        <is>
+          <t>Corps strict (aucun champ inconnu, `tenantId` refusé) : `years` entier 1 à 30 ; `valueGrowthRate`, `rentGrowthRate`, `expenseGrowthRate` de −0,5 à 1 ; `vacancyRate` de 0 à 1 ; les cinq champs sont obligatoires</t>
+        </is>
+      </c>
+      <c r="H712" t="inlineStr">
+        <is>
+          <t>`assumptions`, `saved: true`, `updatedAt`</t>
+        </is>
+      </c>
+      <c r="I712" t="inlineStr">
+        <is>
+          <t>Retrouver les hypothèses de projection d'un bien (synchronisées)</t>
+        </is>
+      </c>
+      <c r="J712" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_EDIT</t>
+        </is>
+      </c>
+      <c r="K712" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L712" t="inlineStr">
+        <is>
+          <t>PUT /tenants/:tenantId/properties/:propertyId/yield/assumptions</t>
+        </is>
+      </c>
+      <c r="M712" t="inlineStr">
+        <is>
+          <t>PROPERTIES_EDIT (`requirePropertyPermission`)</t>
+        </is>
+      </c>
+      <c r="N712" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O712" t="inlineStr">
+        <is>
+          <t>Biens &gt; fiche bien &gt; onglet Patrimoine ; Patrimoine &gt; Performance</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D713" t="inlineStr">
+        <is>
+          <t>Performance du patrimoine</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr">
+        <is>
+          <t>Consulter les ratios bancaires d'un bien (DSCR, LTV, cash-on-cash, TRI)</t>
+        </is>
+      </c>
+      <c r="F713" t="inlineStr">
+        <is>
+          <t>Lire les quatre ratios qu'exige une banque, chacun avec sa définition en info-bulle. DSCR = (loyers annuels effectifs − charges d'exploitation) / mensualités d'emprunt des 12 prochains mois (loyers effectifs = loyers × (1 − vacance des hypothèses)) ; LTV = capital restant dû des prêts actifs / valeur estimée ; cash-on-cash = (loyers effectifs − charges − mensualités) / fonds propres investis (coût de revient − capital emprunté des prêts actifs) ; TRI = taux de rentabilité interne du bien avant financement sur l'horizon projeté (coût de revient en flux initial négatif, flux annuels projetés, valeur projetée en valeur terminale ; résolution numérique bornée). Un ratio indéterminable vaut `null` avec un code de raison (aucun prêt actif, aucune mensualité à venir sur 12 mois, aucune valorisation, prix d'acquisition inconnu, fonds propres nuls, non convergent) et s'affiche « — » avec la raison, jamais 0. DSCR en ratio (1,25 x), les trois autres en %.</t>
+        </is>
+      </c>
+      <c r="G713" t="inlineStr">
+        <is>
+          <t>Param `propertyId` + hypothèses de projection en query (facultatives : sinon celles enregistrées pour le bien, sinon les défauts)</t>
+        </is>
+      </c>
+      <c r="H713" t="inlineStr">
+        <is>
+          <t>`ratios: { dscr, ltv, cashOnCash, irr }`, chacun `{ value: nombre ou null, reason: code ou null }`</t>
+        </is>
+      </c>
+      <c r="I713" t="inlineStr">
+        <is>
+          <t>Consulter le rendement d'un bien ; Consulter les emprunts ; Consulter les valorisations</t>
+        </is>
+      </c>
+      <c r="J713" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K713" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L713" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/properties/:propertyId/yield ; GET /tenants/:tenantId/patrimoine/performance?propertyId=</t>
+        </is>
+      </c>
+      <c r="M713" t="inlineStr">
+        <is>
+          <t>PROPERTIES_VIEW (`requireAnyPropertyPermission`)</t>
+        </is>
+      </c>
+      <c r="N713" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O713" t="inlineStr">
+        <is>
+          <t>Biens &gt; fiche bien &gt; onglet Patrimoine (carte « Ratios bancaires ») ; Patrimoine &gt; Performance</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(patrimoine): liens sécurisés et canaux WhatsApp/e-mail du patrimoine (spec 031)
- lib/secure-links : lien à jeton aléatoire de 256 bits, haché SHA-256 en base
  (le clair n'est jamais stocké ni journalisé), expiration, révocation,
  consultation journalisée, refus uniforme (404) ; modèle SecureLink, migration
  additive 20261007110000.
- Route publique POST /api/public/secure-links/owner-monthly-report (jeton dans
  le corps, fragment d'URL côté partage), limiteur par IP, en-têtes no-store,
  parseur JSON propre borné à 1 Ko ; page publique /rapport-proprietaire.
- Rapport mensuel d'un propriétaire : envoi par WhatsApp ou e-mail avec lien,
  routeur de canaux (canal préféré, consentement revérifié), job mensuel
  désactivé par défaut ; clés WhatsApp opt-in par agence.
- Écran : section « Rapport mensuel et liens sécurisés » sur la fiche d'un relevé.
- Spec 031, DATA_MODELS.md, SECURITY.md, wiki (7 lignes).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -189,8 +189,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O711" headerRowCount="1">
-  <autoFilter ref="A1:O711"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O718" headerRowCount="1">
+  <autoFilter ref="A1:O718"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Domaine (regroupement agent)"/>
     <tableColumn id="2" name="Pack(s)"/>
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O711"/>
+  <dimension ref="A1:O718"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -55475,6 +55475,545 @@
       <c r="O711" s="2" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" s="2" t="inlineStr">
+        <is>
+          <t>Gestion locative</t>
+        </is>
+      </c>
+      <c r="B712" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C712" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE (menu) / RENTAL (feature déclarée sur l'entrée « Relevés »)</t>
+        </is>
+      </c>
+      <c r="D712" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine › Relevés</t>
+        </is>
+      </c>
+      <c r="E712" s="2" t="inlineStr">
+        <is>
+          <t>Envoyer le rapport du mois au propriétaire (WhatsApp ou e-mail)</t>
+        </is>
+      </c>
+      <c r="F712" s="2" t="inlineStr">
+        <is>
+          <t>Envoyer au propriétaire un lien sécurisé vers le rapport mensuel de son relevé, par son canal préféré (WhatsApp ou e-mail), un seul canal par message. Refusé (403 `OWN_ASSETS_ONLY`) à un compte Patrimoine seul.</t>
+        </is>
+      </c>
+      <c r="G712" s="2" t="inlineStr">
+        <is>
+          <t>Aucun corps ; relevé existant de l'agence</t>
+        </is>
+      </c>
+      <c r="H712" s="2" t="inlineStr">
+        <is>
+          <t>Résultat `{ sent, channel, reason? }` : 202 si envoyé, 200 sinon (raisons `NO_ELIGIBLE_CHANNEL`, `EVENT_DISABLED`, `SEND_FAILED`). Lien créé puis révoqué automatiquement si l'envoi échoue sur tous les canaux ; 409 si le relevé est un brouillon (`DRAFT`) ou calculé avec une version obsolète.</t>
+        </is>
+      </c>
+      <c r="I712" s="2" t="inlineStr">
+        <is>
+          <t>Générer un relevé propriétaire (relevé non brouillon) ; consentement WhatsApp ou e-mail du propriétaire (CrmContact) ; événement `OWNER_MONTHLY_REPORT_SENT` activé (e-mail : actif par défaut ; WhatsApp : désactivé par défaut, à activer dans la configuration de l'agence) ; fournisseurs configurés</t>
+        </is>
+      </c>
+      <c r="J712" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — OWNER_STATEMENTS_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
+        </is>
+      </c>
+      <c r="K712" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L712" s="2" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/owner-statements/:statementId/send-monthly-report</t>
+        </is>
+      </c>
+      <c r="M712" s="2" t="inlineStr">
+        <is>
+          <t>OWNER_STATEMENTS_EDIT</t>
+        </is>
+      </c>
+      <c r="N712" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O712" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine › Relevés</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" s="2" t="inlineStr">
+        <is>
+          <t>Gestion locative</t>
+        </is>
+      </c>
+      <c r="B713" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C713" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE (menu) / RENTAL (feature déclarée sur l'entrée « Relevés »)</t>
+        </is>
+      </c>
+      <c r="D713" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine › Relevés</t>
+        </is>
+      </c>
+      <c r="E713" s="2" t="inlineStr">
+        <is>
+          <t>Créer / copier un lien sécurisé de rapport mensuel</t>
+        </is>
+      </c>
+      <c r="F713" s="2" t="inlineStr">
+        <is>
+          <t>Générer un lien public en lecture seule vers le rapport mensuel d'un relevé, à transmettre soi-même au propriétaire. Le jeton (32 octets aléatoires) n'est affiché qu'une fois et n'est stocké que haché.</t>
+        </is>
+      </c>
+      <c r="G713" s="2" t="inlineStr">
+        <is>
+          <t>`ttlDays` optionnel (1 à 30 jours, 7 par défaut)</t>
+        </is>
+      </c>
+      <c r="H713" s="2" t="inlineStr">
+        <is>
+          <t>Lien `…/rapport-proprietaire#&lt;jeton&gt;` et date d'expiration (201) ; 409 si le relevé est un brouillon ou calculé avec une version obsolète</t>
+        </is>
+      </c>
+      <c r="I713" s="2" t="inlineStr">
+        <is>
+          <t>Générer un relevé propriétaire</t>
+        </is>
+      </c>
+      <c r="J713" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — OWNER_STATEMENTS_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
+        </is>
+      </c>
+      <c r="K713" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L713" s="2" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/owner-statements/:statementId/secure-links</t>
+        </is>
+      </c>
+      <c r="M713" s="2" t="inlineStr">
+        <is>
+          <t>OWNER_STATEMENTS_EDIT</t>
+        </is>
+      </c>
+      <c r="N713" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O713" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine › Relevés</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" s="2" t="inlineStr">
+        <is>
+          <t>Gestion locative</t>
+        </is>
+      </c>
+      <c r="B714" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C714" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE (menu) / RENTAL (feature déclarée sur l'entrée « Relevés »)</t>
+        </is>
+      </c>
+      <c r="D714" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine › Relevés</t>
+        </is>
+      </c>
+      <c r="E714" s="2" t="inlineStr">
+        <is>
+          <t>Lister les liens sécurisés actifs d'un relevé</t>
+        </is>
+      </c>
+      <c r="F714" s="2" t="inlineStr">
+        <is>
+          <t>Voir les liens encore valides d'un relevé (création, expiration, nombre de consultations, dernière consultation).</t>
+        </is>
+      </c>
+      <c r="G714" s="2" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="H714" s="2" t="inlineStr">
+        <is>
+          <t>Liste des liens actifs, sans jeton ni empreinte</t>
+        </is>
+      </c>
+      <c r="I714" s="2" t="inlineStr">
+        <is>
+          <t>Créer / copier un lien sécurisé de rapport mensuel</t>
+        </is>
+      </c>
+      <c r="J714" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — OWNER_STATEMENTS_VIEW (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
+        </is>
+      </c>
+      <c r="K714" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L714" s="2" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/owner-statements/:statementId/secure-links</t>
+        </is>
+      </c>
+      <c r="M714" s="2" t="inlineStr">
+        <is>
+          <t>OWNER_STATEMENTS_VIEW</t>
+        </is>
+      </c>
+      <c r="N714" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O714" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine › Relevés</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" s="2" t="inlineStr">
+        <is>
+          <t>Gestion locative</t>
+        </is>
+      </c>
+      <c r="B715" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C715" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE (menu) / RENTAL (feature déclarée sur l'entrée « Relevés »)</t>
+        </is>
+      </c>
+      <c r="D715" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine › Relevés</t>
+        </is>
+      </c>
+      <c r="E715" s="2" t="inlineStr">
+        <is>
+          <t>Révoquer un lien sécurisé</t>
+        </is>
+      </c>
+      <c r="F715" s="2" t="inlineStr">
+        <is>
+          <t>Rendre immédiatement un lien inutilisable (même refus que pour un lien inconnu ou expiré).</t>
+        </is>
+      </c>
+      <c r="G715" s="2" t="inlineStr">
+        <is>
+          <t>`linkId` du lien</t>
+        </is>
+      </c>
+      <c r="H715" s="2" t="inlineStr">
+        <is>
+          <t>`{ revoked: true }` ; 404 si le lien n'appartient pas à ce relevé et à l'agence</t>
+        </is>
+      </c>
+      <c r="I715" s="2" t="inlineStr">
+        <is>
+          <t>Créer / copier un lien sécurisé de rapport mensuel</t>
+        </is>
+      </c>
+      <c r="J715" s="2" t="inlineStr">
+        <is>
+          <t>Collaborateur agence — OWNER_STATEMENTS_EDIT (Administrateur et Gestionnaire par défaut ; ni Agent ni Comptable)</t>
+        </is>
+      </c>
+      <c r="K715" s="2" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L715" s="2" t="inlineStr">
+        <is>
+          <t>DELETE /tenants/:tenantId/owner-statements/:statementId/secure-links/:linkId</t>
+        </is>
+      </c>
+      <c r="M715" s="2" t="inlineStr">
+        <is>
+          <t>OWNER_STATEMENTS_EDIT</t>
+        </is>
+      </c>
+      <c r="N715" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O715" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine › Relevés</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" s="2" t="inlineStr">
+        <is>
+          <t>Portails externes</t>
+        </is>
+      </c>
+      <c r="B716" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C716" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D716" s="2" t="inlineStr">
+        <is>
+          <t>Rapport mensuel propriétaire (lien public)</t>
+        </is>
+      </c>
+      <c r="E716" s="2" t="inlineStr">
+        <is>
+          <t>Consulter le rapport mensuel d'un propriétaire par lien sécurisé</t>
+        </is>
+      </c>
+      <c r="F716" s="2" t="inlineStr">
+        <is>
+          <t>Afficher en lecture seule, sans connexion, le relevé du mois d'un seul propriétaire (totaux, lignes par bien) et l'imprimer ou l'enregistrer en PDF depuis le navigateur. Jeton dans le fragment de l'URL, envoyé en corps de POST ; limiteur de débit par IP ; chaque consultation est journalisée.</t>
+        </is>
+      </c>
+      <c r="G716" s="2" t="inlineStr">
+        <is>
+          <t>`token` (corps JSON), lu dans le fragment `#&lt;jeton&gt;` de la page `/rapport-proprietaire`</t>
+        </is>
+      </c>
+      <c r="H716" s="2" t="inlineStr">
+        <is>
+          <t>Rapport (agence, propriétaire, période, totaux dont retenue à la source et dépôt de garantie conservé, lignes par bien) ; refus uniforme 404 (inconnu, expiré, révoqué, corps invalide) ; 429 au-delà de 30 requêtes par minute et par IP ; en-têtes no-store et noindex ; la page affiche « Service momentanément indisponible » sur panne serveur</t>
+        </is>
+      </c>
+      <c r="I716" s="2" t="inlineStr">
+        <is>
+          <t>Envoyer le rapport du mois au propriétaire (WhatsApp ou e-mail) ou Créer / copier un lien sécurisé de rapport mensuel</t>
+        </is>
+      </c>
+      <c r="J716" s="2" t="inlineStr">
+        <is>
+          <t>Toute personne détenant un lien valide (propriétaire destinataire)</t>
+        </is>
+      </c>
+      <c r="K716" s="2" t="inlineStr">
+        <is>
+          <t>Public (sans connexion)</t>
+        </is>
+      </c>
+      <c r="L716" s="2" t="inlineStr">
+        <is>
+          <t>POST /api/public/secure-links/owner-monthly-report</t>
+        </is>
+      </c>
+      <c r="M716" s="2" t="inlineStr">
+        <is>
+          <t>Aucune (jeton à usage unique de lecture, haché en base)</t>
+        </is>
+      </c>
+      <c r="N716" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O716" s="2" t="inlineStr">
+        <is>
+          <t>Page publique /rapport-proprietaire#&lt;jeton&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" s="2" t="inlineStr">
+        <is>
+          <t>Gestion locative</t>
+        </is>
+      </c>
+      <c r="B717" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C717" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE (menu) / RENTAL (feature déclarée sur l'entrée « Relevés »)</t>
+        </is>
+      </c>
+      <c r="D717" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine — Notifications propriétaire</t>
+        </is>
+      </c>
+      <c r="E717" s="2" t="inlineStr">
+        <is>
+          <t>Envoi mensuel automatique du rapport aux propriétaires</t>
+        </is>
+      </c>
+      <c r="F717" s="2" t="inlineStr">
+        <is>
+          <t>Envoyer chaque mois, sans action manuelle, le rapport du mois précédent (relevés non brouillons, une seule fois par relevé) aux propriétaires consentants. Tâche planifiée quotidienne, active les 10 premiers jours du mois.</t>
+        </is>
+      </c>
+      <c r="G717" s="2" t="inlineStr">
+        <is>
+          <t>Aucune (tâche planifiée) ; variable `PATRIMOINE_MONTHLY_REPORT_JOB_ENABLED`</t>
+        </is>
+      </c>
+      <c r="H717" s="2" t="inlineStr">
+        <is>
+          <t>Messages WhatsApp ou e-mail avec lien sécurisé ; journal d'audit `PATRIMOINE_OWNER_MONTHLY_REPORT_SENT`</t>
+        </is>
+      </c>
+      <c r="I717" s="2" t="inlineStr">
+        <is>
+          <t>Envoyer le rapport du mois au propriétaire (WhatsApp ou e-mail)</t>
+        </is>
+      </c>
+      <c r="J717" s="2" t="inlineStr">
+        <is>
+          <t>Aucun (tâche système)</t>
+        </is>
+      </c>
+      <c r="K717" s="2" t="inlineStr">
+        <is>
+          <t>Aucun (tâche planifiée)</t>
+        </is>
+      </c>
+      <c r="L717" s="2" t="inlineStr">
+        <is>
+          <t>Aucune (tâche planifiée `jobs/owner-monthly-report-job.ts`)</t>
+        </is>
+      </c>
+      <c r="M717" s="2" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="N717" s="2" t="inlineStr">
+        <is>
+          <t>Disponible (désactivé par défaut)</t>
+        </is>
+      </c>
+      <c r="O717" s="2" t="inlineStr">
+        <is>
+          <t>Aucun</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" s="2" t="inlineStr">
+        <is>
+          <t>Gestion locative</t>
+        </is>
+      </c>
+      <c r="B718" s="2" t="inlineStr">
+        <is>
+          <t>Agence, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C718" s="2" t="inlineStr">
+        <is>
+          <t>PATRIMOINE (menu) / RENTAL (feature déclarée sur l'entrée « Relevés »)</t>
+        </is>
+      </c>
+      <c r="D718" s="2" t="inlineStr">
+        <is>
+          <t>Patrimoine — Notifications propriétaire</t>
+        </is>
+      </c>
+      <c r="E718" s="2" t="inlineStr">
+        <is>
+          <t>Alertes d'échéance de bail et de document à renouveler par WhatsApp</t>
+        </is>
+      </c>
+      <c r="F718" s="2" t="inlineStr">
+        <is>
+          <t>Prévenir le propriétaire d'une fin de bail ou d'un document arrivant à échéance par son canal préféré (WhatsApp ou e-mail, repli sur l'autre), avec consentement vérifié et anti-doublon ; un contact e-mail seul reçoit toujours l'e-mail comme avant ; les clés WhatsApp `OWNER_*` sont désactivées par défaut (opt-in par agence).</t>
+        </is>
+      </c>
+      <c r="G718" s="2" t="inlineStr">
+        <is>
+          <t>Aucune (tâche planifiée quotidienne) ; événements WhatsApp `OWNER_LEASE_ENDING_SOON` et `OWNER_DOCUMENT_EXPIRY_ALERT`, e-mail `LEASE_ENDING_SOON` et `DOCUMENT_EXPIRY_ALERT`</t>
+        </is>
+      </c>
+      <c r="H718" s="2" t="inlineStr">
+        <is>
+          <t>Message WhatsApp ou e-mail au propriétaire</t>
+        </is>
+      </c>
+      <c r="I718" s="2" t="inlineStr">
+        <is>
+          <t>Consentement WhatsApp ou e-mail du propriétaire ; événement activé dans la configuration de l'agence</t>
+        </is>
+      </c>
+      <c r="J718" s="2" t="inlineStr">
+        <is>
+          <t>Aucun (tâche système)</t>
+        </is>
+      </c>
+      <c r="K718" s="2" t="inlineStr">
+        <is>
+          <t>Aucun (tâche planifiée)</t>
+        </is>
+      </c>
+      <c r="L718" s="2" t="inlineStr">
+        <is>
+          <t>Aucune (tâche planifiée `jobs/document-expiry-alert-job.ts`)</t>
+        </is>
+      </c>
+      <c r="M718" s="2" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="N718" s="2" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O718" s="2" t="inlineStr">
+        <is>
+          <t>Aucun</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: rétention, scellés quotidiens et vérification d'intégrité du journal d'audit, phase 5 (ADR-006)
- marqueurs anti-doublon hors d'AuditLog (table notification_markers)
- scellés chaînés par racine de Merkle (audit_seals), fonction SQL de purge gardée
- job quotidien (scellement, purge opt-in, vérification), GET /api/admin/audit/integrity
- carte « Intégrité du journal » dans la console plateforme
- docs : spec 023, ADR-006, RUNBOOK, SECURITY, wiki, HANDOFF

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Leurqh2Hminex89pSKXM7W
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -189,8 +189,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O713" headerRowCount="1">
-  <autoFilter ref="A1:O711"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O715" headerRowCount="1">
+  <autoFilter ref="A1:O715"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Domaine (regroupement agent)"/>
     <tableColumn id="2" name="Pack(s)"/>
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O713"/>
+  <dimension ref="A1:O715"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -53591,7 +53591,7 @@
       </c>
       <c r="H687" t="inlineStr">
         <is>
-          <t>E-mail « Fin de bail prochaine » (gabarit `LEASE_ENDING_SOON`, personnalisable) ; entree `AuditLog` (`PATRIMOINE_LEASE_END_ALERT_SENT`) posee comme marque anti-doublon</t>
+          <t>E-mail « Fin de bail prochaine » (gabarit `LEASE_ENDING_SOON`, personnalisable) ; marque anti-doublon inscrite dans la table `notification_markers` (type `lease_end`), hors du journal d'audit</t>
         </is>
       </c>
       <c r="I687" t="inlineStr">
@@ -53668,7 +53668,7 @@
       </c>
       <c r="H688" t="inlineStr">
         <is>
-          <t>E-mail « Alerte fin de prêt » (gabarit `LOAN_MATURITY_ALERT`, personnalisable) ; entree `AuditLog` (`PATRIMOINE_LOAN_MATURITY_ALERT_SENT`) posee comme marque anti-doublon</t>
+          <t>E-mail « Alerte fin de prêt » (gabarit `LOAN_MATURITY_ALERT`, personnalisable) ; marque anti-doublon inscrite dans la table `notification_markers` (type `loan_maturity`), hors du journal d'audit</t>
         </is>
       </c>
       <c r="I688" t="inlineStr">
@@ -53745,7 +53745,7 @@
       </c>
       <c r="H689" t="inlineStr">
         <is>
-          <t>E-mail « Rappel programme de travaux » (gabarit `WORK_PROGRAM_REMINDER`, personnalisable) ; entree `AuditLog` (`PATRIMOINE_WORK_UPCOMING_ALERT_SENT`) posee comme marque anti-doublon</t>
+          <t>E-mail « Rappel programme de travaux » (gabarit `WORK_PROGRAM_REMINDER`, personnalisable) ; marque anti-doublon inscrite dans la table `notification_markers` (type `work_upcoming`), hors du journal d'audit</t>
         </is>
       </c>
       <c r="I689" t="inlineStr">
@@ -55629,6 +55629,160 @@
       <c r="O713" t="inlineStr">
         <is>
           <t>Administration &gt; Journaux d'audit &gt; Exporter en CSV</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>Administration plateforme</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>N/A (plateforme)</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>Administration plateforme</t>
+        </is>
+      </c>
+      <c r="D714" t="inlineStr">
+        <is>
+          <t>Statistiques et audit</t>
+        </is>
+      </c>
+      <c r="E714" t="inlineStr">
+        <is>
+          <t>Vérifier l'intégrité du journal d'audit</t>
+        </is>
+      </c>
+      <c r="F714" t="inlineStr">
+        <is>
+          <t>Contrôler que le journal n'a été ni modifié ni amputé : recalcule la racine de Merkle de chaque journée scellée (une partition = jour UTC × agence ou plateforme × visibilité) et la compare au scellé, puis vérifie le chaînage de tous les scellés. Lecture seule, à la demande (jamais automatique). Limité à 10 vérifications par 10 minutes et par utilisateur</t>
+        </is>
+      </c>
+      <c r="G714" t="inlineStr">
+        <is>
+          <t>Query facultative, schéma strict : `from`, `to` (AAAA-MM-JJ, jours UTC, `from` ≤ `to`). Sans période : les 500 scellés les plus récents ; tout autre paramètre est refusé en 400</t>
+        </is>
+      </c>
+      <c r="H714" t="inlineStr">
+        <is>
+          <t>`{ ok, chain {ok, sealsChecked, brokenAtSeq?, head {seq, sealDate, chainHash}}, partitions {checked, ok, expired, lateRows[], tampered[], truncated} }`. Statuts d'une partition : OK ; EXPIRED (purgée par la rétention, normal) ; LATE_ROWS (lignes arrivées après le scellé, à regarder) ; ROWS_MISSING et ALTERED (incident). Chaque consultation est tracée (`AUDIT_VIEWED`)</t>
+        </is>
+      </c>
+      <c r="I714" t="inlineStr">
+        <is>
+          <t>Consulter les journaux d'audit</t>
+        </is>
+      </c>
+      <c r="J714" t="inlineStr">
+        <is>
+          <t>Collaborateur plateforme avec PLATFORM_AUDIT_VIEW (super-admin par défaut)</t>
+        </is>
+      </c>
+      <c r="K714" t="inlineStr">
+        <is>
+          <t>Super-admin</t>
+        </is>
+      </c>
+      <c r="L714" t="inlineStr">
+        <is>
+          <t>GET /api/admin/audit/integrity</t>
+        </is>
+      </c>
+      <c r="M714" t="inlineStr">
+        <is>
+          <t>PLATFORM_AUDIT_VIEW + limiteur `auditIntegrityRateLimiter`</t>
+        </is>
+      </c>
+      <c r="N714" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O714" t="inlineStr">
+        <is>
+          <t>Administration &gt; Journaux d'audit &gt; Intégrité du journal (bouton « Vérifier l'intégrité »)</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>Administration plateforme</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>N/A (plateforme)</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>Administration plateforme</t>
+        </is>
+      </c>
+      <c r="D715" t="inlineStr">
+        <is>
+          <t>Statistiques et audit</t>
+        </is>
+      </c>
+      <c r="E715" t="inlineStr">
+        <is>
+          <t>Sceller, purger et surveiller le journal d'audit (tâche planifiée)</t>
+        </is>
+      </c>
+      <c r="F715" t="inlineStr">
+        <is>
+          <t>Chaque jour à 2 h 30 UTC : scelle les journées révolues (après `AUDIT_SEAL_GRACE_DAYS` jours, 2 par défaut) en une racine de Merkle chaînée au scellé précédent ; purge les lignes scellées plus anciennes que la rétention (`AUDIT_RETENTION_TENANT_MONTHS` 24 mois pour les lignes visibles de l'agence, `AUDIT_RETENTION_PLATFORM_MONTHS` 60 mois pour les lignes réservées à la plateforme) SEULEMENT si `AUDIT_PURGE_ENABLED=true` (désactivée par défaut, irréversible) ; revérifie la chaîne et les 7 derniers jours ; journalise la tête de chaîne à ancrer hors de la base. La purge refuse une date limite de moins de 180 jours et ne supprime jamais une ligne non scellée</t>
+        </is>
+      </c>
+      <c r="G715" t="inlineStr">
+        <is>
+          <t>Aucune (tâche planifiée `audit-maintenance-job`) ; variables `AUDIT_RETENTION_TENANT_MONTHS`, `AUDIT_RETENTION_PLATFORM_MONTHS`, `AUDIT_SEAL_GRACE_DAYS`, `AUDIT_PURGE_ENABLED`</t>
+        </is>
+      </c>
+      <c r="H715" t="inlineStr">
+        <is>
+          <t>Scellés (`audit_seals`, ajout seul) ; événements `AUDIT_SEALED`, `AUDIT_PURGED` (écrit dans la même transaction que la suppression) et `AUDIT_INTEGRITY_FAILED` (critique) réservés à la plateforme ; log de la tête de chaîne</t>
+        </is>
+      </c>
+      <c r="I715" t="inlineStr">
+        <is>
+          <t>Consulter les journaux d'audit</t>
+        </is>
+      </c>
+      <c r="J715" t="inlineStr">
+        <is>
+          <t>Système (tâche planifiée)</t>
+        </is>
+      </c>
+      <c r="K715" t="inlineStr">
+        <is>
+          <t>— (job serveur)</t>
+        </is>
+      </c>
+      <c r="L715" t="inlineStr">
+        <is>
+          <t>N/A — job cron interne (`packages/api/src/jobs/audit-maintenance-job.ts`), pas de route API</t>
+        </is>
+      </c>
+      <c r="M715" t="inlineStr">
+        <is>
+          <t>Aucune (exécution serveur, hors requête HTTP)</t>
+        </is>
+      </c>
+      <c r="N715" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O715" t="inlineStr">
+        <is>
+          <t>Aucun (technique)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(patrimoine): corrections de la recette navigateur de la vague A
- Sélecteur de bien à recherche serveur et chargement progressif (Performance et
  Trésorerie prévisionnelle) : plus de plafond à 100 biens (BUG 001, 007).
- Fiche bien : le profil fiscal se rafraîchit après une valorisation (002) ;
  les charges de l'année excluent les dépenses capitalisées, onglet et vue
  consolidée (010) ; bouton « Enregistrer les détenteurs » qui se replie à 375 px (012).
- Page publique du rapport : une seule requête sous StrictMode (004), changement de
  fragment pris en compte et réponse tardive ignorée (005), échec transitoire non
  mis en cache.
- Messages d'erreur des dépenses avec accents + test de garde (008), message du
  relevé brouillon exact (006), note « taxe couverte par une dépense récurrente »
  du plan de trésorerie (009), lignes de l'estimation fiscale traduisibles (011).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -4070,7 +4070,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Calculer rendement brut/net/net-net, plus-value latente, projection à horizon, pour tout le portefeuille (sans `propertyId`) ou pour un bien précis ; avec `propertyId`, le net-net et la plus-value latente sont `null` tant que le prix d'acquisition du bien est inconnu. Rendements arrondis (et non tronqués), affichés au format français ; le net-net projeté se rapporte au plus élevé du coût de revient et de la valeur projetée, si bien que brut ≥ net ≥ net-net à tout horizon.</t>
+          <t>Calculer rendement brut/net/net-net, plus-value latente, projection à horizon, pour tout le portefeuille (sans `propertyId`) ou pour un bien précis ; avec `propertyId`, le net-net et la plus-value latente sont `null` tant que le prix d'acquisition du bien est inconnu. Rendements arrondis (et non tronqués), affichés au format français ; le net-net projeté se rapporte au plus élevé du coût de revient et de la valeur projetée, si bien que brut ≥ net ≥ net-net à tout horizon. À l'écran, le sélecteur de bien recherche côté serveur (titre, adresse, référence) et charge les biens par pages, sans plafond à 100 biens.</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -56353,7 +56353,7 @@
       </c>
       <c r="F723" t="inlineStr">
         <is>
-          <t>Restreindre le plan à un seul bien du patrimoine.</t>
+          <t>Restreindre le plan à un seul bien du patrimoine. Le sélecteur de bien recherche côté serveur (titre, adresse, référence) et charge les biens par pages : aucun plafond à 100 biens.</t>
         </is>
       </c>
       <c r="G723" t="inlineStr">
@@ -56517,7 +56517,7 @@
       </c>
       <c r="H725" t="inlineStr">
         <is>
-          <t>Lignes avec `source`, marque « estimation indicative » pour une taxe aux paramètres à valider ; `sources[]` avec statut et motif</t>
+          <t>Lignes avec `source`, marque « estimation indicative » pour une taxe aux paramètres à valider ; `sources[]` avec statut et motif Pour la taxe foncière non estimable, `sources[].coveredByRecurringExpenseCount` indique les biens écartés parce qu'une dépense périodique de taxe les couvre déjà (affiché sous la source).</t>
         </is>
       </c>
       <c r="I725" t="inlineStr">

</xml_diff>

<commit_message>
fix(patrimoine): corrections de la recette des vagues B et C (anomalies 2026-10-02-001 à 015)
B1/B2 : jours avant échéance des polices, erreurs de validation par champ,
étiquette « À valider » en liste foncière, filtres bien/police des sinistres,
pièce justificative de police, case « Étape obligatoire », pièces verrouillées
sur sinistre clos, menu Patrimoine masqué sans PROPERTIES_VIEW et écran de refus.
B3 : une seule consultation par ouverture, pas d'amorçage d'authentification
sur les pages publiques à jeton, mise en page mobile et colonne Actions.
C4 : pas de rapprochement Montant/Surface, surface plafonnée à 500 000 m².
C5 : hôtes *.localhost acceptés en simulateur, statut du détail d'échéance
aligné sur la liste, lien refusé sur une échéance en brouillon à venir.
Inscription : le front envoie confirmPassword.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -189,8 +189,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O791" headerRowCount="1">
-  <autoFilter ref="A1:O791"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O792" headerRowCount="1">
+  <autoFilter ref="A1:O792"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Domaine (regroupement agent)"/>
     <tableColumn id="2" name="Pack(s)"/>
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O791"/>
+  <dimension ref="A1:O792"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -8305,7 +8305,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>Suivre les échéances (par bail, par locataire, en retard...). Le statut est reclassé à l'affichage : une échéance échue et non soldée apparaît « En retard » (Brouillon comprise) même si le job quotidien n'a pas tourné.</t>
+          <t>Suivre les échéances (par bail, par locataire, en retard...). Le statut est reclassé à l'affichage : une échéance échue et non soldée apparaît « En retard » (Brouillon comprise) même si le job quotidien n'a pas tourné. Le détail d'une échéance affiche le même statut reclassé que la liste.</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -39798,7 +39798,7 @@
       </c>
       <c r="F508" s="2" t="inlineStr">
         <is>
-          <t>Menus masqués pour l'utilisateur courant (et éventuellement une agence donnée)</t>
+          <t>Menus masqués pour l'utilisateur courant (et éventuellement une agence donnée) Renvoie aussi les permissions du compte, ce qui permet à la coquille de masquer les entrées Biens/Patrimoine (Sinistres, Régularisation foncière, Accès partagés) pour un rôle sans PROPERTIES_VIEW.</t>
         </is>
       </c>
       <c r="G508" s="2" t="inlineStr">
@@ -39808,7 +39808,7 @@
       </c>
       <c r="H508" s="2" t="inlineStr">
         <is>
-          <t>`{disabledMenuKeys[]}`</t>
+          <t>`{disabledMenuKeys[]}` + `permissions[]` du compte</t>
         </is>
       </c>
       <c r="I508" s="2" t="inlineStr">
@@ -40029,12 +40029,12 @@
       </c>
       <c r="F511" s="2" t="inlineStr">
         <is>
-          <t>Création de compte + envoi d'un e-mail de vérification. L'e-mail est rédigé dans la langue préférée du compte, sinon celle de la requête, sinon le français.</t>
+          <t>Création de compte + envoi d'un e-mail de vérification. L'e-mail est rédigé dans la langue préférée du compte, sinon celle de la requête, sinon le français. La page envoie aussi la confirmation du mot de passe.</t>
         </is>
       </c>
       <c r="G511" s="2" t="inlineStr">
         <is>
-          <t>`email, password, fullName`</t>
+          <t>`email, password, fullName` + `confirmPassword`</t>
         </is>
       </c>
       <c r="H511" s="2" t="inlineStr">
@@ -56738,7 +56738,7 @@
       </c>
       <c r="F728" t="inlineStr">
         <is>
-          <t>Lister les polices d'un bien ou de l'agence avec leur statut dérivé (à venir, active, expire bientôt, expirée)</t>
+          <t>Lister les polices d'un bien ou de l'agence avec leur statut dérivé (à venir, active, expire bientôt, expirée) La liste affiche une colonne « Échéance » (« Dans N jours », « Expire aujourd'hui », « Expirée depuis N jours »).</t>
         </is>
       </c>
       <c r="G728" t="inlineStr">
@@ -56815,7 +56815,7 @@
       </c>
       <c r="F729" t="inlineStr">
         <is>
-          <t>Enregistrer une police (multirisque habitation, multirisque immeuble, responsabilité propriétaire, autre) sur un bien</t>
+          <t>Enregistrer une police (multirisque habitation, multirisque immeuble, responsabilité propriétaire, autre) sur un bien La modale de police propose le champ « Pièce justificative ».</t>
         </is>
       </c>
       <c r="G729" t="inlineStr">
@@ -56969,7 +56969,7 @@
       </c>
       <c r="F731" t="inlineStr">
         <is>
-          <t>Corriger les dates, la prime, les notes ou la pièce d'une police</t>
+          <t>Corriger les dates, la prime, les notes ou la pièce d'une police La modale de police propose le champ « Pièce justificative ».</t>
         </is>
       </c>
       <c r="G731" t="inlineStr">
@@ -57123,7 +57123,7 @@
       </c>
       <c r="F733" t="inlineStr">
         <is>
-          <t>Suivre les sinistres d'un bien, ou de toute l'agence, filtrés par statut</t>
+          <t>Suivre les sinistres d'un bien, ou de toute l'agence, filtrés par statut La page Sinistres filtre par bien et par police.</t>
         </is>
       </c>
       <c r="G733" t="inlineStr">
@@ -57585,7 +57585,7 @@
       </c>
       <c r="F739" t="inlineStr">
         <is>
-          <t>Joindre un document du bien (photo avant ou après, devis, rapport d'expertise, courrier de l'assureur, facture) à un sinistre</t>
+          <t>Joindre un document du bien (photo avant ou après, devis, rapport d'expertise, courrier de l'assureur, facture) à un sinistre Sur un sinistre clos, les pièces ne sont plus modifiables dans l'écran (ni ajout ni retrait).</t>
         </is>
       </c>
       <c r="G739" t="inlineStr">
@@ -57662,7 +57662,7 @@
       </c>
       <c r="F740" t="inlineStr">
         <is>
-          <t>Détacher une pièce d'un sinistre sans supprimer le document du bien</t>
+          <t>Détacher une pièce d'un sinistre sans supprimer le document du bien Sur un sinistre clos, les pièces ne sont plus modifiables dans l'écran (ni ajout ni retrait).</t>
         </is>
       </c>
       <c r="G740" t="inlineStr">
@@ -58355,7 +58355,7 @@
       </c>
       <c r="F749" t="inlineStr">
         <is>
-          <t>Suivre tous les dossiers de régularisation foncière de l'agence avec leur avancement, leurs frais engagés et leurs échéances</t>
+          <t>Suivre tous les dossiers de régularisation foncière de l'agence avec leur avancement, leurs frais engagés et leurs échéances Un dossier de la filière CI_ACD porte l'étiquette « À valider » dans la liste.</t>
         </is>
       </c>
       <c r="G749" t="inlineStr">
@@ -58817,7 +58817,7 @@
       </c>
       <c r="F755" t="inlineStr">
         <is>
-          <t>Renseigner l'échéance, les frais engagés en XOF, les notes et la pièce justificative d'une étape</t>
+          <t>Renseigner l'échéance, les frais engagés en XOF, les notes et la pièce justificative d'une étape Dans le tiroir d'une étape d'un dossier à filière personnalisée, la case « Étape obligatoire » règle `required`.</t>
         </is>
       </c>
       <c r="G755" t="inlineStr">
@@ -59490,7 +59490,7 @@
       </c>
       <c r="F764" t="inlineStr">
         <is>
-          <t>Faire reconnaître chaque colonne comme un champ de la nature (proposition automatique, correction à la main) ; l'étape est sautée quand le rapprochement est parfait.</t>
+          <t>Faire reconnaître chaque colonne comme un champ de la nature (proposition automatique, correction à la main) ; l'étape est sautée quand le rapprochement est parfait. Le rapprochement automatique n'associe plus « Montant » à « Surface ».</t>
         </is>
       </c>
       <c r="G764" t="inlineStr">
@@ -59562,7 +59562,7 @@
       </c>
       <c r="F765" t="inlineStr">
         <is>
-          <t>Voir pour chaque ligne les valeurs reconnues (nombres « 1 250 000,50 », dates JJ/MM/AAAA, type de bien, commune du référentiel géographique), les erreurs en clair avec le numéro de ligne du fichier, corriger les cellules et décocher des lignes ; aucune écriture n'a lieu avant la validation. La valeur réellement lue est affichée sous les cellules numériques et de date (« Lu : … ») ; un CSV lu en Windows-1252 est signalé par un avertissement ; une formule (= ou @ en tête) est refusée quel que soit le champ.</t>
+          <t>Voir pour chaque ligne les valeurs reconnues (nombres « 1 250 000,50 », dates JJ/MM/AAAA, type de bien, commune du référentiel géographique), les erreurs en clair avec le numéro de ligne du fichier, corriger les cellules et décocher des lignes ; aucune écriture n'a lieu avant la validation. La valeur réellement lue est affichée sous les cellules numériques et de date (« Lu : … ») ; un CSV lu en Windows-1252 est signalé par un avertissement ; une formule (= ou @ en tête) est refusée quel que soit le champ. La surface est plafonnée à 500 000 m² (au-delà : erreur de ligne en clair).</t>
         </is>
       </c>
       <c r="G765" t="inlineStr">
@@ -60394,7 +60394,7 @@
       </c>
       <c r="F776" t="inlineStr">
         <is>
-          <t>Donner à un notaire, un expert-comptable ou un banquier un accès en lecture seule, sans compte, à des biens ou entités choisis, avec des rubriques précises, des documents explicitement partagés et une échéance (ou un accès permanent). Un lien sécurisé est émis et envoyé par e-mail au bénéficiaire ; son URL n'est affichée qu'une fois.</t>
+          <t>Donner à un notaire, un expert-comptable ou un banquier un accès en lecture seule, sans compte, à des biens ou entités choisis, avec des rubriques précises, des documents explicitement partagés et une échéance (ou un accès permanent). Un lien sécurisé est émis et envoyé par e-mail au bénéficiaire ; son URL n'est affichée qu'une fois. Dans l'écran agence, la colonne Actions de la liste est épinglée.</t>
         </is>
       </c>
       <c r="G776" t="inlineStr">
@@ -60933,7 +60933,7 @@
       </c>
       <c r="F783" t="inlineStr">
         <is>
-          <t>Afficher, sans connexion, les biens du périmètre et les seules rubriques accordées (valorisations, rendement et ratios, emprunts, dépenses, baux et loyers, titres et propriété, documents partageables), avec un bandeau « Accès en lecture seule accordé par &lt;agence&gt; ». Jeton dans le fragment de l'URL, envoyé en corps de POST ; limiteur de débit par IP ; chaque consultation est journalisée. Aucune coordonnée ni identité de locataire n'est renvoyée.</t>
+          <t>Afficher, sans connexion, les biens du périmètre et les seules rubriques accordées (valorisations, rendement et ratios, emprunts, dépenses, baux et loyers, titres et propriété, documents partageables), avec un bandeau « Accès en lecture seule accordé par &lt;agence&gt; ». Jeton dans le fragment de l'URL, envoyé en corps de POST ; limiteur de débit par IP ; chaque consultation est journalisée. Aucune coordonnée ni identité de locataire n'est renvoyée. La page publique ne lance pas l'amorçage d'authentification (aucun appel /auth/me ni /auth/refresh), n'envoie qu'une consultation par ouverture et a une mise en page adaptée au mobile.</t>
         </is>
       </c>
       <c r="G783" t="inlineStr">
@@ -61087,7 +61087,7 @@
       </c>
       <c r="F785" t="inlineStr">
         <is>
-          <t>Envoyer au locataire, par son canal préféré (WhatsApp ou e-mail, un seul canal par message, avec consentement), un lien sécurisé vers UNE échéance de loyer : il paiera le reste dû en Mobile Money sans compte. Durée de validité 7 jours par défaut (30 au plus). Le lien est créé seulement si un canal est éligible et révoqué si tous les envois échouent ; aucun lien n'est conservé si rien n'est envoyé.</t>
+          <t>Envoyer au locataire, par son canal préféré (WhatsApp ou e-mail, un seul canal par message, avec consentement), un lien sécurisé vers UNE échéance de loyer : il paiera le reste dû en Mobile Money sans compte. Durée de validité 7 jours par défaut (30 au plus). Le lien est créé seulement si un canal est éligible et révoqué si tous les envois échouent ; aucun lien n'est conservé si rien n'est envoyé. La création et l'envoi sont refusés (400) sur une échéance encore en brouillon à venir. En mode simulateur, les hôtes *.localhost sont acceptés pour l'URL de paiement.</t>
         </is>
       </c>
       <c r="G785" t="inlineStr">
@@ -61164,7 +61164,7 @@
       </c>
       <c r="F786" t="inlineStr">
         <is>
-          <t>Créer un lien de paiement d'une échéance sans l'envoyer, pour le transmettre soi-même (messagerie, SMS personnel, en main propre). L'URL complète n'est affichée qu'à la création : elle ne peut pas être relue ensuite.</t>
+          <t>Créer un lien de paiement d'une échéance sans l'envoyer, pour le transmettre soi-même (messagerie, SMS personnel, en main propre). L'URL complète n'est affichée qu'à la création : elle ne peut pas être relue ensuite. La création est refusée sur une échéance encore en brouillon à venir ; en mode simulateur, les hôtes *.localhost sont acceptés pour l'URL de paiement.</t>
         </is>
       </c>
       <c r="G786" t="inlineStr">
@@ -61595,6 +61595,83 @@
       <c r="O791" t="inlineStr">
         <is>
           <t>Communication &gt; Notifications e-mail ; Communication &gt; Notifications WhatsApp</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr">
+        <is>
+          <t>Parc immobilier</t>
+        </is>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>Agence, Promoteur, Opérateur intégré, Patrimoine Essentiel, Patrimoine Pro</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>PATRIMOINE</t>
+        </is>
+      </c>
+      <c r="D792" t="inlineStr">
+        <is>
+          <t>Menu Patrimoine et accès refusé</t>
+        </is>
+      </c>
+      <c r="E792" t="inlineStr">
+        <is>
+          <t>Masquer les entrées Patrimoine sans PROPERTIES_VIEW et afficher « Accès non autorisé » sur 403</t>
+        </is>
+      </c>
+      <c r="F792" t="inlineStr">
+        <is>
+          <t>Pour un rôle sans PROPERTIES_VIEW, les entrées Biens/Patrimoine (dont Sinistres, Régularisation foncière, Accès partagés) sont masquées du menu ; une réponse 403 sur Sinistres, la liste et le détail foncier ou Accès partagés affiche l'écran « Accès non autorisé ». Les erreurs de validation serveur des écrans assurances affichent le champ fautif et son message.</t>
+        </is>
+      </c>
+      <c r="G792" t="inlineStr">
+        <is>
+          <t>Permissions du compte (GET /roles/menu-access/me)</t>
+        </is>
+      </c>
+      <c r="H792" t="inlineStr">
+        <is>
+          <t>Menu filtré ; écran « Accès non autorisé »</t>
+        </is>
+      </c>
+      <c r="I792" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J792" t="inlineStr">
+        <is>
+          <t>Collaborateur agence sans PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="K792" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L792" t="inlineStr">
+        <is>
+          <t>GET /api/roles/menu-access/me</t>
+        </is>
+      </c>
+      <c r="M792" t="inlineStr">
+        <is>
+          <t>PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="N792" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O792" t="inlineStr">
+        <is>
+          <t>Patrimoine (entrées masquées)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(copilot): page de chat plein écran et dictée (étape 1 du plan v2)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NipnEzc6N8uvDDXG2M7jms
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sous-fonctionnalites" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legende Packs-Modules" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes et points ouverts" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sous-fonctionnalites" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Legende Packs-Modules" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Notes et points ouverts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -189,7 +189,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O848" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O850" headerRowCount="1">
   <autoFilter ref="A1:O848"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Domaine (regroupement agent)"/>
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O848"/>
+  <dimension ref="A1:O850"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -53857,7 +53857,7 @@
       </c>
       <c r="O690" s="2" t="inlineStr">
         <is>
-          <t>Bouton flottant Assistant (Ctrl/Cmd+J), toutes pages d'agence</t>
+          <t>Bouton flottant Assistant (Ctrl/Cmd+J), toutes pages d'agence ; menu « Assistant » (zone Plus, section Commercial et communication) quand l'assistant est activé</t>
         </is>
       </c>
     </row>
@@ -53889,7 +53889,7 @@
       </c>
       <c r="F691" s="2" t="inlineStr">
         <is>
-          <t>Ouvre le tiroir de conversation (côté « fin » : à droite en français, à gauche en arabe) et envoie l'échange au fournisseur LLM en flux SSE : texte progressif, cartes de résultats (biens, baux, documents, proposition), suggestions selon l'écran courant, arrêt de la réponse et nouvelle conversation. Conversation non persistée ; l'assistant n'écrit jamais lui-même. Limites : 20 messages, 4 000 caractères chacun, 24 000 au total ; 20 requêtes/min et 300/jour par utilisateur et par agence, plus un plafond par agence tous collaborateurs confondus (`AI_TENANT_MINUTE_LIMIT` 100/min, `AI_TENANT_DAILY_LIMIT` 3000/jour) ; limiteurs en mémoire, par instance d'API ; 4 tours et 8 appels d'outils maximum. L'invite système est construite par agence et ne cite que les capacités des outils exposés (permissions et modules souscrits) ; un appel d'outil d'un module non souscrit (modèle qui en invente un) est refusé poliment (résultat `MODULE_NOT_INCLUDED`, journal d'audit `AI_TOOL_DENIED`) et n'est jamais exécuté.</t>
+          <t>Ouvre le tiroir de conversation (côté « fin » : à droite en français, à gauche en arabe ; bouton « Ouvrir en pleine page » vers la page Assistant) et envoie l'échange au fournisseur LLM en flux SSE : texte progressif, cartes de résultats (biens, baux, documents, proposition), suggestions selon l'écran courant, arrêt de la réponse et nouvelle conversation. Conversation non persistée ; l'assistant n'écrit jamais lui-même. Limites : 20 messages, 4 000 caractères chacun, 24 000 au total ; 20 requêtes/min et 300/jour par utilisateur et par agence, plus un plafond par agence tous collaborateurs confondus (`AI_TENANT_MINUTE_LIMIT` 100/min, `AI_TENANT_DAILY_LIMIT` 3000/jour) ; limiteurs en mémoire, par instance d'API ; 4 tours et 8 appels d'outils maximum. L'invite système est construite par agence et ne cite que les capacités des outils exposés (permissions et modules souscrits) ; un appel d'outil d'un module non souscrit (modèle qui en invente un) est refusé poliment (résultat `MODULE_NOT_INCLUDED`, journal d'audit `AI_TOOL_DENIED`) et n'est jamais exécuté.</t>
         </is>
       </c>
       <c r="G691" s="2" t="inlineStr">
@@ -53934,7 +53934,7 @@
       </c>
       <c r="O691" s="2" t="inlineStr">
         <is>
-          <t>Bouton flottant Assistant (Ctrl/Cmd+J), toutes pages d'agence</t>
+          <t>Bouton flottant Assistant (Ctrl/Cmd+J), toutes pages d'agence ; menu « Assistant » (zone Plus, section Commercial et communication) quand l'assistant est activé</t>
         </is>
       </c>
     </row>
@@ -65979,6 +65979,160 @@
       <c r="O848" t="inlineStr">
         <is>
           <t>Agence &gt; Paramètres de l'agence &gt; carte « SMS »</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>Communication et Documents</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>Agence, Syndic, Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="D849" t="inlineStr">
+        <is>
+          <t>Assistant IA ImmoCopilot</t>
+        </is>
+      </c>
+      <c r="E849" t="inlineStr">
+        <is>
+          <t>Discuter avec l'assistant en pleine page</t>
+        </is>
+      </c>
+      <c r="F849" t="inlineStr">
+        <is>
+          <t>Page de chat plein écran (route `/tenant/:tenantId/assistant`, entrée de menu « Assistant ») : fil des messages défilant en haut, zone de saisie fixée en bas (Entrée envoie, Maj+Entrée saute une ligne, la zone grandit avec le texte), emplacement vide à droite réservé aux futurs artefacts (replié sous 992 px). Même conversation, mêmes cartes et mêmes limites que le tiroir (flux `POST /api/tenants/:tenantId/ai/chat`) ; la conversation reste en mémoire et n'est pas reprise entre le tiroir et la page. Si l'assistant est désactivé, la page l'indique et l'entrée de menu est masquée. Ctrl/Cmd+J ouvre toujours le tiroir.</t>
+        </is>
+      </c>
+      <c r="G849" t="inlineStr">
+        <is>
+          <t>Message saisi ; contexte de l'écran courant</t>
+        </is>
+      </c>
+      <c r="H849" t="inlineStr">
+        <is>
+          <t>Réponse en flux, cartes de résultats et propositions (même rendu que le tiroir)</t>
+        </is>
+      </c>
+      <c r="I849" t="inlineStr">
+        <is>
+          <t>Statut de l'assistant (activé)</t>
+        </is>
+      </c>
+      <c r="J849" t="inlineStr">
+        <is>
+          <t>Collaborateurs de l'agence ; chaque outil vérifie sa propre permission</t>
+        </is>
+      </c>
+      <c r="K849" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L849" t="inlineStr">
+        <is>
+          <t>Aucune route nouvelle : écran web qui réutilise `POST /api/tenants/:tenantId/ai/chat` et `GET /api/tenants/:tenantId/ai/status`</t>
+        </is>
+      </c>
+      <c r="M849" t="inlineStr">
+        <is>
+          <t>Aucune permission propre à l'écran (voir « Discuter avec l'assistant (flux en direct) »)</t>
+        </is>
+      </c>
+      <c r="N849" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O849" t="inlineStr">
+        <is>
+          <t>Menu « Assistant » (zone Plus), bouton « Ouvrir en pleine page » du tiroir</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>Communication et Documents</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>Agence, Syndic, Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="D850" t="inlineStr">
+        <is>
+          <t>Assistant IA ImmoCopilot</t>
+        </is>
+      </c>
+      <c r="E850" t="inlineStr">
+        <is>
+          <t>Dicter un message à l'assistant</t>
+        </is>
+      </c>
+      <c r="F850" t="inlineStr">
+        <is>
+          <t>Bouton micro dans la zone de saisie (page et tiroir) : reconnaissance vocale du navigateur (Web Speech API, `SpeechRecognition` / `webkitSpeechRecognition`), dans la langue active de l'interface (fr-FR, en-US, ar). Le texte provisoire s'affiche dans la zone pendant la dictée, le texte définitif s'y insère ; jamais d'envoi automatique. État « Écoute en cours… » visible et libellé accessible ; refus de permission du micro ou autre erreur signalés par un message discret. Bouton masqué si le navigateur n'a pas l'API. Aucune donnée audio n'est envoyée à notre serveur (le navigateur peut utiliser son propre service de reconnaissance).</t>
+        </is>
+      </c>
+      <c r="G850" t="inlineStr">
+        <is>
+          <t>Voix de l'utilisateur (micro du navigateur)</t>
+        </is>
+      </c>
+      <c r="H850" t="inlineStr">
+        <is>
+          <t>Texte inséré dans la zone de saisie</t>
+        </is>
+      </c>
+      <c r="I850" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J850" t="inlineStr">
+        <is>
+          <t>Collaborateurs de l'agence ayant accès à l'assistant</t>
+        </is>
+      </c>
+      <c r="K850" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L850" t="inlineStr">
+        <is>
+          <t>Aucune (traitement dans le navigateur)</t>
+        </is>
+      </c>
+      <c r="M850" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="N850" t="inlineStr">
+        <is>
+          <t>Disponible (selon le navigateur ; Chrome et Edge, Safari partiel, Firefox sans prise en charge)</t>
+        </is>
+      </c>
+      <c r="O850" t="inlineStr">
+        <is>
+          <t>Zone de saisie de l'assistant (page et tiroir)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(copilot): panneau artefact — tableaux, textes, graphiques, téléchargement (étape 2 du plan v2)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NipnEzc6N8uvDDXG2M7jms
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -189,7 +189,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O850" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O853" headerRowCount="1">
   <autoFilter ref="A1:O848"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Domaine (regroupement agent)"/>
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O850"/>
+  <dimension ref="A1:O853"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -53899,7 +53899,7 @@
       </c>
       <c r="H691" s="2" t="inlineStr">
         <is>
-          <t>Flux `text/event-stream` : `meta`, `text_delta`, `tool_status`, `property_results`, `lease_results`, `document_list`, `action_proposal`, `error`, `done` (ping toutes les 15 s). Avant l'ouverture du flux : JSON typé (400 corps invalide, 403, 429 `RATE_LIMITED`, 503 `AI_DISABLED`)</t>
+          <t>Flux `text/event-stream` : `meta`, `text_delta`, `tool_status`, `property_results`, `lease_results`, `document_list`, `action_proposal`, `artifact`, `error`, `done` (ping toutes les 15 s). Avant l'ouverture du flux : JSON typé (400 corps invalide, 403, 429 `RATE_LIMITED`, 503 `AI_DISABLED`)</t>
         </is>
       </c>
       <c r="I691" s="2" t="inlineStr">
@@ -66010,7 +66010,7 @@
       </c>
       <c r="F849" t="inlineStr">
         <is>
-          <t>Page de chat plein écran (route `/tenant/:tenantId/assistant`, entrée de menu « Assistant ») : fil des messages défilant en haut, zone de saisie fixée en bas (Entrée envoie, Maj+Entrée saute une ligne, la zone grandit avec le texte), emplacement vide à droite réservé aux futurs artefacts (replié sous 992 px). Même conversation, mêmes cartes et mêmes limites que le tiroir (flux `POST /api/tenants/:tenantId/ai/chat`) ; la conversation reste en mémoire et n'est pas reprise entre le tiroir et la page. Si l'assistant est désactivé, la page l'indique et l'entrée de menu est masquée. Ctrl/Cmd+J ouvre toujours le tiroir.</t>
+          <t>Page de chat plein écran (route `/tenant/:tenantId/assistant`, entrée de menu « Assistant ») : fil des messages défilant en haut, zone de saisie fixée en bas (Entrée envoie, Maj+Entrée saute une ligne, la zone grandit avec le texte), panneau d'artefacts à droite (tableaux, textes, graphiques ; voir « Consulter un résultat dans le panneau d'artefacts »), en tiroir plein écran sous 992 px. Même conversation, mêmes cartes et mêmes limites que le tiroir (flux `POST /api/tenants/:tenantId/ai/chat`) ; la conversation reste en mémoire et n'est pas reprise entre le tiroir et la page. Si l'assistant est désactivé, la page l'indique et l'entrée de menu est masquée. Ctrl/Cmd+J ouvre toujours le tiroir.</t>
         </is>
       </c>
       <c r="G849" t="inlineStr">
@@ -66133,6 +66133,237 @@
       <c r="O850" t="inlineStr">
         <is>
           <t>Zone de saisie de l'assistant (page et tiroir)</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr">
+        <is>
+          <t>Communication et Documents</t>
+        </is>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>Agence, Syndic, Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="D851" t="inlineStr">
+        <is>
+          <t>Assistant IA ImmoCopilot</t>
+        </is>
+      </c>
+      <c r="E851" t="inlineStr">
+        <is>
+          <t>Consulter un résultat dans le panneau d'artefacts</t>
+        </is>
+      </c>
+      <c r="F851" t="inlineStr">
+        <is>
+          <t>Affiche à droite de la page Assistant (tiroir plein écran sous 992 px) les tableaux, textes et graphiques publiés par l'assistant. Le panneau apparaît seul à l'arrivée d'un artefact sur grand écran ; sous 992 px il s'ouvre quand on clique la pastille « Ouvrir : &lt;titre&gt; » du message ou le bouton « Résultats (n) ». Plusieurs artefacts : sélecteur dans l'en-tête, le dernier reçu est affiché ; bouton Fermer ; nouvelle conversation = panneau vidé. Tableau : tri par colonne, défilement horizontal et vertical, pagination de 50 lignes, nombres/devises/dates formatés selon la langue (alignement logique en arabe), mention « tronqué » ; texte : Markdown sûr (jamais de HTML) ; graphique (barres, courbes, secteurs) : titre, libellé accessible et tableau de données de repli, couleurs du thème. Défensif : tout artefact mal formé est ignoré, l'affichage est borné (500 lignes, 20 colonnes, 20 000 caractères, 200 points, 6 séries). Dans le tiroir, la pastille n'est pas cliquable (ouvrir la page pleine). Conversation en mémoire seulement.</t>
+        </is>
+      </c>
+      <c r="G851" t="inlineStr">
+        <is>
+          <t>Événement SSE `artifact` reçu pendant le flux (aucune saisie)</t>
+        </is>
+      </c>
+      <c r="H851" t="inlineStr">
+        <is>
+          <t>Panneau d'artefacts (tableau, texte ou graphique) et pastille de renvoi dans le message</t>
+        </is>
+      </c>
+      <c r="I851" t="inlineStr">
+        <is>
+          <t>Discuter avec l'assistant en pleine page</t>
+        </is>
+      </c>
+      <c r="J851" t="inlineStr">
+        <is>
+          <t>Collaborateurs de l'agence ayant accès à l'assistant</t>
+        </is>
+      </c>
+      <c r="K851" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L851" t="inlineStr">
+        <is>
+          <t>Aucune route nouvelle : écran web qui consomme l'événement `artifact` de `POST /api/tenants/:tenantId/ai/chat`</t>
+        </is>
+      </c>
+      <c r="M851" t="inlineStr">
+        <is>
+          <t>Aucune permission propre à l'écran</t>
+        </is>
+      </c>
+      <c r="N851" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O851" t="inlineStr">
+        <is>
+          <t>Page Assistant (menu « Assistant », zone Plus), panneau à droite</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr">
+        <is>
+          <t>Communication et Documents</t>
+        </is>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>Agence, Syndic, Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="D852" t="inlineStr">
+        <is>
+          <t>Assistant IA ImmoCopilot</t>
+        </is>
+      </c>
+      <c r="E852" t="inlineStr">
+        <is>
+          <t>Télécharger un artefact de l'assistant</t>
+        </is>
+      </c>
+      <c r="F852" t="inlineStr">
+        <is>
+          <t>Bouton « Télécharger » du panneau, entièrement côté navigateur à partir des données déjà reçues (aucun appel serveur) : tableau en CSV (UTF-8 avec BOM, séparateur « ; » en français et arabe, « , » en anglais) ou Excel .xlsx (exceljs, chargé à la demande) ; texte en .md ; graphique en image .png (SVG sérialisé vers canvas) ou CSV des données. Protection contre l'injection de formules : toute cellule texte (et tout en-tête) commençant par = + - @ tabulation ou retour chariot est préfixée d'une apostrophe dans le CSV et le XLSX. Noms de fichiers assainis à partir du titre.</t>
+        </is>
+      </c>
+      <c r="G852" t="inlineStr">
+        <is>
+          <t>Choix du format dans le menu Télécharger</t>
+        </is>
+      </c>
+      <c r="H852" t="inlineStr">
+        <is>
+          <t>Fichier .csv, .xlsx, .md ou .png enregistré par le navigateur</t>
+        </is>
+      </c>
+      <c r="I852" t="inlineStr">
+        <is>
+          <t>Consulter un résultat dans le panneau d'artefacts</t>
+        </is>
+      </c>
+      <c r="J852" t="inlineStr">
+        <is>
+          <t>Collaborateurs de l'agence ayant accès à l'assistant</t>
+        </is>
+      </c>
+      <c r="K852" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L852" t="inlineStr">
+        <is>
+          <t>Aucune (traitement dans le navigateur)</t>
+        </is>
+      </c>
+      <c r="M852" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="N852" t="inlineStr">
+        <is>
+          <t>Disponible (PNG : le rendu dépend du navigateur)</t>
+        </is>
+      </c>
+      <c r="O852" t="inlineStr">
+        <is>
+          <t>Page Assistant, panneau d'artefacts &gt; Télécharger</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr">
+        <is>
+          <t>Communication et Documents</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>Agence, Syndic, Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="D853" t="inlineStr">
+        <is>
+          <t>Assistant IA ImmoCopilot</t>
+        </is>
+      </c>
+      <c r="E853" t="inlineStr">
+        <is>
+          <t>Publier un tableau, un texte ou un graphique dans le panneau</t>
+        </is>
+      </c>
+      <c r="F853" t="inlineStr">
+        <is>
+          <t>Outil `show_artifact` (lecture seule) : le modèle publie dans le panneau latéral un tableau, un texte Markdown ou un graphique construit à partir de résultats d'outils déjà reçus. L'outil ne lit rien en base et n'élargit aucun accès ; l'identifiant de l'artefact est généré par le serveur, jamais par le modèle ; HTML refusé partout (titres, libellés, cellules, Markdown), tailles bornées (500 lignes, 20 colonnes, 20 000 caractères de Markdown, 200 points de graphique, 6 séries), lignes excédentaires tronquées (mention « tronqué »).</t>
+        </is>
+      </c>
+      <c r="G853" t="inlineStr">
+        <is>
+          <t>Type (`table`, `markdown`, `chart`), titre, colonnes/lignes, contenu ou série selon le type</t>
+        </is>
+      </c>
+      <c r="H853" t="inlineStr">
+        <is>
+          <t>Événement `artifact` {kind, id, title, …} dans le flux</t>
+        </is>
+      </c>
+      <c r="I853" t="inlineStr">
+        <is>
+          <t>Discuter avec l'assistant (flux en direct)</t>
+        </is>
+      </c>
+      <c r="J853" t="inlineStr">
+        <is>
+          <t>Collaborateurs de l'agence détenteurs de PROPERTIES_VIEW (socle des outils de lecture) ; refusé au super-admin et aux clients de portail</t>
+        </is>
+      </c>
+      <c r="K853" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L853" t="inlineStr">
+        <is>
+          <t>POST `/api/tenants/:tenantId/ai/chat` (outil `show_artifact`)</t>
+        </is>
+      </c>
+      <c r="M853" t="inlineStr">
+        <is>
+          <t>`PROPERTIES_VIEW` (outil `show_artifact`) + `authenticate` + `requireTenantAccess` + `requireTenantCollaborator` + `requireAiAssistantAccess`</t>
+        </is>
+      </c>
+      <c r="N853" t="inlineStr">
+        <is>
+          <t>Disponible (désactivé par défaut, AI_PROVIDER)</t>
+        </is>
+      </c>
+      <c r="O853" t="inlineStr">
+        <is>
+          <t>Page Assistant, panneau d'artefacts</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(copilot): passerelle générique en lecture — catalogue des routes et outils list_capabilities/call_read (étape 3 du plan v2)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NipnEzc6N8uvDDXG2M7jms
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -189,7 +189,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O853" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O855" headerRowCount="1">
   <autoFilter ref="A1:O848"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Domaine (regroupement agent)"/>
@@ -242,7 +242,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotesPointsOuverts" displayName="NotesPointsOuverts" ref="A1:D37" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotesPointsOuverts" displayName="NotesPointsOuverts" ref="A1:D38" headerRowCount="1">
   <autoFilter ref="A1:D37"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Domaine"/>
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O853"/>
+  <dimension ref="A1:O855"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -66364,6 +66364,160 @@
       <c r="O853" t="inlineStr">
         <is>
           <t>Page Assistant, panneau d'artefacts</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr">
+        <is>
+          <t>Communication et Documents</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>Agence, Syndic, Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="D854" t="inlineStr">
+        <is>
+          <t>Assistant IA ImmoCopilot</t>
+        </is>
+      </c>
+      <c r="E854" t="inlineStr">
+        <is>
+          <t>Chercher une consultation disponible dans l'application</t>
+        </is>
+      </c>
+      <c r="F854" t="inlineStr">
+        <is>
+          <t>Outil `list_capabilities` (lecture seule) : cherche dans le catalogue généré des routes GET d'agence (`packages/api/src/lib/ai/gateway/catalog.generated.json`, produit par `npm run ai:catalog` à partir de la pile Express réelle) celles que l'interface permet de consulter : par mots-clés et/ou module (finance, rental, crm, syndics, patrimoine…). Au plus 20 résultats (id, chemin, module, résumé, paramètres de chemin) ; sans argument, la liste des modules. Filtre selon les permissions connues de l'utilisateur quand le catalogue les connaît (sinon laisse passer : l'appel réel tranche). Les routes sensibles (chemin évoquant un secret, un jeton, une invitation, la passerelle de paiement) n'apparaissent jamais ; le catalogue ne contient ni route DELETE ni écriture destructrice (/delete /remove /destroy /purge). Un test (`ai.catalog.test.ts`) échoue tant que le catalogue commité diffère de la pile Express.</t>
+        </is>
+      </c>
+      <c r="G854" t="inlineStr">
+        <is>
+          <t>`query` (mots-clés) et/ou `module`, facultatifs</t>
+        </is>
+      </c>
+      <c r="H854" t="inlineStr">
+        <is>
+          <t>Événement `tool_status` ; résultat renvoyé au modèle seulement : {total, items[{id, path, module, summary, pathParams}]} ou liste des modules</t>
+        </is>
+      </c>
+      <c r="I854" t="inlineStr">
+        <is>
+          <t>Discuter avec l'assistant (flux en direct)</t>
+        </is>
+      </c>
+      <c r="J854" t="inlineStr">
+        <is>
+          <t>Collaborateurs de l'agence détenteurs de PROPERTIES_VIEW (socle des outils de lecture) ; refusé au super-admin et aux clients de portail</t>
+        </is>
+      </c>
+      <c r="K854" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L854" t="inlineStr">
+        <is>
+          <t>POST `/api/tenants/:tenantId/ai/chat` (outil `list_capabilities`)</t>
+        </is>
+      </c>
+      <c r="M854" t="inlineStr">
+        <is>
+          <t>`PROPERTIES_VIEW` (outil `list_capabilities`) + authenticate + requireTenantAccess + requireTenantCollaborator + requireAiAssistantAccess</t>
+        </is>
+      </c>
+      <c r="N854" t="inlineStr">
+        <is>
+          <t>Disponible (désactivé par défaut, AI_PROVIDER)</t>
+        </is>
+      </c>
+      <c r="O854" t="inlineStr">
+        <is>
+          <t>Page Assistant et tiroir (aucun écran propre)</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="inlineStr">
+        <is>
+          <t>Communication et Documents</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>Agence, Syndic, Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="D855" t="inlineStr">
+        <is>
+          <t>Assistant IA ImmoCopilot</t>
+        </is>
+      </c>
+      <c r="E855" t="inlineStr">
+        <is>
+          <t>Consulter une donnée de l'application (passerelle en lecture)</t>
+        </is>
+      </c>
+      <c r="F855" t="inlineStr">
+        <is>
+          <t>Outil `call_read` (lecture seule) : exécute une route GET du catalogue sous l'identité et les permissions de l'utilisateur, par une requête loopback de l'API vers elle-même (127.0.0.1 et PORT de la configuration, jamais une URL fournie par le modèle) qui rejoue l'authentification du chat. Toute la chaîne réelle s'applique (authentification, accès à l'agence, permission de la route, abonnement, garde Prisma, limiteurs) : le catalogue n'est qu'un index. N'accepte qu'un id GET non sensible du catalogue ; `:tenantId` imposé par le serveur, autres paramètres de chemin = UUID ou jeton simple, 20 clés de requête au plus. Délai 10 s, abandon avec le chat, JSON seulement (sinon « contenu non textuel, non affiché »), lecture plafonnée à 2 Mio. Avant retour au modèle : clés évoquant un secret (password, secret, token, apiKey, authorization, hash…) remplacées par « [masqué] » à toute profondeur (iban et rib restent visibles), tableaux &gt; 50 éléments, chaînes &gt; 500 caractères et profondeur &gt; 6 tronqués, total d'environ 12 000 caractères. Erreurs HTTP renvoyées sous la forme {status, message}, sans pile. Les routes d'écriture ne sont pas appelables à ce stade.</t>
+        </is>
+      </c>
+      <c r="G855" t="inlineStr">
+        <is>
+          <t>`capabilityId` (id renvoyé par `list_capabilities`), `pathParams` et `query` facultatifs</t>
+        </is>
+      </c>
+      <c r="H855" t="inlineStr">
+        <is>
+          <t>Résultat renvoyé au modèle : {ok, status, truncated?, data} ou {ok:false, status, message}</t>
+        </is>
+      </c>
+      <c r="I855" t="inlineStr">
+        <is>
+          <t>Chercher une consultation disponible dans l'application</t>
+        </is>
+      </c>
+      <c r="J855" t="inlineStr">
+        <is>
+          <t>Collaborateurs de l'agence détenteurs de PROPERTIES_VIEW (socle des outils de lecture) ; refusé au super-admin et aux clients de portail ; la route appelée applique en plus ses propres permissions</t>
+        </is>
+      </c>
+      <c r="K855" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L855" t="inlineStr">
+        <is>
+          <t>POST `/api/tenants/:tenantId/ai/chat` (outil `call_read`), qui appelle en loopback la route GET choisie</t>
+        </is>
+      </c>
+      <c r="M855" t="inlineStr">
+        <is>
+          <t>`PROPERTIES_VIEW` (outil `call_read`) + permissions de la route appelée (vérifiées par sa chaîne réelle) + authenticate + requireTenantAccess + requireTenantCollaborator + requireAiAssistantAccess</t>
+        </is>
+      </c>
+      <c r="N855" t="inlineStr">
+        <is>
+          <t>Disponible (désactivé par défaut, AI_PROVIDER)</t>
+        </is>
+      </c>
+      <c r="O855" t="inlineStr">
+        <is>
+          <t>Page Assistant et tiroir (aucun écran propre)</t>
         </is>
       </c>
     </row>
@@ -66969,7 +67123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -67792,6 +67946,28 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Communication et Documents</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Passerelle IA en lecture : catalogue sans schéma, outils réservés aux détenteurs de PROPERTIES_VIEW</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Le catalogue des consultations (list_capabilities, call_read) ne porte ni schéma de requête ni schéma de corps : le modèle découvre les filtres par essai. Les outils exigent PROPERTIES_VIEW (socle des outils de lecture) : un rôle sans cette permission, même s'il peut consulter d'autres écrans, ne reçoit pas la passerelle. Une route GET qui n'expose aucune permission lisible est proposée à tous, l'appel réel tranche.</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Étape 4 du plan ImmoCopilot v2 (écritures avec aperçu) : décider d'enrichir le catalogue (schémas Zod) et de lever la dépendance à PROPERTIES_VIEW.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
feat(copilot): écritures avec plan, avant/après et accord explicite (étape 4 du plan v2)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NipnEzc6N8uvDDXG2M7jms
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -189,7 +189,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O855" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O858" headerRowCount="1">
   <autoFilter ref="A1:O848"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Domaine (regroupement agent)"/>
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O855"/>
+  <dimension ref="A1:O858"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -53899,7 +53899,7 @@
       </c>
       <c r="H691" s="2" t="inlineStr">
         <is>
-          <t>Flux `text/event-stream` : `meta`, `text_delta`, `tool_status`, `property_results`, `lease_results`, `document_list`, `action_proposal`, `artifact`, `error`, `done` (ping toutes les 15 s). Avant l'ouverture du flux : JSON typé (400 corps invalide, 403, 429 `RATE_LIMITED`, 503 `AI_DISABLED`)</t>
+          <t>Flux `text/event-stream` : `meta`, `text_delta`, `tool_status`, `property_results`, `lease_results`, `document_list`, `action_proposal`, `write_plan`, `artifact`, `error`, `done` (ping toutes les 15 s). Avant l'ouverture du flux : JSON typé (400 corps invalide, 403, 429 `RATE_LIMITED`, 503 `AI_DISABLED`)</t>
         </is>
       </c>
       <c r="I691" s="2" t="inlineStr">
@@ -66518,6 +66518,237 @@
       <c r="O855" t="inlineStr">
         <is>
           <t>Page Assistant et tiroir (aucun écran propre)</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr">
+        <is>
+          <t>Communication et Documents</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>Agence, Syndic, Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="D856" t="inlineStr">
+        <is>
+          <t>Assistant IA ImmoCopilot</t>
+        </is>
+      </c>
+      <c r="E856" t="inlineStr">
+        <is>
+          <t>Valider un plan d'écriture proposé (carte d'accord)</t>
+        </is>
+      </c>
+      <c r="F856" t="inlineStr">
+        <is>
+          <t>Quand l'assistant veut modifier des données, la conversation affiche une carte d'accord et rien n'est modifié avant l'approbation. Bandeau « Action à valider — rien n'a encore été modifié » ; titre, type (Création, Modification, Action), module et méthode en langage clair ; section « Ce que l'assistant va faire » (étapes numérotées, étiquetée « Expliqué par l'assistant », texte brut) ; section « Données concernées » (étiquetée « Calculé par le serveur ») : enregistrement visé puis tableau Champ / Avant / Après (valeurs formatées selon la langue, valeurs longues repliables, « [masqué] » tel quel, mention « liste tronquée »), puis avertissements du serveur. Boutons « Approuver et exécuter » et « Refuser » ; décompte d'expiration, boutons désactivés à l'expiration ; verrou contre le double envoi. Après décision la carte est figée : statut, heure, message du serveur et aperçu replié du résultat en texte brut ; un échec (refus du serveur, jeton expiré ou déjà utilisé, erreur réseau) est expliqué. Même carte dans le tiroir et la page plein écran</t>
+        </is>
+      </c>
+      <c r="G856" t="inlineStr">
+        <is>
+          <t>Événement SSE `write_plan` (plan : jeton, expiration, route du catalogue, étapes, cible, changements avant/après, avertissements, indicateurs de sensibilité) ; clic sur Approuver : POST `{proposalToken, confirmation?}`</t>
+        </is>
+      </c>
+      <c r="H856" t="inlineStr">
+        <is>
+          <t>Carte figée : exécuté (message + aperçu du résultat), échec, refusé ou expiré ; réponse `{kind: 'capability', proposalId, ok, status, message, resultPreview}`</t>
+        </is>
+      </c>
+      <c r="I856" t="inlineStr">
+        <is>
+          <t>Discuter avec l'assistant (flux en direct)</t>
+        </is>
+      </c>
+      <c r="J856" t="inlineStr">
+        <is>
+          <t>Collaborateurs de l'agence ; l'exécution rejoue côté serveur les permissions de la route exécutée ; refusé au super-admin et aux clients de portail</t>
+        </is>
+      </c>
+      <c r="K856" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L856" t="inlineStr">
+        <is>
+          <t>POST `/api/tenants/:tenantId/ai/actions/execute`</t>
+        </is>
+      </c>
+      <c r="M856" t="inlineStr">
+        <is>
+          <t>`authenticate` + `requireTenantAccess` + `requireTenantCollaborator` + `requireAiAssistantAccess` ; permissions de la route du catalogue exécutée, revérifiées par le serveur au moment de l'approbation (détail côté API)</t>
+        </is>
+      </c>
+      <c r="N856" t="inlineStr">
+        <is>
+          <t>Disponible (désactivé par défaut, AI_PROVIDER)</t>
+        </is>
+      </c>
+      <c r="O856" t="inlineStr">
+        <is>
+          <t>Bouton flottant Assistant (Ctrl/Cmd+J), toutes pages d'agence ; page Assistant</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr">
+        <is>
+          <t>Communication et Documents</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>Agence, Syndic, Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="D857" t="inlineStr">
+        <is>
+          <t>Assistant IA ImmoCopilot</t>
+        </is>
+      </c>
+      <c r="E857" t="inlineStr">
+        <is>
+          <t>Confirmer un plan sensible par la saisie du mot CONFIRMER</t>
+        </is>
+      </c>
+      <c r="F857" t="inlineStr">
+        <is>
+          <t>Pour une route marquée sensible (effets de bord externes : paiements, envois d'e-mails ou de SMS, signatures), la carte d'accord s'affiche avec une alerte rouge qui donne la raison, et le bouton « Approuver et exécuter » reste désactivé tant que l'utilisateur n'a pas saisi exactement le mot CONFIRMER (respect de la casse) ; la touche Entrée dans ce champ n'approuve jamais. Le mot saisi est envoyé comme `confirmation` et revérifié par le serveur</t>
+        </is>
+      </c>
+      <c r="G857" t="inlineStr">
+        <is>
+          <t>Mot de confirmation saisi dans la carte ; POST `{proposalToken, confirmation}`</t>
+        </is>
+      </c>
+      <c r="H857" t="inlineStr">
+        <is>
+          <t>Même résultat que « Valider un plan d'écriture proposé » ; refus serveur si la confirmation est absente ou inexacte</t>
+        </is>
+      </c>
+      <c r="I857" t="inlineStr">
+        <is>
+          <t>Valider un plan d'écriture proposé (carte d'accord)</t>
+        </is>
+      </c>
+      <c r="J857" t="inlineStr">
+        <is>
+          <t>Collaborateurs de l'agence ; l'exécution rejoue côté serveur les permissions de la route exécutée ; refusé au super-admin et aux clients de portail</t>
+        </is>
+      </c>
+      <c r="K857" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L857" t="inlineStr">
+        <is>
+          <t>POST `/api/tenants/:tenantId/ai/actions/execute`</t>
+        </is>
+      </c>
+      <c r="M857" t="inlineStr">
+        <is>
+          <t>`authenticate` + `requireTenantAccess` + `requireTenantCollaborator` + `requireAiAssistantAccess` ; permissions de la route du catalogue exécutée, revérifiées par le serveur au moment de l'approbation (détail côté API)</t>
+        </is>
+      </c>
+      <c r="N857" t="inlineStr">
+        <is>
+          <t>Disponible (désactivé par défaut, AI_PROVIDER)</t>
+        </is>
+      </c>
+      <c r="O857" t="inlineStr">
+        <is>
+          <t>Bouton flottant Assistant (Ctrl/Cmd+J), toutes pages d'agence ; page Assistant</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr">
+        <is>
+          <t>Communication et Documents</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>Agence, Syndic, Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="D858" t="inlineStr">
+        <is>
+          <t>Assistant IA ImmoCopilot</t>
+        </is>
+      </c>
+      <c r="E858" t="inlineStr">
+        <is>
+          <t>Refuser un plan d'écriture</t>
+        </is>
+      </c>
+      <c r="F858" t="inlineStr">
+        <is>
+          <t>Bouton « Refuser » de la carte d'accord : la carte passe à « Action refusée — rien n'a été modifié », sans aucun appel au serveur (le jeton expire de lui-même) ; la conversation continue. L'assistant n'est pas informé automatiquement du refus : l'utilisateur peut le lui dire dans un message</t>
+        </is>
+      </c>
+      <c r="G858" t="inlineStr">
+        <is>
+          <t>Clic sur Refuser (aucune donnée envoyée)</t>
+        </is>
+      </c>
+      <c r="H858" t="inlineStr">
+        <is>
+          <t>Carte figée « Refusé » avec l'heure de la décision ; aucune écriture</t>
+        </is>
+      </c>
+      <c r="I858" t="inlineStr">
+        <is>
+          <t>Valider un plan d'écriture proposé (carte d'accord)</t>
+        </is>
+      </c>
+      <c r="J858" t="inlineStr">
+        <is>
+          <t>Collaborateurs de l'agence ; l'exécution rejoue côté serveur les permissions de la route exécutée ; refusé au super-admin et aux clients de portail</t>
+        </is>
+      </c>
+      <c r="K858" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L858" t="inlineStr">
+        <is>
+          <t>Aucune (action locale dans le navigateur)</t>
+        </is>
+      </c>
+      <c r="M858" t="inlineStr">
+        <is>
+          <t>Aucune (aucun appel serveur)</t>
+        </is>
+      </c>
+      <c r="N858" t="inlineStr">
+        <is>
+          <t>Disponible (désactivé par défaut, AI_PROVIDER)</t>
+        </is>
+      </c>
+      <c r="O858" t="inlineStr">
+        <is>
+          <t>Bouton flottant Assistant (Ctrl/Cmd+J), toutes pages d'agence ; page Assistant</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(copilot): correctifs de l'audit de sécurité — query, parent, sensibilité, listes remplacées, refus révocable
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NipnEzc6N8uvDDXG2M7jms
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -189,7 +189,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O858" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O860" headerRowCount="1">
   <autoFilter ref="A1:O848"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Domaine (regroupement agent)"/>
@@ -242,7 +242,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotesPointsOuverts" displayName="NotesPointsOuverts" ref="A1:D38" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotesPointsOuverts" displayName="NotesPointsOuverts" ref="A1:D39" headerRowCount="1">
   <autoFilter ref="A1:D37"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Domaine"/>
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O858"/>
+  <dimension ref="A1:O860"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -66472,7 +66472,7 @@
       </c>
       <c r="F855" t="inlineStr">
         <is>
-          <t>Outil `call_read` (lecture seule) : exécute une route GET du catalogue sous l'identité et les permissions de l'utilisateur, par une requête loopback de l'API vers elle-même (127.0.0.1 et PORT de la configuration, jamais une URL fournie par le modèle) qui rejoue l'authentification du chat. Toute la chaîne réelle s'applique (authentification, accès à l'agence, permission de la route, abonnement, garde Prisma, limiteurs) : le catalogue n'est qu'un index. N'accepte qu'un id GET non sensible du catalogue ; `:tenantId` imposé par le serveur, autres paramètres de chemin = UUID ou jeton simple, 20 clés de requête au plus. Délai 10 s, abandon avec le chat, JSON seulement (sinon « contenu non textuel, non affiché »), lecture plafonnée à 2 Mio. Avant retour au modèle : clés évoquant un secret (password, secret, token, apiKey, authorization, hash…) remplacées par « [masqué] » à toute profondeur (iban et rib restent visibles), tableaux &gt; 50 éléments, chaînes &gt; 500 caractères et profondeur &gt; 6 tronqués, total d'environ 12 000 caractères. Erreurs HTTP renvoyées sous la forme {status, message}, sans pile. Les routes d'écriture ne sont pas appelables à ce stade.</t>
+          <t>Outil `call_read` (lecture seule) : exécute une route GET du catalogue sous l'identité et les permissions de l'utilisateur, par une requête loopback de l'API vers elle-même (127.0.0.1 et PORT de la configuration, jamais une URL fournie par le modèle) qui rejoue l'authentification du chat. Toute la chaîne réelle s'applique (authentification, accès à l'agence, permission de la route, abonnement, garde Prisma, limiteurs) : le catalogue n'est qu'un index. N'accepte qu'un id GET non sensible du catalogue ; `:tenantId` imposé par le serveur, autres paramètres de chemin = UUID ou jeton simple, 20 clés de requête au plus. Délai 10 s, abandon avec le chat, JSON seulement (sinon « contenu non textuel, non affiché »), lecture plafonnée à 2 Mio. Avant retour au modèle : clés évoquant un secret (password, secret, token, apiKey, authorization, hash…) remplacées par « [masqué] » à toute profondeur (iban et rib restent visibles), tableaux &gt; 50 éléments, chaînes &gt; 500 caractères et profondeur &gt; 6 tronqués, total d'environ 12 000 caractères. Erreurs HTTP renvoyées sous la forme {status, message}, sans pile. Les routes d'écriture ne passent jamais par `call_read` : elles passent par `plan_write` puis un accord explicite.</t>
         </is>
       </c>
       <c r="G855" t="inlineStr">
@@ -66747,6 +66747,160 @@
         </is>
       </c>
       <c r="O858" t="inlineStr">
+        <is>
+          <t>Bouton flottant Assistant (Ctrl/Cmd+J), toutes pages d'agence ; page Assistant</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="inlineStr">
+        <is>
+          <t>Communication et Documents</t>
+        </is>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>Agence, Syndic, Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="D859" t="inlineStr">
+        <is>
+          <t>Assistant IA ImmoCopilot</t>
+        </is>
+      </c>
+      <c r="E859" t="inlineStr">
+        <is>
+          <t>Proposer une écriture à valider (plan d'écriture)</t>
+        </is>
+      </c>
+      <c r="F859" t="inlineStr">
+        <is>
+          <t>Outil `plan_write` : le modèle propose de modifier des données ; rien n'est écrit à ce stade. N'accepte qu'un id POST, PUT ou PATCH du catalogue (jamais DELETE, jamais une route destructive ni sensible-interdite) ; `:tenantId` imposé par le serveur. Le serveur LIT l'état actuel de l'enregistrement par un GET loopback et CALCULE lui-même les changements avant/après : le modèle ne fournit que le titre et les étapes. Clés évoquant un secret masquées (« [masqué] »). 30 changements affichés au plus : au-delà, liste tronquée et saisie obligatoire du mot CONFIRMER. Actions sensibles (paiement, remboursement, envoi, signature, validation ou clôture, droits et comptes, imports et opérations en masse) : confirmation tapée « CONFIRMER ». 3 plans au plus par requête de chat. Le plan est livré avec un jeton signé à usage unique, valable 900 s (AI_WRITE_PLAN_TTL_SECONDS) et lié à la requête approuvée (planHash)</t>
+        </is>
+      </c>
+      <c r="G859" t="inlineStr">
+        <is>
+          <t>`capabilityId` (id POST/PUT/PATCH du catalogue), `pathParams`, `query` et `body` facultatifs, titre et étapes en texte</t>
+        </is>
+      </c>
+      <c r="H859" t="inlineStr">
+        <is>
+          <t>Plan renvoyé au chat (événement `write_plan`) : jeton, expiration, route, étapes, cible, changements avant/après calculés par le serveur, avertissements, indicateurs de sensibilité ; aucune écriture</t>
+        </is>
+      </c>
+      <c r="I859" t="inlineStr">
+        <is>
+          <t>Chercher une consultation disponible dans l'application</t>
+        </is>
+      </c>
+      <c r="J859" t="inlineStr">
+        <is>
+          <t>Collaborateurs de l'agence détenteurs de PROPERTIES_VIEW (socle des outils) ; refusé au super-admin et aux clients de portail ; la route ciblée applique ses propres permissions à l'exécution</t>
+        </is>
+      </c>
+      <c r="K859" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L859" t="inlineStr">
+        <is>
+          <t>POST `/api/tenants/:tenantId/ai/chat` (outil `plan_write`)</t>
+        </is>
+      </c>
+      <c r="M859" t="inlineStr">
+        <is>
+          <t>`PROPERTIES_VIEW` (outil `plan_write`) + authenticate + requireTenantAccess + requireTenantCollaborator + requireAiAssistantAccess</t>
+        </is>
+      </c>
+      <c r="N859" t="inlineStr">
+        <is>
+          <t>Disponible (désactivé par défaut, AI_PROVIDER)</t>
+        </is>
+      </c>
+      <c r="O859" t="inlineStr">
+        <is>
+          <t>Page Assistant et tiroir (aucun écran propre)</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="inlineStr">
+        <is>
+          <t>Communication et Documents</t>
+        </is>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>Agence, Syndic, Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="D860" t="inlineStr">
+        <is>
+          <t>Assistant IA ImmoCopilot</t>
+        </is>
+      </c>
+      <c r="E860" t="inlineStr">
+        <is>
+          <t>Exécuter une écriture après accord explicite</t>
+        </is>
+      </c>
+      <c r="F860" t="inlineStr">
+        <is>
+          <t>Après clic sur « Approuver et exécuter » (et saisie de CONFIRMER si requis), le serveur vérifie la signature du jeton, son expiration, son usage unique, l'utilisateur et l'agence, puis exécute la route réelle par une requête loopback sous l'identité de la personne qui confirme : la permission et l'abonnement de la route réelle s'appliquent donc. Délai 30 s. Audit sans corps de requête ni secret. Réponse avec `resultPreview` masqué. 10 confirmations par minute. Rejeu d'un jeton : PROPOSAL_ALREADY_USED ; confirmation absente ou inexacte : CONFIRMATION_REQUIRED sans consommer le jeton. Aucune suppression possible. Module d'abonnement CORE : l'entrée `/ai/actions` ne dépend plus du module RENTAL (la génération de quittance vérifie toujours RENTAL)</t>
+        </is>
+      </c>
+      <c r="G860" t="inlineStr">
+        <is>
+          <t>`proposalToken` ; `confirmation` (« CONFIRMER ») si requis</t>
+        </is>
+      </c>
+      <c r="H860" t="inlineStr">
+        <is>
+          <t>`{kind: 'capability', proposalId, ok, status, message, resultPreview}` ; erreurs PROPOSAL_ALREADY_USED, CONFIRMATION_REQUIRED, jeton expiré ou invalide</t>
+        </is>
+      </c>
+      <c r="I860" t="inlineStr">
+        <is>
+          <t>Proposer une écriture à valider (plan d'écriture)</t>
+        </is>
+      </c>
+      <c r="J860" t="inlineStr">
+        <is>
+          <t>Collaborateurs de l'agence ; l'exécution rejoue côté serveur les permissions de la route exécutée ; refusé au super-admin et aux clients de portail</t>
+        </is>
+      </c>
+      <c r="K860" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L860" t="inlineStr">
+        <is>
+          <t>POST `/api/tenants/:tenantId/ai/actions/execute`</t>
+        </is>
+      </c>
+      <c r="M860" t="inlineStr">
+        <is>
+          <t>`authenticate` + `requireTenantAccess` + `requireTenantCollaborator` + `requireAiAssistantAccess` ; permissions de la route du catalogue exécutée, vérifiées par la chaîne réelle sous l'identité du confirmant</t>
+        </is>
+      </c>
+      <c r="N860" t="inlineStr">
+        <is>
+          <t>Disponible (désactivé par défaut, AI_PROVIDER)</t>
+        </is>
+      </c>
+      <c r="O860" t="inlineStr">
         <is>
           <t>Bouton flottant Assistant (Ctrl/Cmd+J), toutes pages d'agence ; page Assistant</t>
         </is>
@@ -67354,7 +67508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -68195,7 +68349,29 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Étape 4 du plan ImmoCopilot v2 (écritures avec aperçu) : décider d'enrichir le catalogue (schémas Zod) et de lever la dépendance à PROPERTIES_VIEW.</t>
+          <t>Étape 4 du plan ImmoCopilot v2 (écritures avec aperçu) livrée : plan_write puis exécution après accord. Reste à décider d'enrichir le catalogue (schémas Zod) et de lever la dépendance à PROPERTIES_VIEW.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Communication et Documents</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Écritures IA : limites</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Le catalogue ne porte aucun schéma de corps : le modèle devine les champs et c'est la route réelle qui valide. Certains POST sont en réalité des lectures (search, export) et passent par un plan d'écriture lourd. Les routes multipart (envoi de fichiers) ne sont pas gérées. Un échec après la réclamation du jeton consomme le plan : il faut en demander un nouveau. Les limiteurs (3 plans par requête de chat, 10 confirmations par minute) sont en mémoire, par instance.</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Décider d'ajouter des schémas de corps au catalogue, de distinguer les POST en lecture, et de passer les limiteurs sur un stockage partagé si l'API tourne sur plusieurs instances.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(wiki): refus de plan révocable, détail des plans d'écriture
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NipnEzc6N8uvDDXG2M7jms
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -189,7 +189,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O860" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O861" headerRowCount="1">
   <autoFilter ref="A1:O848"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Domaine (regroupement agent)"/>
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O860"/>
+  <dimension ref="A1:O861"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -66626,7 +66626,7 @@
       </c>
       <c r="F857" t="inlineStr">
         <is>
-          <t>Pour une route marquée sensible (effets de bord externes : paiements, envois d'e-mails ou de SMS, signatures), la carte d'accord s'affiche avec une alerte rouge qui donne la raison, et le bouton « Approuver et exécuter » reste désactivé tant que l'utilisateur n'a pas saisi exactement le mot CONFIRMER (respect de la casse) ; la touche Entrée dans ce champ n'approuve jamais. Le mot saisi est envoyé comme `confirmation` et revérifié par le serveur</t>
+          <t>Pour une route marquée sensible (effets de bord externes : paiements, envois d'e-mails ou de SMS, signatures), la carte d'accord s'affiche avec une alerte rouge qui donne la raison, et le bouton « Approuver et exécuter » reste désactivé tant que l'utilisateur n'a pas saisi exactement le mot CONFIRMER (respect de la casse) ; la touche Entrée dans ce champ n'approuve jamais. Le mot saisi est envoyé comme `confirmation` et revérifié par le serveur. La saisie est aussi exigée pour une requête non vide, une liste remplacée, plus de 30 changements et un corps touchant rôles/permissions/statut/mot de passe/e-mail d'un utilisateur (voir « Proposer une écriture à valider »)</t>
         </is>
       </c>
       <c r="G857" t="inlineStr">
@@ -66636,7 +66636,7 @@
       </c>
       <c r="H857" t="inlineStr">
         <is>
-          <t>Même résultat que « Valider un plan d'écriture proposé » ; refus serveur si la confirmation est absente ou inexacte</t>
+          <t>Même résultat que « Valider un plan d'écriture proposé » ; confirmation absente ou inexacte : CONFIRMATION_REQUIRED (400), carte en attente, jeton non consommé</t>
         </is>
       </c>
       <c r="I857" t="inlineStr">
@@ -66703,12 +66703,12 @@
       </c>
       <c r="F858" t="inlineStr">
         <is>
-          <t>Bouton « Refuser » de la carte d'accord : la carte passe à « Action refusée — rien n'a été modifié », sans aucun appel au serveur (le jeton expire de lui-même) ; la conversation continue. L'assistant n'est pas informé automatiquement du refus : l'utilisateur peut le lui dire dans un message</t>
+          <t>Bouton « Refuser » de la carte d'accord : la carte passe à « Action refusée — rien n'a été modifié » et la conversation continue ; en « meilleur effort », l'interface appelle aussi la route de révocation du jeton (voir « Refuser une écriture proposée (révocation du jeton) »), sans bloquer le refus si l'appel échoue. L'assistant n'est pas informé automatiquement du refus : l'utilisateur peut le lui dire dans un message</t>
         </is>
       </c>
       <c r="G858" t="inlineStr">
         <is>
-          <t>Clic sur Refuser (aucune donnée envoyée)</t>
+          <t>Clic sur Refuser ; POST `{proposalToken}` envoyé en meilleur effort</t>
         </is>
       </c>
       <c r="H858" t="inlineStr">
@@ -66733,12 +66733,12 @@
       </c>
       <c r="L858" t="inlineStr">
         <is>
-          <t>Aucune (action locale dans le navigateur)</t>
+          <t>POST `/api/tenants/:tenantId/ai/actions/reject` (meilleur effort ; l'état de la carte est local)</t>
         </is>
       </c>
       <c r="M858" t="inlineStr">
         <is>
-          <t>Aucune (aucun appel serveur)</t>
+          <t>Voir « Refuser une écriture proposée (révocation du jeton) »</t>
         </is>
       </c>
       <c r="N858" t="inlineStr">
@@ -66780,7 +66780,7 @@
       </c>
       <c r="F859" t="inlineStr">
         <is>
-          <t>Outil `plan_write` : le modèle propose de modifier des données ; rien n'est écrit à ce stade. N'accepte qu'un id POST, PUT ou PATCH du catalogue (jamais DELETE, jamais une route destructive ni sensible-interdite) ; `:tenantId` imposé par le serveur. Le serveur LIT l'état actuel de l'enregistrement par un GET loopback et CALCULE lui-même les changements avant/après : le modèle ne fournit que le titre et les étapes. Clés évoquant un secret masquées (« [masqué] »). 30 changements affichés au plus : au-delà, liste tronquée et saisie obligatoire du mot CONFIRMER. Actions sensibles (paiement, remboursement, envoi, signature, validation ou clôture, droits et comptes, imports et opérations en masse) : confirmation tapée « CONFIRMER ». 3 plans au plus par requête de chat. Le plan est livré avec un jeton signé à usage unique, valable 900 s (AI_WRITE_PLAN_TTL_SECONDS) et lié à la requête approuvée (planHash)</t>
+          <t>Outil `plan_write` : le modèle propose de modifier des données ; rien n'est écrit à ce stade. N'accepte qu'un id POST, PUT ou PATCH du catalogue (jamais DELETE, jamais une route destructive ni sensible-interdite) ; `:tenantId` imposé par le serveur. Le serveur LIT l'état actuel de l'enregistrement par un GET loopback et CALCULE lui-même les changements avant/après : le modèle ne fournit que le titre et les étapes. Clés évoquant un secret masquées (« [masqué] »). 30 changements affichés au plus : au-delà, liste tronquée et saisie obligatoire du mot CONFIRMER. Actions sensibles (paiement, remboursement, envoi, signature, validation ou clôture, droits et comptes, imports et opérations en masse) : confirmation tapée « CONFIRMER ». 3 plans au plus par requête de chat. Le plan est livré avec un jeton signé à usage unique, valable 900 s (AI_WRITE_PLAN_TTL_SECONDS) et lié à la requête approuvée (planHash). La carte d'accord montre aussi : les paramètres de requête envoyés à la route (« Paramètres envoyés à la route »), les identifiants du parent visé pour une création imbriquée (« Éléments visés », le serveur lisant lui-même le parent), l'heure de lecture de l'état « avant » (« État lu à HH:MM » : les données ont pu changer depuis), les listes remplacées (« Liste remplacée : N éléments retirés ») et les champs protégés (« [masqué] » avec avertissement). La saisie du mot CONFIRMER est exigée pour : les actions sensibles (paiements, envois, signature, droits d'accès et comptes, clôtures/verrouillages, fins de contrat, annulations, cessions, archivages, publication, abonnement), une requête non vide (paramètres de requête), une liste remplacée, plus de 30 changements, et un corps touchant rôles, permissions, statut, mot de passe ou e-mail d'un utilisateur</t>
         </is>
       </c>
       <c r="G859" t="inlineStr">
@@ -66790,7 +66790,7 @@
       </c>
       <c r="H859" t="inlineStr">
         <is>
-          <t>Plan renvoyé au chat (événement `write_plan`) : jeton, expiration, route, étapes, cible, changements avant/après calculés par le serveur, avertissements, indicateurs de sensibilité ; aucune écriture</t>
+          <t>Plan renvoyé au chat (événement `write_plan`) : jeton, expiration, route, étapes, cible, changements avant/après calculés par le serveur, avertissements, indicateurs de sensibilité ; aucune écriture ; la carte affiche aussi les paramètres de requête, les éléments visés du parent, l'heure de lecture de l'état « avant », les listes remplacées et les champs [masqué] avec leur avertissement</t>
         </is>
       </c>
       <c r="I859" t="inlineStr">
@@ -66857,7 +66857,7 @@
       </c>
       <c r="F860" t="inlineStr">
         <is>
-          <t>Après clic sur « Approuver et exécuter » (et saisie de CONFIRMER si requis), le serveur vérifie la signature du jeton, son expiration, son usage unique, l'utilisateur et l'agence, puis exécute la route réelle par une requête loopback sous l'identité de la personne qui confirme : la permission et l'abonnement de la route réelle s'appliquent donc. Délai 30 s. Audit sans corps de requête ni secret. Réponse avec `resultPreview` masqué. 10 confirmations par minute. Rejeu d'un jeton : PROPOSAL_ALREADY_USED ; confirmation absente ou inexacte : CONFIRMATION_REQUIRED sans consommer le jeton. Aucune suppression possible. Module d'abonnement CORE : l'entrée `/ai/actions` ne dépend plus du module RENTAL (la génération de quittance vérifie toujours RENTAL)</t>
+          <t>Après clic sur « Approuver et exécuter » (et saisie de CONFIRMER si requis), le serveur vérifie la signature du jeton, son expiration, son usage unique, l'utilisateur et l'agence, puis exécute la route réelle par une requête loopback sous l'identité de la personne qui confirme : la permission et l'abonnement de la route réelle s'appliquent donc. Délai 30 s. Audit sans corps de requête ni secret. Réponse avec `resultPreview` masqué. 10 confirmations par minute. Rejeu d'un jeton : PROPOSAL_ALREADY_USED ; confirmation absente ou inexacte : CONFIRMATION_REQUIRED sans consommer le jeton. Aucune suppression possible. Module d'abonnement CORE : l'entrée `/ai/actions` ne dépend plus du module RENTAL (la génération de quittance vérifie toujours RENTAL). Une confirmation sans le mot exigé répond CONFIRMATION_REQUIRED (400) : la carte reste en attente et le jeton n'est pas consommé. L'aperçu du résultat (`resultPreview`) masque les secrets et retire les chemins disque</t>
         </is>
       </c>
       <c r="G860" t="inlineStr">
@@ -66867,7 +66867,7 @@
       </c>
       <c r="H860" t="inlineStr">
         <is>
-          <t>`{kind: 'capability', proposalId, ok, status, message, resultPreview}` ; erreurs PROPOSAL_ALREADY_USED, CONFIRMATION_REQUIRED, jeton expiré ou invalide</t>
+          <t>`{kind: 'capability', proposalId, ok, status, message, resultPreview}` ; erreurs PROPOSAL_ALREADY_USED, CONFIRMATION_REQUIRED, jeton expiré ou invalide ; CONFIRMATION_REQUIRED (400) laisse la carte en attente sans consommer le jeton ; aperçu sans secrets ni chemins disque</t>
         </is>
       </c>
       <c r="I860" t="inlineStr">
@@ -66901,6 +66901,83 @@
         </is>
       </c>
       <c r="O860" t="inlineStr">
+        <is>
+          <t>Bouton flottant Assistant (Ctrl/Cmd+J), toutes pages d'agence ; page Assistant</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" t="inlineStr">
+        <is>
+          <t>Communication et Documents</t>
+        </is>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>Agence, Syndic, Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="D861" t="inlineStr">
+        <is>
+          <t>Assistant IA ImmoCopilot</t>
+        </is>
+      </c>
+      <c r="E861" t="inlineStr">
+        <is>
+          <t>Refuser une écriture proposée (révocation du jeton)</t>
+        </is>
+      </c>
+      <c r="F861" t="inlineStr">
+        <is>
+          <t>Au clic sur « Refuser », l'interface demande au serveur de révoquer le jeton du plan : le serveur vérifie la signature, l'utilisateur et l'agence, puis CONSOMME le jeton (usage unique) et audite AI_PROPOSAL_REJECTED ; le jeton ne peut plus être exécuté. Idempotent : jeton déjà utilisé ou expiré, réponse 200 `{rejected:false}`. Accessible même avec un abonnement en lecture seule (READ_LIKE_POSTS). Appel en « meilleur effort » : un échec réseau n'empêche pas la carte de passer à « Refusé »</t>
+        </is>
+      </c>
+      <c r="G861" t="inlineStr">
+        <is>
+          <t>`proposalToken`</t>
+        </is>
+      </c>
+      <c r="H861" t="inlineStr">
+        <is>
+          <t>`{rejected: true}` si le jeton a été révoqué, `{rejected: false}` (200) s'il était déjà utilisé ou expiré ; audit AI_PROPOSAL_REJECTED</t>
+        </is>
+      </c>
+      <c r="I861" t="inlineStr">
+        <is>
+          <t>Proposer une écriture à valider (plan d'écriture)</t>
+        </is>
+      </c>
+      <c r="J861" t="inlineStr">
+        <is>
+          <t>Collaborateurs de l'agence ; l'exécution rejoue côté serveur les permissions de la route exécutée ; refusé au super-admin et aux clients de portail</t>
+        </is>
+      </c>
+      <c r="K861" t="inlineStr">
+        <is>
+          <t>Agence (collaborateur)</t>
+        </is>
+      </c>
+      <c r="L861" t="inlineStr">
+        <is>
+          <t>POST `/api/tenants/:tenantId/ai/actions/reject`</t>
+        </is>
+      </c>
+      <c r="M861" t="inlineStr">
+        <is>
+          <t>`authenticate` + `requireTenantAccess` + `requireTenantCollaborator` + `requireAiAssistantAccess` ; accessible en abonnement lecture seule (READ_LIKE_POSTS)</t>
+        </is>
+      </c>
+      <c r="N861" t="inlineStr">
+        <is>
+          <t>Disponible (désactivé par défaut, AI_PROVIDER)</t>
+        </is>
+      </c>
+      <c r="O861" t="inlineStr">
         <is>
           <t>Bouton flottant Assistant (Ctrl/Cmd+J), toutes pages d'agence ; page Assistant</t>
         </is>

</xml_diff>

<commit_message>
fix(copilot): correctifs de la recette navigateur — mobile, PNG, tiroir, carte d'accord, quota de refus
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NipnEzc6N8uvDDXG2M7jms
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -53812,7 +53812,7 @@
       </c>
       <c r="F690" s="2" t="inlineStr">
         <is>
-          <t>Interroge l'assistant à l'ouverture de la coquille d'agence : indique s'il est activé et quels outils l'utilisateur peut employer (permissions RBAC et, en mode `enforce`, modules de l'abonnement). Le bouton flottant « Assistant » (raccourci Ctrl/Cmd+J) n'apparaît que si `enabled` est vrai ; toute erreur de statut le masque Le fournisseur et le modèle effectifs viennent du réglage plateforme (écran « Assistant IA » de l'administration) ou, à défaut, des variables AI_*. L'accueil du tiroir (message et suggestions) ne cite que les capacités des outils autorisés : sans gestion locative, ni baux ni quittances ne sont annoncés.</t>
+          <t>Interroge l'assistant à l'ouverture de la coquille d'agence : indique s'il est activé et quels outils l'utilisateur peut employer (permissions RBAC et, en mode `enforce`, modules de l'abonnement). Le bouton flottant « Assistant » (raccourci Ctrl/Cmd+J) n'apparaît que si `enabled` est vrai, et jamais sur la page plein écran Assistant ; toute erreur de statut le masque. La requête est partagée entre les composants montés ensemble (un seul appel par agence, réutilisé 5 s). La page Assistant distingue trois indisponibilités : désactivé pour l'agence, non disponible pour ce compte (HTTP 403, ex. super-admin) et aucune agence rattachée (404 ou identifiant absent) Le fournisseur et le modèle effectifs viennent du réglage plateforme (écran « Assistant IA » de l'administration) ou, à défaut, des variables AI_*. L'accueil du tiroir (message et suggestions) ne cite que les capacités des outils autorisés : sans gestion locative, ni baux ni quittances ne sont annoncés.</t>
         </is>
       </c>
       <c r="G690" s="2" t="inlineStr">
@@ -53889,7 +53889,7 @@
       </c>
       <c r="F691" s="2" t="inlineStr">
         <is>
-          <t>Ouvre le tiroir de conversation (côté « fin » : à droite en français, à gauche en arabe ; bouton « Ouvrir en pleine page » vers la page Assistant) et envoie l'échange au fournisseur LLM en flux SSE : texte progressif, cartes de résultats (biens, baux, documents, proposition), suggestions selon l'écran courant, arrêt de la réponse et nouvelle conversation. Conversation non persistée ; l'assistant n'écrit jamais lui-même. Limites : 20 messages, 4 000 caractères chacun, 24 000 au total ; 20 requêtes/min et 300/jour par utilisateur et par agence, plus un plafond par agence tous collaborateurs confondus (`AI_TENANT_MINUTE_LIMIT` 100/min, `AI_TENANT_DAILY_LIMIT` 3000/jour) ; limiteurs en mémoire, par instance d'API ; 4 tours et 8 appels d'outils maximum. L'invite système est construite par agence et ne cite que les capacités des outils exposés (permissions et modules souscrits) ; un appel d'outil d'un module non souscrit (modèle qui en invente un) est refusé poliment (résultat `MODULE_NOT_INCLUDED`, journal d'audit `AI_TOOL_DENIED`) et n'est jamais exécuté.</t>
+          <t>Ouvre le tiroir de conversation (côté « fin » : à droite en français, à gauche en arabe ; icône « Ouvrir en pleine page » (infobulle) vers la page Assistant ; les actions de l'en-tête sont des icônes seules, sans débordement à 375 px) et envoie l'échange au fournisseur LLM en flux SSE : texte progressif, cartes de résultats (biens, baux, documents, proposition), suggestions selon l'écran courant, arrêt de la réponse et nouvelle conversation. Conversation non persistée ; l'assistant n'écrit jamais lui-même. Limites : 20 messages, 4 000 caractères chacun, 24 000 au total ; 20 requêtes/min et 300/jour par utilisateur et par agence, plus un plafond par agence tous collaborateurs confondus (`AI_TENANT_MINUTE_LIMIT` 100/min, `AI_TENANT_DAILY_LIMIT` 3000/jour) ; limiteurs en mémoire, par instance d'API ; 4 tours et 8 appels d'outils maximum. L'invite système est construite par agence et ne cite que les capacités des outils exposés (permissions et modules souscrits) ; un appel d'outil d'un module non souscrit (modèle qui en invente un) est refusé poliment (résultat `MODULE_NOT_INCLUDED`, journal d'audit `AI_TOOL_DENIED`) et n'est jamais exécuté.</t>
         </is>
       </c>
       <c r="G691" s="2" t="inlineStr">
@@ -66010,7 +66010,7 @@
       </c>
       <c r="F849" t="inlineStr">
         <is>
-          <t>Page de chat plein écran (route `/tenant/:tenantId/assistant`, entrée de menu « Assistant ») : fil des messages défilant en haut, zone de saisie fixée en bas (Entrée envoie, Maj+Entrée saute une ligne, la zone grandit avec le texte), panneau d'artefacts à droite (tableaux, textes, graphiques ; voir « Consulter un résultat dans le panneau d'artefacts »), en tiroir plein écran sous 992 px. Même conversation, mêmes cartes et mêmes limites que le tiroir (flux `POST /api/tenants/:tenantId/ai/chat`) ; la conversation reste en mémoire et n'est pas reprise entre le tiroir et la page. Si l'assistant est désactivé, la page l'indique et l'entrée de menu est masquée. Ctrl/Cmd+J ouvre toujours le tiroir.</t>
+          <t>Page de chat plein écran (route `/tenant/:tenantId/assistant`, entrée de menu « Assistant ») : fil des messages défilant en haut, zone de saisie fixée en bas (Entrée envoie, Maj+Entrée saute une ligne, la zone grandit avec le texte), panneau d'artefacts à droite (tableaux, textes, graphiques ; voir « Consulter un résultat dans le panneau d'artefacts »), en tiroir plein écran sous 992 px. Même conversation, mêmes cartes et mêmes limites que le tiroir (flux `POST /api/tenants/:tenantId/ai/chat`) ; la conversation reste en mémoire et n'est pas reprise entre le tiroir et la page. Si l'assistant est désactivé, la page l'indique et l'entrée de menu est masquée. Sur cette page le bouton flottant est masqué et Ctrl/Cmd+J place le curseur dans la zone de saisie (aucun tiroir par-dessus). La page tient exactement dans la fenêtre sous 992 px (barre d'onglets comprise) : la ligne micro/Envoyer reste visible et cliquable. Si l'assistant est indisponible, le message dit pourquoi : désactivé pour l'agence, non disponible pour ce compte, ou aucune agence rattachée.</t>
         </is>
       </c>
       <c r="G849" t="inlineStr">
@@ -66055,7 +66055,7 @@
       </c>
       <c r="O849" t="inlineStr">
         <is>
-          <t>Menu « Assistant » (zone Plus), bouton « Ouvrir en pleine page » du tiroir</t>
+          <t>Menu « Assistant » (zone Plus), icône « Ouvrir en pleine page » du tiroir</t>
         </is>
       </c>
     </row>
@@ -66164,7 +66164,7 @@
       </c>
       <c r="F851" t="inlineStr">
         <is>
-          <t>Affiche à droite de la page Assistant (tiroir plein écran sous 992 px) les tableaux, textes et graphiques publiés par l'assistant. Le panneau apparaît seul à l'arrivée d'un artefact sur grand écran ; sous 992 px il s'ouvre quand on clique la pastille « Ouvrir : &lt;titre&gt; » du message ou le bouton « Résultats (n) ». Plusieurs artefacts : sélecteur dans l'en-tête, le dernier reçu est affiché ; bouton Fermer ; nouvelle conversation = panneau vidé. Tableau : tri par colonne, défilement horizontal et vertical, pagination de 50 lignes, nombres/devises/dates formatés selon la langue (alignement logique en arabe), mention « tronqué » ; texte : Markdown sûr (jamais de HTML) ; graphique (barres, courbes, secteurs) : titre, libellé accessible et tableau de données de repli, couleurs du thème. Défensif : tout artefact mal formé est ignoré, l'affichage est borné (500 lignes, 20 colonnes, 20 000 caractères, 200 points, 6 séries). Dans le tiroir, la pastille n'est pas cliquable (ouvrir la page pleine). Conversation en mémoire seulement.</t>
+          <t>Affiche à droite de la page Assistant (tiroir plein écran sous 992 px) les tableaux, textes et graphiques publiés par l'assistant. Le panneau apparaît seul à l'arrivée d'un artefact sur grand écran ; sous 992 px il s'ouvre quand on clique la pastille « Ouvrir : &lt;titre&gt; » du message ou le bouton « Résultats (n) ». Plusieurs artefacts : sélecteur dans l'en-tête, le dernier reçu est affiché ; bouton Fermer ; nouvelle conversation = panneau vidé. Tableau : tri par colonne, défilement horizontal et vertical, pagination de 50 lignes, nombres, dates et devises (0 décimale pour un entier, sinon 2) formatés selon la langue (alignement logique en arabe, valeurs isolées pour ne pas retourner « -5 Villa »), statuts et types connus (Disponible, Loué…) traduits, mention « tronqué » ; texte : Markdown sûr (titres # à ### en h3–h5, jamais de HTML) ; graphique (barres, courbes, secteurs) : titre, libellé accessible et tableau de données de repli, couleurs du thème. Défensif : tout artefact mal formé est ignoré, l'affichage est borné (500 lignes, 20 colonnes, 20 000 caractères, 200 points, 6 séries). Dans le tiroir, la pastille n'est pas cliquable (ouvrir la page pleine). Conversation en mémoire seulement.</t>
         </is>
       </c>
       <c r="G851" t="inlineStr">
@@ -66241,7 +66241,7 @@
       </c>
       <c r="F852" t="inlineStr">
         <is>
-          <t>Bouton « Télécharger » du panneau, entièrement côté navigateur à partir des données déjà reçues (aucun appel serveur) : tableau en CSV (UTF-8 avec BOM, séparateur « ; » en français et arabe, « , » en anglais) ou Excel .xlsx (exceljs, chargé à la demande) ; texte en .md ; graphique en image .png (SVG sérialisé vers canvas) ou CSV des données. Protection contre l'injection de formules : toute cellule texte (et tout en-tête) commençant par = + - @ tabulation ou retour chariot est préfixée d'une apostrophe dans le CSV et le XLSX. Noms de fichiers assainis à partir du titre.</t>
+          <t>Bouton « Télécharger » du panneau, entièrement côté navigateur à partir des données déjà reçues (aucun appel serveur) : tableau en CSV (UTF-8 avec BOM, séparateur « ; » en français et arabe, « , » en anglais) ou Excel .xlsx (exceljs, chargé à la demande) ; texte en .md ; graphique en image .png (SVG du graphe — jamais l'icône de la légende — sérialisé vers canvas à 2× la taille affichée, sur le fond du thème, polices et couleurs figées, légende redessinée sous le graphique) ou CSV des données. Protection contre l'injection de formules : toute cellule texte (et tout en-tête) commençant par = + - @ tabulation ou retour chariot est préfixée d'une apostrophe dans le CSV et le XLSX. Noms de fichiers assainis à partir du titre.</t>
         </is>
       </c>
       <c r="G852" t="inlineStr">
@@ -66549,7 +66549,7 @@
       </c>
       <c r="F856" t="inlineStr">
         <is>
-          <t>Quand l'assistant veut modifier des données, la conversation affiche une carte d'accord et rien n'est modifié avant l'approbation. Bandeau « Action à valider — rien n'a encore été modifié » ; titre, type (Création, Modification, Action), module et méthode en langage clair ; section « Ce que l'assistant va faire » (étapes numérotées, étiquetée « Expliqué par l'assistant », texte brut) ; section « Données concernées » (étiquetée « Calculé par le serveur ») : enregistrement visé puis tableau Champ / Avant / Après (valeurs formatées selon la langue, valeurs longues repliables, « [masqué] » tel quel, mention « liste tronquée »), puis avertissements du serveur. Boutons « Approuver et exécuter » et « Refuser » ; décompte d'expiration, boutons désactivés à l'expiration ; verrou contre le double envoi. Après décision la carte est figée : statut, heure, message du serveur et aperçu replié du résultat en texte brut ; un échec (refus du serveur, jeton expiré ou déjà utilisé, erreur réseau) est expliqué. Même carte dans le tiroir et la page plein écran</t>
+          <t>Quand l'assistant veut modifier des données, la conversation affiche une carte d'accord et rien n'est modifié avant l'approbation. Bandeau « Action à valider — rien n'a encore été modifié » ; titre, type (Création, Modification, Action), module et méthode en langage clair ; section « Ce que l'assistant va faire » (étapes numérotées, étiquetée « Expliqué par l'assistant », texte brut) ; section « Données concernées » (étiquetée « Calculé par le serveur ») : enregistrement visé (un identifiant brut est qualifié « Enregistrement (identifiant …) ») puis tableau Champ / Avant / Après (noms de champs rendus lisibles, nom technique en infobulle) (valeurs formatées selon la langue, valeurs longues repliables, « [masqué] » tel quel, mention « liste tronquée »), puis avertissements du serveur. Boutons « Approuver et exécuter » et « Refuser » ; décompte d'expiration, boutons désactivés à l'expiration ; verrou contre le double envoi. Après décision la carte est figée : statut, heure, message du serveur et aperçu replié du résultat en texte brut ; un échec (refus du serveur, jeton expiré ou déjà utilisé, erreur réseau) est expliqué. Même carte dans le tiroir et la page plein écran</t>
         </is>
       </c>
       <c r="G856" t="inlineStr">
@@ -67383,6 +67383,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat(web): régler les menus d'un rôle agence par agence
Onglet « Menus » de Rôles et permissions : pour un rôle d'agence ou de
portail, un sélecteur d'agence précède l'arbre ; rien n'est éditable avant
le choix, et l'enregistrement ne touche que l'agence choisie. Les rôles
plateforme se règlent sans agence. Confirmation avant de changer d'agence
avec des modifications non enregistrées.

Classeur des fonctionnalités mis à jour (routes menu-access et écran).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sous-fonctionnalites" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Legende Packs-Modules" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Notes et points ouverts" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sous-fonctionnalites" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legende Packs-Modules" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes et points ouverts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -39798,7 +39798,7 @@
       </c>
       <c r="F508" s="2" t="inlineStr">
         <is>
-          <t>Menus masqués pour l'utilisateur courant (et éventuellement une agence donnée) Renvoie aussi les permissions du compte, ce qui permet à la coquille de masquer les entrées Biens/Patrimoine (Sinistres, Régularisation foncière, Accès partagés) pour un rôle sans PROPERTIES_VIEW.</t>
+          <t>Menus masqués pour l'utilisateur courant dans l'agence demandée : seules les coupures posées pour CETTE agence s'appliquent (sans agence : coupures du périmètre plateforme). Renvoie aussi les permissions du compte, ce qui permet à la coquille de masquer les entrées Biens/Patrimoine (Sinistres, Régularisation foncière, Accès partagés) pour un rôle sans PROPERTIES_VIEW.</t>
         </is>
       </c>
       <c r="G508" s="2" t="inlineStr">
@@ -39870,29 +39870,29 @@
       </c>
       <c r="E509" s="2" t="inlineStr">
         <is>
-          <t>Consulter la carte des menus par rôle</t>
+          <t>Consulter la carte des menus par rôle et par agence</t>
         </is>
       </c>
       <c r="F509" s="2" t="inlineStr">
         <is>
-          <t>Vue d'ensemble : quels menus sont coupés pour quel rôle</t>
+          <t>Vue d'ensemble : quels menus sont coupés pour quel rôle, dans l'agence choisie (ou au niveau plateforme pour les rôles plateforme). Aucun héritage entre agences ni depuis la plateforme.</t>
         </is>
       </c>
       <c r="G509" s="2" t="inlineStr">
         <is>
+          <t>Query `tenantId?` (agence ; absent = périmètre plateforme)</t>
+        </is>
+      </c>
+      <c r="H509" s="2" t="inlineStr">
+        <is>
+          <t>Carte rôle → menus désactivés pour ce périmètre ; 404 si l’agence n’existe pas</t>
+        </is>
+      </c>
+      <c r="I509" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H509" s="2" t="inlineStr">
-        <is>
-          <t>Carte rôle → menus désactivés</t>
-        </is>
-      </c>
-      <c r="I509" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="J509" s="2" t="inlineStr">
         <is>
           <t>Super-admin</t>
@@ -39920,7 +39920,7 @@
       </c>
       <c r="O509" s="2" t="inlineStr">
         <is>
-          <t>Administration &gt; Rôles et permissions</t>
+          <t>Administration &gt; Rôles et permissions &gt; onglet Menus (sélecteur d’agence)</t>
         </is>
       </c>
     </row>
@@ -39952,22 +39952,22 @@
       </c>
       <c r="F510" s="2" t="inlineStr">
         <is>
-          <t>Définit quelles entrées de menu sont visibles pour un rôle (ou persona portail propriétaire/locataire)</t>
+          <t>Définit quelles entrées de menu sont visibles pour un rôle (ou persona portail propriétaire/locataire) dans UNE agence ; les autres agences ne sont pas touchées. L'écran demande de choisir l'agence avant d'afficher l'arbre des menus d'un rôle d'agence.</t>
         </is>
       </c>
       <c r="G510" s="2" t="inlineStr">
         <is>
-          <t>`roleKey` (ou pseudo-clé PORTAL_OWNER/PORTAL_RENTER), `menus: {menuKey: boolean}`</t>
+          <t>`roleKey` (ou pseudo-clé PORTAL_OWNER/PORTAL_RENTER), `menus: {menuKey: boolean}`, query `tenantId` obligatoire pour un rôle d’agence ou de portail, interdit pour un rôle plateforme</t>
         </is>
       </c>
       <c r="H510" s="2" t="inlineStr">
         <is>
-          <t>Décisions de menu mises à jour</t>
+          <t>Décisions de menu de ce rôle mises à jour pour ce périmètre seulement</t>
         </is>
       </c>
       <c r="I510" s="2" t="inlineStr">
         <is>
-          <t>Rôle (ou pseudo-rôle) existant</t>
+          <t>Rôle (ou pseudo-rôle) existant ; agence existante</t>
         </is>
       </c>
       <c r="J510" s="2" t="inlineStr">
@@ -39997,7 +39997,7 @@
       </c>
       <c r="O510" s="2" t="inlineStr">
         <is>
-          <t>Administration &gt; Rôles et permissions</t>
+          <t>Administration &gt; Rôles et permissions &gt; onglet Menus (sélecteur d’agence)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(copilot,users): garde-fous de désactivation, libellé de la cible, refus de lecture audité (recette passage 2)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NipnEzc6N8uvDDXG2M7jms
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -242,7 +242,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotesPointsOuverts" displayName="NotesPointsOuverts" ref="A1:D39" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotesPointsOuverts" displayName="NotesPointsOuverts" ref="A1:D40" headerRowCount="1">
   <autoFilter ref="A1:D37"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Domaine"/>
@@ -41492,7 +41492,7 @@
       </c>
       <c r="F530" s="2" t="inlineStr">
         <is>
-          <t>Change les rôles assignés à un membre</t>
+          <t>Change les rôles assignés à un membre. Retirer le rôle TENANT_ADMIN au dernier administrateur actif de l'agence est refusé (409).</t>
         </is>
       </c>
       <c r="G530" s="2" t="inlineStr">
@@ -41502,7 +41502,7 @@
       </c>
       <c r="H530" s="2" t="inlineStr">
         <is>
-          <t>Membre mis à jour</t>
+          <t>Membre mis à jour; erreur 409 si l'opération retirerait le rôle TENANT_ADMIN au dernier administrateur actif de l'agence</t>
         </is>
       </c>
       <c r="I530" s="2" t="inlineStr">
@@ -41569,7 +41569,7 @@
       </c>
       <c r="F531" s="2" t="inlineStr">
         <is>
-          <t>Coupe l'accès d'un membre à l'agence</t>
+          <t>Coupe l'accès d'un membre à l'agence. Refus 409 de l'auto-désactivation et de la désactivation du dernier administrateur actif de l'agence (membre actif portant TENANT_ADMIN) ; désactiver un membre déjà désactivé répond 409 (et non plus 400). Voir Notes « Dernier administrateur : course possible ».</t>
         </is>
       </c>
       <c r="G531" s="2" t="inlineStr">
@@ -41579,7 +41579,7 @@
       </c>
       <c r="H531" s="2" t="inlineStr">
         <is>
-          <t>Membership désactivé</t>
+          <t>Membership désactivé; erreur 409 si auto-désactivation, dernier administrateur actif ou membre déjà désactivé</t>
         </is>
       </c>
       <c r="I531" s="2" t="inlineStr">
@@ -66472,7 +66472,7 @@
       </c>
       <c r="F855" t="inlineStr">
         <is>
-          <t>Outil `call_read` (lecture seule) : exécute une route GET du catalogue sous l'identité et les permissions de l'utilisateur, par une requête loopback de l'API vers elle-même (127.0.0.1 et PORT de la configuration, jamais une URL fournie par le modèle) qui rejoue l'authentification du chat. Toute la chaîne réelle s'applique (authentification, accès à l'agence, permission de la route, abonnement, garde Prisma, limiteurs) : le catalogue n'est qu'un index. N'accepte qu'un id GET non sensible du catalogue ; `:tenantId` imposé par le serveur, autres paramètres de chemin = UUID ou jeton simple, 20 clés de requête au plus. Délai 10 s, abandon avec le chat, JSON seulement (sinon « contenu non textuel, non affiché »), lecture plafonnée à 2 Mio. Avant retour au modèle : clés évoquant un secret (password, secret, token, apiKey, authorization, hash…) remplacées par « [masqué] » à toute profondeur (iban et rib restent visibles), tableaux &gt; 50 éléments, chaînes &gt; 500 caractères et profondeur &gt; 6 tronqués, total d'environ 12 000 caractères. Erreurs HTTP renvoyées sous la forme {status, message}, sans pile. Les routes d'écriture ne passent jamais par `call_read` : elles passent par `plan_write` puis un accord explicite.</t>
+          <t>Outil `call_read` (lecture seule) : exécute une route GET du catalogue sous l'identité et les permissions de l'utilisateur, par une requête loopback de l'API vers elle-même (127.0.0.1 et PORT de la configuration, jamais une URL fournie par le modèle) qui rejoue l'authentification du chat. Toute la chaîne réelle s'applique (authentification, accès à l'agence, permission de la route, abonnement, garde Prisma, limiteurs) : le catalogue n'est qu'un index. N'accepte qu'un id GET non sensible du catalogue ; `:tenantId` imposé par le serveur, autres paramètres de chemin = UUID ou jeton simple, 20 clés de requête au plus. Délai 10 s, abandon avec le chat, JSON seulement (sinon « contenu non textuel, non affiché »), lecture plafonnée à 2 Mio. Avant retour au modèle : clés évoquant un secret (password, secret, token, apiKey, authorization, hash…) remplacées par « [masqué] » à toute profondeur (iban et rib restent visibles), tableaux &gt; 50 éléments, chaînes &gt; 500 caractères et profondeur &gt; 6 tronqués, total d'environ 12 000 caractères. Erreurs HTTP renvoyées sous la forme {status, message}, sans pile. Les routes d'écriture ne passent jamais par `call_read` : elles passent par `plan_write` puis un accord explicite. Un refus de permission (401/403) de la route réelle est traité comme un refus de l'assistant (statut d'outil « forbidden », audit AI_TOOL_DENIED), et non comme un résultat normal renvoyé au modèle.</t>
         </is>
       </c>
       <c r="G855" t="inlineStr">
@@ -66549,7 +66549,7 @@
       </c>
       <c r="F856" t="inlineStr">
         <is>
-          <t>Quand l'assistant veut modifier des données, la conversation affiche une carte d'accord et rien n'est modifié avant l'approbation. Bandeau « Action à valider — rien n'a encore été modifié » ; titre, type (Création, Modification, Action), module et méthode en langage clair ; section « Ce que l'assistant va faire » (étapes numérotées, étiquetée « Expliqué par l'assistant », texte brut) ; section « Données concernées » (étiquetée « Calculé par le serveur ») : enregistrement visé (un identifiant brut est qualifié « Enregistrement (identifiant …) ») puis tableau Champ / Avant / Après (noms de champs rendus lisibles, nom technique en infobulle) (valeurs formatées selon la langue, valeurs longues repliables, « [masqué] » tel quel, mention « liste tronquée »), puis avertissements du serveur. Boutons « Approuver et exécuter » et « Refuser » ; décompte d'expiration, boutons désactivés à l'expiration ; verrou contre le double envoi. Après décision la carte est figée : statut, heure, message du serveur et aperçu replié du résultat en texte brut ; un échec (refus du serveur, jeton expiré ou déjà utilisé, erreur réseau) est expliqué. Même carte dans le tiroir et la page plein écran</t>
+          <t>Quand l'assistant veut modifier des données, la conversation affiche une carte d'accord et rien n'est modifié avant l'approbation. Bandeau « Action à valider — rien n'a encore été modifié » ; titre, type (Création, Modification, Action), module et méthode en langage clair ; section « Ce que l'assistant va faire » (étapes numérotées, étiquetée « Expliqué par l'assistant », texte brut) ; section « Données concernées » (étiquetée « Calculé par le serveur ») : enregistrement visé (un identifiant brut est qualifié « Enregistrement (identifiant …) ») puis tableau Champ / Avant / Après (noms de champs rendus lisibles, nom technique en infobulle) (valeurs formatées selon la langue, valeurs longues repliables, « [masqué] » tel quel, mention « liste tronquée »), puis avertissements du serveur. Boutons « Approuver et exécuter » et « Refuser » ; décompte d'expiration, boutons désactivés à l'expiration ; verrou contre le double envoi. Après décision la carte est figée : statut, heure, message du serveur et aperçu replié du résultat en texte brut ; un échec (refus du serveur, jeton expiré ou déjà utilisé, erreur réseau) est expliqué. Même carte dans le tiroir et la page plein écran Pour une écriture sur un utilisateur (route `users/:id`), le serveur ajoute l'avertissement « Cette action modifie l'accès de &lt;nom&gt; » ; le libellé de la personne visée est lu dans la réponse de la route (prénom + nom, sinon e-mail).</t>
         </is>
       </c>
       <c r="G856" t="inlineStr">
@@ -66780,7 +66780,7 @@
       </c>
       <c r="F859" t="inlineStr">
         <is>
-          <t>Outil `plan_write` : le modèle propose de modifier des données ; rien n'est écrit à ce stade. N'accepte qu'un id POST, PUT ou PATCH du catalogue (jamais DELETE, jamais une route destructive ni sensible-interdite) ; `:tenantId` imposé par le serveur. Le serveur LIT l'état actuel de l'enregistrement par un GET loopback et CALCULE lui-même les changements avant/après : le modèle ne fournit que le titre et les étapes. Clés évoquant un secret masquées (« [masqué] »). 30 changements affichés au plus : au-delà, liste tronquée et saisie obligatoire du mot CONFIRMER. Actions sensibles (paiement, remboursement, envoi, signature, validation ou clôture, droits et comptes, imports et opérations en masse) : confirmation tapée « CONFIRMER ». 3 plans au plus par requête de chat. Le plan est livré avec un jeton signé à usage unique, valable 900 s (AI_WRITE_PLAN_TTL_SECONDS) et lié à la requête approuvée (planHash). La carte d'accord montre aussi : les paramètres de requête envoyés à la route (« Paramètres envoyés à la route »), les identifiants du parent visé pour une création imbriquée (« Éléments visés », le serveur lisant lui-même le parent), l'heure de lecture de l'état « avant » (« État lu à HH:MM » : les données ont pu changer depuis), les listes remplacées (« Liste remplacée : N éléments retirés ») et les champs protégés (« [masqué] » avec avertissement). La saisie du mot CONFIRMER est exigée pour : les actions sensibles (paiements, envois, signature, droits d'accès et comptes, clôtures/verrouillages, fins de contrat, annulations, cessions, archivages, publication, abonnement), une requête non vide (paramètres de requête), une liste remplacée, plus de 30 changements, et un corps touchant rôles, permissions, statut, mot de passe ou e-mail d'un utilisateur</t>
+          <t>Outil `plan_write` : le modèle propose de modifier des données ; rien n'est écrit à ce stade. N'accepte qu'un id POST, PUT ou PATCH du catalogue (jamais DELETE, jamais une route destructive ni sensible-interdite) ; `:tenantId` imposé par le serveur. Le serveur LIT l'état actuel de l'enregistrement par un GET loopback et CALCULE lui-même les changements avant/après : le modèle ne fournit que le titre et les étapes. Clés évoquant un secret masquées (« [masqué] »). 30 changements affichés au plus : au-delà, liste tronquée et saisie obligatoire du mot CONFIRMER. Actions sensibles (paiement, remboursement, envoi, signature, validation ou clôture, droits et comptes, imports et opérations en masse) : confirmation tapée « CONFIRMER ». 3 plans au plus par requête de chat. Le plan est livré avec un jeton signé à usage unique, valable 900 s (AI_WRITE_PLAN_TTL_SECONDS) et lié à la requête approuvée (planHash). La carte d'accord montre aussi : les paramètres de requête envoyés à la route (« Paramètres envoyés à la route »), les identifiants du parent visé pour une création imbriquée (« Éléments visés », le serveur lisant lui-même le parent), l'heure de lecture de l'état « avant » (« État lu à HH:MM » : les données ont pu changer depuis), les listes remplacées (« Liste remplacée : N éléments retirés ») et les champs protégés (« [masqué] » avec avertissement). La saisie du mot CONFIRMER est exigée pour : les actions sensibles (paiements, envois, signature, droits d'accès et comptes, clôtures/verrouillages, fins de contrat, annulations, cessions, archivages, publication, abonnement), une requête non vide (paramètres de requête), une liste remplacée, plus de 30 changements, et un corps touchant rôles, permissions, statut, mot de passe ou e-mail d'un utilisateur Pour une écriture sur un utilisateur (route `users/:id`), le serveur ajoute l'avertissement « Cette action modifie l'accès de &lt;nom&gt; » ; le libellé de la personne visée est lu dans la réponse de la route (prénom + nom, sinon e-mail).</t>
         </is>
       </c>
       <c r="G859" t="inlineStr">
@@ -67383,7 +67383,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
@@ -67586,7 +67585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -68453,6 +68452,28 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Administration plateforme</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Dernier administrateur : course possible</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Le contrôle du dernier administrateur actif (désactivation d'un membre, retrait du rôle TENANT_ADMIN) se fait avant la transaction, sans verrou : deux désactivations simultanées des deux seuls administrateurs pourraient théoriquement passer toutes les deux (voir SECURITY §13). Non couvert : désactivation de compte au niveau plateforme et suspension de l'agence.</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Confirmer si un verrou (ou un contrôle dans la transaction) est nécessaire ; décider si la désactivation de compte plateforme et la suspension de l'agence doivent aussi être protégées.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
docs(stock): mise en service Meta, spécification et wiki de l'inventaire WhatsApp
- DEPLOIEMENT.md : section « Lot 041 — Inventaire WhatsApp » (variables,
  refus de deploy.sh, staging en log + simulateur + fake, mise en service
  Meta pas à pas, retour arrière) et comptes de recette des chefs de chantier.
- Spécification : correctifs de relecture déjà codés (limiteur du webhook,
  messages de plus de 7 jours ignorés, activation HMAC et essai réservé,
  purges quel que soit le transport, plafond des appels à l'IA, simulateur
  filtré par agence).
- Wiki des fonctionnalités : 16 sous-fonctionnalités « Inventaire par
  WhatsApp » et trois lignes modifiées (906 lignes).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -189,7 +189,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O891" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SousFonctionnalites" displayName="SousFonctionnalites" ref="A1:O907" headerRowCount="1">
   <autoFilter ref="A1:O891"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Domaine (regroupement agent)"/>
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O891"/>
+  <dimension ref="A1:O907"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -20096,7 +20096,7 @@
       </c>
       <c r="H252" s="2" t="inlineStr">
         <is>
-          <t>Détail de l'inventaire ; attendus et écarts masqués tant que le comptage est en cours (sauf pour qui voit le stock du lieu), visibles après sa clôture</t>
+          <t>Détail de l'inventaire ; attendus et écarts masqués tant que le comptage est en cours (sauf pour qui voit le stock du lieu), visibles après sa clôture ; lot 041 : pastille « Ouvert par WhatsApp », badge « WhatsApp » et bouton photo sur les lignes comptées par le bot (captures lues à part, `GET …/whatsapp/counts/:countId/captures`, sans effet sur l'écran en cas de 403 ou 404)</t>
         </is>
       </c>
       <c r="I252" s="2" t="inlineStr">
@@ -22088,7 +22088,7 @@
       </c>
       <c r="F278" s="2" t="inlineStr">
         <is>
-          <t>Voir les faits au-dessus des seuils (écart, sortie ou rebut important, réception, achat en espèces, auto-validation)</t>
+          <t>Voir les faits au-dessus des seuils (écart, sortie ou rebut important, réception, achat en espèces, auto-validation, inventaire de chantier clos par WhatsApp)</t>
         </is>
       </c>
       <c r="G278" s="2" t="inlineStr">
@@ -44418,7 +44418,7 @@
       </c>
       <c r="F568" s="2" t="inlineStr">
         <is>
-          <t>Liste des packs/extensions/mises en route disponibles</t>
+          <t>Liste des packs/extensions/mises en route disponibles (dont l'option Inventaire WhatsApp EXT_INVENTAIRE_WHATSAPP : blocs de 500 photos analysées par mois, avec Promoteur ou Opérateur intégré, sans dépassement facturé)</t>
         </is>
       </c>
       <c r="G568" s="2" t="inlineStr">
@@ -69290,6 +69290,1238 @@
       <c r="O891" t="inlineStr">
         <is>
           <t>Bouton flottant Assistant (Ctrl/Cmd+J), toutes pages d'agence ; page Assistant</t>
+        </is>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>Promoteur, Opérateur intégré (option Inventaire WhatsApp, EXT_INVENTAIRE_WHATSAPP)</t>
+        </is>
+      </c>
+      <c r="C892" t="inlineStr">
+        <is>
+          <t>CONSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D892" t="inlineStr">
+        <is>
+          <t>Inventaire par WhatsApp</t>
+        </is>
+      </c>
+      <c r="E892" t="inlineStr">
+        <is>
+          <t>Inscrire un chef de chantier</t>
+        </is>
+      </c>
+      <c r="F892" t="inlineStr">
+        <is>
+          <t>Relier le numéro WhatsApp d'un Chef de chantier à ses chantiers et lui remettre un code d'activation</t>
+        </is>
+      </c>
+      <c r="G892" t="inlineStr">
+        <is>
+          <t>`userId` (membre actif détenteur du rôle Chef de chantier), `phone` (format ivoirien ou E.164), `siteIds` (1 à 10 chantiers ouverts et basculés au stock) ; listes d'aide `eligible-members` et `eligible-sites`</t>
+        </is>
+      </c>
+      <c r="H892" t="inlineStr">
+        <is>
+          <t>201 — inscription `PENDING_ACTIVATION` et code à 6 chiffres affiché une seule fois (valable 72 heures, 5 essais), numéro du bot ; code stocké en empreinte HMAC à clé serveur. 409 si le membre n'est pas éligible, déjà inscrit, ou si le numéro est déjà inscrit (sur toute la plateforme, refus neutre) ; 404 pour un chantier d'une autre agence</t>
+        </is>
+      </c>
+      <c r="I892" t="inlineStr">
+        <is>
+          <t>Attribuer le rôle Chef de chantier ; Basculer un chantier au stock</t>
+        </is>
+      </c>
+      <c r="J892" t="inlineStr">
+        <is>
+          <t>TENANT_ADMIN (droit de paramétrer la finance)</t>
+        </is>
+      </c>
+      <c r="K892" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L892" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/finance/stock/whatsapp/registrations ; GET /tenants/:tenantId/finance/stock/whatsapp/eligible-members ; GET /tenants/:tenantId/finance/stock/whatsapp/eligible-sites</t>
+        </is>
+      </c>
+      <c r="M892" t="inlineStr">
+        <is>
+          <t>FINANCE_SETTINGS_MANAGE</t>
+        </is>
+      </c>
+      <c r="N892" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O892" t="inlineStr">
+        <is>
+          <t>Finance &gt; Chantiers et stock &gt; Gestion du stock &gt; WhatsApp &gt; Chefs de chantier — bouton « Inscrire un chef de chantier »</t>
+        </is>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>Promoteur, Opérateur intégré (option Inventaire WhatsApp, EXT_INVENTAIRE_WHATSAPP)</t>
+        </is>
+      </c>
+      <c r="C893" t="inlineStr">
+        <is>
+          <t>CONSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D893" t="inlineStr">
+        <is>
+          <t>Inventaire par WhatsApp</t>
+        </is>
+      </c>
+      <c r="E893" t="inlineStr">
+        <is>
+          <t>Lister les chefs de chantier inscrits</t>
+        </is>
+      </c>
+      <c r="F893" t="inlineStr">
+        <is>
+          <t>Voir qui peut compter par WhatsApp, l'état de chaque inscription et de son accès</t>
+        </is>
+      </c>
+      <c r="G893" t="inlineStr">
+        <is>
+          <t>Aucune saisie ; détail par `registrationId`</t>
+        </is>
+      </c>
+      <c r="H893" t="inlineStr">
+        <is>
+          <t>Inscriptions (membre, numéro masqué, chantiers et leur éligibilité, statut, accès relu en base : rôle retiré, adhésion inactive, option absente…, dernier message)</t>
+        </is>
+      </c>
+      <c r="I893" t="inlineStr">
+        <is>
+          <t>Inscrire un chef de chantier</t>
+        </is>
+      </c>
+      <c r="J893" t="inlineStr">
+        <is>
+          <t>TENANT_ADMIN (droit de paramétrer la finance)</t>
+        </is>
+      </c>
+      <c r="K893" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L893" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/finance/stock/whatsapp/registrations ; GET /tenants/:tenantId/finance/stock/whatsapp/registrations/:registrationId</t>
+        </is>
+      </c>
+      <c r="M893" t="inlineStr">
+        <is>
+          <t>FINANCE_SETTINGS_MANAGE</t>
+        </is>
+      </c>
+      <c r="N893" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O893" t="inlineStr">
+        <is>
+          <t>Finance &gt; Chantiers et stock &gt; Gestion du stock &gt; WhatsApp &gt; Chefs de chantier</t>
+        </is>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>Promoteur, Opérateur intégré (option Inventaire WhatsApp, EXT_INVENTAIRE_WHATSAPP)</t>
+        </is>
+      </c>
+      <c r="C894" t="inlineStr">
+        <is>
+          <t>CONSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D894" t="inlineStr">
+        <is>
+          <t>Inventaire par WhatsApp</t>
+        </is>
+      </c>
+      <c r="E894" t="inlineStr">
+        <is>
+          <t>Modifier les chantiers d'un chef inscrit</t>
+        </is>
+      </c>
+      <c r="F894" t="inlineStr">
+        <is>
+          <t>Changer les chantiers sur lesquels un chef compte</t>
+        </is>
+      </c>
+      <c r="G894" t="inlineStr">
+        <is>
+          <t>Chemin `registrationId`, `siteIds` (1 à 10, chacun de l'agence, ouvert et basculé au stock)</t>
+        </is>
+      </c>
+      <c r="H894" t="inlineStr">
+        <is>
+          <t>Inscription mise à jour ; 409 `STOCK_WHATSAPP_SITE_NOT_ELIGIBLE` (avec `data.siteIds`) pour un chantier non éligible</t>
+        </is>
+      </c>
+      <c r="I894" t="inlineStr">
+        <is>
+          <t>Inscrire un chef de chantier</t>
+        </is>
+      </c>
+      <c r="J894" t="inlineStr">
+        <is>
+          <t>TENANT_ADMIN (droit de paramétrer la finance)</t>
+        </is>
+      </c>
+      <c r="K894" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L894" t="inlineStr">
+        <is>
+          <t>PATCH /tenants/:tenantId/finance/stock/whatsapp/registrations/:registrationId</t>
+        </is>
+      </c>
+      <c r="M894" t="inlineStr">
+        <is>
+          <t>FINANCE_SETTINGS_MANAGE</t>
+        </is>
+      </c>
+      <c r="N894" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O894" t="inlineStr">
+        <is>
+          <t>Finance &gt; Chantiers et stock &gt; Gestion du stock &gt; WhatsApp &gt; Chefs de chantier — action « Modifier les chantiers »</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>Promoteur, Opérateur intégré (option Inventaire WhatsApp, EXT_INVENTAIRE_WHATSAPP)</t>
+        </is>
+      </c>
+      <c r="C895" t="inlineStr">
+        <is>
+          <t>CONSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D895" t="inlineStr">
+        <is>
+          <t>Inventaire par WhatsApp</t>
+        </is>
+      </c>
+      <c r="E895" t="inlineStr">
+        <is>
+          <t>Régénérer le code d'activation</t>
+        </is>
+      </c>
+      <c r="F895" t="inlineStr">
+        <is>
+          <t>Remettre un nouveau code à un chef qui l'a perdu ou bloqué</t>
+        </is>
+      </c>
+      <c r="G895" t="inlineStr">
+        <is>
+          <t>Chemin `registrationId` (inscription en attente d'activation)</t>
+        </is>
+      </c>
+      <c r="H895" t="inlineStr">
+        <is>
+          <t>Nouveau code affiché une fois ; essais remis à zéro, ancien code invalidé ; 409 si l'inscription n'est pas en attente</t>
+        </is>
+      </c>
+      <c r="I895" t="inlineStr">
+        <is>
+          <t>Inscrire un chef de chantier</t>
+        </is>
+      </c>
+      <c r="J895" t="inlineStr">
+        <is>
+          <t>TENANT_ADMIN (droit de paramétrer la finance)</t>
+        </is>
+      </c>
+      <c r="K895" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L895" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/finance/stock/whatsapp/registrations/:registrationId/regenerate-code</t>
+        </is>
+      </c>
+      <c r="M895" t="inlineStr">
+        <is>
+          <t>FINANCE_SETTINGS_MANAGE</t>
+        </is>
+      </c>
+      <c r="N895" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O895" t="inlineStr">
+        <is>
+          <t>Finance &gt; Chantiers et stock &gt; Gestion du stock &gt; WhatsApp &gt; Chefs de chantier — action « Régénérer le code »</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>Promoteur, Opérateur intégré (option Inventaire WhatsApp, EXT_INVENTAIRE_WHATSAPP)</t>
+        </is>
+      </c>
+      <c r="C896" t="inlineStr">
+        <is>
+          <t>CONSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D896" t="inlineStr">
+        <is>
+          <t>Inventaire par WhatsApp</t>
+        </is>
+      </c>
+      <c r="E896" t="inlineStr">
+        <is>
+          <t>Révoquer un chef de chantier</t>
+        </is>
+      </c>
+      <c r="F896" t="inlineStr">
+        <is>
+          <t>Retirer à un chef l'accès à l'inventaire par WhatsApp</t>
+        </is>
+      </c>
+      <c r="G896" t="inlineStr">
+        <is>
+          <t>Chemin `registrationId`, `reason?` (500 caractères au plus)</t>
+        </is>
+      </c>
+      <c r="H896" t="inlineStr">
+        <is>
+          <t>Inscription `REVOKED`, session ouverte fermée, proposition en attente abandonnée ; le bot refuse ses messages suivants (M06) ; numéro de nouveau inscriptible</t>
+        </is>
+      </c>
+      <c r="I896" t="inlineStr">
+        <is>
+          <t>Inscrire un chef de chantier</t>
+        </is>
+      </c>
+      <c r="J896" t="inlineStr">
+        <is>
+          <t>TENANT_ADMIN (droit de paramétrer la finance)</t>
+        </is>
+      </c>
+      <c r="K896" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L896" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/finance/stock/whatsapp/registrations/:registrationId/revoke</t>
+        </is>
+      </c>
+      <c r="M896" t="inlineStr">
+        <is>
+          <t>FINANCE_SETTINGS_MANAGE</t>
+        </is>
+      </c>
+      <c r="N896" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O896" t="inlineStr">
+        <is>
+          <t>Finance &gt; Chantiers et stock &gt; Gestion du stock &gt; WhatsApp &gt; Chefs de chantier — action « Révoquer »</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>Promoteur, Opérateur intégré (option Inventaire WhatsApp, EXT_INVENTAIRE_WHATSAPP)</t>
+        </is>
+      </c>
+      <c r="C897" t="inlineStr">
+        <is>
+          <t>CONSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D897" t="inlineStr">
+        <is>
+          <t>Inventaire par WhatsApp</t>
+        </is>
+      </c>
+      <c r="E897" t="inlineStr">
+        <is>
+          <t>Activer son inscription par le code</t>
+        </is>
+      </c>
+      <c r="F897" t="inlineStr">
+        <is>
+          <t>Prouver au bot qu'on utilise bien le numéro inscrit, et consentir à recevoir ses réponses</t>
+        </is>
+      </c>
+      <c r="G897" t="inlineStr">
+        <is>
+          <t>Message WhatsApp dont les seuls chiffres forment le code (« 482 913 »), depuis le numéro inscrit</t>
+        </is>
+      </c>
+      <c r="H897" t="inlineStr">
+        <is>
+          <t>Inscription `ACTIVE` et message de bienvenue (M02) ; sinon « Code incorrect, il vous reste n essai(s) » (M03), blocage au 5e échec ou après 72 heures (M04). Essai réservé avant toute comparaison ; message journalisé sans son texte</t>
+        </is>
+      </c>
+      <c r="I897" t="inlineStr">
+        <is>
+          <t>Inscrire un chef de chantier</t>
+        </is>
+      </c>
+      <c r="J897" t="inlineStr">
+        <is>
+          <t>TENANT_SITE_MANAGER (Chef de chantier inscrit)</t>
+        </is>
+      </c>
+      <c r="K897" t="inlineStr">
+        <is>
+          <t>WhatsApp (bot)</t>
+        </is>
+      </c>
+      <c r="L897" t="inlineStr">
+        <is>
+          <t>POST /api/webhooks/whatsapp-cloud/events (Meta) ou POST /tenants/:tenantId/finance/stock/whatsapp/simulator/messages (recette)</t>
+        </is>
+      </c>
+      <c r="M897" t="inlineStr">
+        <is>
+          <t>— (signature X-Hub-Signature-256)</t>
+        </is>
+      </c>
+      <c r="N897" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O897" t="inlineStr">
+        <is>
+          <t>Hors application : conversation WhatsApp avec le numéro du bot</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>Promoteur, Opérateur intégré (option Inventaire WhatsApp, EXT_INVENTAIRE_WHATSAPP)</t>
+        </is>
+      </c>
+      <c r="C898" t="inlineStr">
+        <is>
+          <t>CONSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D898" t="inlineStr">
+        <is>
+          <t>Inventaire par WhatsApp</t>
+        </is>
+      </c>
+      <c r="E898" t="inlineStr">
+        <is>
+          <t>Compter le stock par photo WhatsApp</t>
+        </is>
+      </c>
+      <c r="F898" t="inlineStr">
+        <is>
+          <t>Compter un article de son chantier en envoyant sa photo, sans voir le stock attendu</t>
+        </is>
+      </c>
+      <c r="G898" t="inlineStr">
+        <is>
+          <t>Photo (JPEG, PNG ou WebP, 10 Mo au plus, une à la fois) ; réponse « 1 » (valider), le nombre exact, ou « 0 » (annuler) ; « 1 / 2 / 0 » pour ajouter, remplacer ou annuler quand l'article est déjà compté ; commandes FIN, CHANTIER, AIDE</t>
+        </is>
+      </c>
+      <c r="H898" t="inlineStr">
+        <is>
+          <t>Ligne écrite dans l'inventaire `DRAFT` du lieu (ouvert par le bot au besoin, source WHATSAPP), comptée par le chef, à l'aveugle ; FIN clôt l'inventaire ouvert par le bot (lignes « non comptées » créées, alerte « Inventaire de chantier clos par WhatsApp ») ou le laisse ouvert s'il vient du bureau. Photo et empreinte gardées comme preuve. Aucun mouvement, aucune validation par WhatsApp</t>
+        </is>
+      </c>
+      <c r="I898" t="inlineStr">
+        <is>
+          <t>Activer son inscription par le code ; Ouvrir un inventaire physique</t>
+        </is>
+      </c>
+      <c r="J898" t="inlineStr">
+        <is>
+          <t>TENANT_SITE_MANAGER (Chef de chantier inscrit, actif, rôle relu en base à chaque message)</t>
+        </is>
+      </c>
+      <c r="K898" t="inlineStr">
+        <is>
+          <t>WhatsApp (bot)</t>
+        </is>
+      </c>
+      <c r="L898" t="inlineStr">
+        <is>
+          <t>POST /api/webhooks/whatsapp-cloud/events (Meta) ou POST /tenants/:tenantId/finance/stock/whatsapp/simulator/messages (recette)</t>
+        </is>
+      </c>
+      <c r="M898" t="inlineStr">
+        <is>
+          <t>STOCK_COUNT (rôle Chef de chantier) ; option d'abonnement en `enforce`</t>
+        </is>
+      </c>
+      <c r="N898" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O898" t="inlineStr">
+        <is>
+          <t>Hors application : conversation WhatsApp avec le numéro du bot</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>Promoteur, Opérateur intégré (option Inventaire WhatsApp, EXT_INVENTAIRE_WHATSAPP)</t>
+        </is>
+      </c>
+      <c r="C899" t="inlineStr">
+        <is>
+          <t>CONSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D899" t="inlineStr">
+        <is>
+          <t>Inventaire par WhatsApp</t>
+        </is>
+      </c>
+      <c r="E899" t="inlineStr">
+        <is>
+          <t>Analyser une photo de stock par l'IA</t>
+        </is>
+      </c>
+      <c r="F899" t="inlineStr">
+        <is>
+          <t>Proposer au chef un article et un total à partir de la photo</t>
+        </is>
+      </c>
+      <c r="G899" t="inlineStr">
+        <is>
+          <t>Photo stockée (EXIF retiré), 300 articles candidats au plus (référence, libellé, unité, famille ; jamais de solde), article imposé par le chef le cas échéant</t>
+        </is>
+      </c>
+      <c r="H899" t="inlineStr">
+        <is>
+          <t>Proposition (article, méthode : sacs empilés, fagot, palette, autre ; détail du comptage, total arrondi à 4 décimales, confiance ; phrase de prudence sous 0,7) ou refus : photo trop sombre ou floue (M18), sans matériau (M18b), article non reconnu (M19, le chef tape son nom), échec ou délai (M22, photo conservée). Quota réservé avant l'appel et rendu en cas d'échec ; plafond des appels (5 échecs par heure et par chef, deux fois le quota par mois)</t>
+        </is>
+      </c>
+      <c r="I899" t="inlineStr">
+        <is>
+          <t>Compter le stock par photo WhatsApp</t>
+        </is>
+      </c>
+      <c r="J899" t="inlineStr">
+        <is>
+          <t>Système (fournisseur de vision : Gemini, OpenRouter ; faux fournisseur en recette)</t>
+        </is>
+      </c>
+      <c r="K899" t="inlineStr">
+        <is>
+          <t>WhatsApp (bot)</t>
+        </is>
+      </c>
+      <c r="L899" t="inlineStr">
+        <is>
+          <t>— (appel interne, aucune route)</t>
+        </is>
+      </c>
+      <c r="M899" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N899" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O899" t="inlineStr">
+        <is>
+          <t>Hors application ; réglages visibles dans Finance &gt; Chantiers et stock &gt; Gestion du stock &gt; WhatsApp (passerelle)</t>
+        </is>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>Promoteur, Opérateur intégré (option Inventaire WhatsApp, EXT_INVENTAIRE_WHATSAPP)</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>CONSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D900" t="inlineStr">
+        <is>
+          <t>Inventaire par WhatsApp</t>
+        </is>
+      </c>
+      <c r="E900" t="inlineStr">
+        <is>
+          <t>Consulter les comptages terrain</t>
+        </is>
+      </c>
+      <c r="F900" t="inlineStr">
+        <is>
+          <t>Rapprocher, par lieu et par article, le stock théorique et le dernier comptage physique (WhatsApp ou web)</t>
+        </is>
+      </c>
+      <c r="G900" t="inlineStr">
+        <is>
+          <t>Query `siteId?`, `locationId?`, `itemId?`, `source?` (WHATSAPP ou WEB), `cursor?`, `limit?` (200 au plus)</t>
+        </is>
+      </c>
+      <c r="H900" t="inlineStr">
+        <is>
+          <t>Lignes : lieu, article, stock théorique (masqué « Comptage en cours » pendant un comptage pour qui ne valide pas), dernier comptage, date, chef, source, statut ; valeurs seulement avec STOCK_VALUES_VIEW ; aucune colonne d'écart</t>
+        </is>
+      </c>
+      <c r="I900" t="inlineStr">
+        <is>
+          <t>Compter le stock par photo WhatsApp</t>
+        </is>
+      </c>
+      <c r="J900" t="inlineStr">
+        <is>
+          <t>TENANT_ADMIN, TENANT_MANAGER, TENANT_ACCOUNTANT, TENANT_STOREKEEPER (Magasinier)</t>
+        </is>
+      </c>
+      <c r="K900" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L900" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/finance/stock/whatsapp/field-counts</t>
+        </is>
+      </c>
+      <c r="M900" t="inlineStr">
+        <is>
+          <t>STOCK_VIEW</t>
+        </is>
+      </c>
+      <c r="N900" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O900" t="inlineStr">
+        <is>
+          <t>Finance &gt; Chantiers et stock &gt; Gestion du stock &gt; Comptages terrain</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>Promoteur, Opérateur intégré (option Inventaire WhatsApp, EXT_INVENTAIRE_WHATSAPP)</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>CONSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D901" t="inlineStr">
+        <is>
+          <t>Inventaire par WhatsApp</t>
+        </is>
+      </c>
+      <c r="E901" t="inlineStr">
+        <is>
+          <t>Consulter la preuve photo d'un comptage</t>
+        </is>
+      </c>
+      <c r="F901" t="inlineStr">
+        <is>
+          <t>Vérifier la photo, l'heure du serveur, l'empreinte et l'analyse derrière une ligne comptée par WhatsApp</t>
+        </is>
+      </c>
+      <c r="G901" t="inlineStr">
+        <is>
+          <t>Chemin `captureId` (lien « Voir la photo » des comptages terrain ou de l'inventaire, `?capture=`) ; liste filtrable des captures</t>
+        </is>
+      </c>
+      <c r="H901" t="inlineStr">
+        <is>
+          <t>Capture : photo (lue à l'ouverture, jamais en statique), heure du serveur, empreinte SHA-256 copiable, analyse (méthode, total proposé, confiance), ce que le chef a fait (validée, corrigée, ajoutée, remplacée, annulée, sans réponse), photo retirée le cas échéant ; captures d'un inventaire (source, ligne, nombre de photos)</t>
+        </is>
+      </c>
+      <c r="I901" t="inlineStr">
+        <is>
+          <t>Compter le stock par photo WhatsApp</t>
+        </is>
+      </c>
+      <c r="J901" t="inlineStr">
+        <is>
+          <t>TENANT_ADMIN, TENANT_MANAGER, TENANT_ACCOUNTANT, TENANT_STOREKEEPER (Magasinier)</t>
+        </is>
+      </c>
+      <c r="K901" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L901" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/finance/stock/whatsapp/captures ; GET /tenants/:tenantId/finance/stock/whatsapp/captures/:captureId ; GET /tenants/:tenantId/finance/stock/whatsapp/captures/:captureId/file ; GET /tenants/:tenantId/finance/stock/whatsapp/counts/:countId/captures</t>
+        </is>
+      </c>
+      <c r="M901" t="inlineStr">
+        <is>
+          <t>STOCK_VIEW</t>
+        </is>
+      </c>
+      <c r="N901" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O901" t="inlineStr">
+        <is>
+          <t>Finance &gt; Chantiers et stock &gt; Gestion du stock &gt; Comptages terrain (tiroir « Voir la photo ») ; Gestion du stock &gt; Inventaire (bouton photo d'une ligne)</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>Promoteur, Opérateur intégré (option Inventaire WhatsApp, EXT_INVENTAIRE_WHATSAPP)</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr">
+        <is>
+          <t>CONSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D902" t="inlineStr">
+        <is>
+          <t>Inventaire par WhatsApp</t>
+        </is>
+      </c>
+      <c r="E902" t="inlineStr">
+        <is>
+          <t>Retirer la photo d'un comptage</t>
+        </is>
+      </c>
+      <c r="F902" t="inlineStr">
+        <is>
+          <t>Effacer une photo qui ne devait pas être gardée (une personne y figure)</t>
+        </is>
+      </c>
+      <c r="G902" t="inlineStr">
+        <is>
+          <t>Chemin `captureId`, `reason` (3 à 500 caractères)</t>
+        </is>
+      </c>
+      <c r="H902" t="inlineStr">
+        <is>
+          <t>Fichier effacé ; la capture, le comptage et l'empreinte restent, avec la date, l'auteur et le motif du retrait</t>
+        </is>
+      </c>
+      <c r="I902" t="inlineStr">
+        <is>
+          <t>Consulter la preuve photo d'un comptage</t>
+        </is>
+      </c>
+      <c r="J902" t="inlineStr">
+        <is>
+          <t>TENANT_ADMIN</t>
+        </is>
+      </c>
+      <c r="K902" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L902" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/finance/stock/whatsapp/captures/:captureId/remove-photo</t>
+        </is>
+      </c>
+      <c r="M902" t="inlineStr">
+        <is>
+          <t>STOCK_DISPOSE</t>
+        </is>
+      </c>
+      <c r="N902" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O902" t="inlineStr">
+        <is>
+          <t>Finance &gt; Chantiers et stock &gt; Gestion du stock &gt; Comptages terrain (tiroir de preuve) — bouton « Retirer la photo »</t>
+        </is>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>Promoteur, Opérateur intégré (option Inventaire WhatsApp, EXT_INVENTAIRE_WHATSAPP)</t>
+        </is>
+      </c>
+      <c r="C903" t="inlineStr">
+        <is>
+          <t>CONSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D903" t="inlineStr">
+        <is>
+          <t>Inventaire par WhatsApp</t>
+        </is>
+      </c>
+      <c r="E903" t="inlineStr">
+        <is>
+          <t>Consulter la conversation WhatsApp d'un chef</t>
+        </is>
+      </c>
+      <c r="F903" t="inlineStr">
+        <is>
+          <t>Relire les échanges entre un chef et le bot autour d'un comptage</t>
+        </is>
+      </c>
+      <c r="G903" t="inlineStr">
+        <is>
+          <t>Query `registrationId?` ; chemin `sessionId`</t>
+        </is>
+      </c>
+      <c r="H903" t="inlineStr">
+        <is>
+          <t>Sessions (chantier, état, ouverture, clôture) et bulles de la conversation (180 jours au plus) ; 403 `STOCK_WHATSAPP_CONVERSATION_FORBIDDEN` sans le droit</t>
+        </is>
+      </c>
+      <c r="I903" t="inlineStr">
+        <is>
+          <t>Compter le stock par photo WhatsApp</t>
+        </is>
+      </c>
+      <c r="J903" t="inlineStr">
+        <is>
+          <t>TENANT_ADMIN (paramétrage de la finance ou validation des inventaires)</t>
+        </is>
+      </c>
+      <c r="K903" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L903" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/finance/stock/whatsapp/sessions ; GET /tenants/:tenantId/finance/stock/whatsapp/sessions/:sessionId/messages</t>
+        </is>
+      </c>
+      <c r="M903" t="inlineStr">
+        <is>
+          <t>FINANCE_SETTINGS_MANAGE ou STOCK_COUNT_VALIDATE</t>
+        </is>
+      </c>
+      <c r="N903" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O903" t="inlineStr">
+        <is>
+          <t>Finance &gt; Chantiers et stock &gt; Gestion du stock &gt; Comptages terrain (tiroir de preuve) — bouton « Voir la conversation »</t>
+        </is>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>Promoteur, Opérateur intégré (option Inventaire WhatsApp, EXT_INVENTAIRE_WHATSAPP)</t>
+        </is>
+      </c>
+      <c r="C904" t="inlineStr">
+        <is>
+          <t>CONSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D904" t="inlineStr">
+        <is>
+          <t>Inventaire par WhatsApp</t>
+        </is>
+      </c>
+      <c r="E904" t="inlineStr">
+        <is>
+          <t>Suivre le quota mensuel de photos</t>
+        </is>
+      </c>
+      <c r="F904" t="inlineStr">
+        <is>
+          <t>Savoir combien de photos analysées l'agence a consommées ce mois-ci, et l'état de la passerelle</t>
+        </is>
+      </c>
+      <c r="G904" t="inlineStr">
+        <is>
+          <t>Aucune saisie</t>
+        </is>
+      </c>
+      <c r="H904" t="inlineStr">
+        <is>
+          <t>Passerelle (journal, Meta, désactivée ; numéro du bot ; fournisseur de vision), quota du mois civil UTC (utilisées, plafond = 500 par bloc souscrit, source : option, secours `warn`/`off`, aucune) ; « Option non souscrite » en `enforce` sans option</t>
+        </is>
+      </c>
+      <c r="I904" t="inlineStr">
+        <is>
+          <t>Compter le stock par photo WhatsApp</t>
+        </is>
+      </c>
+      <c r="J904" t="inlineStr">
+        <is>
+          <t>TENANT_ADMIN (droit de paramétrer la finance)</t>
+        </is>
+      </c>
+      <c r="K904" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L904" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/finance/stock/whatsapp/overview</t>
+        </is>
+      </c>
+      <c r="M904" t="inlineStr">
+        <is>
+          <t>FINANCE_SETTINGS_MANAGE</t>
+        </is>
+      </c>
+      <c r="N904" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O904" t="inlineStr">
+        <is>
+          <t>Finance &gt; Chantiers et stock &gt; Gestion du stock &gt; WhatsApp (en-tête)</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>Promoteur, Opérateur intégré (option Inventaire WhatsApp, EXT_INVENTAIRE_WHATSAPP)</t>
+        </is>
+      </c>
+      <c r="C905" t="inlineStr">
+        <is>
+          <t>CONSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D905" t="inlineStr">
+        <is>
+          <t>Inventaire par WhatsApp</t>
+        </is>
+      </c>
+      <c r="E905" t="inlineStr">
+        <is>
+          <t>Simuler une conversation WhatsApp (recette)</t>
+        </is>
+      </c>
+      <c r="F905" t="inlineStr">
+        <is>
+          <t>Jouer, sans Meta, les messages d'un chef inscrit ou d'un numéro inconnu et faire avancer l'horloge</t>
+        </is>
+      </c>
+      <c r="G905" t="inlineStr">
+        <is>
+          <t>Inscription de l'agence ou numéro libre ; texte, photo (multipart, 10 Mo, légende `fake:…`) ou réponse de bouton ; avance de 10 ou 30 minutes</t>
+        </is>
+      </c>
+      <c r="H905" t="inlineStr">
+        <is>
+          <t>Message traité par le même moteur que le webhook ; conversation relue ; relance (M23) et expiration (M24) jouées. 404 `STOCK_WHATSAPP_SIMULATOR_UNAVAILABLE` hors transport `log` (et en production sans `WHATSAPP_INVENTORY_SIMULATOR=1`) ; un numéro d'une autre agence est refusé</t>
+        </is>
+      </c>
+      <c r="I905" t="inlineStr">
+        <is>
+          <t>Inscrire un chef de chantier</t>
+        </is>
+      </c>
+      <c r="J905" t="inlineStr">
+        <is>
+          <t>TENANT_ADMIN (droit de paramétrer la finance)</t>
+        </is>
+      </c>
+      <c r="K905" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L905" t="inlineStr">
+        <is>
+          <t>POST /tenants/:tenantId/finance/stock/whatsapp/simulator/messages ; GET /tenants/:tenantId/finance/stock/whatsapp/simulator/conversation ; POST /tenants/:tenantId/finance/stock/whatsapp/simulator/sessions/:sessionId/advance</t>
+        </is>
+      </c>
+      <c r="M905" t="inlineStr">
+        <is>
+          <t>FINANCE_SETTINGS_MANAGE</t>
+        </is>
+      </c>
+      <c r="N905" t="inlineStr">
+        <is>
+          <t>Disponible (staging et développement seulement)</t>
+        </is>
+      </c>
+      <c r="O905" t="inlineStr">
+        <is>
+          <t>Finance &gt; Chantiers et stock &gt; Gestion du stock &gt; WhatsApp &gt; Simulateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>Promoteur, Opérateur intégré (option Inventaire WhatsApp, EXT_INVENTAIRE_WHATSAPP)</t>
+        </is>
+      </c>
+      <c r="C906" t="inlineStr">
+        <is>
+          <t>CONSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D906" t="inlineStr">
+        <is>
+          <t>Inventaire par WhatsApp</t>
+        </is>
+      </c>
+      <c r="E906" t="inlineStr">
+        <is>
+          <t>Consulter les mesures de l'inventaire WhatsApp</t>
+        </is>
+      </c>
+      <c r="F906" t="inlineStr">
+        <is>
+          <t>Juger l'usage et la fiabilité du comptage par photo, sans mesure par personne</t>
+        </is>
+      </c>
+      <c r="G906" t="inlineStr">
+        <is>
+          <t>Query `month?` (AAAA-MM)</t>
+        </is>
+      </c>
+      <c r="H906" t="inlineStr">
+        <is>
+          <t>Mesures de l'agence entière : photos analysées, délai médian jusqu'à la confirmation, part validée sans correction, couverture photo des lignes, photos illisibles, articles non reconnus, analyses en échec</t>
+        </is>
+      </c>
+      <c r="I906" t="inlineStr">
+        <is>
+          <t>Compter le stock par photo WhatsApp</t>
+        </is>
+      </c>
+      <c r="J906" t="inlineStr">
+        <is>
+          <t>TENANT_ADMIN (droit de paramétrer la finance)</t>
+        </is>
+      </c>
+      <c r="K906" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L906" t="inlineStr">
+        <is>
+          <t>GET /tenants/:tenantId/finance/stock/whatsapp/overview</t>
+        </is>
+      </c>
+      <c r="M906" t="inlineStr">
+        <is>
+          <t>FINANCE_SETTINGS_MANAGE</t>
+        </is>
+      </c>
+      <c r="N906" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O906" t="inlineStr">
+        <is>
+          <t>Finance &gt; Chantiers et stock &gt; Gestion du stock &gt; WhatsApp &gt; Mesures</t>
+        </is>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>Promoteur, Opérateur intégré</t>
+        </is>
+      </c>
+      <c r="C907" t="inlineStr">
+        <is>
+          <t>CONSTRUCTION</t>
+        </is>
+      </c>
+      <c r="D907" t="inlineStr">
+        <is>
+          <t>Inventaire par WhatsApp</t>
+        </is>
+      </c>
+      <c r="E907" t="inlineStr">
+        <is>
+          <t>Attribuer le rôle Chef de chantier</t>
+        </is>
+      </c>
+      <c r="F907" t="inlineStr">
+        <is>
+          <t>Permettre à un collaborateur de compter le stock de ses chantiers par WhatsApp, sans voir le stock ni les valeurs</t>
+        </is>
+      </c>
+      <c r="G907" t="inlineStr">
+        <is>
+          <t>`roleIds` incluant TENANT_SITE_MANAGER</t>
+        </is>
+      </c>
+      <c r="H907" t="inlineStr">
+        <is>
+          <t>Collaborateur Chef de chantier : seul droit STOCK_COUNT (ni STOCK_VIEW ni valeurs) ; inscriptible au bot. Un rôle retiré coupe l'accès WhatsApp au message suivant</t>
+        </is>
+      </c>
+      <c r="I907" t="inlineStr">
+        <is>
+          <t>Modifier les rôles d'un collaborateur</t>
+        </is>
+      </c>
+      <c r="J907" t="inlineStr">
+        <is>
+          <t>Collaborateur USERS_EDIT ; super-admin</t>
+        </is>
+      </c>
+      <c r="K907" t="inlineStr">
+        <is>
+          <t>Agence</t>
+        </is>
+      </c>
+      <c r="L907" t="inlineStr">
+        <is>
+          <t>PATCH /api/tenants/:tenantId/users/:userId</t>
+        </is>
+      </c>
+      <c r="M907" t="inlineStr">
+        <is>
+          <t>USERS_EDIT</t>
+        </is>
+      </c>
+      <c r="N907" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="O907" t="inlineStr">
+        <is>
+          <t>Agence &gt; Collaborateurs &gt; fiche</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(wiki): réappliquer les lignes de désactivation, d'accès et de refus après la fusion
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NipnEzc6N8uvDDXG2M7jms
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sous-fonctionnalites" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legende Packs-Modules" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes et points ouverts" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sous-fonctionnalites" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Legende Packs-Modules" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Notes et points ouverts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -242,7 +242,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotesPointsOuverts" displayName="NotesPointsOuverts" ref="A1:D39" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotesPointsOuverts" displayName="NotesPointsOuverts" ref="A1:D40" headerRowCount="1">
   <autoFilter ref="A1:D37"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Domaine"/>
@@ -43802,7 +43802,7 @@
       </c>
       <c r="F560" s="2" t="inlineStr">
         <is>
-          <t>Change les rôles assignés à un membre</t>
+          <t>Change les rôles assignés à un membre. Retirer TENANT_ADMIN au dernier administrateur actif de l'agence est refusé (409)</t>
         </is>
       </c>
       <c r="G560" s="2" t="inlineStr">
@@ -43812,7 +43812,7 @@
       </c>
       <c r="H560" s="2" t="inlineStr">
         <is>
-          <t>Membre mis à jour</t>
+          <t>Membre mis à jour ; erreur 409 si le dernier administrateur actif perd TENANT_ADMIN</t>
         </is>
       </c>
       <c r="I560" s="2" t="inlineStr">
@@ -43879,7 +43879,7 @@
       </c>
       <c r="F561" s="2" t="inlineStr">
         <is>
-          <t>Coupe l'accès d'un membre à l'agence</t>
+          <t>Coupe l'accès d'un membre à l'agence. Refus 409 de l'auto-désactivation et de la désactivation du dernier administrateur actif de l'agence (TENANT_ADMIN actif) ; un membre déjà désactivé répond 409 (et non plus 400). Voir la note « Dernier administrateur : course possible »</t>
         </is>
       </c>
       <c r="G561" s="2" t="inlineStr">
@@ -43889,7 +43889,7 @@
       </c>
       <c r="H561" s="2" t="inlineStr">
         <is>
-          <t>Membership désactivé</t>
+          <t>Membership désactivé ; erreurs 409 : auto-désactivation, dernier administrateur actif, membre déjà désactivé</t>
         </is>
       </c>
       <c r="I561" s="2" t="inlineStr">
@@ -68782,7 +68782,7 @@
       </c>
       <c r="F885" t="inlineStr">
         <is>
-          <t>Outil `call_read` (lecture seule) : exécute une route GET du catalogue sous l'identité et les permissions de l'utilisateur, par une requête loopback de l'API vers elle-même (127.0.0.1 et PORT de la configuration, jamais une URL fournie par le modèle) qui rejoue l'authentification du chat. Toute la chaîne réelle s'applique (authentification, accès à l'agence, permission de la route, abonnement, garde Prisma, limiteurs) : le catalogue n'est qu'un index. N'accepte qu'un id GET non sensible du catalogue ; `:tenantId` imposé par le serveur, autres paramètres de chemin = UUID ou jeton simple, 20 clés de requête au plus. Délai 10 s, abandon avec le chat, JSON seulement (sinon « contenu non textuel, non affiché »), lecture plafonnée à 2 Mio. Avant retour au modèle : clés évoquant un secret (password, secret, token, apiKey, authorization, hash…) remplacées par « [masqué] » à toute profondeur (iban et rib restent visibles), tableaux &gt; 50 éléments, chaînes &gt; 500 caractères et profondeur &gt; 6 tronqués, total d'environ 12 000 caractères. Erreurs HTTP renvoyées sous la forme {status, message}, sans pile. Les routes d'écriture ne passent jamais par `call_read` : elles passent par `plan_write` puis un accord explicite.</t>
+          <t>Outil `call_read` (lecture seule) : exécute une route GET du catalogue sous l'identité et les permissions de l'utilisateur, par une requête loopback de l'API vers elle-même (127.0.0.1 et PORT de la configuration, jamais une URL fournie par le modèle) qui rejoue l'authentification du chat. Toute la chaîne réelle s'applique (authentification, accès à l'agence, permission de la route, abonnement, garde Prisma, limiteurs) : le catalogue n'est qu'un index. N'accepte qu'un id GET non sensible du catalogue ; `:tenantId` imposé par le serveur, autres paramètres de chemin = UUID ou jeton simple, 20 clés de requête au plus. Délai 10 s, abandon avec le chat, JSON seulement (sinon « contenu non textuel, non affiché »), lecture plafonnée à 2 Mio. Avant retour au modèle : clés évoquant un secret (password, secret, token, apiKey, authorization, hash…) remplacées par « [masqué] » à toute profondeur (iban et rib restent visibles), tableaux &gt; 50 éléments, chaînes &gt; 500 caractères et profondeur &gt; 6 tronqués, total d'environ 12 000 caractères. Erreurs HTTP renvoyées sous la forme {status, message}, sans pile. Les routes d'écriture ne passent jamais par `call_read` : elles passent par `plan_write` puis un accord explicite. Un refus 401 ou 403 de la route réelle est un refus de l'assistant (statut d'outil « forbidden », audit AI_TOOL_DENIED), et non un résultat normal.</t>
         </is>
       </c>
       <c r="G885" t="inlineStr">
@@ -68859,7 +68859,7 @@
       </c>
       <c r="F886" t="inlineStr">
         <is>
-          <t>Quand l'assistant veut modifier des données, la conversation affiche une carte d'accord et rien n'est modifié avant l'approbation. Bandeau « Action à valider — rien n'a encore été modifié » ; titre, type (Création, Modification, Action), module et méthode en langage clair ; section « Ce que l'assistant va faire » (étapes numérotées, étiquetée « Expliqué par l'assistant », texte brut) ; section « Données concernées » (étiquetée « Calculé par le serveur ») : enregistrement visé (un identifiant brut est qualifié « Enregistrement (identifiant …) ») puis tableau Champ / Avant / Après (noms de champs rendus lisibles, nom technique en infobulle) (valeurs formatées selon la langue, valeurs longues repliables, « [masqué] » tel quel, mention « liste tronquée »), puis avertissements du serveur. Boutons « Approuver et exécuter » et « Refuser » ; décompte d'expiration, boutons désactivés à l'expiration ; verrou contre le double envoi. Après décision la carte est figée : statut, heure, message du serveur et aperçu replié du résultat en texte brut ; un échec (refus du serveur, jeton expiré ou déjà utilisé, erreur réseau) est expliqué. Même carte dans le tiroir et la page plein écran</t>
+          <t>Quand l'assistant veut modifier des données, la conversation affiche une carte d'accord et rien n'est modifié avant l'approbation. Bandeau « Action à valider — rien n'a encore été modifié » ; titre, type (Création, Modification, Action), module et méthode en langage clair ; section « Ce que l'assistant va faire » (étapes numérotées, étiquetée « Expliqué par l'assistant », texte brut) ; section « Données concernées » (étiquetée « Calculé par le serveur ») : enregistrement visé (un identifiant brut est qualifié « Enregistrement (identifiant …) ») puis tableau Champ / Avant / Après (noms de champs rendus lisibles, nom technique en infobulle) (valeurs formatées selon la langue, valeurs longues repliables, « [masqué] » tel quel, mention « liste tronquée »), puis avertissements du serveur. Boutons « Approuver et exécuter » et « Refuser » ; décompte d'expiration, boutons désactivés à l'expiration ; verrou contre le double envoi. Après décision la carte est figée : statut, heure, message du serveur et aperçu replié du résultat en texte brut ; un échec (refus du serveur, jeton expiré ou déjà utilisé, erreur réseau) est expliqué. Même carte dans le tiroir et la page plein écran. Pour une écriture sur un utilisateur (route `users/:id`), le serveur ajoute l'avertissement « Cette action modifie l'accès de &lt;nom&gt; » ; le libellé de la personne visée est lu dans la réponse (prénom + nom, sinon e-mail)</t>
         </is>
       </c>
       <c r="G886" t="inlineStr">
@@ -69090,7 +69090,7 @@
       </c>
       <c r="F889" t="inlineStr">
         <is>
-          <t>Outil `plan_write` : le modèle propose de modifier des données ; rien n'est écrit à ce stade. N'accepte qu'un id POST, PUT ou PATCH du catalogue (jamais DELETE, jamais une route destructive ni sensible-interdite) ; `:tenantId` imposé par le serveur. Le serveur LIT l'état actuel de l'enregistrement par un GET loopback et CALCULE lui-même les changements avant/après : le modèle ne fournit que le titre et les étapes. Clés évoquant un secret masquées (« [masqué] »). 30 changements affichés au plus : au-delà, liste tronquée et saisie obligatoire du mot CONFIRMER. Actions sensibles (paiement, remboursement, envoi, signature, validation ou clôture, droits et comptes, imports et opérations en masse) : confirmation tapée « CONFIRMER ». 3 plans au plus par requête de chat. Le plan est livré avec un jeton signé à usage unique, valable 900 s (AI_WRITE_PLAN_TTL_SECONDS) et lié à la requête approuvée (planHash). La carte d'accord montre aussi : les paramètres de requête envoyés à la route (« Paramètres envoyés à la route »), les identifiants du parent visé pour une création imbriquée (« Éléments visés », le serveur lisant lui-même le parent), l'heure de lecture de l'état « avant » (« État lu à HH:MM » : les données ont pu changer depuis), les listes remplacées (« Liste remplacée : N éléments retirés ») et les champs protégés (« [masqué] » avec avertissement). La saisie du mot CONFIRMER est exigée pour : les actions sensibles (paiements, envois, signature, droits d'accès et comptes, clôtures/verrouillages, fins de contrat, annulations, cessions, archivages, publication, abonnement), une requête non vide (paramètres de requête), une liste remplacée, plus de 30 changements, et un corps touchant rôles, permissions, statut, mot de passe ou e-mail d'un utilisateur</t>
+          <t>Outil `plan_write` : le modèle propose de modifier des données ; rien n'est écrit à ce stade. N'accepte qu'un id POST, PUT ou PATCH du catalogue (jamais DELETE, jamais une route destructive ni sensible-interdite) ; `:tenantId` imposé par le serveur. Le serveur LIT l'état actuel de l'enregistrement par un GET loopback et CALCULE lui-même les changements avant/après : le modèle ne fournit que le titre et les étapes. Clés évoquant un secret masquées (« [masqué] »). 30 changements affichés au plus : au-delà, liste tronquée et saisie obligatoire du mot CONFIRMER. Actions sensibles (paiement, remboursement, envoi, signature, validation ou clôture, droits et comptes, imports et opérations en masse) : confirmation tapée « CONFIRMER ». 3 plans au plus par requête de chat. Le plan est livré avec un jeton signé à usage unique, valable 900 s (AI_WRITE_PLAN_TTL_SECONDS) et lié à la requête approuvée (planHash). La carte d'accord montre aussi : les paramètres de requête envoyés à la route (« Paramètres envoyés à la route »), les identifiants du parent visé pour une création imbriquée (« Éléments visés », le serveur lisant lui-même le parent), l'heure de lecture de l'état « avant » (« État lu à HH:MM » : les données ont pu changer depuis), les listes remplacées (« Liste remplacée : N éléments retirés ») et les champs protégés (« [masqué] » avec avertissement). La saisie du mot CONFIRMER est exigée pour : les actions sensibles (paiements, envois, signature, droits d'accès et comptes, clôtures/verrouillages, fins de contrat, annulations, cessions, archivages, publication, abonnement), une requête non vide (paramètres de requête), une liste remplacée, plus de 30 changements, et un corps touchant rôles, permissions, statut, mot de passe ou e-mail d'un utilisateur. Pour une écriture sur un utilisateur (route `users/:id`), le serveur ajoute l'avertissement « Cette action modifie l'accès de &lt;nom&gt; » ; le libellé de la personne visée est lu dans la réponse (prénom + nom, sinon e-mail)</t>
         </is>
       </c>
       <c r="G889" t="inlineStr">
@@ -71127,7 +71127,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -71994,6 +71994,28 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Administration plateforme</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Dernier administrateur : course possible</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Le contrôle du dernier administrateur actif (désactivation ou retrait de TENANT_ADMIN) se fait avant la transaction, sans verrou : deux désactivations simultanées des deux seuls administrateurs pourraient théoriquement passer (voir SECURITY §13).</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Non couvert : désactivation de compte au niveau plateforme et suspension de l'agence. À confirmer : verrou ou contrôle dans la transaction si le risque est jugé réel.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
feat(menus): défaut commun et surcharge par agence
Décision du 2026-10-05 : les lots 040/041 coupent une fois, pour toutes les
agences, les menus hors stock des rôles Magasinier et Chef de chantier.

- `tenant_id` NULL = défaut de toutes les agences pour un rôle d'agence ou de
  portail (périmètre plateforme pour un rôle PLATFORM) ; agence = surcharge.
  Résolution par (rôle, menu) : agence, sinon défaut, sinon autorisé.
- Migration sans copie : les décisions existantes deviennent le défaut.
- PUT sans tenantId écrit le défaut ; `{}` avec tenantId rend l'agence au défaut.
- Écran Menus : « Toutes les agences (défaut) » ou une agence, tags
  « Hérite du défaut » / « Réglage propre à l'agence », « Revenir au défaut ».
- DEPLOIEMENT.md (étapes 040/041), DATA_MODELS.md et classeur à jour.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -42108,7 +42108,7 @@
       </c>
       <c r="F538" s="2" t="inlineStr">
         <is>
-          <t>Menus masqués pour l'utilisateur courant dans l'agence demandée : seules les coupures posées pour CETTE agence s'appliquent (sans agence : coupures du périmètre plateforme). Renvoie aussi les permissions du compte, ce qui permet à la coquille de masquer les entrées Biens/Patrimoine (Sinistres, Régularisation foncière, Accès partagés) pour un rôle sans PROPERTIES_VIEW.</t>
+          <t>Menus masqués pour l'utilisateur courant dans l'agence demandée : pour chaque rôle et chaque menu, le réglage propre à l'agence l'emporte, sinon le réglage par défaut de toutes les agences s'applique (sans agence : réglages du périmètre plateforme). Renvoie aussi les permissions du compte, ce qui permet à la coquille de masquer les entrées Biens/Patrimoine (Sinistres, Régularisation foncière, Accès partagés) pour un rôle sans PROPERTIES_VIEW.</t>
         </is>
       </c>
       <c r="G538" s="2" t="inlineStr">
@@ -42180,17 +42180,17 @@
       </c>
       <c r="E539" s="2" t="inlineStr">
         <is>
-          <t>Consulter la carte des menus par rôle et par agence</t>
+          <t>Consulter la carte des menus par rôle (défaut ou agence)</t>
         </is>
       </c>
       <c r="F539" s="2" t="inlineStr">
         <is>
-          <t>Vue d'ensemble : quels menus sont coupés pour quel rôle, dans l'agence choisie (ou au niveau plateforme pour les rôles plateforme). Aucun héritage entre agences ni depuis la plateforme.</t>
+          <t>Vue d'ensemble des menus coupés par rôle : sans agence, le réglage par défaut de toutes les agences (et celui des rôles plateforme) ; avec une agence, les réglages propres à cette agence.</t>
         </is>
       </c>
       <c r="G539" s="2" t="inlineStr">
         <is>
-          <t>Query `tenantId?` (agence ; absent = périmètre plateforme)</t>
+          <t>Query `tenantId?` (agence ; absent = défaut de toutes les agences / plateforme)</t>
         </is>
       </c>
       <c r="H539" s="2" t="inlineStr">
@@ -42230,7 +42230,7 @@
       </c>
       <c r="O539" s="2" t="inlineStr">
         <is>
-          <t>Administration &gt; Rôles et permissions &gt; onglet Menus (sélecteur d’agence)</t>
+          <t>Administration &gt; Rôles et permissions &gt; onglet Menus (choix « Toutes les agences (défaut) » ou une agence)</t>
         </is>
       </c>
     </row>
@@ -42262,12 +42262,12 @@
       </c>
       <c r="F540" s="2" t="inlineStr">
         <is>
-          <t>Définit quelles entrées de menu sont visibles pour un rôle (ou persona portail propriétaire/locataire) dans UNE agence ; les autres agences ne sont pas touchées. L'écran demande de choisir l'agence avant d'afficher l'arbre des menus d'un rôle d'agence.</t>
+          <t>Définit quelles entrées de menu sont visibles pour un rôle (ou persona portail propriétaire/locataire) : soit par défaut pour toutes les agences (« Toutes les agences (défaut) »), soit pour une seule agence, dont le réglage remplace alors le défaut. « Revenir au défaut » efface le réglage propre de l'agence (carte vide).</t>
         </is>
       </c>
       <c r="G540" s="2" t="inlineStr">
         <is>
-          <t>`roleKey` (ou pseudo-clé PORTAL_OWNER/PORTAL_RENTER), `menus: {menuKey: boolean}`, query `tenantId` obligatoire pour un rôle d’agence ou de portail, interdit pour un rôle plateforme</t>
+          <t>`roleKey` (ou pseudo-clé PORTAL_OWNER/PORTAL_RENTER), `menus: {menuKey: boolean}` (500 entrées max), query `tenantId?` (absent = défaut de toutes les agences pour un rôle d’agence ou de portail ; interdit pour un rôle plateforme)</t>
         </is>
       </c>
       <c r="H540" s="2" t="inlineStr">
@@ -42307,7 +42307,7 @@
       </c>
       <c r="O540" s="2" t="inlineStr">
         <is>
-          <t>Administration &gt; Rôles et permissions &gt; onglet Menus (sélecteur d’agence)</t>
+          <t>Administration &gt; Rôles et permissions &gt; onglet Menus (choix « Toutes les agences (défaut) » ou une agence)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(copilot): refuser les créations imbriquées sans parent lisible, libellés traduits, tests du patrimoine déterministes
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NipnEzc6N8uvDDXG2M7jms
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -242,7 +242,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotesPointsOuverts" displayName="NotesPointsOuverts" ref="A1:D40" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotesPointsOuverts" displayName="NotesPointsOuverts" ref="A1:D41" headerRowCount="1">
   <autoFilter ref="A1:D37"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Domaine"/>
@@ -69090,7 +69090,7 @@
       </c>
       <c r="F889" t="inlineStr">
         <is>
-          <t>Outil `plan_write` : le modèle propose de modifier des données ; rien n'est écrit à ce stade. N'accepte qu'un id POST, PUT ou PATCH du catalogue (jamais DELETE, jamais une route destructive ni sensible-interdite) ; `:tenantId` imposé par le serveur. Le serveur LIT l'état actuel de l'enregistrement par un GET loopback et CALCULE lui-même les changements avant/après : le modèle ne fournit que le titre et les étapes. Clés évoquant un secret masquées (« [masqué] »). 30 changements affichés au plus : au-delà, liste tronquée et saisie obligatoire du mot CONFIRMER. Actions sensibles (paiement, remboursement, envoi, signature, validation ou clôture, droits et comptes, imports et opérations en masse) : confirmation tapée « CONFIRMER ». 3 plans au plus par requête de chat. Le plan est livré avec un jeton signé à usage unique, valable 900 s (AI_WRITE_PLAN_TTL_SECONDS) et lié à la requête approuvée (planHash). La carte d'accord montre aussi : les paramètres de requête envoyés à la route (« Paramètres envoyés à la route »), les identifiants du parent visé pour une création imbriquée (« Éléments visés », le serveur lisant lui-même le parent), l'heure de lecture de l'état « avant » (« État lu à HH:MM » : les données ont pu changer depuis), les listes remplacées (« Liste remplacée : N éléments retirés ») et les champs protégés (« [masqué] » avec avertissement). La saisie du mot CONFIRMER est exigée pour : les actions sensibles (paiements, envois, signature, droits d'accès et comptes, clôtures/verrouillages, fins de contrat, annulations, cessions, archivages, publication, abonnement), une requête non vide (paramètres de requête), une liste remplacée, plus de 30 changements, et un corps touchant rôles, permissions, statut, mot de passe ou e-mail d'un utilisateur. Pour une écriture sur un utilisateur (route `users/:id`), le serveur ajoute l'avertissement « Cette action modifie l'accès de &lt;nom&gt; » ; le libellé de la personne visée est lu dans la réponse (prénom + nom, sinon e-mail)</t>
+          <t>Outil `plan_write` : le modèle propose de modifier des données ; rien n'est écrit à ce stade. N'accepte qu'un id POST, PUT ou PATCH du catalogue (jamais DELETE, jamais une route destructive ni sensible-interdite) ; `:tenantId` imposé par le serveur. Le serveur LIT l'état actuel de l'enregistrement par un GET loopback et CALCULE lui-même les changements avant/après : le modèle ne fournit que le titre et les étapes. Clés évoquant un secret masquées (« [masqué] »). 30 changements affichés au plus : au-delà, liste tronquée et saisie obligatoire du mot CONFIRMER. Actions sensibles (paiement, remboursement, envoi, signature, validation ou clôture, droits et comptes, imports et opérations en masse) : confirmation tapée « CONFIRMER ». 3 plans au plus par requête de chat. Le plan est livré avec un jeton signé à usage unique, valable 900 s (AI_WRITE_PLAN_TTL_SECONDS) et lié à la requête approuvée (planHash). La carte d'accord montre aussi : les paramètres de requête envoyés à la route (« Paramètres envoyés à la route »), les identifiants du parent visé pour une création imbriquée (« Éléments visés », le serveur lisant lui-même le parent), l'heure de lecture de l'état « avant » (« État lu à HH:MM » : les données ont pu changer depuis), les listes remplacées (« Liste remplacée : N éléments retirés ») et les champs protégés (« [masqué] » avec avertissement). La saisie du mot CONFIRMER est exigée pour : les actions sensibles (paiements, envois, signature, droits d'accès et comptes, clôtures/verrouillages, fins de contrat, annulations, cessions, archivages, publication, abonnement), une requête non vide (paramètres de requête), une liste remplacée, plus de 30 changements, et un corps touchant rôles, permissions, statut, mot de passe ou e-mail d'un utilisateur. Pour une écriture sur un utilisateur (route `users/:id`), le serveur ajoute l'avertissement « Cette action modifie l'accès de &lt;nom&gt; » ; le libellé de la personne visée est lu dans la réponse (prénom + nom, sinon e-mail). Pour une création imbriquée, si le serveur ne peut pas lire la ressource parente visée (aucune route de lecture du parent dans le catalogue, ou lecture refusée/introuvable), le plan est refusé (« Impossible de vérifier la ressource parente visée ») et aucun jeton n'est émis.</t>
         </is>
       </c>
       <c r="G889" t="inlineStr">
@@ -71127,7 +71127,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -72016,6 +72016,28 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Communication et Documents</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Créations imbriquées non planifiables par l'assistant</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>3 routes du catalogue n'ont pas de route GET pour leur parent et sont donc refusées par plan_write (« Impossible de vérifier la ressource parente visée ») : `POST /api/tenants/:tenantId/crm/deals/:dealId/properties/:propertyId/status/legacy`, `POST …/syndics/:syndicId/lots/:lotId/compte/ajustements`, `POST …/syndics/:syndicId/lots/:lotId/paiements/apercu` (cette dernière ressemble à un simple aperçu de calcul : plutôt une lecture). Un GET `…/syndics/:syndicId/lots/:lotId` les rendrait planifiables.</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>À faire / à confirmer : ajouter cette route de lecture du lot, ou classer `apercu` comme lecture.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
fix(copilot): list_capabilities liste les routes d'écriture (kind write) pour plan_write
Le prompt et plan_write faisaient chercher la route d'écriture avec
list_capabilities, qui ne renvoyait que les routes GET : un vrai modèle
bouclait puis échouait (« trop d'étapes »). kind: 'write' renvoie
exactement les routes que findWritableEntry accepte (jamais DELETE ni
sensibles, filtrées par permission), chaque entrée porte sa méthode, et le
prompt demande de chercher par module d'abord.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sous-fonctionnalites" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Legende Packs-Modules" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Notes et points ouverts" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sous-fonctionnalites" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legende Packs-Modules" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes et points ouverts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -68705,7 +68705,7 @@
       </c>
       <c r="F884" t="inlineStr">
         <is>
-          <t>Outil `list_capabilities` (lecture seule) : cherche dans le catalogue généré des routes GET d'agence (`packages/api/src/lib/ai/gateway/catalog.generated.json`, produit par `npm run ai:catalog` à partir de la pile Express réelle) celles que l'interface permet de consulter : par mots-clés et/ou module (finance, rental, crm, syndics, patrimoine…). Au plus 20 résultats (id, chemin, module, résumé, paramètres de chemin) ; sans argument, la liste des modules. Filtre selon les permissions connues de l'utilisateur quand le catalogue les connaît (sinon laisse passer : l'appel réel tranche). Les routes sensibles (chemin évoquant un secret, un jeton, une invitation, la passerelle de paiement) n'apparaissent jamais ; le catalogue ne contient ni route DELETE ni écriture destructrice (/delete /remove /destroy /purge). Un test (`ai.catalog.test.ts`) échoue tant que le catalogue commité diffère de la pile Express.</t>
+          <t>Outil `list_capabilities` (n'écrit rien) : cherche dans le catalogue généré des routes d'agence (GET par défaut ; avec `kind: "write"`, les routes POST/PUT/PATCH non sensibles et permises que `plan_write` accepte, jamais DELETE) (`packages/api/src/lib/ai/gateway/catalog.generated.json`, produit par `npm run ai:catalog` à partir de la pile Express réelle) celles que l'interface permet de consulter : par mots-clés et/ou module (finance, rental, crm, syndics, patrimoine…). Au plus 20 résultats (id, chemin, module, résumé, paramètres de chemin) ; sans argument, la liste des modules. Filtre selon les permissions connues de l'utilisateur quand le catalogue les connaît (sinon laisse passer : l'appel réel tranche). Les routes sensibles (chemin évoquant un secret, un jeton, une invitation, la passerelle de paiement) n'apparaissent jamais ; le catalogue ne contient ni route DELETE ni écriture destructrice (/delete /remove /destroy /purge). Un test (`ai.catalog.test.ts`) échoue tant que le catalogue commité diffère de la pile Express.</t>
         </is>
       </c>
       <c r="G884" t="inlineStr">

</xml_diff>

<commit_message>
feat(copilot): valider à sec le corps d'un plan d'écriture et nommer les champs en erreur
plan_write valide le corps proposé contre le schéma Zod réel de 11 routes
(biens, CRM, baux) avant d'afficher la carte d'accord : un corps incomplet
est refusé au modèle (chemin, absent ou invalide, valeurs permises, jamais la
valeur saisie) sans jeton ni audit. Les autres routes gardent leur plan avec
l'avertissement « non vérifiée à l'avance ». L'exécution renvoie fieldErrors
et la carte d'échec liste les champs avec leur libellé traduit. Le masquage
des valeurs citées ne dépend plus de la langue.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
+++ b/docs/fonctionnalites/ImmoTopia_Wiki_Fonctionnalites.xlsx
@@ -69090,7 +69090,7 @@
       </c>
       <c r="F889" t="inlineStr">
         <is>
-          <t>Outil `plan_write` : le modèle propose de modifier des données ; rien n'est écrit à ce stade. N'accepte qu'un id POST, PUT ou PATCH du catalogue (jamais DELETE, jamais une route destructive ni sensible-interdite) ; `:tenantId` imposé par le serveur. Le serveur LIT l'état actuel de l'enregistrement par un GET loopback et CALCULE lui-même les changements avant/après : le modèle ne fournit que le titre et les étapes. Clés évoquant un secret masquées (« [masqué] »). 30 changements affichés au plus : au-delà, liste tronquée et saisie obligatoire du mot CONFIRMER. Actions sensibles (paiement, remboursement, envoi, signature, validation ou clôture, droits et comptes, imports et opérations en masse) : confirmation tapée « CONFIRMER ». 3 plans au plus par requête de chat. Le plan est livré avec un jeton signé à usage unique, valable 900 s (AI_WRITE_PLAN_TTL_SECONDS) et lié à la requête approuvée (planHash). La carte d'accord montre aussi : les paramètres de requête envoyés à la route (« Paramètres envoyés à la route »), les identifiants du parent visé pour une création imbriquée (« Éléments visés », le serveur lisant lui-même le parent), l'heure de lecture de l'état « avant » (« État lu à HH:MM » : les données ont pu changer depuis), les listes remplacées (« Liste remplacée : N éléments retirés ») et les champs protégés (« [masqué] » avec avertissement). La saisie du mot CONFIRMER est exigée pour : les actions sensibles (paiements, envois, signature, droits d'accès et comptes, clôtures/verrouillages, fins de contrat, annulations, cessions, archivages, publication, abonnement), une requête non vide (paramètres de requête), une liste remplacée, plus de 30 changements, et un corps touchant rôles, permissions, statut, mot de passe ou e-mail d'un utilisateur. Pour une écriture sur un utilisateur (route `users/:id`), le serveur ajoute l'avertissement « Cette action modifie l'accès de &lt;nom&gt; » ; le libellé de la personne visée est lu dans la réponse (prénom + nom, sinon e-mail) Pour une création imbriquée, si le serveur ne peut pas lire la ressource parente visée (aucune route de lecture du parent dans le catalogue, ou lecture refusée/introuvable), le plan est refusé (« Impossible de vérifier la ressource parente visée ») et aucun jeton n'est émis.</t>
+          <t>Outil `plan_write` : le modèle propose de modifier des données ; rien n'est écrit à ce stade. N'accepte qu'un id POST, PUT ou PATCH du catalogue (jamais DELETE, jamais une route destructive ni sensible-interdite) ; `:tenantId` imposé par le serveur. Le serveur LIT l'état actuel de l'enregistrement par un GET loopback et CALCULE lui-même les changements avant/après : le modèle ne fournit que le titre et les étapes. Clés évoquant un secret masquées (« [masqué] »). 30 changements affichés au plus : au-delà, liste tronquée et saisie obligatoire du mot CONFIRMER. Actions sensibles (paiement, remboursement, envoi, signature, validation ou clôture, droits et comptes, imports et opérations en masse) : confirmation tapée « CONFIRMER ». 3 plans au plus par requête de chat. Le plan est livré avec un jeton signé à usage unique, valable 900 s (AI_WRITE_PLAN_TTL_SECONDS) et lié à la requête approuvée (planHash). La carte d'accord montre aussi : les paramètres de requête envoyés à la route (« Paramètres envoyés à la route »), les identifiants du parent visé pour une création imbriquée (« Éléments visés », le serveur lisant lui-même le parent), l'heure de lecture de l'état « avant » (« État lu à HH:MM » : les données ont pu changer depuis), les listes remplacées (« Liste remplacée : N éléments retirés ») et les champs protégés (« [masqué] » avec avertissement). La saisie du mot CONFIRMER est exigée pour : les actions sensibles (paiements, envois, signature, droits d'accès et comptes, clôtures/verrouillages, fins de contrat, annulations, cessions, archivages, publication, abonnement), une requête non vide (paramètres de requête), une liste remplacée, plus de 30 changements, et un corps touchant rôles, permissions, statut, mot de passe ou e-mail d'un utilisateur. Pour une écriture sur un utilisateur (route `users/:id`), le serveur ajoute l'avertissement « Cette action modifie l'accès de &lt;nom&gt; » ; le libellé de la personne visée est lu dans la réponse (prénom + nom, sinon e-mail) Pour une création imbriquée, si le serveur ne peut pas lire la ressource parente visée (aucune route de lecture du parent dans le catalogue, ou lecture refusée/introuvable), le plan est refusé (« Impossible de vérifier la ressource parente visée ») et aucun jeton n'est émis. Valide à sec le corps proposé contre le schéma de la route pour 11 routes (biens POST/PUT, CRM contacts, deals, activités, conversion et rôles, baux POST/PATCH) : un corps incomplet ou invalide est refusé AVANT l'affichage de la carte, et le modèle reçoit les champs fautifs (chemin, absent ou invalide, valeurs permises) pour les demander à l'utilisateur. Pour les autres routes, le plan porte l'avertissement « Cette route n'a pas pu être vérifiée à l'avance ».</t>
         </is>
       </c>
       <c r="G889" t="inlineStr">
@@ -69167,7 +69167,7 @@
       </c>
       <c r="F890" t="inlineStr">
         <is>
-          <t>Après clic sur « Approuver et exécuter » (et saisie de CONFIRMER si requis), le serveur vérifie la signature du jeton, son expiration, son usage unique, l'utilisateur et l'agence, puis exécute la route réelle par une requête loopback sous l'identité de la personne qui confirme : la permission et l'abonnement de la route réelle s'appliquent donc. Délai 30 s. Audit sans corps de requête ni secret. Réponse avec `resultPreview` masqué. 10 confirmations par minute. Rejeu d'un jeton : PROPOSAL_ALREADY_USED ; confirmation absente ou inexacte : CONFIRMATION_REQUIRED sans consommer le jeton. Aucune suppression possible. Module d'abonnement CORE : l'entrée `/ai/actions` ne dépend plus du module RENTAL (la génération de quittance vérifie toujours RENTAL). Une confirmation sans le mot exigé répond CONFIRMATION_REQUIRED (400) : la carte reste en attente et le jeton n'est pas consommé. L'aperçu du résultat (`resultPreview`) masque les secrets et retire les chemins disque</t>
+          <t>Après clic sur « Approuver et exécuter » (et saisie de CONFIRMER si requis), le serveur vérifie la signature du jeton, son expiration, son usage unique, l'utilisateur et l'agence, puis exécute la route réelle par une requête loopback sous l'identité de la personne qui confirme : la permission et l'abonnement de la route réelle s'appliquent donc. Délai 30 s. Audit sans corps de requête ni secret. Réponse avec `resultPreview` masqué. 10 confirmations par minute. Rejeu d'un jeton : PROPOSAL_ALREADY_USED ; confirmation absente ou inexacte : CONFIRMATION_REQUIRED sans consommer le jeton. Aucune suppression possible. Module d'abonnement CORE : l'entrée `/ai/actions` ne dépend plus du module RENTAL (la génération de quittance vérifie toujours RENTAL). Une confirmation sans le mot exigé répond CONFIRMATION_REQUIRED (400) : la carte reste en attente et le jeton n'est pas consommé. L'aperçu du résultat (`resultPreview`) masque les secrets et retire les chemins disque Si la route refuse malgré tout (400 de validation), la carte d'échec liste les champs en erreur avec leur libellé traduit (`fieldErrors` : 10 au plus, jamais la valeur saisie ni les champs secrets).</t>
         </is>
       </c>
       <c r="G890" t="inlineStr">

</xml_diff>